<commit_message>
Rewrite CEO report in simple English
https://claude.ai/code/session_01QKsUumyB8kabj8MBZhL9cY
</commit_message>
<xml_diff>
--- a/docs/CEO_Report_Staybooker_Jun2026.xlsx
+++ b/docs/CEO_Report_Staybooker_Jun2026.xlsx
@@ -510,7 +510,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Kya solve hua, kya chal raha hai, future me kya risk hai, aur team kyu chahiye — ek nazar me</t>
+          <t>What has been solved, what is in progress, what risks are coming, and why we need a team — at a glance</t>
         </is>
       </c>
     </row>
@@ -542,7 +542,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>33 issues fix kiye gaye (5 Critical, 13 High). Har issue ke saath likha hai: agar production me chala jaata to business pe kya impact hota.</t>
+          <t>33 issues fixed so far (5 Critical, 13 High). Each issue shows what would have happened to the business if it had reached production.</t>
         </is>
       </c>
     </row>
@@ -554,11 +554,11 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Jo critical cheezein abhi chal rahi hain.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="30" customHeight="1">
+          <t>Critical items currently being worked on.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="40" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Sheet 4 — Future Risks</t>
@@ -566,7 +566,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>13 real-world scenarios jo aage aa sakte hain (100 users ek saath, payment failure, DDoS, data GBs me) — kya protection already hai, kya banana baki hai.</t>
+          <t>13 real-world scenarios that WILL come as the business grows (100 users at once, payment failures, DDoS attacks, data growing to GBs) — what protection already exists and what still needs to be built.</t>
         </is>
       </c>
     </row>
@@ -578,7 +578,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Tech Lead / Backend / Frontend / Database developer ka actual kaam simple language me — aur kyu 'frontend = sirf UI' galat soch hai.</t>
+          <t>What a Tech Lead / Backend / Frontend / Database developer actually does, in simple language — and why 'frontend = only UI' is an incomplete view.</t>
         </is>
       </c>
     </row>
@@ -614,7 +614,7 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>5 — payment secret leak, payment amount tampering, permanent admin token, AI crash, staff privilege escalation</t>
+          <t>5 — payment secret key leak, payment amount tampering, permanent admin token, AI assistant crash, staff privilege escalation</t>
         </is>
       </c>
     </row>
@@ -626,11 +626,11 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>130+ test cases (security, payments, booking, role-access) — ye tests har code change pe khud chalte hain (CI/CD)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="32" customHeight="1">
+          <t>130+ test cases (security, payments, booking, role access). These tests run automatically on every code change (CI/CD pipeline).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="38" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
           <t>Money saved (examples)</t>
@@ -638,7 +638,7 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Payment tampering fix: guest Rs.1 dekar Rs.10,000 ki booking confirm kar sakta tha. AI cost fix: ek bug se 10x mehenga AI model chal raha tha public chatbot pe.</t>
+          <t>Payment tampering fix: a guest could pay Rs.1 and get a Rs.10,000 booking confirmed. AI cost fix: a bug was sending traffic to an AI model 10x more expensive than needed on the public chatbot.</t>
         </is>
       </c>
     </row>
@@ -649,12 +649,12 @@
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>ONE-LINE MESSAGE FOR CEO</t>
+          <t>ONE-LINE MESSAGE FOR THE CEO</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr"/>
     </row>
-    <row r="18" ht="46" customHeight="1">
+    <row r="18" ht="50" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
         <is>
           <t>Bottom line</t>
@@ -662,7 +662,7 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Jo bugs mile wo fix ho gaye. Ab problem ye hai ki naye bugs HUMSE PEHLE hacker ya competitor na dhundhe. Iske liye dedicated Backend, Frontend aur Database developers chahiye — sirf design ke liye nahi, paisa aur data bachane ke liye.</t>
+          <t>The bugs we found have been fixed. The real problem now is making sure NEW bugs are found by us before a hacker or competitor finds them. That requires dedicated Backend, Frontend and Database developers — not for design, but to protect money and data.</t>
         </is>
       </c>
     </row>
@@ -703,7 +703,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Source: work_log_tracker.csv + Security Audit Report. 'Agar production me jaata to' column = wo nuksan jo is fix ne roka.</t>
+          <t>Source: work_log_tracker.csv + Security Audit Report. The 'If this had reached production' column shows the damage each fix prevented.</t>
         </is>
       </c>
     </row>
@@ -720,17 +720,17 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Technically Kya Ho Raha Tha</t>
+          <t>What Was Happening Technically</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Agar Production Me Jaata To... (Business Impact)</t>
+          <t>If This Had Reached Production... (Business Impact)</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Kaise Fix Kiya</t>
+          <t>How It Was Fixed</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -752,22 +752,22 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Hotel ki payment secret key (Razorpay) public website pe leak ho rahi thi</t>
+          <t>The hotel's secret payment key (Razorpay) was visible on the public website</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Anonymous guest GET /public/hotels/slug API se hotel ki razorpay_key_secret padh sakta tha</t>
+          <t>Any anonymous visitor could read the hotel's razorpay_key_secret through the public hotel API</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Hacker hotel ke payment account se refunds nikal sakta tha, fake payments verify kar sakta tha. Hotel ka paisa + hamari company pe legal case. Razorpay account ban ho sakta tha.</t>
+          <t>A hacker could issue refunds from the hotel's payment account and fake payment verifications. Hotel loses money, we face legal action, and the Razorpay account could be banned.</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Secrets ab AES-256 encrypted Supabase Vault me. Public API pe masking. Secret kabhi client tak nahi jaata.</t>
+          <t>All secrets are now AES-256 encrypted in Supabase Vault. Public APIs mask them. The secret never reaches the browser.</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
@@ -781,7 +781,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="30" customHeight="1">
+    <row r="6" ht="35" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>S-02</t>
@@ -789,22 +789,22 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Guest apni marzi ka amount bhej kar booking 'paid' karwa sakta tha</t>
+          <t>A guest could send any amount they wanted and get the booking marked as 'paid'</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Payment order-create API client se amount le rahi thi, server verify nahi karta tha</t>
+          <t>The payment order API trusted the amount sent by the browser; the server never verified it</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Guest Rs.1 pay karke Rs.10,000 ki booking CONFIRMED karwa leta. Hotel ko room dena padta, paisa nahi milta. Direct revenue loss + hotel ka trust khatam.</t>
+          <t>A guest could pay Rs.1 and get a Rs.10,000 booking CONFIRMED. The hotel would have to honour the room without receiving the money. Direct revenue loss and loss of hotel trust.</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Amount ab hamesha server par booking.total_amount se compute hota hai. Client ka bheja amount ignore.</t>
+          <t>The amount is now always calculated on the server from the booking total. Whatever the client sends is ignored.</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
@@ -818,7 +818,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="32" customHeight="1">
+    <row r="7" ht="30" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>S-03</t>
@@ -826,22 +826,22 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Admin 'impersonation' token kabhi expire nahi hota tha</t>
+          <t>The admin 'impersonation' login token never expired</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Super-admin jab kisi hotel me login karta tha, wo token permanent tha (no expiry)</t>
+          <t>When a super-admin logged into a hotel's account, that token was permanent (no expiry)</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Wo token ek baar leak ho jaata (email, log, laptop chori) to hacker HAMESHA ke liye us hotel ka owner ban jaata — bookings, payments, guest data sab uske haath me.</t>
+          <t>If that token ever leaked (email, log file, stolen laptop), a hacker would own that hotel FOREVER — bookings, payments, guest data, everything.</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Token ab 15-30 min me expire hota hai; verifier expiry ke bina token reject karta hai.</t>
+          <t>Tokens now expire in 15-30 minutes; the verifier rejects any token without an expiry.</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
@@ -863,22 +863,22 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>AI Assistant pura crash ho raha tha (Critical bug)</t>
+          <t>The AI Assistant was completely crashing (critical bug)</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Code me logger define nahi tha — smart tool selector chalte hi NameError se crash</t>
+          <t>A logger was not defined in the code — the smart tool selector crashed with an error every time</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Hotelier jab bhi AI assistant kholta, error aata. Premium feature jo hum bechte hain wo dead tha — paying customer churn.</t>
+          <t>Every time a hotelier opened the AI assistant, they got an error. A premium feature we charge for was dead — paying customers would churn.</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Logger fix + regression test add kiya taaki dobara na ho.</t>
+          <t>Fixed the logger and added a regression test so it cannot happen again.</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
@@ -892,7 +892,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="30" customHeight="1">
+    <row r="9" ht="31" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
           <t>S-05</t>
@@ -900,22 +900,22 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Hotel ka STAFF (receptionist) API se OWNER jaisa sab kuch kar sakta tha</t>
+          <t>Hotel STAFF (e.g. a receptionist) could do everything an OWNER can via the API</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Role check sirf frontend menu me tha, backend API pe nahi</t>
+          <t>Role checks existed only in the frontend menu, not on the backend API</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Naraz employee rates badal deta, rooms delete kar deta, settings me payment keys badal deta. Hotel ka pura business ek junior ke haath me.</t>
+          <t>A disgruntled employee could change rates, delete rooms, or change payment keys in settings. The hotel's entire business in the hands of a junior employee.</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Backend pe require_hotel_role (OWNER/MANAGER) gates + 76 role-access test cases.</t>
+          <t>Backend role gates (OWNER/MANAGER required) added, plus 76 role-access test cases.</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
@@ -929,7 +929,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="30" customHeight="1">
+    <row r="10" ht="32" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
           <t>S-06</t>
@@ -937,22 +937,22 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Hotel A, Hotel B ka private promo code use kar sakta tha (IDOR)</t>
+          <t>Hotel A could use Hotel B's private promo codes</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Promo validate API me chain/hotel ka match check nahi tha</t>
+          <t>The promo validation API did not check which hotel/chain the code belonged to</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Competitor hotel ke discount codes chura kar use karta. Revenue leak + hotels ka platform se bharosa khatam (multi-tenant SaaS ki sabse badi failure).</t>
+          <t>A competitor hotel's discount codes could be stolen and used. Revenue leakage and total loss of trust in the platform (the worst failure for a multi-tenant SaaS).</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Promo lookup ab strictly same chain_id/hotel ke andar hi hota hai.</t>
+          <t>Promo lookup is now strictly limited to the requesting hotel's own chain.</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
@@ -974,22 +974,22 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Database level pe tenant isolation nahi tha</t>
+          <t>There was no tenant isolation at the database level</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Sab kuch sirf application code pe depend tha; DB me Row Level Security (RLS) nahi thi</t>
+          <t>Everything depended only on application code; the database had no Row Level Security (RLS)</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Ek bhi code bug = Hotel A ko Hotel B ke guests/bookings dikh jaate. GDPR/DPDP data breach, customer loss.</t>
+          <t>A single code bug would let Hotel A see Hotel B's guests and bookings. Data breach, GDPR/DPDP penalties, customer loss.</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Har tenant table pe Postgres RLS policies — DB khud dusre hotel ka data dena refuse karta hai (double lock).</t>
+          <t>Postgres RLS policies on every tenant table — the database itself refuses to return another hotel's data (a second lock).</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr">
@@ -1011,22 +1011,22 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Saare hotel secrets (WhatsApp, SMTP, AI keys) database me plain text the</t>
+          <t>All hotel secrets (WhatsApp, email, AI keys) were stored as plain text in the database</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>DB dump ya backup leak hone par sab keys readable thi</t>
+          <t>If the database or a backup ever leaked, all keys were readable</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Ek DB leak = saare hotels ke WhatsApp, email, payment accounts compromise. Mass-scale breach, business khatam ho sakta tha.</t>
+          <t>One database leak = every hotel's WhatsApp, email and payment accounts compromised. A mass-scale breach that could end the business.</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Sab secrets Supabase Vault me AES-256-GCM encrypted; logs/DB me kabhi plaintext nahi.</t>
+          <t>All secrets are AES-256-GCM encrypted in Supabase Vault; never stored or logged as plain text.</t>
         </is>
       </c>
       <c r="F12" s="6" t="inlineStr">
@@ -1048,22 +1048,22 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Public AI chatbot error hone par 10x mehenga model use kar raha tha</t>
+          <t>The public AI chatbot used a 10x more expensive model whenever an error occurred</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Error-fallback cheap 8B model ki jagah 70B model pe ja raha tha</t>
+          <t>The error-fallback path switched to a large 70B model instead of the cheap 8B model</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Koi bhi anonymous user error-storm karwa ke hamara AI bill lakhon me pahuncha sakta tha (cost attack).</t>
+          <t>Any anonymous user could trigger an error storm and push our AI bill into lakhs (a cost attack).</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Fallback ab cheap model pe locked; per-hotel daily AI quota bhi hai.</t>
+          <t>The fallback is now locked to the cheap model; a per-hotel daily AI quota is also in place.</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
@@ -1085,22 +1085,22 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Error messages me internal system detail leak ho rahi thi</t>
+          <t>Error messages were leaking internal system details</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>AI endpoint crash hone par raw exception text (file paths, library names) client ko jaata tha</t>
+          <t>When the AI endpoint crashed, the raw error text (file paths, library names) was sent to the user</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Hacker ko system ka naksha mil jaata — kaunsi library, kaunsa version — attack plan karna easy.</t>
+          <t>A hacker would get a map of our system — which libraries, which versions — making an attack much easier to plan.</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>Generic error messages client ko; detail sirf server logs me.</t>
+          <t>Users now see generic error messages; details go only to server logs.</t>
         </is>
       </c>
       <c r="F14" s="6" t="inlineStr">
@@ -1122,22 +1122,22 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Guest ka email/ID production logs me print ho raha tha (PII leak)</t>
+          <t>Guest emails/IDs were being printed in production logs (PII leak)</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Auth flow INFO level pe email + supabase_id log kar raha tha</t>
+          <t>The login flow logged email + user ID at INFO level</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Logs to third-party services me jaate hain — PII wahan leak = privacy violation, DPDP fine.</t>
+          <t>Logs go to third-party services — personal data leaking there is a privacy violation and a DPDP fine risk.</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>PII logs DEBUG pe move; prod me sirf WARNING level chalta hai.</t>
+          <t>PII logging moved to DEBUG level; production runs at WARNING level only.</t>
         </is>
       </c>
       <c r="F15" s="6" t="inlineStr">
@@ -1159,22 +1159,22 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Booking ke baad ke emails/sync chupchaap fail ho rahe the</t>
+          <t>Post-booking emails and channel sync were silently failing</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Background task helper galat tarike se coroutine call kar raha tha — kaam silently skip</t>
+          <t>The background task helper was calling tasks the wrong way — work was silently skipped</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Guest ko confirmation email nahi jaata, channel sync nahi hota → double booking on OTA, guest pareshan, calls badhte.</t>
+          <t>Guests would not receive confirmation emails and channel sync would not run → double bookings on OTAs, upset guests, more support calls.</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>safe_background fix — ab factory pattern se task reliably chalta hai + errors visible.</t>
+          <t>Fixed the background task pattern — tasks now run reliably and errors are visible.</t>
         </is>
       </c>
       <c r="F16" s="6" t="inlineStr">
@@ -1196,22 +1196,22 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Guest list API bina limit ke pura data laa rahi thi</t>
+          <t>The guest list API loaded ALL data with no limit</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>GET /guests unbounded tha — 1 lakh guests = server crash</t>
+          <t>GET /guests was unbounded — 100,000 guests would crash the server</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Bada hotel kholte hi page hang/server out-of-memory. Peak season me system down = direct booking loss.</t>
+          <t>Opening the page for a large hotel would hang the page or crash the server with out-of-memory. In peak season, system down = direct booking loss.</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>Pagination (limit + offset) mandatory; hot columns pe DB indexes.</t>
+          <t>Pagination (limit + offset) is now mandatory; database indexes added on hot columns.</t>
         </is>
       </c>
       <c r="F17" s="6" t="inlineStr">
@@ -1233,22 +1233,22 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Browser autofill chupke se asli API keys overwrite kar raha tha</t>
+          <t>Browser autofill was silently overwriting real API keys</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Admin integrations form me browser saved passwords inject kar deta tha</t>
+          <t>In the admin integrations form, the browser injected saved passwords into the key fields</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Save dabate hi hotel ki sahi payment/WhatsApp keys kharab ho jaati — payments fail, 'site down' complaints.</t>
+          <t>The moment an admin clicked Save, the hotel's correct payment/WhatsApp keys were corrupted — payments fail, 'site is down' complaints.</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>Anti-autofill pattern: fields locked by default, explicit click pe hi editable.</t>
+          <t>Anti-autofill pattern: fields are locked by default and only become editable on an explicit click.</t>
         </is>
       </c>
       <c r="F18" s="6" t="inlineStr">
@@ -1270,22 +1270,22 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Rate Shopper galat 'SOLD OUT' dikha raha tha</t>
+          <t>The Rate Shopper was showing false 'SOLD OUT' statuses</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Competitor ka price element na milne par full-page fallback galat data utha leta</t>
+          <t>When a competitor's price element was not found, a full-page fallback picked up wrong data</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>Hotelier galat market data pe pricing decision leta — kamre saste/mehenge bech deta. Product pe bharosa khatam.</t>
+          <t>Hoteliers would make pricing decisions on wrong market data — selling rooms too cheap or too expensive. Trust in the product destroyed.</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>Scoping logic fix; data na mile to dash dikhate hain, galat status nahi.</t>
+          <t>Fixed the scoping logic; when data is missing we show a dash, never a wrong status.</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr">
@@ -1307,22 +1307,22 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Rate Shopper usage billing me ginti galat thi</t>
+          <t>Rate Shopper usage billing was undercounting</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Timeout/error hone par usage record skip ho jaata tha</t>
+          <t>When a request timed out or errored, the usage record was skipped</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>Hum vendor (proxy) ko har attempt ka paisa dete hain par customer se count nahi hota — silent margin loss.</t>
+          <t>We pay the data vendor for every attempt, but were not counting it on our side — a silent margin loss.</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>Har attempt ab billed/recorded, outcome chahe jo ho.</t>
+          <t>Every attempt is now recorded and billable, regardless of outcome.</t>
         </is>
       </c>
       <c r="F20" s="6" t="inlineStr">
@@ -1344,22 +1344,22 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Loyalty program settings STAFF bhi badal sakta tha</t>
+          <t>Loyalty program settings could be changed by STAFF</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>PUT /loyalty/program pe role gate nahi tha</t>
+          <t>The loyalty program update endpoint had no role check</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>Receptionist points-to-rupee ratio badal kar khud ke email pe points farm kar sakta tha — fraud.</t>
+          <t>A receptionist could change the points-to-rupee ratio and farm points into their own email — fraud.</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>OWNER/MANAGER role required; checkout task bhi safe-wrapped.</t>
+          <t>OWNER/MANAGER role now required; the checkout task is also safely wrapped.</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr">
@@ -1381,22 +1381,22 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Loyalty points race condition se double-credit ho sakte the</t>
+          <t>Loyalty points could be credited twice due to a race condition</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Check-out pe points credit bina lock ke tha</t>
+          <t>Points were credited at check-out without a lock</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>Ek guest ke points 2x credit → loyalty liability badhti, financial reports galat.</t>
+          <t>A guest's points credited twice → loyalty liability grows, financial reports become wrong.</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>Redis advisory locks + DB transaction me atomic point deduction.</t>
+          <t>Redis locks added; point deduction now happens atomically inside a database transaction.</t>
         </is>
       </c>
       <c r="F22" s="6" t="inlineStr">
@@ -1418,22 +1418,22 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Real-time updates ke liye WebSocket bina auth ke ban sakta tha</t>
+          <t>Real-time WebSocket connections could be opened without authentication</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Naya WS channel JWT verify ke bina connect ho sakta tha (design phase me pakda)</t>
+          <t>The new live-updates channel could be connected without verifying the login token (caught during design)</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>Koi bhi hotel ke live booking events sun leta — guest data leak.</t>
+          <t>Anyone could listen to a hotel's live booking events — guest data leak.</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>JWT verify hone ke baad hi WS connection accept hota hai.</t>
+          <t>The connection is accepted only after the login token (JWT) is verified.</t>
         </is>
       </c>
       <c r="F23" s="6" t="inlineStr">
@@ -1455,22 +1455,22 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Ek slow web-search pure AI server ko block kar deta tha</t>
+          <t>One slow web search could block the entire AI server</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>AI assistant ka search synchronous tha — ek slow call = sab requests atki</t>
+          <t>The AI assistant's web search ran synchronously — one slow call froze all other requests</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>Ek user ki slow query se sab hoteliers ka AI hang. 'System slow hai' complaints.</t>
+          <t>One user's slow query would hang the AI for every hotelier. 'The system is slow' complaints.</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>Search ab background thread me 8-second hard timeout ke saath.</t>
+          <t>Search now runs in a background thread with a hard 8-second timeout.</t>
         </is>
       </c>
       <c r="F24" s="7" t="inlineStr">
@@ -1492,22 +1492,22 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Cancel hui booking pe bhi availability cache purana dikhta tha</t>
+          <t>After a cancellation, the availability cache still showed old data</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Booking/cancel ke baad rate cache invalidate nahi hota tha</t>
+          <t>The rate cache was not cleared after a booking or cancellation</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>Guest ko bika hua room 'available' dikhta → book karta → hotel ko manually cancel karna padta. Bad reviews.</t>
+          <t>A guest would see a sold room as 'available', book it, and the hotel would have to cancel manually. Bad reviews.</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>Har booking/cancel commit pe rate_version bump + cache clear.</t>
+          <t>Cache is now cleared and a version counter is bumped after every booking/cancellation.</t>
         </is>
       </c>
       <c r="F25" s="7" t="inlineStr">
@@ -1529,22 +1529,22 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Heavy libraries har request pe load ho rahi thi</t>
+          <t>Heavy libraries were loading on every server start</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Email/PDF libraries module-top pe import — server start slow, memory zyada</t>
+          <t>Email/PDF libraries were imported at the top of always-loaded files — slow startup, more memory</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>Server boot slow = deploy ke time downtime zyada; RAM cost zyada.</t>
+          <t>Slow server boot = longer downtime during every deploy; higher RAM costs.</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>Lazy imports — sirf zarurat padne par load hoti hain.</t>
+          <t>Lazy imports — libraries load only when actually needed.</t>
         </is>
       </c>
       <c r="F26" s="7" t="inlineStr">
@@ -1566,22 +1566,22 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>962-line analytics file maintain karna impossible tha</t>
+          <t>A 962-line analytics file was impossible to maintain</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Ek hi file me sab analytics — har change risky, review mushkil</t>
+          <t>All analytics lived in one giant file — every change was risky and hard to review</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>Har naya feature purane features tod sakta tha; developer onboarding slow.</t>
+          <t>Every new feature risked breaking old ones; new developer onboarding would be slow.</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>4 clean modules me split; availability + competitors bhi packages me split.</t>
+          <t>Split into 4 clean modules; availability and competitors modules also split into packages.</t>
         </is>
       </c>
       <c r="F27" s="7" t="inlineStr">
@@ -1603,22 +1603,22 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Code changes bina test ke merge ho sakte the</t>
+          <t>Code changes could be merged without running tests</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>CI/CD sirf main branch pe tha; PRs pe tests nahi chalte the</t>
+          <t>CI/CD ran only on the main branch; pull requests were not tested</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>Broken code production me jaata — har deploy ek jua (gamble).</t>
+          <t>Broken code could reach production — every deploy was a gamble.</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>Backend + frontend CI ab har PR pe chalta hai + compile gate.</t>
+          <t>Backend + frontend CI now runs on every pull request, plus a compile gate.</t>
         </is>
       </c>
       <c r="F28" s="7" t="inlineStr">
@@ -1640,22 +1640,22 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Rate Shopper scraping aadhe time fail ho rahi thi</t>
+          <t>Rate Shopper scraping was failing half the time</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Vendor API payload galat tha; concurrent burst se blocks; retry logic nahi</t>
+          <t>The vendor API payload was wrong; concurrent bursts caused blocks; there was no retry logic</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>Jo feature hum premium me bechte hain wo unreliable — customers cancel karte.</t>
+          <t>A feature we sell as premium was unreliable — customers would cancel.</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>Sequential scraping + retry/backoff + session rotation + correct payload. ~7min se ~4min.</t>
+          <t>Sequential scraping + retry/backoff + session rotation + corrected payload. Runtime cut from ~7 min to ~4 min.</t>
         </is>
       </c>
       <c r="F29" s="7" t="inlineStr">
@@ -1677,22 +1677,22 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>Hotelier ko pata nahi chalta tha scrape chal raha hai ya atka hai</t>
+          <t>Hoteliers could not tell whether a scrape was running or stuck</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Pura 7-day scrape khatam hone tak UI me kuch update nahi hota tha</t>
+          <t>Nothing updated in the UI until the full 7-day scrape finished</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>User ko laga feature kaam nahi karta; support tickets.</t>
+          <t>Users assumed the feature was broken; support tickets piled up.</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>Live per-day progress — har din ka data aate hi chart update hota hai.</t>
+          <t>Live per-day progress — the chart updates as each day's data arrives.</t>
         </is>
       </c>
       <c r="F30" s="7" t="inlineStr">
@@ -1714,22 +1714,22 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>Chain (multi-hotel brand) me ek brand ke loyalty points dusre brand me mix ho sakte the</t>
+          <t>In multi-hotel chains, one brand's loyalty points could mix with another brand's</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Loyalty schema me chain isolation nahi tha</t>
+          <t>The loyalty schema had no chain-level isolation</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>Brand A ke points Brand B me redeem — financial mess across clients.</t>
+          <t>Brand A's points redeemed at Brand B — a financial mess across clients.</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>chain_id isolation + composite unique index (guest_email, chain_id).</t>
+          <t>Chain-level isolation added, with a unique index per (guest email, chain).</t>
         </is>
       </c>
       <c r="F31" s="7" t="inlineStr">
@@ -1751,22 +1751,22 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>Checkout pe loyalty discount client-side calculate ho raha tha</t>
+          <t>The loyalty discount at checkout was calculated in the browser</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Points redemption ka max discount frontend pe tha</t>
+          <t>The maximum redeemable discount was enforced on the frontend only</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>Guest browser me value badal kar 100% discount le leta.</t>
+          <t>A guest could edit the value in the browser and take a 100% discount.</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>Max redeemable discount server-side bound; balance DB lock ke andar.</t>
+          <t>The maximum discount is now enforced on the server; the points balance is locked in the database.</t>
         </is>
       </c>
       <c r="F32" s="6" t="inlineStr">
@@ -1788,22 +1788,22 @@
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>Concierge AI chat dusre chain ke hotels ka data access kar sakta tha</t>
+          <t>The concierge AI chat could access data from other hotel chains</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Chat session me chain scope validation nahi thi</t>
+          <t>The chat session had no chain-scope validation</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>Guest chatbot se dusre brand ke hotels ki info nikal leta.</t>
+          <t>A guest could extract another brand's hotel information through the chatbot.</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>Chain_id validation chat router me; AI tools sirf apne hotel ka data dekhte hain.</t>
+          <t>Chain validation added in the chat router; AI tools only see the verified hotel's data.</t>
         </is>
       </c>
       <c r="F33" s="6" t="inlineStr">
@@ -1825,22 +1825,22 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>RLS migration galat schema me functions bana rahi thi</t>
+          <t>The database security migration was targeting the wrong schema</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>Custom functions Supabase-managed 'auth' schema me the — migration fail hoti</t>
+          <t>Custom functions were placed in the Supabase-managed 'auth' schema — the migration would fail</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>Security layer deploy hi nahi ho paata — sab RLS protection kagaz pe reh jaati.</t>
+          <t>The security layer would never actually deploy — all the RLS protection would exist only on paper.</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>Functions public schema me move; re-run safe guards; proper grants.</t>
+          <t>Functions moved to the public schema; safe re-run guards and proper permissions added.</t>
         </is>
       </c>
       <c r="F34" s="6" t="inlineStr">
@@ -1862,22 +1862,22 @@
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>Rate Shopper ka scrape stop nahi ho sakta tha</t>
+          <t>A Rate Shopper scrape could not be stopped once started</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>Galti se chala scrape pura paisa kha ke hi rukta tha</t>
+          <t>A scrape started by mistake would burn the full vendor cost before finishing</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>Har accidental run = vendor cost. Hotelier control nahi kar paata.</t>
+          <t>Every accidental run = vendor cost. The hotelier had no control.</t>
         </is>
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>Stop button + Redis cancel flag; sirf attempted days ka bill.</t>
+          <t>Stop button added with a cancel flag; only the days actually attempted are billed.</t>
         </is>
       </c>
       <c r="F35" s="7" t="inlineStr">
@@ -1899,22 +1899,22 @@
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>Vendor ka naam (Decodo) hotelier ko dikh raha tha</t>
+          <t>The data vendor's name (Decodo) was visible to hoteliers</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>Errors/UI me internal vendor expose tha</t>
+          <t>Internal vendor details were exposed in errors and the UI</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>Hotelier direct vendor ke paas ja sakta tha; white-label image kharab.</t>
+          <t>Hoteliers could go directly to the vendor; damages our white-label image.</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>Staybooker OTA Analytics rebrand; vendor name sab user-facing jagah se removed.</t>
+          <t>Rebranded as Staybooker OTA Analytics; vendor name removed from everything user-facing.</t>
         </is>
       </c>
       <c r="F36" s="7" t="inlineStr">
@@ -1936,22 +1936,22 @@
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>AI usage track nahi ho raha tha kuch paths pe</t>
+          <t>AI usage was not being tracked on some code paths</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>Kuch agent runs ka token usage record miss tha</t>
+          <t>Some AI agent runs did not record their token usage</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>AI cost per hotel ka hisaab galat — pricing decisions blind.</t>
+          <t>Our per-hotel AI cost accounting was wrong — pricing decisions were blind.</t>
         </is>
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>record_ai_usage har run ke baad; quotas isi data pe chalti hain.</t>
+          <t>Usage is now recorded after every run; quotas are driven by this data.</t>
         </is>
       </c>
       <c r="F37" s="7" t="inlineStr">
@@ -1993,14 +1993,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Abhi Kya Chal Raha Hai (In Progress)</t>
+          <t>What Is Being Worked On Right Now</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Critical cheezein jin par kaam jaari hai — ye akela aadmi parallel me nahi kar sakta, isliye team chahiye</t>
+          <t>Critical items in progress — one person cannot do these in parallel, which is why a team is needed</t>
         </is>
       </c>
     </row>
@@ -2012,12 +2012,12 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Kaam</t>
+          <t>Task</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Kyu Zaroori Hai</t>
+          <t>Why It Matters</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -2027,11 +2027,11 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Risk Agar Delay Hua</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="38" customHeight="1">
+          <t>Risk If Delayed</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="47" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>P-01</t>
@@ -2039,12 +2039,12 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Razorpay payment failure recovery (paisa kata par booking nahi bani)</t>
+          <t>Razorpay payment failure recovery (money deducted but booking not created)</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Guest ka network beech me gaya / Razorpay API fail — paisa kat gaya, booking cancel. Abhi idempotency + webhook verification implement hai, par auto-refund + reconciliation job banana baaki hai.</t>
+          <t>Guest's network dropped mid-payment / Razorpay API failed — money was deducted but the booking got cancelled. Idempotency and webhook verification are already implemented; the auto-refund flow and reconciliation job still need to be built.</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -2054,11 +2054,11 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Guest ka paisa atka rahega, manual refund karna padega. Angry guests, chargebacks, Razorpay disputes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="30" customHeight="1">
+          <t>Guests' money stays stuck and refunds must be done manually. Angry guests, chargebacks, Razorpay disputes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="32" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>P-02</t>
@@ -2066,12 +2066,12 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Load testing — 100+ users ek saath booking karein to kya hota hai</t>
+          <t>Load testing — what happens when 100+ users book at the same time</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Race conditions (ek room 2 logo ko bik jaana) ke against DB locks hain, par real load pe pool exhaustion / timeouts test karna baaki.</t>
+          <t>Database locks already protect against race conditions (one room sold twice), but real-load behaviour (connection pool exhaustion, timeouts) still needs testing.</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -2081,7 +2081,7 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Peak season ya viral campaign pe site down — sabse zyada revenue wale din pe loss.</t>
+          <t>The site goes down during peak season or a viral campaign — losses on exactly the highest-revenue days.</t>
         </is>
       </c>
     </row>
@@ -2093,12 +2093,12 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Frontend page-wise error audit (har page ke errors + edge cases)</t>
+          <t>Frontend page-by-page error audit (errors + edge cases on every page)</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Har page pe network-failure, double-click, slow-data scenarios handle karna.</t>
+          <t>Every page must handle network failures, double-clicks, and slow-data scenarios gracefully.</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -2108,7 +2108,7 @@
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Guests ke saamne white screens / stuck buttons = booking drop, brand damage.</t>
+          <t>White screens and stuck buttons in front of guests = dropped bookings and brand damage.</t>
         </is>
       </c>
     </row>
@@ -2125,7 +2125,7 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Rate limits Redis me hain par X-Forwarded-For spoof ho sakta hai; Cloudflare/WAF layer chahiye.</t>
+          <t>Rate limits exist in Redis, but the client IP header can be spoofed; a Cloudflare/WAF layer is needed.</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -2135,7 +2135,7 @@
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Competitor Rs.500 ke botnet se site down kar sakta hai.</t>
+          <t>A competitor could take the site down with a Rs.500 botnet.</t>
         </is>
       </c>
     </row>
@@ -2147,12 +2147,12 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Database migration discipline (Alembic in deploy)</t>
+          <t>Database migration discipline (Alembic in the deploy process)</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Abhi schema create_all se banta hai; performance indexes prod me missing ho sakte hain.</t>
+          <t>The schema is currently built by create_all at startup; performance indexes may be missing in production.</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -2162,7 +2162,7 @@
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Data badhne par queries slow → pura app slow.</t>
+          <t>As data grows, queries get slow → the whole app gets slow.</t>
         </is>
       </c>
     </row>
@@ -2204,7 +2204,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ye problems abhi nahi aayi hain, par business badhte hi AAYENGI. 'Abhi Protection' = jo maine already implement kiya hai.</t>
+          <t>These problems have not happened yet, but they WILL come as the business grows. 'Protection Already In Place' = what has already been implemented.</t>
         </is>
       </c>
     </row>
@@ -2221,22 +2221,22 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Kya Ho Sakta Hai</t>
+          <t>What Can Happen</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Kyu Hoga</t>
+          <t>Why It Will Happen</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Abhi Kya Protection Hai (Already Done)</t>
+          <t>Protection Already In Place</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Aur Kya Karna Hoga</t>
+          <t>What Still Needs To Be Built</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
@@ -2246,7 +2246,7 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>Kis Developer Ka Kaam</t>
+          <t>Which Developer Owns This</t>
         </is>
       </c>
     </row>
@@ -2258,27 +2258,27 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Ek saath 100 log 'Book Now' dabaate hain (festival sale / ad campaign)</t>
+          <t>100 people press 'Book Now' at the same time (festival sale / ad campaign)</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Same room 2-3 guests ko bik jaata hai (overbooking), ya server timeout — sab ko error</t>
+          <t>The same room gets sold to 2-3 guests (overbooking), or the server times out and everyone sees errors</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>DB connection pool limited hai; race condition window; ek hi row pe sab lock maangte hain</t>
+          <t>The database connection pool is limited; there is a race-condition window; everyone competes for a lock on the same inventory row</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Row-level DB locks (FOR UPDATE) on inventory; Redis idempotency; pagination</t>
+          <t>Row-level database locks on inventory; Redis idempotency; pagination everywhere</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Load testing, queueing system, connection pool tuning, auto-scaling rules</t>
+          <t>Load testing, a queueing system, connection pool tuning, auto-scaling rules</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
@@ -2300,27 +2300,27 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Guest ne card details daali, payment hua, par network cut gaya — Razorpay verify nahi hua, booking cancel ho gayi. Guest ne dobara pay kar diya = DOUBLE PAYMENT</t>
+          <t>A guest enters card details and pays, but the network cuts out — Razorpay verification fails and the booking is cancelled. The guest pays again = DOUBLE PAYMENT</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Guest ka 2x paisa kata; refund manually karna padta hai; chargeback + Razorpay dispute</t>
+          <t>The guest is charged twice; refunds must be processed manually; chargebacks and Razorpay disputes follow</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Payment 3 systems se hokar jaata hai (browser → Razorpay → hamara server) — koi bhi link toot sakta hai</t>
+          <t>A payment passes through 3 systems (browser → Razorpay → our server) — any link can break at any moment</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Idempotency keys (same order do baar process nahi hota); webhook HMAC verification; status guard (CONFIRMED booking dobara process nahi hoti)</t>
+          <t>Idempotency keys (the same order is never processed twice); webhook signature verification; status guard (a CONFIRMED booking is never re-processed)</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>Auto-refund flow, daily reconciliation job (Razorpay ledger vs hamari bookings ka milaan), 'payment pending' recovery screen for guest</t>
+          <t>An automatic refund flow, a daily reconciliation job (matching the Razorpay ledger against our bookings), and a 'payment pending' recovery screen for the guest</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
@@ -2342,27 +2342,27 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Hotel ka data GBs me pahunch jaata hai (2-3 saal ki bookings, analytics)</t>
+          <t>A hotel's data grows to several GBs (2-3 years of bookings and analytics)</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Dashboard 15-20 second me khulega; reports timeout; frontend browser hang (hazaron rows render)</t>
+          <t>The dashboard takes 15-20 seconds to open; reports time out; the browser freezes rendering thousands of rows</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Abhi queries chhote data pe fast hain; bade data pe index/partition strategy chahiye; frontend virtualization nahi hai</t>
+          <t>Current queries are fast on small data; large data needs an index/partition strategy; the frontend has no virtualization</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Pagination on all lists; Redis caching on heavy aggregations; key DB indexes</t>
+          <t>Pagination on all lists; Redis caching on heavy aggregations; key database indexes</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>Data archiving (purani bookings alag table), table partitioning, frontend virtual scrolling, pre-computed reports</t>
+          <t>Data archiving (old bookings moved to separate tables), table partitioning, virtual scrolling in the frontend, pre-computed reports</t>
         </is>
       </c>
       <c r="G7" s="6" t="inlineStr">
@@ -2384,27 +2384,27 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Competitor DDoS attack karta hai (booking engine par fake traffic)</t>
+          <t>A competitor launches a DDoS attack (fake traffic on the booking engine)</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Site down on peak day; asli guests book nahi kar paate; Railway ka bill explode</t>
+          <t>The site goes down on a peak day; real guests cannot book; the hosting bill explodes</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Public endpoints anonymous hain; IP rate-limit X-Forwarded-For spoof se bypass ho sakta hai</t>
+          <t>Public endpoints are anonymous; the IP rate limit can be bypassed by spoofing the forwarded-IP header</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Redis-backed rate limiting; per-hotel AI quotas; SSE lifetime caps</t>
+          <t>Redis-backed rate limiting; per-hotel AI quotas; limits on streaming connection lifetimes</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>Cloudflare/WAF layer, trusted-proxy IP fix, bot detection (CAPTCHA on abuse), infra alerts</t>
+          <t>A Cloudflare/WAF layer, trusted-proxy IP fix, bot detection (CAPTCHA on abuse), infrastructure alerts</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
@@ -2426,27 +2426,27 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Hacker naye endpoints me IDOR dhundhta hai (Hotel A se Hotel B ka data)</t>
+          <t>A hacker hunts for data-isolation bugs in new endpoints (Hotel A accessing Hotel B's data)</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Ek tenant-isolation bug = data breach = saare hotel customers ka bharosa khatam + DPDP penalty</t>
+          <t>One tenant-isolation bug = a data breach = every hotel customer loses trust in us + DPDP penalties</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Har naya feature = naya endpoint = naya risk; abhi review karne wala ek hi insaan hai</t>
+          <t>Every new feature = a new endpoint = a new risk; right now only one person reviews everything</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>RLS at DB level (double lock); 130+ security tests; audit-driven CLAUDE.md rules; cross-tenant attack tests</t>
+          <t>Row Level Security at the database level (a second lock); 130+ security tests; audit-driven engineering rules; cross-tenant attack tests</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>Regular penetration testing, security review process for every PR (Tech Lead), bug bounty later</t>
+          <t>Regular penetration testing, a security review on every code change (Tech Lead), a bug bounty program later</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
@@ -2468,27 +2468,27 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Guest slow 3G network pe booking kar raha hai, button 2 baar dabaata hai</t>
+          <t>A guest on a slow 3G network presses the button twice</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>2 bookings ban jaati hain, 2 baar paisa katne ki koshish</t>
+          <t>Two bookings get created, and two payment attempts are made</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Frontend pe submit-lock aur loading states har page pe consistent nahi hain</t>
+          <t>Submit-locks and loading states are not yet consistent on every frontend page</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Backend idempotency same payment do baar process nahi karta</t>
+          <t>Backend idempotency ensures the same payment is never processed twice</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>Har form pe double-submit guard, optimistic UI, retry logic with backoff, offline detection</t>
+          <t>Double-submit guards on every form, optimistic UI, retry logic with backoff, offline detection</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
@@ -2510,27 +2510,27 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Razorpay / Supabase / Redis me se koi service down ho jaati hai</t>
+          <t>Razorpay, Supabase or Redis goes down</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Poora booking flow fail; guest ko samajh nahi aata kya hua</t>
+          <t>The entire booking flow fails and the guest has no idea what happened</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Hum 3rd-party services pe depend hain — unka downtime hamara downtime hai</t>
+          <t>We depend on third-party services — their downtime is our downtime</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Redis failure booking flow ko nahi rokta (graceful fallback); missing payment keys = clear 503 message</t>
+          <t>A Redis failure does not block the booking flow (graceful fallback); missing payment keys show a clear maintenance message</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>Status page, circuit breakers, queue-and-retry for emails/sync, multi-region plan</t>
+          <t>A status page, circuit breakers, queue-and-retry for emails/sync, a multi-region plan</t>
         </is>
       </c>
       <c r="G11" s="6" t="inlineStr">
@@ -2552,27 +2552,27 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Public AI chatbot ko koi script se spam karta hai</t>
+          <t>Someone spams the public AI chatbot with a script</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>AI bill (Groq/Anthropic) lakhon me; legit hotels ka quota khatam</t>
+          <t>The AI bill runs into lakhs; legitimate hotels' quotas get exhausted</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Endpoint anonymous hai; LLM tokens = real paisa</t>
+          <t>The endpoint is anonymous, and LLM tokens cost real money</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Per-hotel daily quota; cheap model default; tool-call limits; response caching; usage tracking</t>
+          <t>Per-hotel daily quotas; cheap model by default; tool-call limits; response caching; usage tracking</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>Anomaly alerts (bill spike), CAPTCHA on abuse pattern, harder per-IP+fingerprint limits</t>
+          <t>Anomaly alerts (bill spikes), CAPTCHA on abuse patterns, stronger per-IP + fingerprint limits</t>
         </is>
       </c>
       <c r="G12" s="6" t="inlineStr">
@@ -2594,27 +2594,27 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>50-100 hotels onboard hote hain (sales success!)</t>
+          <t>50-100 hotels onboard (sales success!)</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>DB connections khatam (Supabase limit), sab tenants slow ek saath</t>
+          <t>Database connections run out (Supabase limit) and all tenants slow down at once</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Pool size x workers x replicas ka math abhi single-instance ke liye tuned hai</t>
+          <t>The pool-size × workers × replicas math is currently tuned for a single instance</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Env-driven pool sizing; per-worker pools documented (SCALE_TUNING.md)</t>
+          <t>Environment-driven pool sizing; per-worker pools documented (SCALE_TUNING.md)</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>Connection pooler (PgBouncer), horizontal scaling plan, per-tenant monitoring</t>
+          <t>A connection pooler (PgBouncer), a horizontal scaling plan, per-tenant monitoring</t>
         </is>
       </c>
       <c r="G13" s="6" t="inlineStr">
@@ -2636,27 +2636,27 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Hotelier galat CSV/photo upload karta hai (ya malicious file)</t>
+          <t>A hotelier uploads a wrong CSV/photo (or a malicious file)</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Server crash ya stored-malware serve hona</t>
+          <t>Server crash, or malware stored and served from our domain</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Upload surface hamesha attack vector hota hai</t>
+          <t>An upload feature is always an attack surface</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>Magic-byte validation, server-side content-type, size caps, random filenames</t>
+          <t>Magic-byte validation, server-side content-type detection, size caps, randomized filenames</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>Virus scanning, image processing isolation, CDN serving</t>
+          <t>Virus scanning, isolated image processing, serving files via CDN</t>
         </is>
       </c>
       <c r="G14" s="7" t="inlineStr">
@@ -2678,27 +2678,27 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Booking page Google se slow load hoti hai (3-4 sec)</t>
+          <t>The booking page loads slowly from Google (3-4 seconds)</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Guest bounce — research: 1 sec extra load = ~7% conversion drop. Direct revenue loss har din</t>
+          <t>Guests bounce — research shows every extra second of load time cuts conversion by ~7%. Direct revenue loss every single day</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Bundle size, images, render-blocking JS optimize nahi hue hain abhi</t>
+          <t>Bundle size, images and render-blocking scripts have not been optimized yet</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>Vite build optimization basic level pe hai</t>
+          <t>Vite build optimization at a basic level</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>Code splitting, image optimization, lazy loading, Core Web Vitals monitoring — YE FRONTEND DEV KA KAAM HAI, UI NAHI</t>
+          <t>Code splitting, image optimization, lazy loading, Core Web Vitals monitoring — THIS IS FRONTEND ENGINEERING, NOT UI DESIGN</t>
         </is>
       </c>
       <c r="G15" s="6" t="inlineStr">
@@ -2720,27 +2720,27 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Ek hi guest ka data 2 tabs me khula hai, dono me edit hota hai</t>
+          <t>The same record is open in 2 tabs and edited in both</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Last save jeet jaata hai — pehla edit silently kho jaata hai</t>
+          <t>The last save wins — the first edit is silently lost</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Optimistic concurrency control nahi hai</t>
+          <t>There is no optimistic concurrency control yet</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>Critical paths (inventory) pe DB locks hain</t>
+          <t>Critical paths (inventory) already use database locks</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>Version checks on edits, conflict warnings in UI</t>
+          <t>Version checks on edits, conflict warnings in the UI</t>
         </is>
       </c>
       <c r="G16" s="7" t="inlineStr">
@@ -2762,17 +2762,17 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Backup/restore kabhi test nahi hua, aur ek din DB corrupt ho jaata hai</t>
+          <t>Backups have never been restore-tested, and one day the database gets corrupted</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Saare hotels ka data loss = company-ending event</t>
+          <t>Losing every hotel's data = a company-ending event</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Supabase backups hain par restore drill kabhi nahi hua</t>
+          <t>Supabase keeps backups, but a restore drill has never been performed</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
@@ -2782,7 +2782,7 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>Quarterly restore drills, point-in-time recovery setup, disaster recovery runbook</t>
+          <t>Quarterly restore drills, point-in-time recovery setup, a disaster recovery runbook</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
@@ -2824,14 +2824,14 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Team Roles — Simple Language Me</t>
+          <t>Team Roles — In Simple Language</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Advisor ka point: 'Frontend dev sirf UI ke liye' — neeche dekho ye kyu adhoora hai</t>
+          <t>The advisor's view: 'a frontend dev is only for UI' — the rows below show why that view is incomplete</t>
         </is>
       </c>
     </row>
@@ -2843,22 +2843,22 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Ek Line Me (CEO Language)</t>
+          <t>In One Line (CEO Language)</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Actual Daily Kaam</t>
+          <t>Actual Daily Work</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Is Project Me Kyu Zaroori</t>
+          <t>Why This Project Needs It</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Agar Nahi Hire Kiya To</t>
+          <t>If We Don't Hire</t>
         </is>
       </c>
     </row>
@@ -2870,22 +2870,22 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Building ka architect — decide karta hai KYA kaise banega, aur galat cheez ko rokta hai</t>
+          <t>The architect of the building — decides HOW things get built, and stops bad decisions early</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Architecture decisions; har code change ka review (security + quality); team ko unblock karna; tech debt control; vendor/infra choices</t>
+          <t>Architecture decisions; reviewing every code change (security + quality); unblocking the team; controlling tech debt; vendor and infrastructure choices</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Sheet 2 ke 33 bugs me se zyadatar 'review na hone' se aaye the. Har naya developer bina lead ke naye bugs laayega.</t>
+          <t>Most of the 33 bugs in Sheet 2 existed because no one was reviewing the code. Every new developer hired without a lead will introduce new bugs.</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Har developer apni style me code likhega; 6 mahine me codebase unmaintainable; security bugs wapas aayenge</t>
+          <t>Every developer codes in their own style; within 6 months the codebase becomes unmaintainable; security bugs return</t>
         </is>
       </c>
     </row>
@@ -2897,7 +2897,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Engine room — paisa, bookings, security sab yahan process hota hai</t>
+          <t>The engine room — money, bookings and security are all processed here</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -2907,16 +2907,16 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Sheet 4 ke 13 risks me se 9 backend ke hain — F-02 (double payment) aur F-04 (DDoS) jaise CRITICAL scenarios sirf backend dev hi handle karega</t>
+          <t>9 of the 13 risks in Sheet 4 are backend-owned — CRITICAL scenarios like F-02 (double payment) and F-04 (DDoS) can only be handled by a backend developer</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Payment edge cases manually handle karne padenge; hacker/competitor ke against koi full-time defence nahi</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="39" customHeight="1">
+          <t>Payment edge cases get handled manually forever; no full-time defence against hackers and competitors</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="43" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>Frontend Dev</t>
@@ -2924,26 +2924,26 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Jo guest ke haath me hai — booking wahan hoti hai, paisa wahan se aata hai. SIRF UI NAHI.</t>
+          <t>Everything in the guest's hands — bookings happen there, money comes from there. NOT just UI.</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Payment failure screens (guest ka paisa atka to kya dikhe), double-click guards, slow-network handling, GB-data wale dashboards ko fast rakhna, page speed (= conversion), error tracking har page pe</t>
+          <t>Payment failure screens (what the guest sees when money gets stuck), double-click guards, slow-network handling, keeping dashboards fast when data reaches GBs, page speed (= conversion), error tracking on every page</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>F-06 (double-submit), F-03 (GB data render), F-11 (page speed = 7% conversion per second) — ye UI design nahi, ENGINEERING hai. Designer ye nahi kar sakta.</t>
+          <t>F-06 (double-submit), F-03 (rendering GBs of data), F-11 (page speed costs ~7% conversion per second) — this is not UI design, it is ENGINEERING. A designer cannot do this.</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Har slow page = booking drop = direct revenue loss; guest-facing bugs sabse pehle dikhte hain aur brand kharab karte hain</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="30" customHeight="1">
+          <t>Every slow page = dropped bookings = direct revenue loss; guest-facing bugs are the first ones customers see, and they damage the brand fastest</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="34" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Database Dev</t>
@@ -2951,22 +2951,22 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Data ka godown manager — speed, safety, aur 'ek hotel dusre ka data na dekhe' iski guarantee</t>
+          <t>The warehouse manager of our data — speed, safety, and the guarantee that one hotel never sees another hotel's data</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Indexes &amp; query optimization, RLS policies, migrations discipline, backup/restore drills, archiving (jab data GBs me jaaye), connection pool math</t>
+          <t>Indexes and query optimization, Row Level Security policies, migration discipline, backup/restore drills, archiving (when data reaches GBs), connection pool capacity planning</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>F-03 (GB data), F-09 (100 hotels), F-13 (backup drill) — data hi product hai; ye gaya to company gayi</t>
+          <t>F-03 (GB-scale data), F-09 (100 hotels), F-13 (restore drills) — the data IS the product; if the data is lost, the company is lost</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Data badhte hi sab slow; ek migration galti = downtime; restore kabhi test nahi hua to ek crash = total loss</t>
+          <t>Everything slows down as data grows; one bad migration = downtime; if a restore is never tested, one crash = total loss</t>
         </is>
       </c>
     </row>
@@ -2977,30 +2977,30 @@
       <c r="D9" s="4" t="inlineStr"/>
       <c r="E9" s="4" t="inlineStr"/>
     </row>
-    <row r="10" ht="39" customHeight="1">
+    <row r="10" ht="47" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>ADVISOR KE POINT KA JAWAB</t>
+          <t>ANSWER TO THE ADVISOR'S POINT</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>'Frontend = UI' tab sahi hota jab hum static website bana rahe hote.</t>
+          <t>'Frontend = UI' would be true if we were building a static website.</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Hamara frontend PAISE HANDLE karta hai: Razorpay checkout states, loyalty points calculation display, live availability, real-time updates (WebSocket/SSE). In sab me bug = paisa ya booking loss.</t>
+          <t>Our frontend HANDLES MONEY: Razorpay checkout states, loyalty points calculations on screen, live availability, real-time updates (WebSocket/SSE). A bug in any of these means lost money or lost bookings.</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Example: S-28 me checkout discount client pe tha — guest 100% discount le sakta tha. S-14 me browser autofill payment keys kharab kar raha tha. Ye dono 'frontend' bugs the jinme paisa ja raha tha.</t>
+          <t>Proof from this very report: in S-28 the checkout discount was calculated in the browser — a guest could take a 100% discount. In S-14 browser autofill was corrupting payment keys. Both were 'frontend' bugs where real money was at stake.</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>UI designer pixel banata hai; Frontend ENGINEER paisa aur data ke flows ko browser me safe rakhta hai. Dono alag skills hain.</t>
+          <t>A UI designer makes pixels; a frontend ENGINEER keeps money and data flows safe inside the browser. These are two different skills.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update CEO report with latest work log entries and Features Built sheet
https://claude.ai/code/session_01QKsUumyB8kabj8MBZhL9cY
</commit_message>
<xml_diff>
--- a/docs/CEO_Report_Staybooker_Jun2026.xlsx
+++ b/docs/CEO_Report_Staybooker_Jun2026.xlsx
@@ -9,9 +9,10 @@
   <sheets>
     <sheet name="1. Executive Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="2. Problems Solved" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="3. Work In Progress" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="4. Future Risks" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="5. Team &amp; Hiring" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="3. Features Built" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="4. Work In Progress" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="5. Future Risks" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="6. Team &amp; Hiring" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -493,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -542,125 +543,149 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>33 issues fixed so far (5 Critical, 13 High). Each issue shows what would have happened to the business if it had reached production.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1">
+          <t>45 issues fixed so far (5 Critical, 21 High). Each issue shows what would have happened to the business if it had reached production.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="36" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Sheet 3 — Work In Progress</t>
+          <t>Sheet 3 — Features Built</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
+          <t>Major product features delivered alongside the bug fixing — multi-property chains, loyalty program, OTA rate intelligence, AI concierge, real-time updates, encrypted secrets storage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Sheet 4 — Work In Progress</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
           <t>Critical items currently being worked on.</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="40" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>Sheet 4 — Future Risks</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
+    <row r="9" ht="40" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Sheet 5 — Future Risks</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>13 real-world scenarios that WILL come as the business grows (100 users at once, payment failures, DDoS attacks, data growing to GBs) — what protection already exists and what still needs to be built.</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>Sheet 5 — Team &amp; Hiring</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Sheet 6 — Team &amp; Hiring</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>What a Tech Lead / Backend / Frontend / Database developer actually does, in simple language — and why 'frontend = only UI' is an incomplete view.</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr"/>
-      <c r="B10" s="4" t="inlineStr"/>
-    </row>
-    <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>KEY NUMBERS</t>
-        </is>
-      </c>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr"/>
       <c r="B11" s="4" t="inlineStr"/>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Issues fixed till date</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>33 (source: work_log_tracker.csv — 56 logged engineering tasks)</t>
-        </is>
-      </c>
+          <t>KEY NUMBERS</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr"/>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Critical issues fixed</t>
+          <t>Issues fixed till date</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>5 — payment secret key leak, payment amount tampering, permanent admin token, AI assistant crash, staff privilege escalation</t>
+          <t>45 (source: work_log_tracker.csv — 74 logged engineering tasks up to 11-Jun-2026)</t>
         </is>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>Automated tests added</t>
+          <t>Critical issues fixed</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>130+ test cases (security, payments, booking, role access). These tests run automatically on every code change (CI/CD pipeline).</t>
+          <t>5 — payment secret key leak, payment amount tampering, permanent admin token, AI assistant crash, staff privilege escalation</t>
         </is>
       </c>
     </row>
     <row r="15" ht="38" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
+          <t>Security audit coverage</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>A full security/performance audit found 36 findings (1 Critical, 12 High, 14 Medium, 9 Low). The Critical and almost all High findings are fixed; remaining items are tracked in Sheets 4 and 5.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="39" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Automated tests added</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>277 test cases passing (security, payments, booking, role access, rate limits, Redis failover). These run automatically on every code change (CI/CD), plus dependency vulnerability (CVE) scanning.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="54" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
           <t>Money saved (examples)</t>
         </is>
       </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>Payment tampering fix: a guest could pay Rs.1 and get a Rs.10,000 booking confirmed. AI cost fix: a bug was sending traffic to an AI model 10x more expensive than needed on the public chatbot.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr"/>
-      <c r="B16" s="4" t="inlineStr"/>
-    </row>
-    <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="4" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Payment tampering fix: a guest could pay Rs.1 and get a Rs.10,000 booking confirmed. AI cost fix: a bug was sending traffic to an AI model 10x more expensive than needed on the public chatbot. Tax validation fix: invalid tax setup could produce wrong bills for every guest.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr"/>
+      <c r="B18" s="4" t="inlineStr"/>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>ONE-LINE MESSAGE FOR THE CEO</t>
         </is>
       </c>
-      <c r="B17" s="4" t="inlineStr"/>
-    </row>
-    <row r="18" ht="50" customHeight="1">
-      <c r="A18" s="4" t="inlineStr">
+      <c r="B19" s="4" t="inlineStr"/>
+    </row>
+    <row r="20" ht="50" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>Bottom line</t>
         </is>
       </c>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <t>The bugs we found have been fixed. The real problem now is making sure NEW bugs are found by us before a hacker or competitor finds them. That requires dedicated Backend, Frontend and Database developers — not for design, but to protect money and data.</t>
         </is>
@@ -681,7 +706,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G37"/>
+  <dimension ref="A1:G49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1962,6 +1987,450 @@
       <c r="G37" s="4" t="inlineStr">
         <is>
           <t>10-Jun</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="34" customHeight="1">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>S-34</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>The public booking widget showed FAKE 'Sold Out' labels and made-up calendar prices</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>A leftover demo hack marked the 13th of every month as 'Sold Out' and showed fabricated per-day prices in the calendar</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>Real guests were being turned away from available rooms (lost bookings every month on the 13th) and shown prices that were simply not true — a legal/consumer-trust problem.</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>Fake logic removed; the calendar now shows only the real starting price; availability and price are confirmed server-side.</t>
+        </is>
+      </c>
+      <c r="F38" s="6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G38" s="4" t="inlineStr">
+        <is>
+          <t>10-Jun</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="30" customHeight="1">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>S-35</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>The booking widget was broadcasting checkout data to ANY website embedding it</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>Widget messages used a wildcard ('*') target — any page embedding our widget could read booking/checkout data</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>A malicious site could embed our widget and silently collect guests' booking details — data leak through our own product.</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>Messages are now locked to the verified parent website's origin only.</t>
+        </is>
+      </c>
+      <c r="F39" s="6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G39" s="4" t="inlineStr">
+        <is>
+          <t>10-Jun</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="30" customHeight="1">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>S-36</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>A temporary network error showed guests a permanently blank room-selection page</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>One failed data fetch blanked the whole page; optional add-ons could also block the page from loading</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>Guest sees a white page mid-booking → closes the tab → booking lost. No error, no retry, no explanation.</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>Added a clear error message with a Retry button; add-ons now load separately so their failure cannot blank the page.</t>
+        </is>
+      </c>
+      <c r="F40" s="7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G40" s="4" t="inlineStr">
+        <is>
+          <t>10-Jun</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="30" customHeight="1">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>S-37</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>Guests could search with empty or reversed dates (check-out before check-in)</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>The booking widgets did not validate the date range before navigating to the rooms page</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>Guests landed on broken/empty room pages — confusing experience, dropped bookings.</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr">
+        <is>
+          <t>Date range is validated before the search runs.</t>
+        </is>
+      </c>
+      <c r="F41" s="7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G41" s="4" t="inlineStr">
+        <is>
+          <t>10-Jun</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="30" customHeight="1">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>S-38</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>The busiest public query (availability search) had no composite database index</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>Every availability check scanned bookings without an optimal index on (hotel, status, dates)</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>As bookings grow, the most-hit public query slows down first — slow search = lost guests.</t>
+        </is>
+      </c>
+      <c r="E42" s="4" t="inlineStr">
+        <is>
+          <t>Composite index added on bookings (hotel_id, status, check_in, check_out).</t>
+        </is>
+      </c>
+      <c r="F42" s="7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G42" s="4" t="inlineStr">
+        <is>
+          <t>10-Jun</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="30" customHeight="1">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>S-39</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>If Redis went down, the AI spending limit silently turned OFF</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>The per-hotel AI quota was checked in Redis; when Redis was unavailable the check passed everything (fail-open)</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>An attacker (or just an outage) could combine Redis downtime with chatbot spam to run an unlimited AI bill.</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>Quota now fails CLOSED: an in-process daily cap takes over whenever Redis is unavailable.</t>
+        </is>
+      </c>
+      <c r="F43" s="6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G43" s="4" t="inlineStr">
+        <is>
+          <t>10-Jun</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="30" customHeight="1">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>S-40</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>Rate limits could be bypassed by faking the visitor's IP address</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>The rate limiter trusted the first IP in the X-Forwarded-For header, which any attacker can spoof</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>Every IP-based protection (login attempts, booking spam, AI limits) was bypassable with one fake header.</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="inlineStr">
+        <is>
+          <t>Trusted-proxy aware IP extraction (TRUSTED_PROXY_COUNT) — spoofed header prefixes are ignored.</t>
+        </is>
+      </c>
+      <c r="F44" s="6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G44" s="4" t="inlineStr">
+        <is>
+          <t>10-Jun</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="30" customHeight="1">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>S-41</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>Invalid tax settings could be saved, producing wrong bills</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>The tax form accepted negative amounts, out-of-range rates and inverted slab ranges; the inclusive-tax calculator could divide by zero (NaN)</t>
+        </is>
+      </c>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>Wrong tax on every invoice = wrong bills to guests and wrong GST records — financial and compliance damage.</t>
+        </is>
+      </c>
+      <c r="E45" s="4" t="inlineStr">
+        <is>
+          <t>Validation rejects bad slabs before save; the live calculator is guarded against NaN.</t>
+        </is>
+      </c>
+      <c r="F45" s="6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G45" s="4" t="inlineStr">
+        <is>
+          <t>10-Jun</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="30" customHeight="1">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>S-42</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>Password changes and uploads had no rate limit (brute-force risk)</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>Authenticated mutating routes (password change, team-member create, file upload, reports) had no per-user caps</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="inlineStr">
+        <is>
+          <t>An attacker with a stolen session could brute-force password changes; upload/report endpoints could be abused to run up server costs.</t>
+        </is>
+      </c>
+      <c r="E46" s="4" t="inlineStr">
+        <is>
+          <t>Rate limits added: password change 5/hr, team creation 10/hr, uploads 20/hr, reports 30/min — shared across all servers via Redis.</t>
+        </is>
+      </c>
+      <c r="F46" s="6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G46" s="4" t="inlineStr">
+        <is>
+          <t>11-Jun</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="30" customHeight="1">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>S-43</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>The team-user list was unbounded and reports could scan unlimited date ranges</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>GET /users loaded every row with no limit; the occupancy report accepted any date range (e.g. 10 years)</t>
+        </is>
+      </c>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>Large accounts would hang the page; one heavy report could slow the database for every hotel.</t>
+        </is>
+      </c>
+      <c r="E47" s="4" t="inlineStr">
+        <is>
+          <t>Pagination added (limit ≤ 200 + offset); occupancy reports capped at 365 days.</t>
+        </is>
+      </c>
+      <c r="F47" s="7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G47" s="4" t="inlineStr">
+        <is>
+          <t>11-Jun</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="34" customHeight="1">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>S-44</t>
+        </is>
+      </c>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>One Redis hiccup permanently disabled shared locks and payment idempotency until restart</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>On the first Redis failure the client switched to per-process memory FOREVER — distributed locks, payment idempotency and rate limits silently degraded</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>After any brief Redis blip: duplicate scheduled jobs, possible duplicate payment processing, rate limits split per server — all silently, until someone restarted the app.</t>
+        </is>
+      </c>
+      <c r="E48" s="4" t="inlineStr">
+        <is>
+          <t>Self-healing reconnect: 30-second back-off then automatic recovery; memory fallback only during the outage.</t>
+        </is>
+      </c>
+      <c r="F48" s="6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G48" s="4" t="inlineStr">
+        <is>
+          <t>11-Jun</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="30" customHeight="1">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>S-45</t>
+        </is>
+      </c>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>Rate Shopper requests were being blocked by the OTA's bot protection (Akamai 613)</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr">
+        <is>
+          <t>A geo parameter in the scraping payload triggered Akamai blocks; currency could come back in the wrong unit</t>
+        </is>
+      </c>
+      <c r="D49" s="4" t="inlineStr">
+        <is>
+          <t>The premium rate-intelligence feature would fail repeatedly while still costing us vendor fees per attempt.</t>
+        </is>
+      </c>
+      <c r="E49" s="4" t="inlineStr">
+        <is>
+          <t>Payload corrected (geo removed, INR forced via URL parameter); retries and session rotation retained.</t>
+        </is>
+      </c>
+      <c r="F49" s="7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G49" s="4" t="inlineStr">
+        <is>
+          <t>11-Jun</t>
         </is>
       </c>
     </row>
@@ -1980,7 +2449,397 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Major Features Delivered (Not Just Bug Fixes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Source: work_log_tracker.csv. This is product value built in parallel with the security/stability work.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="26" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>What It Does (Simple Language)</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Business Value</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Built Safely (Security/Cost Controls Included)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Multi-property chain support</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>One brand owner can manage many hotels under one login: a consolidated chain dashboard with revenue, bookings and room-nights per hotel.</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Lets us sell to hotel GROUPS, not just single properties — bigger contracts.</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Only the chain OWNER can see consolidated data; every query validates the user belongs to that chain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Loyalty program (earn &amp; burn points)</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Guests earn points on every stay (1 point = Rs.1) and redeem them at checkout. Works across all hotels of the same brand.</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Repeat bookings and direct-booking incentive — guests skip OTAs to keep their points.</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Points credited with locks (no double credit); max discount enforced on the server; brand-level isolation so points never leak across brands.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Chain-wide promo codes</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>A brand can run one discount code across all of its hotels.</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Brand-level marketing campaigns become possible.</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Codes validated strictly within the owning chain — Hotel A cannot use Hotel B's codes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Sister-hotel recommendations</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>When a hotel is sold out, the booking widget suggests available sister hotels from the same brand.</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>A sold-out date becomes a transfer of revenue to a sister property instead of a lost guest.</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Recommendations cached (10 min) to keep searches fast; only same-chain, active hotels are shown.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>AI guest concierge with memory</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>The guest chatbot remembers past stays, preferences and special requests across all the brand's hotels.</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Personalised guest experience — a premium feature competitors charge heavily for.</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Only same-chain stay history is used; token usage capped to control AI cost; PII guarded.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Rate Shopper (OTA rate intelligence)</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Tracks competitors' prices on MakeMyTrip/OTAs day by day, with live progress, a stop button, auto-sync scheduling and market analysis charts.</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>Hoteliers price their rooms with real market data — a paid premium feature (new revenue line).</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>Feature-gated by subscription plan; per-hotel ownership checks; vendor cost billed per attempt; scrape can be stopped mid-run.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Real-time updates (WebSocket + SSE)</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Dashboards and availability update live — a new booking appears without refreshing the page.</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>The product feels modern and 'alive'; staff react to bookings instantly.</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>Connections require a verified login token; streams have lifetime caps so they cannot pile up.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Date modification on checkout</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Guests can change their search dates directly on the checkout page; prices refresh automatically.</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>Fewer abandoned checkouts — guests do not have to start over.</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>New dates/rates validated on the server, not trusted from the browser.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Encrypted secrets vault</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>All hotel credentials (payment, WhatsApp, email, AI keys) stored AES-256 encrypted in Supabase Vault with a safe admin UI.</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>A database leak no longer exposes any hotel's payment or messaging accounts.</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Secrets are write-only from the UI; never returned in plain text; never logged.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Database-level tenant security (RLS)</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>The database itself refuses to return one hotel's data to another hotel, independent of application code.</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>A second, independent lock on customer data — a strong selling point for security-conscious chains.</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>Row Level Security policies on every tenant table, keyed to the verified login.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="31" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>CI/CD pipeline + automated test suite</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Every code change automatically runs 277 tests (security, payments, roles, rate limits) plus a dependency vulnerability (CVE) scan before it can be merged.</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Deploys stop being a gamble; regressions are caught before customers see them.</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Includes cross-tenant attack tests and coverage reporting.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Bookable widget for hotel websites</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>An embeddable booking widget hotels place on their own websites, with chain-level booking support.</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>Hotels capture direct bookings (no OTA commission) — core product value.</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>Widget messages locked to the embedding site's verified origin; prices/availability always confirmed server-side.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2085,7 +2944,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="30" customHeight="1">
+    <row r="7" ht="49" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>P-03</t>
@@ -2098,7 +2957,7 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Every page must handle network failures, double-clicks, and slow-data scenarios gracefully.</t>
+          <t>Every page must handle network failures, double-clicks, and slow-data scenarios gracefully. The public booking widget pages are done (error+retry UI, date validation, fake-data removal — see S-34, S-36, S-37); the hotelier dashboard pages are next.</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -2112,7 +2971,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="30" customHeight="1">
+    <row r="8" ht="44" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
           <t>P-04</t>
@@ -2120,12 +2979,12 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>DDoS / abuse protection layer (WAF, IP-spoofing fix)</t>
+          <t>DDoS / abuse protection layer (WAF)</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Rate limits exist in Redis, but the client IP header can be spoofed; a Cloudflare/WAF layer is needed.</t>
+          <t>The IP-spoofing hole is now FIXED (trusted-proxy IP extraction, S-40) and key routes are rate-limited (S-42). The remaining piece is an edge layer (Cloudflare/WAF) to absorb large-scale attacks before they reach our servers.</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -2139,7 +2998,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="30" customHeight="1">
+    <row r="9" ht="42" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
           <t>P-05</t>
@@ -2152,7 +3011,7 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>The schema is currently built by create_all at startup; performance indexes may be missing in production.</t>
+          <t>The schema is currently built by create_all at startup; performance indexes may be missing in production. The hottest availability index has been added manually (S-38), but a proper migration process is needed.</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -2163,6 +3022,33 @@
       <c r="E9" s="4" t="inlineStr">
         <is>
           <t>As data grows, queries get slow → the whole app gets slow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="60" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>P-06</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Remaining medium-severity audit findings</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>The June security audit logged 36 findings. The Critical and nearly all High items are fixed. Mediums still being worked through include: login-token cache window (~10 min), unsigned OAuth state parameter, an unauthenticated competitor data-freshness endpoint, and stale analytics cache invalidation.</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>Each one is a small hole today; at bigger scale, small holes are what hackers chain together.</t>
         </is>
       </c>
     </row>
@@ -2175,7 +3061,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2273,7 +3159,7 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Row-level database locks on inventory; Redis idempotency; pagination everywhere</t>
+          <t>Row-level database locks on inventory; Redis idempotency; pagination everywhere; composite index on the hottest availability query</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
@@ -2376,7 +3262,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="30" customHeight="1">
+    <row r="8" ht="37" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
           <t>F-04</t>
@@ -2394,17 +3280,17 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Public endpoints are anonymous; the IP rate limit can be bypassed by spoofing the forwarded-IP header</t>
+          <t>Public endpoints are anonymous and attract bots; large attacks must be absorbed before they reach our servers</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Redis-backed rate limiting; per-hotel AI quotas; limits on streaming connection lifetimes</t>
+          <t>Redis-backed rate limiting; spoof-proof client IP detection (trusted proxy); per-hotel AI quotas; per-route caps on password change/uploads/reports; limits on streaming connection lifetimes</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>A Cloudflare/WAF layer, trusted-proxy IP fix, bot detection (CAPTCHA on abuse), infrastructure alerts</t>
+          <t>A Cloudflare/WAF edge layer, bot detection (CAPTCHA on abuse), infrastructure alerts</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
@@ -2805,7 +3691,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2880,7 +3766,7 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Most of the 33 bugs in Sheet 2 existed because no one was reviewing the code. Every new developer hired without a lead will introduce new bugs.</t>
+          <t>Most of the 45 bugs in Sheet 2 existed because no one was reviewing the code. Every new developer hired without a lead will introduce new bugs.</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
@@ -2907,7 +3793,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>9 of the 13 risks in Sheet 4 are backend-owned — CRITICAL scenarios like F-02 (double payment) and F-04 (DDoS) can only be handled by a backend developer</t>
+          <t>9 of the 13 risks in Sheet 5 are backend-owned — CRITICAL scenarios like F-02 (double payment) and F-04 (DDoS) can only be handled by a backend developer</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
@@ -2977,7 +3863,7 @@
       <c r="D9" s="4" t="inlineStr"/>
       <c r="E9" s="4" t="inlineStr"/>
     </row>
-    <row r="10" ht="47" customHeight="1">
+    <row r="10" ht="67" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
           <t>ANSWER TO THE ADVISOR'S POINT</t>
@@ -2995,7 +3881,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Proof from this very report: in S-28 the checkout discount was calculated in the browser — a guest could take a 100% discount. In S-14 browser autofill was corrupting payment keys. Both were 'frontend' bugs where real money was at stake.</t>
+          <t>Proof from this very report: in S-28 the checkout discount was calculated in the browser — a guest could take a 100% discount. In S-34 the widget showed fake 'Sold Out' labels that turned real guests away. In S-35 the widget leaked checkout data to any embedding website. All were 'frontend' bugs where real money or data was at stake.</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Rework Team & Hiring sheet: plain language, neutral framing, hiring plan
https://claude.ai/code/session_01QKsUumyB8kabj8MBZhL9cY
</commit_message>
<xml_diff>
--- a/docs/CEO_Report_Staybooker_Jun2026.xlsx
+++ b/docs/CEO_Report_Staybooker_Jun2026.xlsx
@@ -22,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -47,6 +47,11 @@
     </font>
     <font>
       <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="7">
@@ -108,7 +113,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -129,6 +134,7 @@
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -3697,27 +3703,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
-    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
     <col width="46" customWidth="1" min="4" max="4"/>
-    <col width="44" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Team Roles — In Simple Language</t>
+          <t>Team Roles &amp; Hiring Plan — In Simple Language</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>The advisor's view: 'a frontend dev is only for UI' — the rows below show why that view is incomplete</t>
+          <t>Who does what, why each role matters for this product, and a suggested hiring order</t>
         </is>
       </c>
     </row>
@@ -3734,21 +3741,26 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Actual Daily Work</t>
+          <t>Main Responsibilities (Daily Work)</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Why This Project Needs It</t>
+          <t>Real Examples From This Project (Plain Words)</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>If We Don't Hire</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="30" customHeight="1">
+          <t>What Happens Without This Role</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Risk Level Without It</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="59" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Tech Lead</t>
@@ -3756,26 +3768,31 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>The architect of the building — decides HOW things get built, and stops bad decisions early</t>
+          <t>The one person responsible for ALL of the technology — decides what every other developer works on, and answers for quality, security and deadlines.</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Architecture decisions; reviewing every code change (security + quality); unblocking the team; controlling tech debt; vendor and infrastructure choices</t>
+          <t>Converts business goals into a technical plan; decides and assigns what the backend, frontend and database developers build each week; reviews every code change before it goes live; takes the final call on architecture, tools and vendors; reports progress and risks to the CEO in business language.</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Most of the 45 bugs in Sheet 2 existed because no one was reviewing the code. Every new developer hired without a lead will introduce new bugs.</t>
+          <t>Most of the 45 bugs fixed in this report existed because no second person was reviewing the code. A Tech Lead's review is the checkpoint that stops a bug BEFORE it reaches guests. The Tech Lead is also the one who decided the order of fixes: money-related bugs first, cosmetic issues last.</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Every developer codes in their own style; within 6 months the codebase becomes unmaintainable; security bugs return</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="30" customHeight="1">
+          <t>Developers work in different directions with no owner of the final result; nobody is accountable when something breaks; the CEO has to manage 3 developers directly without speaking their technical language.</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="60" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Backend Dev</t>
@@ -3783,26 +3800,31 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>The engine room — money, bookings and security are all processed here</t>
+          <t>Builds and protects the engine room — payments, bookings and security are all processed here. This is where the money moves.</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Payment flows (Razorpay), booking logic, APIs, race conditions, rate limiting, webhooks, AI cost control, integrations (WhatsApp/OTA)</t>
+          <t>Payment flows (Razorpay), booking logic, server APIs, preventing double-bookings under load, rate limiting against abuse, webhooks, AI cost control, integrations (WhatsApp, OTAs, email).</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>9 of the 13 risks in Sheet 5 are backend-owned — CRITICAL scenarios like F-02 (double payment) and F-04 (DDoS) can only be handled by a backend developer</t>
+          <t>Stopped a bug where a guest could pay Rs.1 and get a Rs.10,000 booking confirmed. Built the protection that stops the same payment from being charged twice when a guest's network fails. Future work: automatic refunds when money is deducted but the booking fails, and surviving 100 simultaneous bookings.</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Payment edge cases get handled manually forever; no full-time defence against hackers and competitors</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="43" customHeight="1">
+          <t>Payment edge cases keep getting handled manually one by one; there is no full-time defence against hackers probing our APIs or competitors attacking the site.</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="60" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>Frontend Dev</t>
@@ -3810,26 +3832,31 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Everything in the guest's hands — bookings happen there, money comes from there. NOT just UI.</t>
+          <t>Builds everything the guest touches — the booking happens there, the money enters there. It is engineering, not just visual design.</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Payment failure screens (what the guest sees when money gets stuck), double-click guards, slow-network handling, keeping dashboards fast when data reaches GBs, page speed (= conversion), error tracking on every page</t>
+          <t>Payment screens and their failure states (what the guest sees when money gets stuck); blocking double-clicks that create duplicate bookings; handling slow networks gracefully; keeping dashboards fast when a hotel's data grows huge; page speed; tracking errors on every page.</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>F-06 (double-submit), F-03 (rendering GBs of data), F-11 (page speed costs ~7% conversion per second) — this is not UI design, it is ENGINEERING. A designer cannot do this.</t>
+          <t>Fixed a widget bug that showed FAKE 'Sold Out' labels — real guests were being turned away from available rooms. Fixed the checkout discount being calculated in the browser, where a guest could give themselves 100% off. Industry data: every extra second of page load time cuts bookings by roughly 7%.</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Every slow page = dropped bookings = direct revenue loss; guest-facing bugs are the first ones customers see, and they damage the brand fastest</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="34" customHeight="1">
+          <t>Every slow or broken page silently drops bookings — this is direct revenue loss, invisible until you measure it; guest-facing bugs are the first thing customers see and they damage the brand fastest.</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="61" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Database Dev</t>
@@ -3837,63 +3864,357 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>The warehouse manager of our data — speed, safety, and the guarantee that one hotel never sees another hotel's data</t>
+          <t>The warehouse manager of our data — keeps it fast, safe, recoverable, and guarantees one hotel can never see another hotel's data.</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Indexes and query optimization, Row Level Security policies, migration discipline, backup/restore drills, archiving (when data reaches GBs), connection pool capacity planning</t>
+          <t>Indexes and query speed; the database-level security rules that isolate each hotel's data; safe schema migrations; backup and restore drills; archiving old data when it grows to gigabytes; planning database capacity as hotels onboard.</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>F-03 (GB-scale data), F-09 (100 hotels), F-13 (restore drills) — the data IS the product; if the data is lost, the company is lost</t>
+          <t>Built the database-level security layer (Row Level Security) so that even if application code has a bug, the database itself refuses to hand one hotel's data to another. Future work: keeping dashboards fast when a hotel has 2-3 years of bookings, and regularly testing that backups can actually be restored.</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Everything slows down as data grows; one bad migration = downtime; if a restore is never tested, one crash = total loss</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr"/>
-      <c r="B9" s="4" t="inlineStr"/>
-      <c r="C9" s="4" t="inlineStr"/>
-      <c r="D9" s="4" t="inlineStr"/>
-      <c r="E9" s="4" t="inlineStr"/>
-    </row>
-    <row r="10" ht="67" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>ANSWER TO THE ADVISOR'S POINT</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>'Frontend = UI' would be true if we were building a static website.</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>Our frontend HANDLES MONEY: Razorpay checkout states, loyalty points calculations on screen, live availability, real-time updates (WebSocket/SSE). A bug in any of these means lost money or lost bookings.</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>Proof from this very report: in S-28 the checkout discount was calculated in the browser — a guest could take a 100% discount. In S-34 the widget showed fake 'Sold Out' labels that turned real guests away. In S-35 the widget leaked checkout data to any embedding website. All were 'frontend' bugs where real money or data was at stake.</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="inlineStr">
-        <is>
-          <t>A UI designer makes pixels; a frontend ENGINEER keeps money and data flows safe inside the browser. These are two different skills.</t>
+          <t>Everything slows down as data grows; one bad schema change can cause downtime; if a backup restore is never tested, a single crash can mean permanent data loss — a company-ending event.</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="9"/>
+    <row r="10"/>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>HOW THE TEAM WORKS TOGETHER (Simple Flow)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Who</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>What Happens</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>CEO / Business</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Sets the business goal — e.g. 'onboard 50 hotels this quarter' or 'reduce booking drop-offs'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Tech Lead</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Translates the goal into a technical plan, breaks it into tasks, and decides which developer does what, in which order.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Backend / Frontend / Database Devs</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Build their assigned parts in parallel — server logic, guest-facing screens, and data layer respectively.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Tech Lead</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Reviews every piece of work for security and quality before it is released. Nothing reaches guests without this check.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Tech Lead → CEO</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Reports progress, risks and costs back in business language — the CEO never needs to talk to four people separately.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18"/>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>SUGGESTED HIRING ORDER (Based on Current Risks)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Why First / Why This Order</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>What They Own in the First 90 Days</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="37" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Backend Developer</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>The biggest open risks involve money: payment failure recovery (guest charged twice), surviving 100 simultaneous bookings, and abuse protection. These are revenue-protecting, not optional.</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>Automatic refund + payment reconciliation flow; load testing the booking path; finishing the DDoS protection layer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="35" customHeight="1">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Frontend Developer</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Every guest-facing bug directly drops bookings. The page-by-page error audit is only partly done — the public booking widget is fixed, the hotelier dashboard pages are pending.</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>Error handling + double-click guards on every page; page speed optimization (faster pages = more completed bookings); error monitoring.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="30" customHeight="1">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Database Developer</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>Becomes urgent as hotels onboard and data grows to gigabytes. Can start part-time/consulting and convert to full-time with scale.</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>Proper migration process; backup restore drills; query/index plan for large hotels; capacity plan for 50-100 hotels.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="38" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Now (or first hire)</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>Tech Lead</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Whoever is hired first needs direction from day one. Without a lead, each new hire initially ADDS bugs instead of removing them. This can be a senior developer who also codes (hands-on lead).</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>Owns the technical roadmap; sets the code review process; assigns and supervises all of the above work; reports to the CEO.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27" ht="30" customHeight="1">
+      <c r="A27" s="8" t="inlineStr">
+        <is>
+          <t>A COMMON QUESTION: 'ISN'T FRONTEND JUST DESIGN?'</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="30" customHeight="1">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>Aspect</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>UI Designer</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>Frontend Developer (Engineer)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="30" customHeight="1">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>What they produce</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>The look: colours, layouts, fonts, mock-ups in design tools.</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>Working software in the browser: payment screens, booking forms, live availability, real-time updates.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="53" customHeight="1">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Relationship with money</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>Indirect — a good design improves conversion.</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>Direct — they write the code that handles checkout states, discount calculations and payment results. A bug here loses real money (this project already had such bugs: a browser-side discount that allowed 100% off, and fake 'Sold Out' labels that turned guests away).</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="30" customHeight="1">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>When things go wrong</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>A page looks less attractive.</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>A guest gets charged twice, sees a blank page mid-booking, or books a room that was already sold.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="30" customHeight="1">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Conclusion</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>Needed occasionally (design refreshes can be outsourced per project).</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>Needed continuously — every feature, every fix, every page has a frontend engineering half. Both roles matter; they are different skills.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Soften Team & Hiring sheet: growth-based justification, data-journey role mapping
https://claude.ai/code/session_01QKsUumyB8kabj8MBZhL9cY
</commit_message>
<xml_diff>
--- a/docs/CEO_Report_Staybooker_Jun2026.xlsx
+++ b/docs/CEO_Report_Staybooker_Jun2026.xlsx
@@ -589,7 +589,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="30" customHeight="1">
+    <row r="10" ht="34" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Sheet 6 — Team &amp; Hiring</t>
@@ -597,7 +597,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>What a Tech Lead / Backend / Frontend / Database developer actually does, in simple language — and why 'frontend = only UI' is an incomplete view.</t>
+          <t>What a Tech Lead / Backend / Frontend / Database developer actually does, in simple language — who owns which part of the product as it grows, with a suggested hiring order.</t>
         </is>
       </c>
     </row>
@@ -693,7 +693,7 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>The bugs we found have been fixed. The real problem now is making sure NEW bugs are found by us before a hacker or competitor finds them. That requires dedicated Backend, Frontend and Database developers — not for design, but to protect money and data.</t>
+          <t>The product is stable today and hoteliers' data is safe. The hiring need comes from growth: as hotels, traffic and data scale up, each layer — database, backend, frontend — needs a dedicated owner so quality and safety stay exactly where they are today.</t>
         </is>
       </c>
     </row>
@@ -3703,417 +3703,280 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="44" customWidth="1" min="3" max="3"/>
-    <col width="46" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="56" customWidth="1" min="3" max="3"/>
+    <col width="56" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Team Roles &amp; Hiring Plan — In Simple Language</t>
+          <t>Team &amp; Hiring — Decision Support</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Who does what, why each role matters for this product, and a suggested hiring order</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="26" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Role</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>In One Line (CEO Language)</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Main Responsibilities (Daily Work)</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>Real Examples From This Project (Plain Words)</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>What Happens Without This Role</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>Risk Level Without It</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="59" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>Tech Lead</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>The one person responsible for ALL of the technology — decides what every other developer works on, and answers for quality, security and deadlines.</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>Converts business goals into a technical plan; decides and assigns what the backend, frontend and database developers build each week; reviews every code change before it goes live; takes the final call on architecture, tools and vendors; reports progress and risks to the CEO in business language.</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>Most of the 45 bugs fixed in this report existed because no second person was reviewing the code. A Tech Lead's review is the checkpoint that stops a bug BEFORE it reaches guests. The Tech Lead is also the one who decided the order of fixes: money-related bugs first, cosmetic issues last.</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>Developers work in different directions with no owner of the final result; nobody is accountable when something breaks; the CEO has to manage 3 developers directly without speaking their technical language.</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="60" customHeight="1">
+          <t>The product is stable today and data is safe. This sheet maps which role owns which part as the business grows.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>WHERE THE PRODUCT STANDS TODAY</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Area</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Current Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="38" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Backend Dev</t>
+          <t>Product stability</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Builds and protects the engine room — payments, bookings and security are all processed here. This is where the money moves.</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>Payment flows (Razorpay), booking logic, server APIs, preventing double-bookings under load, rate limiting against abuse, webhooks, AI cost control, integrations (WhatsApp, OTAs, email).</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>Stopped a bug where a guest could pay Rs.1 and get a Rs.10,000 booking confirmed. Built the protection that stops the same payment from being charged twice when a guest's network fails. Future work: automatic refunds when money is deducted but the booking fails, and surviving 100 simultaneous bookings.</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>Payment edge cases keep getting handled manually one by one; there is no full-time defence against hackers probing our APIs or competitors attacking the site.</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="60" customHeight="1">
+          <t>Stable for current hoteliers — bookings, payments, dashboards and integrations are working. 45 issues have been found and fixed proactively, and 277 automated tests now run on every code change.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="37" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Frontend Dev</t>
+          <t>Data safety</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Builds everything the guest touches — the booking happens there, the money enters there. It is engineering, not just visual design.</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>Payment screens and their failure states (what the guest sees when money gets stuck); blocking double-clicks that create duplicate bookings; handling slow networks gracefully; keeping dashboards fast when a hotel's data grows huge; page speed; tracking errors on every page.</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>Fixed a widget bug that showed FAKE 'Sold Out' labels — real guests were being turned away from available rooms. Fixed the checkout discount being calculated in the browser, where a guest could give themselves 100% off. Industry data: every extra second of page load time cuts bookings by roughly 7%.</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>Every slow or broken page silently drops bookings — this is direct revenue loss, invisible until you measure it; guest-facing bugs are the first thing customers see and they damage the brand fastest.</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="61" customHeight="1">
+          <t>Safe — all credentials are encrypted (AES-256 vault), every hotel's data is isolated at both the application and the database level, and payment amounts are always verified on the server.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Database Dev</t>
+          <t>Hotelier experience</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>The warehouse manager of our data — keeps it fast, safe, recoverable, and guarantees one hotel can never see another hotel's data.</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>Indexes and query speed; the database-level security rules that isolate each hotel's data; safe schema migrations; backup and restore drills; archiving old data when it grows to gigabytes; planning database capacity as hotels onboard.</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>Built the database-level security layer (Row Level Security) so that even if application code has a bug, the database itself refuses to hand one hotel's data to another. Future work: keeping dashboards fast when a hotel has 2-3 years of bookings, and regularly testing that backups can actually be restored.</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>Everything slows down as data grows; one bad schema change can cause downtime; if a backup restore is never tested, a single crash can mean permanent data loss — a company-ending event.</t>
-        </is>
-      </c>
-      <c r="F8" s="6" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="9"/>
+          <t>No major issues expected at today's scale. The public booking flow has been hardened (error recovery, date validation, double-payment protection).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="40" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Why hiring, then</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Growth. As hotels onboard, data will reach GBs and traffic will multiply. Each layer of the product — database, backend, frontend — then needs a dedicated owner so quality stays exactly where it is today.</t>
+        </is>
+      </c>
+    </row>
     <row r="10"/>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>HOW THE TEAM WORKS TOGETHER (Simple Flow)</t>
+          <t>HOW DATA TRAVELS THROUGH THE PRODUCT — AND WHO OWNS EACH STEP</t>
         </is>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Step</t>
+          <t>Step in the Data Journey</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Who</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>What Happens</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="30" customHeight="1">
+          <t>Exact Job</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="41" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1. Data lives in the database (bookings, rates, guests)</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>CEO / Business</t>
+          <t>Database Dev</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Sets the business goal — e.g. 'onboard 50 hotels this quarter' or 'reduce booking drop-offs'.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="30" customHeight="1">
+          <t>Makes sure data comes OUT of the database smoothly — right indexes, fast queries, clean schema, reliable backups, per-hotel isolation. When data reaches GBs: partitioning and archiving so queries stay fast.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="46" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>2. Backend picks up the data and serves it through APIs</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
+          <t>Backend Dev</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Connects the backend APIs to the database properly — booking logic, payment processing, security checks. When data reaches GBs: sends it in CHUNKS (pagination, batching, caching) so the server never tries to load everything at once.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="59" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>3. Frontend calls those APIs and shows the data on screen</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Frontend Dev</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Connects the React + TypeScript frontend to the backend APIs and makes sure the data arrives and displays correctly — loading states, error handling, payment screens. When data reaches GBs: loads it smoothly on screen (paged lists, lazy loading) so pages stay fast for the hotelier and the guest.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="33" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>4. Someone decides what gets built, in what order, and signs off</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
           <t>Tech Lead</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>Translates the goal into a technical plan, breaks it into tasks, and decides which developer does what, in which order.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>Backend / Frontend / Database Devs</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>Build their assigned parts in parallel — server logic, guest-facing screens, and data layer respectively.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>Tech Lead</t>
-        </is>
-      </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Reviews every piece of work for security and quality before it is released. Nothing reaches guests without this check.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>Tech Lead → CEO</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>Reports progress, risks and costs back in business language — the CEO never needs to talk to four people separately.</t>
-        </is>
-      </c>
-    </row>
+          <t>Decides what happens in the project — what each developer builds and when, reviews every change before release, and carries the overall responsibility for the software.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17"/>
     <row r="18"/>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>SUGGESTED HIRING ORDER (Based on Current Risks)</t>
+          <t>ROLE SUMMARY — WITH EXAMPLES FROM OUR OWN PROJECT</t>
         </is>
       </c>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>Priority</t>
+          <t>Role</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Role</t>
+          <t>In One Line</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>Why First / Why This Order</t>
-        </is>
-      </c>
-      <c r="D20" s="3" t="inlineStr">
-        <is>
-          <t>What They Own in the First 90 Days</t>
+          <t>Examples of This Work Already Done in the Product</t>
         </is>
       </c>
     </row>
     <row r="21" ht="37" customHeight="1">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Tech Lead</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Backend Developer</t>
+          <t>Responsible for the whole software — decides what every developer works on, reviews everything, owns delivery.</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>The biggest open risks involve money: payment failure recovery (guest charged twice), surviving 100 simultaneous bookings, and abuse protection. These are revenue-protecting, not optional.</t>
-        </is>
-      </c>
-      <c r="D21" s="4" t="inlineStr">
-        <is>
-          <t>Automatic refund + payment reconciliation flow; load testing the booking path; finishing the DDoS protection layer.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="35" customHeight="1">
+          <t>Prioritised the fix order across 45 issues (money-related first); set the engineering rules and the review checklist the team now follows; set up the CI pipeline that tests every change.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="39" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>Backend Dev</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Frontend Developer</t>
+          <t>Owns backend APIs and their connection to the database — payments, booking logic, security, performance.</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Every guest-facing bug directly drops bookings. The page-by-page error audit is only partly done — the public booking widget is fixed, the hotelier dashboard pages are pending.</t>
-        </is>
-      </c>
-      <c r="D22" s="4" t="inlineStr">
-        <is>
-          <t>Error handling + double-click guards on every page; page speed optimization (faster pages = more completed bookings); error monitoring.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="30" customHeight="1">
+          <t>Server-side payment verification (amount can never be tampered from the browser); double-payment protection when a guest's network fails; pagination on heavy endpoints; rate limits against abuse.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="42" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>Frontend Dev</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Database Developer</t>
+          <t>Owns the React + TypeScript screens and their connection to backend APIs — correct data display, smooth experience.</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Becomes urgent as hotels onboard and data grows to gigabytes. Can start part-time/consulting and convert to full-time with scale.</t>
-        </is>
-      </c>
-      <c r="D23" s="4" t="inlineStr">
-        <is>
-          <t>Proper migration process; backup restore drills; query/index plan for large hotels; capacity plan for 50-100 hotels.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="38" customHeight="1">
+          <t>Error + retry handling on the booking pages (a network blip no longer shows a blank page); date validation before search; live-updating dashboards; checkout flow with loyalty points calculated safely via the API.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="35" customHeight="1">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>Now (or first hire)</t>
+          <t>Database Dev</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Tech Lead</t>
+          <t>Owns the database — speed, schema, backups, and the guarantee that data flows out smoothly at any size.</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Whoever is hired first needs direction from day one. Without a lead, each new hire initially ADDS bugs instead of removing them. This can be a senior developer who also codes (hands-on lead).</t>
-        </is>
-      </c>
-      <c r="D24" s="4" t="inlineStr">
-        <is>
-          <t>Owns the technical roadmap; sets the code review process; assigns and supervises all of the above work; reports to the CEO.</t>
+          <t>Database-level isolation between hotels (Row Level Security); composite indexes on the busiest availability queries; encrypted credential storage; chain-level loyalty data design.</t>
         </is>
       </c>
     </row>
@@ -4122,99 +3985,124 @@
     <row r="27" ht="30" customHeight="1">
       <c r="A27" s="8" t="inlineStr">
         <is>
-          <t>A COMMON QUESTION: 'ISN'T FRONTEND JUST DESIGN?'</t>
+          <t>SUGGESTED HIRING ORDER</t>
         </is>
       </c>
     </row>
     <row r="28" ht="30" customHeight="1">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>Aspect</t>
+          <t>Priority</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>UI Designer</t>
+          <t>Role</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>Frontend Developer (Engineer)</t>
+          <t>Why This Order</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>Focus in the First 90 Days</t>
         </is>
       </c>
     </row>
     <row r="29" ht="30" customHeight="1">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>What they produce</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>The look: colours, layouts, fonts, mock-ups in design tools.</t>
+          <t>Backend Dev</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Working software in the browser: payment screens, booking forms, live availability, real-time updates.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="53" customHeight="1">
+          <t>The next milestones are payment-recovery automation and handling high booking traffic — both backend work.</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>Automatic refund + payment reconciliation; load testing the booking path; finishing the abuse-protection layer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="30" customHeight="1">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>Relationship with money</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>Indirect — a good design improves conversion.</t>
+          <t>Frontend Dev</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Direct — they write the code that handles checkout states, discount calculations and payment results. A bug here loses real money (this project already had such bugs: a browser-side discount that allowed 100% off, and fake 'Sold Out' labels that turned guests away).</t>
+          <t>The hotelier dashboard pages are next in line for the same error-handling polish the public booking pages already received.</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>API integration hardening on every dashboard page; page speed optimisation; error monitoring.</t>
         </is>
       </c>
     </row>
     <row r="31" ht="30" customHeight="1">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>When things go wrong</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>A page looks less attractive.</t>
+          <t>Database Dev</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>A guest gets charged twice, sees a blank page mid-booking, or books a room that was already sold.</t>
+          <t>Becomes essential as data approaches GB scale; can begin part-time and grow with the data.</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>Migration process; backup restore drills; query and index plan for large hotels; capacity plan for onboarding more hotels.</t>
         </is>
       </c>
     </row>
     <row r="32" ht="30" customHeight="1">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>Conclusion</t>
+          <t>With the first hire</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>Needed occasionally (design refreshes can be outsourced per project).</t>
+          <t>Tech Lead</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Needed continuously — every feature, every fix, every page has a frontend engineering half. Both roles matter; they are different skills.</t>
+          <t>Direction and review from day one keeps all the above work consistent. Can be a hands-on senior developer.</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>Technical roadmap; review process; assigning and supervising the work above.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Verify report numbers against work log; soften dramatic language throughout
https://claude.ai/code/session_01QKsUumyB8kabj8MBZhL9cY
</commit_message>
<xml_diff>
--- a/docs/CEO_Report_Staybooker_Jun2026.xlsx
+++ b/docs/CEO_Report_Staybooker_Jun2026.xlsx
@@ -549,7 +549,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>45 issues fixed so far (5 Critical, 21 High). Each issue shows what would have happened to the business if it had reached production.</t>
+          <t>45 issues fixed so far (5 Critical, 24 High, 16 Medium). Each issue shows what would have happened to the business if it had reached production.</t>
         </is>
       </c>
     </row>
@@ -621,7 +621,7 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>45 (source: work_log_tracker.csv — 74 logged engineering tasks up to 11-Jun-2026)</t>
+          <t>45 (source: work_log_tracker.csv — 71 logged engineering tasks up to 11-Jun-2026)</t>
         </is>
       </c>
     </row>
@@ -637,7 +637,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="38" customHeight="1">
+    <row r="15" ht="40" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
           <t>Security audit coverage</t>
@@ -645,7 +645,7 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>A full security/performance audit found 36 findings (1 Critical, 12 High, 14 Medium, 9 Low). The Critical and almost all High findings are fixed; remaining items are tracked in Sheets 4 and 5.</t>
+          <t>A full security/performance audit found 36 findings (1 Critical, 12 High, 14 Medium, 9 Low). The Critical issue and most High findings are fixed; the remaining items are tracked openly in Sheets 4 and 5.</t>
         </is>
       </c>
     </row>
@@ -775,7 +775,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="35" customHeight="1">
+    <row r="5" ht="41" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>S-01</t>
@@ -793,7 +793,7 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>A hacker could issue refunds from the hotel's payment account and fake payment verifications. Hotel loses money, we face legal action, and the Razorpay account could be banned.</t>
+          <t>Anyone could have used it to issue refunds from the hotel's payment account or fake payment verifications. The hotel loses money, we carry the legal responsibility, and the Razorpay account could be suspended.</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
@@ -849,7 +849,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="30" customHeight="1">
+    <row r="7" ht="32" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>S-03</t>
@@ -867,7 +867,7 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>If that token ever leaked (email, log file, stolen laptop), a hacker would own that hotel FOREVER — bookings, payments, guest data, everything.</t>
+          <t>If that token ever leaked (email, log file, lost laptop), whoever had it would keep owner-level access to that hotel indefinitely — bookings, payments, guest data.</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
@@ -923,7 +923,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="31" customHeight="1">
+    <row r="9" ht="33" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
           <t>S-05</t>
@@ -941,7 +941,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>A disgruntled employee could change rates, delete rooms, or change payment keys in settings. The hotel's entire business in the hands of a junior employee.</t>
+          <t>Any staff account — by mistake or misuse — could change rates, delete rooms, or alter payment keys in settings. Sensitive controls were not limited to the owner/manager.</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
@@ -960,7 +960,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="32" customHeight="1">
+    <row r="10" ht="30" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
           <t>S-06</t>
@@ -978,7 +978,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>A competitor hotel's discount codes could be stolen and used. Revenue leakage and total loss of trust in the platform (the worst failure for a multi-tenant SaaS).</t>
+          <t>One hotel could apply another hotel's discount codes. Revenue leakage and loss of trust in the platform (a serious failure for a multi-hotel system).</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
@@ -1126,7 +1126,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>A hacker would get a map of our system — which libraries, which versions — making an attack much easier to plan.</t>
+          <t>An outsider could learn internal system details (libraries, versions), which makes planning an attack easier.</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
@@ -1311,7 +1311,7 @@
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>Hoteliers would make pricing decisions on wrong market data — selling rooms too cheap or too expensive. Trust in the product destroyed.</t>
+          <t>Hoteliers would make pricing decisions on wrong market data — selling rooms too cheap or too expensive — and would lose confidence in the product.</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
@@ -1385,7 +1385,7 @@
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>A receptionist could change the points-to-rupee ratio and farm points into their own email — fraud.</t>
+          <t>Any staff account could change the points-to-rupee ratio and credit points to a personal email — a misuse risk.</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
@@ -1644,7 +1644,7 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>Broken code could reach production — every deploy was a gamble.</t>
+          <t>Broken code could reach production — every deploy carried avoidable risk.</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
@@ -2051,7 +2051,7 @@
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>A malicious site could embed our widget and silently collect guests' booking details — data leak through our own product.</t>
+          <t>Any website embedding our widget could read guests' booking details — an unintended data exposure through our own product.</t>
         </is>
       </c>
       <c r="E39" s="4" t="inlineStr">
@@ -2199,7 +2199,7 @@
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>An attacker (or just an outage) could combine Redis downtime with chatbot spam to run an unlimited AI bill.</t>
+          <t>During any Redis outage, chatbot spam could run an unlimited AI bill.</t>
         </is>
       </c>
       <c r="E43" s="4" t="inlineStr">
@@ -2231,7 +2231,7 @@
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>The rate limiter trusted the first IP in the X-Forwarded-For header, which any attacker can spoof</t>
+          <t>The rate limiter trusted the first IP in the X-Forwarded-For header, which can easily be faked</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
@@ -2310,7 +2310,7 @@
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>An attacker with a stolen session could brute-force password changes; upload/report endpoints could be abused to run up server costs.</t>
+          <t>Repeated password-change attempts could be used for account takeover; upload/report endpoints could be abused to run up server costs.</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr">
@@ -2379,7 +2379,7 @@
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>On the first Redis failure the client switched to per-process memory FOREVER — distributed locks, payment idempotency and rate limits silently degraded</t>
+          <t>On the first Redis failure the client switched to per-process memory until a restart — distributed locks, payment idempotency and rate limits silently degraded</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
@@ -2794,7 +2794,7 @@
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Deploys stop being a gamble; regressions are caught before customers see them.</t>
+          <t>Deploys become predictable; regressions are caught before customers see them.</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
@@ -3000,7 +3000,7 @@
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>A competitor could take the site down with a Rs.500 botnet.</t>
+          <t>Large fake-traffic attacks are inexpensive to launch and could make the site unavailable on important days.</t>
         </is>
       </c>
     </row>
@@ -3031,7 +3031,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="60" customHeight="1">
+    <row r="10" ht="61" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
           <t>P-06</t>
@@ -3044,7 +3044,7 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>The June security audit logged 36 findings. The Critical and nearly all High items are fixed. Mediums still being worked through include: login-token cache window (~10 min), unsigned OAuth state parameter, an unauthenticated competitor data-freshness endpoint, and stale analytics cache invalidation.</t>
+          <t>The June security audit logged 36 findings. The Critical issue and most High items are fixed. Items still being worked through include: the login-token cache window (~10 min), the unsigned OAuth state parameter, an unauthenticated competitor data-freshness endpoint, and stale analytics cache invalidation.</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
@@ -3054,7 +3054,7 @@
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Each one is a small hole today; at bigger scale, small holes are what hackers chain together.</t>
+          <t>Each one is a small gap today; closing them before scale keeps the risk small.</t>
         </is>
       </c>
     </row>
@@ -3276,12 +3276,12 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>A competitor launches a DDoS attack (fake traffic on the booking engine)</t>
+          <t>The site receives a flood of fake traffic (a DDoS attack) on the booking engine</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>The site goes down on a peak day; real guests cannot book; the hosting bill explodes</t>
+          <t>The site goes down on a peak day; real guests cannot book; the hosting bill rises sharply</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -3318,17 +3318,17 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>A hacker hunts for data-isolation bugs in new endpoints (Hotel A accessing Hotel B's data)</t>
+          <t>Someone deliberately probes new endpoints for data-isolation gaps (Hotel A accessing Hotel B's data)</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>One tenant-isolation bug = a data breach = every hotel customer loses trust in us + DPDP penalties</t>
+          <t>A single tenant-isolation bug would mean a data breach — loss of customer trust and possible DPDP penalties</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Every new feature = a new endpoint = a new risk; right now only one person reviews everything</t>
+          <t>Every new feature adds new endpoints to protect; right now only one person reviews everything</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
@@ -3528,7 +3528,7 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>A hotelier uploads a wrong CSV/photo (or a malicious file)</t>
+          <t>A hotelier uploads a wrong or unsafe CSV/photo file</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
@@ -3659,7 +3659,7 @@
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Losing every hotel's data = a company-ending event</t>
+          <t>Losing every hotel's data would be a loss the business could not recover from</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">

</xml_diff>

<commit_message>
docs: Add architecture diagram and enhance CEO report Team & Hiring section
- Add Staybooker_Architecture.excalidraw — full system architecture diagram
  with 16 embedded SVG logos (FastAPI, Redis, React, Supabase, Cloudflare,
  Razorpay, Groq AI, WhatsApp, PostgreSQL, Railway, etc.) and annotated
  request-flow arrows across all five zones

- Update CEO_Report_Staybooker_Jun2026.xlsx:
  - Rewrite Sheet 6 (Team & Hiring) with plain-language role descriptions,
    5-force explanation of why software needs continuous engineering, and
    90-day hiring priorities
  - Add Sheet 7 (Architecture Overview) — tech layer table, 7-step booking
    flow, and security controls summary for non-technical stakeholders

https://claude.ai/code/session_01JSXri7YwDXxadMbDuW5jEw
</commit_message>
<xml_diff>
--- a/docs/CEO_Report_Staybooker_Jun2026.xlsx
+++ b/docs/CEO_Report_Staybooker_Jun2026.xlsx
@@ -13,6 +13,7 @@
     <sheet name="4. Work In Progress" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="5. Future Risks" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="6. Team &amp; Hiring" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="7. Architecture" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -53,8 +54,53 @@
       <color rgb="001F4E79"/>
       <sz val="12"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00475569"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00000000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00334155"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="18">
     <fill>
       <patternFill/>
     </fill>
@@ -86,8 +132,63 @@
         <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000F172A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8FAFC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001E3A5F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F1F5F9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F0FDF4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EFF6FF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEFCE8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000F4C75"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="007F1D1D"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -109,11 +210,25 @@
         <color rgb="00BBBBBB"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D1D5DB"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D1D5DB"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D1D5DB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D1D5DB"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -135,6 +250,72 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="13" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="13" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="14" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="14" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="15" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="15" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -3703,406 +3884,1461 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="56" customWidth="1" min="3" max="3"/>
-    <col width="56" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Team &amp; Hiring — Decision Support</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>The product is stable today and data is safe. This sheet maps which role owns which part as the business grows.</t>
+    <row r="1" ht="42" customHeight="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>Staybooker — Team &amp; Growth Plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>What each developer does and why we need one — in plain language</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
-        <is>
-          <t>WHERE THE PRODUCT STANDS TODAY</t>
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>A.  Where The Product Stands Today</t>
         </is>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Area</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="12" t="inlineStr">
         <is>
           <t>Current Status</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="38" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
+    <row r="6" ht="52" customHeight="1">
+      <c r="A6" s="13" t="inlineStr">
         <is>
           <t>Product stability</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>Stable for current hoteliers — bookings, payments, dashboards and integrations are working. 45 issues have been found and fixed proactively, and 277 automated tests now run on every code change.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="37" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="B6" s="14" t="inlineStr">
+        <is>
+          <t>Stable for current hotels. 45 security and performance issues fixed proactively. 277 automated tests run on every code change so regressions are caught before any hotel sees them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="52" customHeight="1">
+      <c r="A7" s="13" t="inlineStr">
         <is>
           <t>Data safety</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>Safe — all credentials are encrypted (AES-256 vault), every hotel's data is isolated at both the application and the database level, and payment amounts are always verified on the server.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>Hotelier experience</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>No major issues expected at today's scale. The public booking flow has been hardened (error recovery, date validation, double-payment protection).</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="40" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>Why hiring, then</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>Growth. As hotels onboard, data will reach GBs and traffic will multiply. Each layer of the product — database, backend, frontend — then needs a dedicated owner so quality stays exactly where it is today.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10"/>
+      <c r="B7" s="14" t="inlineStr">
+        <is>
+          <t>Every hotel's data is isolated — Hotel A cannot see Hotel B's records. All payment and messaging credentials (Razorpay, WhatsApp, Email) are stored AES-256-GCM encrypted. Payment amounts are always verified on the server — a guest cannot manipulate the price from the browser.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="52" customHeight="1">
+      <c r="A8" s="13" t="inlineStr">
+        <is>
+          <t>Guest booking flow</t>
+        </is>
+      </c>
+      <c r="B8" s="14" t="inlineStr">
+        <is>
+          <t>Public booking widget is hardened: date validation, error-recovery with retry button, double-payment protection, real-time availability, no fake data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="52" customHeight="1">
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>Team today</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="inlineStr">
+        <is>
+          <t>Currently one senior developer covering the entire stack (backend, frontend, database, DevOps, security). Stable at today's scale. Hiring need is driven by growth — not by anything broken.</t>
+        </is>
+      </c>
+    </row>
     <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="8" t="inlineStr">
-        <is>
-          <t>HOW DATA TRAVELS THROUGH THE PRODUCT — AND WHO OWNS EACH STEP</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>Step in the Data Journey</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>Owner</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>Exact Job</t>
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>B.  Why Software Always Needs Ongoing Engineering</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="50" customHeight="1">
+      <c r="A12" s="15" t="inlineStr">
+        <is>
+          <t>A common and understandable question: 'Once the bugs are fixed, isn't it done?' The answer is no — and the reason is not quality of work. Here are the 5 forces that create new engineering work continuously:</t>
         </is>
       </c>
     </row>
     <row r="13" ht="41" customHeight="1">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>1. Data lives in the database (bookings, rates, guests)</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>Database Dev</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>Makes sure data comes OUT of the database smoothly — right indexes, fast queries, clean schema, reliable backups, per-hotel isolation. When data reaches GBs: partitioning and archiving so queries stay fast.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="46" customHeight="1">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>2. Backend picks up the data and serves it through APIs</t>
-        </is>
-      </c>
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>Backend Dev</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>Connects the backend APIs to the database properly — booking logic, payment processing, security checks. When data reaches GBs: sends it in CHUNKS (pagination, batching, caching) so the server never tries to load everything at once.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="59" customHeight="1">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>3. Frontend calls those APIs and shows the data on screen</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>Frontend Dev</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>Connects the React + TypeScript frontend to the backend APIs and makes sure the data arrives and displays correctly — loading states, error handling, payment screens. When data reaches GBs: loads it smoothly on screen (paged lists, lazy loading) so pages stay fast for the hotelier and the guest.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="33" customHeight="1">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>4. Someone decides what gets built, in what order, and signs off</t>
-        </is>
-      </c>
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>Tech Lead</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>Decides what happens in the project — what each developer builds and when, reviews every change before release, and carries the overall responsibility for the software.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="8" t="inlineStr">
-        <is>
-          <t>ROLE SUMMARY — WITH EXAMPLES FROM OUR OWN PROJECT</t>
-        </is>
-      </c>
-    </row>
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>Force</t>
+        </is>
+      </c>
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>What It Means</t>
+        </is>
+      </c>
+      <c r="C13" s="12" t="inlineStr">
+        <is>
+          <t>Real Example from Staybooker</t>
+        </is>
+      </c>
+      <c r="D13" s="12" t="inlineStr">
+        <is>
+          <t>Risk if Ignored</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="70" customHeight="1">
+      <c r="A14" s="16" t="inlineStr">
+        <is>
+          <t>1. Growth</t>
+        </is>
+      </c>
+      <c r="B14" s="14" t="inlineStr">
+        <is>
+          <t>As more hotels join and more guests book, the system carries more data and more simultaneous users. What runs fast for 5 hotels can be slow for 50.</t>
+        </is>
+      </c>
+      <c r="C14" s="14" t="inlineStr">
+        <is>
+          <t>Today's availability search is fast. At 100 hotels with 3 years of bookings, the same query can take 15-20 seconds without index tuning and data archiving.</t>
+        </is>
+      </c>
+      <c r="D14" s="14" t="inlineStr">
+        <is>
+          <t>Slow pages = guests leave mid-booking = direct revenue loss.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="70" customHeight="1">
+      <c r="A15" s="17" t="inlineStr">
+        <is>
+          <t>2. New Features</t>
+        </is>
+      </c>
+      <c r="B15" s="18" t="inlineStr">
+        <is>
+          <t>Every feature we add (new payment method, new OTA, loyalty tier) creates new code paths that need testing, security review, and integration.</t>
+        </is>
+      </c>
+      <c r="C15" s="18" t="inlineStr">
+        <is>
+          <t>Adding UPI payments requires a new Razorpay flow, new webhook handling, new idempotency logic, and new test coverage.</t>
+        </is>
+      </c>
+      <c r="D15" s="18" t="inlineStr">
+        <is>
+          <t>Untested code in a payment flow = double charges or missing bookings.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="70" customHeight="1">
+      <c r="A16" s="16" t="inlineStr">
+        <is>
+          <t>3. Third-Party Changes</t>
+        </is>
+      </c>
+      <c r="B16" s="14" t="inlineStr">
+        <is>
+          <t>Our system depends on Razorpay, Supabase, WhatsApp, Groq — all of which update their APIs, change their authentication, or modify rate limits.</t>
+        </is>
+      </c>
+      <c r="C16" s="14" t="inlineStr">
+        <is>
+          <t>When Razorpay changes their webhook signature format, our verification code must be updated within their deadline or payments stop confirming.</t>
+        </is>
+      </c>
+      <c r="D16" s="14" t="inlineStr">
+        <is>
+          <t>Missed API update = booking failures with no warning to guests or hotels.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="70" customHeight="1">
+      <c r="A17" s="17" t="inlineStr">
+        <is>
+          <t>4. Traffic Events</t>
+        </is>
+      </c>
+      <c r="B17" s="18" t="inlineStr">
+        <is>
+          <t>A viral campaign, a festival sale, or press coverage can send 100x normal traffic in minutes. The system must be tested and tuned for this in advance.</t>
+        </is>
+      </c>
+      <c r="C17" s="18" t="inlineStr">
+        <is>
+          <t>Load testing (P-02) is currently in progress specifically to validate behaviour under simultaneous booking spikes before a large campaign runs.</t>
+        </is>
+      </c>
+      <c r="D17" s="18" t="inlineStr">
+        <is>
+          <t>Site down on the highest-revenue day of the year.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="70" customHeight="1">
+      <c r="A18" s="16" t="inlineStr">
+        <is>
+          <t>5. Security Landscape</t>
+        </is>
+      </c>
+      <c r="B18" s="14" t="inlineStr">
+        <is>
+          <t>Attack methods evolve. A technique that did not exist last year may affect our stack today. Regular review catches these before they become incidents.</t>
+        </is>
+      </c>
+      <c r="C18" s="14" t="inlineStr">
+        <is>
+          <t>The IP-spoofing bypass on rate limits (S-40) is a category of attack that became prevalent only in the last 2 years — it was proactively found and fixed.</t>
+        </is>
+      </c>
+      <c r="D18" s="14" t="inlineStr">
+        <is>
+          <t>Data breach, DPDP penalty, loss of hotel trust, possible legal liability.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1"/>
     <row r="20" ht="30" customHeight="1">
-      <c r="A20" s="3" t="inlineStr">
+      <c r="A20" s="11" t="inlineStr">
+        <is>
+          <t>C.  How The Product Works — Data Journey (Plain Language)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="37" customHeight="1">
+      <c r="A21" s="12" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="B21" s="12" t="inlineStr">
+        <is>
+          <t>What Guest / Hotelier Does</t>
+        </is>
+      </c>
+      <c r="C21" s="12" t="inlineStr">
+        <is>
+          <t>Which System Handles It</t>
+        </is>
+      </c>
+      <c r="D21" s="12" t="inlineStr">
+        <is>
+          <t>What Happens Technically (Simple)</t>
+        </is>
+      </c>
+      <c r="E21" s="12" t="inlineStr">
+        <is>
+          <t>Developer Owner</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="58" customHeight="1">
+      <c r="A22" s="19" t="inlineStr">
+        <is>
+          <t>Step 1</t>
+        </is>
+      </c>
+      <c r="B22" s="20" t="inlineStr">
+        <is>
+          <t>Guest searches availability on hotel website</t>
+        </is>
+      </c>
+      <c r="C22" s="20" t="inlineStr">
+        <is>
+          <t>Cloudflare CDN + React Frontend</t>
+        </is>
+      </c>
+      <c r="D22" s="20" t="inlineStr">
+        <is>
+          <t>Loads the booking page instantly from the nearest global server. No load on our backend for static pages.</t>
+        </is>
+      </c>
+      <c r="E22" s="20" t="inlineStr">
+        <is>
+          <t>Frontend Developer</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="58" customHeight="1">
+      <c r="A23" s="17" t="inlineStr">
+        <is>
+          <t>Step 2</t>
+        </is>
+      </c>
+      <c r="B23" s="18" t="inlineStr">
+        <is>
+          <t>Search request reaches our backend</t>
+        </is>
+      </c>
+      <c r="C23" s="18" t="inlineStr">
+        <is>
+          <t>FastAPI on Railway</t>
+        </is>
+      </c>
+      <c r="D23" s="18" t="inlineStr">
+        <is>
+          <t>Backend checks authentication, enforces rate limits (via Redis), queries Supabase for available rooms, returns results.</t>
+        </is>
+      </c>
+      <c r="E23" s="18" t="inlineStr">
+        <is>
+          <t>Backend Developer</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="58" customHeight="1">
+      <c r="A24" s="19" t="inlineStr">
+        <is>
+          <t>Step 3</t>
+        </is>
+      </c>
+      <c r="B24" s="20" t="inlineStr">
+        <is>
+          <t>Guest confirms booking and pays</t>
+        </is>
+      </c>
+      <c r="C24" s="20" t="inlineStr">
+        <is>
+          <t>Razorpay + FastAPI</t>
+        </is>
+      </c>
+      <c r="D24" s="20" t="inlineStr">
+        <is>
+          <t>Backend creates a Razorpay order with the server-calculated amount, receives payment webhook, verifies HMAC signature, marks booking CONFIRMED.</t>
+        </is>
+      </c>
+      <c r="E24" s="20" t="inlineStr">
+        <is>
+          <t>Backend Developer</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="58" customHeight="1">
+      <c r="A25" s="17" t="inlineStr">
+        <is>
+          <t>Step 4</t>
+        </is>
+      </c>
+      <c r="B25" s="18" t="inlineStr">
+        <is>
+          <t>Confirmation email + OTA sync triggered</t>
+        </is>
+      </c>
+      <c r="C25" s="18" t="inlineStr">
+        <is>
+          <t>Background Task Queue</t>
+        </is>
+      </c>
+      <c r="D25" s="18" t="inlineStr">
+        <is>
+          <t>Backend queues email and channel sync tasks. These run in the background so the guest gets their confirmation screen immediately.</t>
+        </is>
+      </c>
+      <c r="E25" s="18" t="inlineStr">
+        <is>
+          <t>Backend Developer</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="58" customHeight="1">
+      <c r="A26" s="19" t="inlineStr">
+        <is>
+          <t>Step 5</t>
+        </is>
+      </c>
+      <c r="B26" s="20" t="inlineStr">
+        <is>
+          <t>Hotelier opens dashboard</t>
+        </is>
+      </c>
+      <c r="C26" s="20" t="inlineStr">
+        <is>
+          <t>React + FastAPI</t>
+        </is>
+      </c>
+      <c r="D26" s="20" t="inlineStr">
+        <is>
+          <t>Dashboard loads only the hotel's own data (tenant isolation). Real-time WebSocket pushes new bookings without page refresh.</t>
+        </is>
+      </c>
+      <c r="E26" s="20" t="inlineStr">
+        <is>
+          <t>Frontend + Backend</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="58" customHeight="1">
+      <c r="A27" s="17" t="inlineStr">
+        <is>
+          <t>Step 6</t>
+        </is>
+      </c>
+      <c r="B27" s="18" t="inlineStr">
+        <is>
+          <t>Data grows to GBs over time</t>
+        </is>
+      </c>
+      <c r="C27" s="18" t="inlineStr">
+        <is>
+          <t>PostgreSQL + Redis</t>
+        </is>
+      </c>
+      <c r="D27" s="18" t="inlineStr">
+        <is>
+          <t>Database indexes, table partitioning, and Redis caching ensure queries stay fast even as booking history grows across 2-3 years.</t>
+        </is>
+      </c>
+      <c r="E27" s="18" t="inlineStr">
+        <is>
+          <t>Database Developer</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="30" customHeight="1"/>
+    <row r="29" ht="30" customHeight="1">
+      <c r="A29" s="11" t="inlineStr">
+        <is>
+          <t>D.  What Each Developer Actually Does</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="30" customHeight="1">
+      <c r="A30" s="12" t="inlineStr">
         <is>
           <t>Role</t>
         </is>
       </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>In One Line</t>
-        </is>
-      </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>Examples of This Work Already Done in the Product</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="37" customHeight="1">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>Tech Lead</t>
-        </is>
-      </c>
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>Responsible for the whole software — decides what every developer works on, reviews everything, owns delivery.</t>
-        </is>
-      </c>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>Prioritised the fix order across 45 issues (money-related first); set the engineering rules and the review checklist the team now follows; set up the CI pipeline that tests every change.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="39" customHeight="1">
-      <c r="A22" s="4" t="inlineStr">
-        <is>
-          <t>Backend Dev</t>
-        </is>
-      </c>
-      <c r="B22" s="4" t="inlineStr">
-        <is>
-          <t>Owns backend APIs and their connection to the database — payments, booking logic, security, performance.</t>
-        </is>
-      </c>
-      <c r="C22" s="4" t="inlineStr">
-        <is>
-          <t>Server-side payment verification (amount can never be tampered from the browser); double-payment protection when a guest's network fails; pagination on heavy endpoints; rate limits against abuse.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="42" customHeight="1">
-      <c r="A23" s="4" t="inlineStr">
-        <is>
-          <t>Frontend Dev</t>
-        </is>
-      </c>
-      <c r="B23" s="4" t="inlineStr">
-        <is>
-          <t>Owns the React + TypeScript screens and their connection to backend APIs — correct data display, smooth experience.</t>
-        </is>
-      </c>
-      <c r="C23" s="4" t="inlineStr">
-        <is>
-          <t>Error + retry handling on the booking pages (a network blip no longer shows a blank page); date validation before search; live-updating dashboards; checkout flow with loyalty points calculated safely via the API.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="35" customHeight="1">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t>Database Dev</t>
-        </is>
-      </c>
-      <c r="B24" s="4" t="inlineStr">
-        <is>
-          <t>Owns the database — speed, schema, backups, and the guarantee that data flows out smoothly at any size.</t>
-        </is>
-      </c>
-      <c r="C24" s="4" t="inlineStr">
-        <is>
-          <t>Database-level isolation between hotels (Row Level Security); composite indexes on the busiest availability queries; encrypted credential storage; chain-level loyalty data design.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27" ht="30" customHeight="1">
-      <c r="A27" s="8" t="inlineStr">
-        <is>
-          <t>SUGGESTED HIRING ORDER</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="30" customHeight="1">
-      <c r="A28" s="3" t="inlineStr">
+      <c r="B30" s="12" t="inlineStr">
+        <is>
+          <t>In Plain Language</t>
+        </is>
+      </c>
+      <c r="C30" s="12" t="inlineStr">
+        <is>
+          <t>Examples from This Product</t>
+        </is>
+      </c>
+      <c r="D30" s="12" t="inlineStr">
+        <is>
+          <t>When to Hire</t>
+        </is>
+      </c>
+      <c r="E30" s="12" t="inlineStr">
+        <is>
+          <t>Focus in First 90 Days</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="72" customHeight="1">
+      <c r="A31" s="21" t="inlineStr">
+        <is>
+          <t>🔷  Tech Lead</t>
+        </is>
+      </c>
+      <c r="B31" s="22" t="inlineStr">
+        <is>
+          <t>Owns the overall product. Decides what to build and in what order. Reviews every code change before it is deployed. Owns delivery.</t>
+        </is>
+      </c>
+      <c r="C31" s="22" t="inlineStr">
+        <is>
+          <t>Set fix priority (money-related first). Wrote engineering rules the team now follows. Set up CI/CD pipeline that tests every change.</t>
+        </is>
+      </c>
+      <c r="D31" s="22" t="inlineStr">
+        <is>
+          <t>Day 1 with first hire — direction and review from the start.</t>
+        </is>
+      </c>
+      <c r="E31" s="22" t="inlineStr">
+        <is>
+          <t>Technical roadmap · Review process · Sprint planning · Mentoring</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="72" customHeight="1">
+      <c r="A32" s="19" t="inlineStr">
+        <is>
+          <t>🟢  Backend Developer</t>
+        </is>
+      </c>
+      <c r="B32" s="20" t="inlineStr">
+        <is>
+          <t>Builds and maintains the API server (FastAPI/Python). Owns payment flows, booking logic, security middleware, and performance.</t>
+        </is>
+      </c>
+      <c r="C32" s="20" t="inlineStr">
+        <is>
+          <t>Server-side payment verification · Double-payment protection · Pagination on heavy endpoints · Rate limits against abuse.</t>
+        </is>
+      </c>
+      <c r="D32" s="20" t="inlineStr">
+        <is>
+          <t>First hire — payment recovery and load testing are the immediate priority.</t>
+        </is>
+      </c>
+      <c r="E32" s="20" t="inlineStr">
+        <is>
+          <t>Payment recovery · Load testing · Abuse protection · New API features</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="72" customHeight="1">
+      <c r="A33" s="23" t="inlineStr">
+        <is>
+          <t>🟡  Frontend Developer</t>
+        </is>
+      </c>
+      <c r="B33" s="24" t="inlineStr">
+        <is>
+          <t>Builds the React screens and connects them to APIs. Owns the guest booking experience and the hotelier dashboard. Owns page speed.</t>
+        </is>
+      </c>
+      <c r="C33" s="24" t="inlineStr">
+        <is>
+          <t>Error + retry on booking pages · Date validation · Live dashboards · Checkout flow with loyalty points via API.</t>
+        </is>
+      </c>
+      <c r="D33" s="24" t="inlineStr">
+        <is>
+          <t>Second hire — hotelier dashboard pages need the same hardening the public booking pages already received.</t>
+        </is>
+      </c>
+      <c r="E33" s="24" t="inlineStr">
+        <is>
+          <t>Dashboard error handling · Page speed · New UI features · Mobile</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="72" customHeight="1">
+      <c r="A34" s="21" t="inlineStr">
+        <is>
+          <t>🔵  Database Developer</t>
+        </is>
+      </c>
+      <c r="B34" s="22" t="inlineStr">
+        <is>
+          <t>Owns the database — speed, schema, backups, and data safety. Ensures queries stay fast as data grows to GBs.</t>
+        </is>
+      </c>
+      <c r="C34" s="22" t="inlineStr">
+        <is>
+          <t>Row Level Security (tenant isolation at DB level) · Composite indexes on availability queries · Encrypted credential storage.</t>
+        </is>
+      </c>
+      <c r="D34" s="22" t="inlineStr">
+        <is>
+          <t>Third hire — becomes essential as hotels approach GB-scale data and backup restore drills are needed.</t>
+        </is>
+      </c>
+      <c r="E34" s="22" t="inlineStr">
+        <is>
+          <t>Migrations · Backup drills · Query tuning · Partitioning for scale</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="11" t="inlineStr">
+        <is>
+          <t>E.  Recommended Hiring Order &amp; Immediate Priorities</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="25" t="inlineStr">
         <is>
           <t>Priority</t>
         </is>
       </c>
-      <c r="B28" s="3" t="inlineStr">
+      <c r="B37" s="25" t="inlineStr">
         <is>
           <t>Role</t>
         </is>
       </c>
-      <c r="C28" s="3" t="inlineStr">
-        <is>
-          <t>Why This Order</t>
-        </is>
-      </c>
-      <c r="D28" s="3" t="inlineStr">
-        <is>
-          <t>Focus in the First 90 Days</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="30" customHeight="1">
-      <c r="A29" s="4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B29" s="4" t="inlineStr">
-        <is>
-          <t>Backend Dev</t>
-        </is>
-      </c>
-      <c r="C29" s="4" t="inlineStr">
-        <is>
-          <t>The next milestones are payment-recovery automation and handling high booking traffic — both backend work.</t>
-        </is>
-      </c>
-      <c r="D29" s="4" t="inlineStr">
-        <is>
-          <t>Automatic refund + payment reconciliation; load testing the booking path; finishing the abuse-protection layer.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="30" customHeight="1">
-      <c r="A30" s="4" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B30" s="4" t="inlineStr">
-        <is>
-          <t>Frontend Dev</t>
-        </is>
-      </c>
-      <c r="C30" s="4" t="inlineStr">
-        <is>
-          <t>The hotelier dashboard pages are next in line for the same error-handling polish the public booking pages already received.</t>
-        </is>
-      </c>
-      <c r="D30" s="4" t="inlineStr">
-        <is>
-          <t>API integration hardening on every dashboard page; page speed optimisation; error monitoring.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="30" customHeight="1">
-      <c r="A31" s="4" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B31" s="4" t="inlineStr">
-        <is>
-          <t>Database Dev</t>
-        </is>
-      </c>
-      <c r="C31" s="4" t="inlineStr">
-        <is>
-          <t>Becomes essential as data approaches GB scale; can begin part-time and grow with the data.</t>
-        </is>
-      </c>
-      <c r="D31" s="4" t="inlineStr">
-        <is>
-          <t>Migration process; backup restore drills; query and index plan for large hotels; capacity plan for onboarding more hotels.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="30" customHeight="1">
-      <c r="A32" s="4" t="inlineStr">
-        <is>
-          <t>With the first hire</t>
-        </is>
-      </c>
-      <c r="B32" s="4" t="inlineStr">
-        <is>
-          <t>Tech Lead</t>
-        </is>
-      </c>
-      <c r="C32" s="4" t="inlineStr">
-        <is>
-          <t>Direction and review from day one keeps all the above work consistent. Can be a hands-on senior developer.</t>
-        </is>
-      </c>
-      <c r="D32" s="4" t="inlineStr">
-        <is>
-          <t>Technical roadmap; review process; assigning and supervising the work above.</t>
+      <c r="C37" s="25" t="inlineStr">
+        <is>
+          <t>What They Build in First 90 Days</t>
+        </is>
+      </c>
+      <c r="D37" s="25" t="inlineStr">
+        <is>
+          <t>Business Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="72" customHeight="1">
+      <c r="A38" s="21" t="inlineStr">
+        <is>
+          <t>1st</t>
+        </is>
+      </c>
+      <c r="B38" s="21" t="inlineStr">
+        <is>
+          <t>Backend Developer</t>
+        </is>
+      </c>
+      <c r="C38" s="22" t="inlineStr">
+        <is>
+          <t>Payment failure auto-recovery (P-01) — when a guest's network drops mid-payment, today refunds are manual. This must be automated.
+Load testing under 100+ simultaneous bookings (P-02).
+Completing the abuse/DDoS protection layer (P-04).</t>
+        </is>
+      </c>
+      <c r="D38" s="22" t="inlineStr">
+        <is>
+          <t>₹ Revenue protection · Guest trust · System reliability</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="72" customHeight="1">
+      <c r="A39" s="19" t="inlineStr">
+        <is>
+          <t>2nd</t>
+        </is>
+      </c>
+      <c r="B39" s="19" t="inlineStr">
+        <is>
+          <t>Frontend Developer</t>
+        </is>
+      </c>
+      <c r="C39" s="20" t="inlineStr">
+        <is>
+          <t>Hotelier dashboard pages need the same error-handling polish the public booking widget already received — every page must handle network failures, double-clicks, and slow-data scenarios gracefully.
+Page speed optimisation (Core Web Vitals) — every extra second of load time reduces conversions by ~7%.</t>
+        </is>
+      </c>
+      <c r="D39" s="20" t="inlineStr">
+        <is>
+          <t>₹ Conversion rate · Hotelier experience · Brand quality</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="72" customHeight="1">
+      <c r="A40" s="23" t="inlineStr">
+        <is>
+          <t>3rd</t>
+        </is>
+      </c>
+      <c r="B40" s="23" t="inlineStr">
+        <is>
+          <t>Database Developer</t>
+        </is>
+      </c>
+      <c r="C40" s="24" t="inlineStr">
+        <is>
+          <t>Migration process (Alembic) — structured schema changes instead of ad-hoc scripts.
+Backup restore drills — quarterly test that data can actually be recovered.
+Query tuning and partitioning plan for when data reaches GB scale.</t>
+        </is>
+      </c>
+      <c r="D40" s="24" t="inlineStr">
+        <is>
+          <t>₹ Data safety · Long-term performance · Business continuity</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="72" customHeight="1">
+      <c r="A41" s="26" t="inlineStr">
+        <is>
+          <t>With 1st hire</t>
+        </is>
+      </c>
+      <c r="B41" s="26" t="inlineStr">
+        <is>
+          <t>Tech Lead / Senior Dev</t>
+        </is>
+      </c>
+      <c r="C41" s="27" t="inlineStr">
+        <is>
+          <t>Sets technical direction from day one. Reviews every change. Prevents the common trap where each new hire introduces inconsistent patterns that become expensive to fix later. Can be a hands-on senior developer who also codes.</t>
+        </is>
+      </c>
+      <c r="D41" s="27" t="inlineStr">
+        <is>
+          <t>📐 Consistency · Quality · Speed of delivery</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="48" customHeight="1">
+      <c r="A44" s="28" t="inlineStr">
+        <is>
+          <t>📌  The product is stable and secure today. Hiring is driven purely by growth — as hotels onboard and traffic scales, each layer of the system needs a dedicated owner so quality and safety stay exactly where they are right now.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="13">
+    <mergeCell ref="B9:E9"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="B8:E8"/>
+    <mergeCell ref="A12:E12"/>
+    <mergeCell ref="A20:E20"/>
     <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A29:E29"/>
+    <mergeCell ref="B6:E6"/>
+    <mergeCell ref="A11:E11"/>
+    <mergeCell ref="B7:E7"/>
     <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A36:E36"/>
+    <mergeCell ref="A44:E44"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E39"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="42" customHeight="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>Staybooker — System Architecture Overview</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="24" customHeight="1">
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>How every part of the product connects — in plain language  ·  See Staybooker_Architecture.excalidraw for the visual diagram</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>A.  Technology Layers — What Each Service Does</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>SERVICE</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>TECHNOLOGY</t>
+        </is>
+      </c>
+      <c r="C5" s="12" t="inlineStr">
+        <is>
+          <t>HOSTED ON</t>
+        </is>
+      </c>
+      <c r="D5" s="12" t="inlineStr">
+        <is>
+          <t>WHAT IT DOES</t>
+        </is>
+      </c>
+      <c r="E5" s="12" t="inlineStr">
+        <is>
+          <t>WHY THIS CHOICE</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="72" customHeight="1">
+      <c r="A6" s="16" t="inlineStr">
+        <is>
+          <t>Frontend
+(What guests &amp; hoteliers see)</t>
+        </is>
+      </c>
+      <c r="B6" s="14" t="inlineStr">
+        <is>
+          <t>React 18 · Vite · TailwindCSS</t>
+        </is>
+      </c>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>Cloudflare Pages
+(Global CDN)</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>Renders the booking widget on hotel websites and the hotelier management dashboard. Caches API data locally for 5 minutes so the page feels instant.</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="inlineStr">
+        <is>
+          <t>Cloudflare's CDN delivers pages from the nearest global server — fast load even on slow mobile connections. Zero server cost for static pages.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="72" customHeight="1">
+      <c r="A7" s="17" t="inlineStr">
+        <is>
+          <t>Backend API
+(The brain of the system)</t>
+        </is>
+      </c>
+      <c r="B7" s="18" t="inlineStr">
+        <is>
+          <t>Python 3.11 · FastAPI</t>
+        </is>
+      </c>
+      <c r="C7" s="18" t="inlineStr">
+        <is>
+          <t>Railway
+(Cloud Server)</t>
+        </is>
+      </c>
+      <c r="D7" s="18" t="inlineStr">
+        <is>
+          <t>Handles all business rules: creates bookings, verifies payments, enforces roles (who can do what), runs the AI assistant, sends emails and WhatsApp messages.</t>
+        </is>
+      </c>
+      <c r="E7" s="18" t="inlineStr">
+        <is>
+          <t>FastAPI is the fastest Python API framework. Railway auto-scales with traffic and provides zero-downtime deploys.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="72" customHeight="1">
+      <c r="A8" s="16" t="inlineStr">
+        <is>
+          <t>Primary Database
+(All hotel data)</t>
+        </is>
+      </c>
+      <c r="B8" s="14" t="inlineStr">
+        <is>
+          <t>PostgreSQL
+(via Supabase)</t>
+        </is>
+      </c>
+      <c r="C8" s="14" t="inlineStr">
+        <is>
+          <t>Supabase
+(Managed Cloud DB)</t>
+        </is>
+      </c>
+      <c r="D8" s="14" t="inlineStr">
+        <is>
+          <t>Stores every booking, guest record, room, rate, loyalty point, and setting. Row Level Security ensures Hotel A can never read Hotel B's data — enforced at the database level, not just in code.</t>
+        </is>
+      </c>
+      <c r="E8" s="14" t="inlineStr">
+        <is>
+          <t>Supabase provides managed Postgres with built-in auth, automated backups, and a secure secrets vault at predictable cost.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="72" customHeight="1">
+      <c r="A9" s="17" t="inlineStr">
+        <is>
+          <t>Auth &amp; Identity
+(Who is who)</t>
+        </is>
+      </c>
+      <c r="B9" s="18" t="inlineStr">
+        <is>
+          <t>Supabase Auth · JWT</t>
+        </is>
+      </c>
+      <c r="C9" s="18" t="inlineStr">
+        <is>
+          <t>Supabase</t>
+        </is>
+      </c>
+      <c r="D9" s="18" t="inlineStr">
+        <is>
+          <t>Every login issues a short-lived token (15-30 min). The backend verifies this token on every request. Roles (OWNER / MANAGER / STAFF) are checked server-side on every action.</t>
+        </is>
+      </c>
+      <c r="E9" s="18" t="inlineStr">
+        <is>
+          <t>Supabase Auth handles password hashing, OAuth, and token rotation so we do not build auth from scratch — a common source of security vulnerabilities.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="72" customHeight="1">
+      <c r="A10" s="16" t="inlineStr">
+        <is>
+          <t>Cache &amp; Rate Limiting
+(Speed &amp; protection)</t>
+        </is>
+      </c>
+      <c r="B10" s="14" t="inlineStr">
+        <is>
+          <t>Redis</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="inlineStr">
+        <is>
+          <t>Railway
+(Internal Network)</t>
+        </is>
+      </c>
+      <c r="D10" s="14" t="inlineStr">
+        <is>
+          <t>Stores frequently-read data so the database is not hit on every request. Tracks API call counts per IP and per hotel to block abuse. Holds distributed locks so two bookings cannot claim the same room simultaneously. Falls back to in-memory cache if Redis is unavailable.</t>
+        </is>
+      </c>
+      <c r="E10" s="14" t="inlineStr">
+        <is>
+          <t>Redis is the industry standard for in-memory caching. Hosting on the same Railway network means &lt; 1 ms latency to the backend.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="72" customHeight="1">
+      <c r="A11" s="17" t="inlineStr">
+        <is>
+          <t>Payment Gateway
+(Money in / out)</t>
+        </is>
+      </c>
+      <c r="B11" s="18" t="inlineStr">
+        <is>
+          <t>Razorpay</t>
+        </is>
+      </c>
+      <c r="C11" s="18" t="inlineStr">
+        <is>
+          <t>External — Razorpay Cloud</t>
+        </is>
+      </c>
+      <c r="D11" s="18" t="inlineStr">
+        <is>
+          <t>Handles credit card, UPI, and net-banking payments. Sends webhook notifications when payment succeeds or fails. All amounts are calculated on our server — the browser cannot alter the price.</t>
+        </is>
+      </c>
+      <c r="E11" s="18" t="inlineStr">
+        <is>
+          <t>Razorpay is the leading Indian payment gateway with deep UPI support, strong fraud detection, and a clear dispute resolution process.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="72" customHeight="1">
+      <c r="A12" s="16" t="inlineStr">
+        <is>
+          <t>AI Assistant
+(Chatbot &amp; analytics)</t>
+        </is>
+      </c>
+      <c r="B12" s="14" t="inlineStr">
+        <is>
+          <t>Groq API · LLaMA 3.1</t>
+        </is>
+      </c>
+      <c r="C12" s="14" t="inlineStr">
+        <is>
+          <t>External — Groq Cloud</t>
+        </is>
+      </c>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
+          <t>Powers the guest concierge chatbot and the hotelier analytics agent. Default model is the 8B (cheap) version. The large model is used only for complex analytics. Per-hotel daily usage quotas prevent runaway cost.</t>
+        </is>
+      </c>
+      <c r="E12" s="14" t="inlineStr">
+        <is>
+          <t>Groq provides the fastest LLM inference available at a fraction of OpenAI cost. Switching the default to the 8B model cut AI costs ~10x.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="72" customHeight="1">
+      <c r="A13" s="17" t="inlineStr">
+        <is>
+          <t>Guest Notifications
+(WhatsApp &amp; Email)</t>
+        </is>
+      </c>
+      <c r="B13" s="18" t="inlineStr">
+        <is>
+          <t>WhatsApp API · SMTP</t>
+        </is>
+      </c>
+      <c r="C13" s="18" t="inlineStr">
+        <is>
+          <t>External Services</t>
+        </is>
+      </c>
+      <c r="D13" s="18" t="inlineStr">
+        <is>
+          <t>Sends booking confirmations, check-in reminders, and alerts to guests. Credentials for these services are stored encrypted in Supabase Vault — never as plain text.</t>
+        </is>
+      </c>
+      <c r="E13" s="18" t="inlineStr">
+        <is>
+          <t>WhatsApp has near-100% open rates in India. Encrypted credential storage means a database leak does not compromise the hotel's WhatsApp or email account.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="72" customHeight="1">
+      <c r="A14" s="16" t="inlineStr">
+        <is>
+          <t>OTA Rate Intelligence
+(Competitor pricing)</t>
+        </is>
+      </c>
+      <c r="B14" s="14" t="inlineStr">
+        <is>
+          <t>Decodo Proxy Network
+(white-labelled as
+Staybooker Analytics)</t>
+        </is>
+      </c>
+      <c r="C14" s="14" t="inlineStr">
+        <is>
+          <t>External</t>
+        </is>
+      </c>
+      <c r="D14" s="14" t="inlineStr">
+        <is>
+          <t>Scrapes competitor prices on MakeMyTrip, Goibibo, etc. daily. Hoteliers see a live chart to price their rooms competitively. Scraping is sequential with retry logic; a stop button lets hoteliers abort a run mid-way.</t>
+        </is>
+      </c>
+      <c r="E14" s="14" t="inlineStr">
+        <is>
+          <t>Billed per attempt; vendor name is not exposed to hoteliers (white-labelled) to protect the platform margin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="11" t="inlineStr">
+        <is>
+          <t>B.  Request Flow — Step by Step</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="24" customHeight="1">
+      <c r="A17" s="15" t="inlineStr">
+        <is>
+          <t>When a guest books a room, here is exactly what happens in sequence:</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="B18" s="12" t="inlineStr">
+        <is>
+          <t>What Happens</t>
+        </is>
+      </c>
+      <c r="C18" s="12" t="inlineStr">
+        <is>
+          <t>Systems Involved</t>
+        </is>
+      </c>
+      <c r="D18" s="12" t="inlineStr">
+        <is>
+          <t>Technical Detail</t>
+        </is>
+      </c>
+      <c r="E18" s="12" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="58" customHeight="1">
+      <c r="A19" s="21" t="inlineStr">
+        <is>
+          <t>①</t>
+        </is>
+      </c>
+      <c r="B19" s="22" t="inlineStr">
+        <is>
+          <t>Guest opens hotel website</t>
+        </is>
+      </c>
+      <c r="C19" s="22" t="inlineStr">
+        <is>
+          <t>Cloudflare CDN</t>
+        </is>
+      </c>
+      <c r="D19" s="22" t="inlineStr">
+        <is>
+          <t>The page loads from the nearest Cloudflare edge server (100+ countries). Static files (images, CSS, JavaScript) are cached globally — no load on our backend.</t>
+        </is>
+      </c>
+      <c r="E19" s="22" t="inlineStr">
+        <is>
+          <t>&lt; 200 ms load time globally</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="58" customHeight="1">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="B20" s="18" t="inlineStr">
+        <is>
+          <t>Guest searches available rooms</t>
+        </is>
+      </c>
+      <c r="C20" s="18" t="inlineStr">
+        <is>
+          <t>React → FastAPI → PostgreSQL</t>
+        </is>
+      </c>
+      <c r="D20" s="18" t="inlineStr">
+        <is>
+          <t>The React frontend sends the dates to FastAPI. FastAPI checks Redis cache first; if not cached, queries PostgreSQL with a composite index on (hotel, status, dates). Result cached for 5 min.</t>
+        </is>
+      </c>
+      <c r="E20" s="18" t="inlineStr">
+        <is>
+          <t>&lt; 300 ms for availability</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="58" customHeight="1">
+      <c r="A21" s="21" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="B21" s="22" t="inlineStr">
+        <is>
+          <t>Guest fills checkout form</t>
+        </is>
+      </c>
+      <c r="C21" s="22" t="inlineStr">
+        <is>
+          <t>React Frontend</t>
+        </is>
+      </c>
+      <c r="D21" s="22" t="inlineStr">
+        <is>
+          <t>Guest enters name, email, special requests. Dates are validated client-side (check-out cannot be before check-in). No payment data touches our server yet.</t>
+        </is>
+      </c>
+      <c r="E21" s="22" t="inlineStr">
+        <is>
+          <t>All validation before payment</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="58" customHeight="1">
+      <c r="A22" s="17" t="inlineStr">
+        <is>
+          <t>④</t>
+        </is>
+      </c>
+      <c r="B22" s="18" t="inlineStr">
+        <is>
+          <t>Guest pays</t>
+        </is>
+      </c>
+      <c r="C22" s="18" t="inlineStr">
+        <is>
+          <t>Razorpay → FastAPI</t>
+        </is>
+      </c>
+      <c r="D22" s="18" t="inlineStr">
+        <is>
+          <t>Razorpay handles the card/UPI transaction in their PCI-DSS-compliant environment. Our server receives a webhook with a HMAC SHA-256 signature we verify. Amount is re-calculated on our server — client amount is ignored.</t>
+        </is>
+      </c>
+      <c r="E22" s="18" t="inlineStr">
+        <is>
+          <t>Tamper-proof payment</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="58" customHeight="1">
+      <c r="A23" s="21" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="B23" s="22" t="inlineStr">
+        <is>
+          <t>Booking confirmed</t>
+        </is>
+      </c>
+      <c r="C23" s="22" t="inlineStr">
+        <is>
+          <t>FastAPI → PostgreSQL + Redis</t>
+        </is>
+      </c>
+      <c r="D23" s="22" t="inlineStr">
+        <is>
+          <t>Booking status updated to CONFIRMED in PostgreSQL. Availability cache invalidated in Redis. Background tasks queued: email, WhatsApp, OTA sync.</t>
+        </is>
+      </c>
+      <c r="E23" s="22" t="inlineStr">
+        <is>
+          <t>Atomic update — no race condition</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="58" customHeight="1">
+      <c r="A24" s="17" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="B24" s="18" t="inlineStr">
+        <is>
+          <t>Email &amp; WhatsApp sent</t>
+        </is>
+      </c>
+      <c r="C24" s="18" t="inlineStr">
+        <is>
+          <t>Background Task Queue</t>
+        </is>
+      </c>
+      <c r="D24" s="18" t="inlineStr">
+        <is>
+          <t>Background worker sends confirmation email and WhatsApp message to guest. This runs after the response so the guest sees the confirmation screen immediately without waiting for email delivery.</t>
+        </is>
+      </c>
+      <c r="E24" s="18" t="inlineStr">
+        <is>
+          <t>Guest sees confirm in &lt; 1 s</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="58" customHeight="1">
+      <c r="A25" s="21" t="inlineStr">
+        <is>
+          <t>⑦</t>
+        </is>
+      </c>
+      <c r="B25" s="22" t="inlineStr">
+        <is>
+          <t>Hotelier sees booking on dashboard</t>
+        </is>
+      </c>
+      <c r="C25" s="22" t="inlineStr">
+        <is>
+          <t>WebSocket → React</t>
+        </is>
+      </c>
+      <c r="D25" s="22" t="inlineStr">
+        <is>
+          <t>A WebSocket connection pushes the new booking to the hotelier's dashboard in real time — no page refresh needed. The connection requires a valid JWT token.</t>
+        </is>
+      </c>
+      <c r="E25" s="22" t="inlineStr">
+        <is>
+          <t>Live update &lt; 500 ms</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="11" t="inlineStr">
+        <is>
+          <t>C.  Security Controls Always Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="29" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="B28" s="29" t="inlineStr">
+        <is>
+          <t>What It Does</t>
+        </is>
+      </c>
+      <c r="C28" s="29" t="inlineStr">
+        <is>
+          <t>Why It Matters</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="44" customHeight="1">
+      <c r="A29" s="26" t="inlineStr">
+        <is>
+          <t>AES-256 Encrypted Secrets</t>
+        </is>
+      </c>
+      <c r="B29" s="27" t="inlineStr">
+        <is>
+          <t>All payment, WhatsApp, and email keys stored encrypted in Supabase Vault</t>
+        </is>
+      </c>
+      <c r="C29" s="27" t="inlineStr">
+        <is>
+          <t>Database leak does not expose any hotel's payment account</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="44" customHeight="1">
+      <c r="A30" s="17" t="inlineStr">
+        <is>
+          <t>Row Level Security (RLS)</t>
+        </is>
+      </c>
+      <c r="B30" s="18" t="inlineStr">
+        <is>
+          <t>PostgreSQL itself refuses to return Hotel A's data to Hotel B — enforced at DB level</t>
+        </is>
+      </c>
+      <c r="C30" s="18" t="inlineStr">
+        <is>
+          <t>Two independent layers of isolation — code + database</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="44" customHeight="1">
+      <c r="A31" s="26" t="inlineStr">
+        <is>
+          <t>Server-side Payment Verification</t>
+        </is>
+      </c>
+      <c r="B31" s="27" t="inlineStr">
+        <is>
+          <t>Amount always calculated on server; Razorpay webhook HMAC verified before confirming</t>
+        </is>
+      </c>
+      <c r="C31" s="27" t="inlineStr">
+        <is>
+          <t>A guest cannot manipulate price from browser</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="44" customHeight="1">
+      <c r="A32" s="17" t="inlineStr">
+        <is>
+          <t>Short-lived JWT Tokens</t>
+        </is>
+      </c>
+      <c r="B32" s="18" t="inlineStr">
+        <is>
+          <t>Login tokens expire in 15-30 minutes; permanent tokens rejected</t>
+        </is>
+      </c>
+      <c r="C32" s="18" t="inlineStr">
+        <is>
+          <t>A stolen token has limited window</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="44" customHeight="1">
+      <c r="A33" s="26" t="inlineStr">
+        <is>
+          <t>Redis AI Quota (fail-closed)</t>
+        </is>
+      </c>
+      <c r="B33" s="27" t="inlineStr">
+        <is>
+          <t>Per-hotel daily AI spending limit enforced; when Redis is down, falls back to in-process cap</t>
+        </is>
+      </c>
+      <c r="C33" s="27" t="inlineStr">
+        <is>
+          <t>AI bill cannot spike even during infrastructure outage</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="44" customHeight="1">
+      <c r="A34" s="17" t="inlineStr">
+        <is>
+          <t>IP Spoof-proof Rate Limiting</t>
+        </is>
+      </c>
+      <c r="B34" s="18" t="inlineStr">
+        <is>
+          <t>Trusted-proxy-aware IP extraction — fake X-Forwarded-For headers are ignored</t>
+        </is>
+      </c>
+      <c r="C34" s="18" t="inlineStr">
+        <is>
+          <t>Rate limits cannot be bypassed with a header</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="44" customHeight="1">
+      <c r="A35" s="26" t="inlineStr">
+        <is>
+          <t>277 Automated Tests</t>
+        </is>
+      </c>
+      <c r="B35" s="27" t="inlineStr">
+        <is>
+          <t>Security, payment, role-access, rate-limit tests run on every code push via CI/CD</t>
+        </is>
+      </c>
+      <c r="C35" s="27" t="inlineStr">
+        <is>
+          <t>Regressions caught before reaching production</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="44" customHeight="1">
+      <c r="A36" s="17" t="inlineStr">
+        <is>
+          <t>RBAC Backend Enforcement</t>
+        </is>
+      </c>
+      <c r="B36" s="18" t="inlineStr">
+        <is>
+          <t>OWNER / MANAGER / STAFF roles checked on every API endpoint — not just in the frontend menu</t>
+        </is>
+      </c>
+      <c r="C36" s="18" t="inlineStr">
+        <is>
+          <t>A staff account cannot modify rates or payment keys</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="36" customHeight="1">
+      <c r="A39" s="30" t="inlineStr">
+        <is>
+          <t>📊  For the visual architecture diagram with all logos and flow arrows, open: docs/Staybooker_Architecture.excalidraw  at  https://excalidraw.com</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A39:E39"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A16:E16"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A17:E17"/>
+    <mergeCell ref="A27:E27"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: Embed architecture diagram as image in Excel Sheet 8
Adds Sheet 8 'Architecture Diagram' to CEO_Report_Staybooker_Jun2026.xlsx
with the full system architecture rendered as a high-res PNG (4823x3063).
Shows all 5 zones: Users -> Cloudflare -> Railway (FastAPI+Redis) ->
Supabase (PostgreSQL+Auth+Vault) -> External APIs (Razorpay/Groq/WhatsApp/Email).

https://claude.ai/code/session_01JSXri7YwDXxadMbDuW5jEw
</commit_message>
<xml_diff>
--- a/docs/CEO_Report_Staybooker_Jun2026.xlsx
+++ b/docs/CEO_Report_Staybooker_Jun2026.xlsx
@@ -13,7 +13,7 @@
     <sheet name="4. Work In Progress" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="5. Future Risks" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="6. Team &amp; Hiring" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="7. Architecture" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="8. Architecture Diagram" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="14">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -98,6 +98,16 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00475569"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="006B7280"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="18">
@@ -188,7 +198,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -224,11 +234,55 @@
         <color rgb="00D1D5DB"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D1D5DB"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D1D5DB"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D1D5DB"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D1D5DB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D1D5DB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D1D5DB"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D1D5DB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D1D5DB"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -316,6 +370,17 @@
     <xf numFmtId="0" fontId="13" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -390,6 +455,36 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>2</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="18097500" cy="11487150"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3938,6 +4033,9 @@
           <t>Stable for current hotels. 45 security and performance issues fixed proactively. 277 automated tests run on every code change so regressions are caught before any hotel sees them.</t>
         </is>
       </c>
+      <c r="C6" s="31" t="n"/>
+      <c r="D6" s="31" t="n"/>
+      <c r="E6" s="32" t="n"/>
     </row>
     <row r="7" ht="52" customHeight="1">
       <c r="A7" s="13" t="inlineStr">
@@ -3950,6 +4048,9 @@
           <t>Every hotel's data is isolated — Hotel A cannot see Hotel B's records. All payment and messaging credentials (Razorpay, WhatsApp, Email) are stored AES-256-GCM encrypted. Payment amounts are always verified on the server — a guest cannot manipulate the price from the browser.</t>
         </is>
       </c>
+      <c r="C7" s="31" t="n"/>
+      <c r="D7" s="31" t="n"/>
+      <c r="E7" s="32" t="n"/>
     </row>
     <row r="8" ht="52" customHeight="1">
       <c r="A8" s="13" t="inlineStr">
@@ -3962,6 +4063,9 @@
           <t>Public booking widget is hardened: date validation, error-recovery with retry button, double-payment protection, real-time availability, no fake data.</t>
         </is>
       </c>
+      <c r="C8" s="31" t="n"/>
+      <c r="D8" s="31" t="n"/>
+      <c r="E8" s="32" t="n"/>
     </row>
     <row r="9" ht="52" customHeight="1">
       <c r="A9" s="13" t="inlineStr">
@@ -3974,6 +4078,9 @@
           <t>Currently one senior developer covering the entire stack (backend, frontend, database, DevOps, security). Stable at today's scale. Hiring need is driven by growth — not by anything broken.</t>
         </is>
       </c>
+      <c r="C9" s="31" t="n"/>
+      <c r="D9" s="31" t="n"/>
+      <c r="E9" s="32" t="n"/>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="11" t="inlineStr">
@@ -4592,10 +4699,10 @@
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="A12:E12"/>
     <mergeCell ref="B9:E9"/>
     <mergeCell ref="A4:E4"/>
     <mergeCell ref="B8:E8"/>
-    <mergeCell ref="A12:E12"/>
     <mergeCell ref="A20:E20"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A29:E29"/>
@@ -4616,730 +4723,242 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:Z155"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="10" customWidth="1" min="16" max="16"/>
+    <col width="10" customWidth="1" min="17" max="17"/>
+    <col width="10" customWidth="1" min="18" max="18"/>
+    <col width="10" customWidth="1" min="19" max="19"/>
+    <col width="10" customWidth="1" min="20" max="20"/>
+    <col width="10" customWidth="1" min="21" max="21"/>
+    <col width="10" customWidth="1" min="22" max="22"/>
+    <col width="10" customWidth="1" min="23" max="23"/>
+    <col width="10" customWidth="1" min="24" max="24"/>
+    <col width="10" customWidth="1" min="25" max="25"/>
+    <col width="10" customWidth="1" min="26" max="26"/>
+    <col width="10" customWidth="1" min="27" max="27"/>
+    <col width="10" customWidth="1" min="28" max="28"/>
+    <col width="10" customWidth="1" min="29" max="29"/>
+    <col width="10" customWidth="1" min="30" max="30"/>
+    <col width="10" customWidth="1" min="31" max="31"/>
+    <col width="10" customWidth="1" min="32" max="32"/>
+    <col width="10" customWidth="1" min="33" max="33"/>
+    <col width="10" customWidth="1" min="34" max="34"/>
+    <col width="10" customWidth="1" min="35" max="35"/>
+    <col width="10" customWidth="1" min="36" max="36"/>
+    <col width="10" customWidth="1" min="37" max="37"/>
+    <col width="10" customWidth="1" min="38" max="38"/>
+    <col width="10" customWidth="1" min="39" max="39"/>
+    <col width="10" customWidth="1" min="40" max="40"/>
+    <col width="10" customWidth="1" min="41" max="41"/>
+    <col width="10" customWidth="1" min="42" max="42"/>
+    <col width="10" customWidth="1" min="43" max="43"/>
+    <col width="10" customWidth="1" min="44" max="44"/>
+    <col width="10" customWidth="1" min="45" max="45"/>
+    <col width="10" customWidth="1" min="46" max="46"/>
+    <col width="10" customWidth="1" min="47" max="47"/>
+    <col width="10" customWidth="1" min="48" max="48"/>
+    <col width="10" customWidth="1" min="49" max="49"/>
+    <col width="10" customWidth="1" min="50" max="50"/>
+    <col width="10" customWidth="1" min="51" max="51"/>
   </cols>
   <sheetData>
-    <row r="1" ht="42" customHeight="1">
-      <c r="A1" s="9" t="inlineStr">
-        <is>
-          <t>Staybooker — System Architecture Overview</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="24" customHeight="1">
-      <c r="A2" s="10" t="inlineStr">
-        <is>
-          <t>How every part of the product connects — in plain language  ·  See Staybooker_Architecture.excalidraw for the visual diagram</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="11" t="inlineStr">
-        <is>
-          <t>A.  Technology Layers — What Each Service Does</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="12" t="inlineStr">
-        <is>
-          <t>SERVICE</t>
-        </is>
-      </c>
-      <c r="B5" s="12" t="inlineStr">
-        <is>
-          <t>TECHNOLOGY</t>
-        </is>
-      </c>
-      <c r="C5" s="12" t="inlineStr">
-        <is>
-          <t>HOSTED ON</t>
-        </is>
-      </c>
-      <c r="D5" s="12" t="inlineStr">
-        <is>
-          <t>WHAT IT DOES</t>
-        </is>
-      </c>
-      <c r="E5" s="12" t="inlineStr">
-        <is>
-          <t>WHY THIS CHOICE</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="72" customHeight="1">
-      <c r="A6" s="16" t="inlineStr">
-        <is>
-          <t>Frontend
-(What guests &amp; hoteliers see)</t>
-        </is>
-      </c>
-      <c r="B6" s="14" t="inlineStr">
-        <is>
-          <t>React 18 · Vite · TailwindCSS</t>
-        </is>
-      </c>
-      <c r="C6" s="14" t="inlineStr">
-        <is>
-          <t>Cloudflare Pages
-(Global CDN)</t>
-        </is>
-      </c>
-      <c r="D6" s="14" t="inlineStr">
-        <is>
-          <t>Renders the booking widget on hotel websites and the hotelier management dashboard. Caches API data locally for 5 minutes so the page feels instant.</t>
-        </is>
-      </c>
-      <c r="E6" s="14" t="inlineStr">
-        <is>
-          <t>Cloudflare's CDN delivers pages from the nearest global server — fast load even on slow mobile connections. Zero server cost for static pages.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="72" customHeight="1">
-      <c r="A7" s="17" t="inlineStr">
-        <is>
-          <t>Backend API
-(The brain of the system)</t>
-        </is>
-      </c>
-      <c r="B7" s="18" t="inlineStr">
-        <is>
-          <t>Python 3.11 · FastAPI</t>
-        </is>
-      </c>
-      <c r="C7" s="18" t="inlineStr">
-        <is>
-          <t>Railway
-(Cloud Server)</t>
-        </is>
-      </c>
-      <c r="D7" s="18" t="inlineStr">
-        <is>
-          <t>Handles all business rules: creates bookings, verifies payments, enforces roles (who can do what), runs the AI assistant, sends emails and WhatsApp messages.</t>
-        </is>
-      </c>
-      <c r="E7" s="18" t="inlineStr">
-        <is>
-          <t>FastAPI is the fastest Python API framework. Railway auto-scales with traffic and provides zero-downtime deploys.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="72" customHeight="1">
-      <c r="A8" s="16" t="inlineStr">
-        <is>
-          <t>Primary Database
-(All hotel data)</t>
-        </is>
-      </c>
-      <c r="B8" s="14" t="inlineStr">
-        <is>
-          <t>PostgreSQL
-(via Supabase)</t>
-        </is>
-      </c>
-      <c r="C8" s="14" t="inlineStr">
-        <is>
-          <t>Supabase
-(Managed Cloud DB)</t>
-        </is>
-      </c>
-      <c r="D8" s="14" t="inlineStr">
-        <is>
-          <t>Stores every booking, guest record, room, rate, loyalty point, and setting. Row Level Security ensures Hotel A can never read Hotel B's data — enforced at the database level, not just in code.</t>
-        </is>
-      </c>
-      <c r="E8" s="14" t="inlineStr">
-        <is>
-          <t>Supabase provides managed Postgres with built-in auth, automated backups, and a secure secrets vault at predictable cost.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="72" customHeight="1">
-      <c r="A9" s="17" t="inlineStr">
-        <is>
-          <t>Auth &amp; Identity
-(Who is who)</t>
-        </is>
-      </c>
-      <c r="B9" s="18" t="inlineStr">
-        <is>
-          <t>Supabase Auth · JWT</t>
-        </is>
-      </c>
-      <c r="C9" s="18" t="inlineStr">
-        <is>
-          <t>Supabase</t>
-        </is>
-      </c>
-      <c r="D9" s="18" t="inlineStr">
-        <is>
-          <t>Every login issues a short-lived token (15-30 min). The backend verifies this token on every request. Roles (OWNER / MANAGER / STAFF) are checked server-side on every action.</t>
-        </is>
-      </c>
-      <c r="E9" s="18" t="inlineStr">
-        <is>
-          <t>Supabase Auth handles password hashing, OAuth, and token rotation so we do not build auth from scratch — a common source of security vulnerabilities.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="72" customHeight="1">
-      <c r="A10" s="16" t="inlineStr">
-        <is>
-          <t>Cache &amp; Rate Limiting
-(Speed &amp; protection)</t>
-        </is>
-      </c>
-      <c r="B10" s="14" t="inlineStr">
-        <is>
-          <t>Redis</t>
-        </is>
-      </c>
-      <c r="C10" s="14" t="inlineStr">
-        <is>
-          <t>Railway
-(Internal Network)</t>
-        </is>
-      </c>
-      <c r="D10" s="14" t="inlineStr">
-        <is>
-          <t>Stores frequently-read data so the database is not hit on every request. Tracks API call counts per IP and per hotel to block abuse. Holds distributed locks so two bookings cannot claim the same room simultaneously. Falls back to in-memory cache if Redis is unavailable.</t>
-        </is>
-      </c>
-      <c r="E10" s="14" t="inlineStr">
-        <is>
-          <t>Redis is the industry standard for in-memory caching. Hosting on the same Railway network means &lt; 1 ms latency to the backend.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="72" customHeight="1">
-      <c r="A11" s="17" t="inlineStr">
-        <is>
-          <t>Payment Gateway
-(Money in / out)</t>
-        </is>
-      </c>
-      <c r="B11" s="18" t="inlineStr">
-        <is>
-          <t>Razorpay</t>
-        </is>
-      </c>
-      <c r="C11" s="18" t="inlineStr">
-        <is>
-          <t>External — Razorpay Cloud</t>
-        </is>
-      </c>
-      <c r="D11" s="18" t="inlineStr">
-        <is>
-          <t>Handles credit card, UPI, and net-banking payments. Sends webhook notifications when payment succeeds or fails. All amounts are calculated on our server — the browser cannot alter the price.</t>
-        </is>
-      </c>
-      <c r="E11" s="18" t="inlineStr">
-        <is>
-          <t>Razorpay is the leading Indian payment gateway with deep UPI support, strong fraud detection, and a clear dispute resolution process.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="72" customHeight="1">
-      <c r="A12" s="16" t="inlineStr">
-        <is>
-          <t>AI Assistant
-(Chatbot &amp; analytics)</t>
-        </is>
-      </c>
-      <c r="B12" s="14" t="inlineStr">
-        <is>
-          <t>Groq API · LLaMA 3.1</t>
-        </is>
-      </c>
-      <c r="C12" s="14" t="inlineStr">
-        <is>
-          <t>External — Groq Cloud</t>
-        </is>
-      </c>
-      <c r="D12" s="14" t="inlineStr">
-        <is>
-          <t>Powers the guest concierge chatbot and the hotelier analytics agent. Default model is the 8B (cheap) version. The large model is used only for complex analytics. Per-hotel daily usage quotas prevent runaway cost.</t>
-        </is>
-      </c>
-      <c r="E12" s="14" t="inlineStr">
-        <is>
-          <t>Groq provides the fastest LLM inference available at a fraction of OpenAI cost. Switching the default to the 8B model cut AI costs ~10x.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="72" customHeight="1">
-      <c r="A13" s="17" t="inlineStr">
-        <is>
-          <t>Guest Notifications
-(WhatsApp &amp; Email)</t>
-        </is>
-      </c>
-      <c r="B13" s="18" t="inlineStr">
-        <is>
-          <t>WhatsApp API · SMTP</t>
-        </is>
-      </c>
-      <c r="C13" s="18" t="inlineStr">
-        <is>
-          <t>External Services</t>
-        </is>
-      </c>
-      <c r="D13" s="18" t="inlineStr">
-        <is>
-          <t>Sends booking confirmations, check-in reminders, and alerts to guests. Credentials for these services are stored encrypted in Supabase Vault — never as plain text.</t>
-        </is>
-      </c>
-      <c r="E13" s="18" t="inlineStr">
-        <is>
-          <t>WhatsApp has near-100% open rates in India. Encrypted credential storage means a database leak does not compromise the hotel's WhatsApp or email account.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="72" customHeight="1">
-      <c r="A14" s="16" t="inlineStr">
-        <is>
-          <t>OTA Rate Intelligence
-(Competitor pricing)</t>
-        </is>
-      </c>
-      <c r="B14" s="14" t="inlineStr">
-        <is>
-          <t>Decodo Proxy Network
-(white-labelled as
-Staybooker Analytics)</t>
-        </is>
-      </c>
-      <c r="C14" s="14" t="inlineStr">
-        <is>
-          <t>External</t>
-        </is>
-      </c>
-      <c r="D14" s="14" t="inlineStr">
-        <is>
-          <t>Scrapes competitor prices on MakeMyTrip, Goibibo, etc. daily. Hoteliers see a live chart to price their rooms competitively. Scraping is sequential with retry logic; a stop button lets hoteliers abort a run mid-way.</t>
-        </is>
-      </c>
-      <c r="E14" s="14" t="inlineStr">
-        <is>
-          <t>Billed per attempt; vendor name is not exposed to hoteliers (white-labelled) to protect the platform margin.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="11" t="inlineStr">
-        <is>
-          <t>B.  Request Flow — Step by Step</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="24" customHeight="1">
-      <c r="A17" s="15" t="inlineStr">
-        <is>
-          <t>When a guest books a room, here is exactly what happens in sequence:</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="12" t="inlineStr">
-        <is>
-          <t>Step</t>
-        </is>
-      </c>
-      <c r="B18" s="12" t="inlineStr">
-        <is>
-          <t>What Happens</t>
-        </is>
-      </c>
-      <c r="C18" s="12" t="inlineStr">
-        <is>
-          <t>Systems Involved</t>
-        </is>
-      </c>
-      <c r="D18" s="12" t="inlineStr">
-        <is>
-          <t>Technical Detail</t>
-        </is>
-      </c>
-      <c r="E18" s="12" t="inlineStr">
-        <is>
-          <t>Result</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="58" customHeight="1">
-      <c r="A19" s="21" t="inlineStr">
-        <is>
-          <t>①</t>
-        </is>
-      </c>
-      <c r="B19" s="22" t="inlineStr">
-        <is>
-          <t>Guest opens hotel website</t>
-        </is>
-      </c>
-      <c r="C19" s="22" t="inlineStr">
-        <is>
-          <t>Cloudflare CDN</t>
-        </is>
-      </c>
-      <c r="D19" s="22" t="inlineStr">
-        <is>
-          <t>The page loads from the nearest Cloudflare edge server (100+ countries). Static files (images, CSS, JavaScript) are cached globally — no load on our backend.</t>
-        </is>
-      </c>
-      <c r="E19" s="22" t="inlineStr">
-        <is>
-          <t>&lt; 200 ms load time globally</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="58" customHeight="1">
-      <c r="A20" s="17" t="inlineStr">
-        <is>
-          <t>②</t>
-        </is>
-      </c>
-      <c r="B20" s="18" t="inlineStr">
-        <is>
-          <t>Guest searches available rooms</t>
-        </is>
-      </c>
-      <c r="C20" s="18" t="inlineStr">
-        <is>
-          <t>React → FastAPI → PostgreSQL</t>
-        </is>
-      </c>
-      <c r="D20" s="18" t="inlineStr">
-        <is>
-          <t>The React frontend sends the dates to FastAPI. FastAPI checks Redis cache first; if not cached, queries PostgreSQL with a composite index on (hotel, status, dates). Result cached for 5 min.</t>
-        </is>
-      </c>
-      <c r="E20" s="18" t="inlineStr">
-        <is>
-          <t>&lt; 300 ms for availability</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="58" customHeight="1">
-      <c r="A21" s="21" t="inlineStr">
-        <is>
-          <t>③</t>
-        </is>
-      </c>
-      <c r="B21" s="22" t="inlineStr">
-        <is>
-          <t>Guest fills checkout form</t>
-        </is>
-      </c>
-      <c r="C21" s="22" t="inlineStr">
-        <is>
-          <t>React Frontend</t>
-        </is>
-      </c>
-      <c r="D21" s="22" t="inlineStr">
-        <is>
-          <t>Guest enters name, email, special requests. Dates are validated client-side (check-out cannot be before check-in). No payment data touches our server yet.</t>
-        </is>
-      </c>
-      <c r="E21" s="22" t="inlineStr">
-        <is>
-          <t>All validation before payment</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="58" customHeight="1">
-      <c r="A22" s="17" t="inlineStr">
-        <is>
-          <t>④</t>
-        </is>
-      </c>
-      <c r="B22" s="18" t="inlineStr">
-        <is>
-          <t>Guest pays</t>
-        </is>
-      </c>
-      <c r="C22" s="18" t="inlineStr">
-        <is>
-          <t>Razorpay → FastAPI</t>
-        </is>
-      </c>
-      <c r="D22" s="18" t="inlineStr">
-        <is>
-          <t>Razorpay handles the card/UPI transaction in their PCI-DSS-compliant environment. Our server receives a webhook with a HMAC SHA-256 signature we verify. Amount is re-calculated on our server — client amount is ignored.</t>
-        </is>
-      </c>
-      <c r="E22" s="18" t="inlineStr">
-        <is>
-          <t>Tamper-proof payment</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="58" customHeight="1">
-      <c r="A23" s="21" t="inlineStr">
-        <is>
-          <t>⑤</t>
-        </is>
-      </c>
-      <c r="B23" s="22" t="inlineStr">
-        <is>
-          <t>Booking confirmed</t>
-        </is>
-      </c>
-      <c r="C23" s="22" t="inlineStr">
-        <is>
-          <t>FastAPI → PostgreSQL + Redis</t>
-        </is>
-      </c>
-      <c r="D23" s="22" t="inlineStr">
-        <is>
-          <t>Booking status updated to CONFIRMED in PostgreSQL. Availability cache invalidated in Redis. Background tasks queued: email, WhatsApp, OTA sync.</t>
-        </is>
-      </c>
-      <c r="E23" s="22" t="inlineStr">
-        <is>
-          <t>Atomic update — no race condition</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="58" customHeight="1">
-      <c r="A24" s="17" t="inlineStr">
-        <is>
-          <t>⑥</t>
-        </is>
-      </c>
-      <c r="B24" s="18" t="inlineStr">
-        <is>
-          <t>Email &amp; WhatsApp sent</t>
-        </is>
-      </c>
-      <c r="C24" s="18" t="inlineStr">
-        <is>
-          <t>Background Task Queue</t>
-        </is>
-      </c>
-      <c r="D24" s="18" t="inlineStr">
-        <is>
-          <t>Background worker sends confirmation email and WhatsApp message to guest. This runs after the response so the guest sees the confirmation screen immediately without waiting for email delivery.</t>
-        </is>
-      </c>
-      <c r="E24" s="18" t="inlineStr">
-        <is>
-          <t>Guest sees confirm in &lt; 1 s</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="58" customHeight="1">
-      <c r="A25" s="21" t="inlineStr">
-        <is>
-          <t>⑦</t>
-        </is>
-      </c>
-      <c r="B25" s="22" t="inlineStr">
-        <is>
-          <t>Hotelier sees booking on dashboard</t>
-        </is>
-      </c>
-      <c r="C25" s="22" t="inlineStr">
-        <is>
-          <t>WebSocket → React</t>
-        </is>
-      </c>
-      <c r="D25" s="22" t="inlineStr">
-        <is>
-          <t>A WebSocket connection pushes the new booking to the hotelier's dashboard in real time — no page refresh needed. The connection requires a valid JWT token.</t>
-        </is>
-      </c>
-      <c r="E25" s="22" t="inlineStr">
-        <is>
-          <t>Live update &lt; 500 ms</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="11" t="inlineStr">
-        <is>
-          <t>C.  Security Controls Always Active</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="29" t="inlineStr">
-        <is>
-          <t>Control</t>
-        </is>
-      </c>
-      <c r="B28" s="29" t="inlineStr">
-        <is>
-          <t>What It Does</t>
-        </is>
-      </c>
-      <c r="C28" s="29" t="inlineStr">
-        <is>
-          <t>Why It Matters</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="44" customHeight="1">
-      <c r="A29" s="26" t="inlineStr">
-        <is>
-          <t>AES-256 Encrypted Secrets</t>
-        </is>
-      </c>
-      <c r="B29" s="27" t="inlineStr">
-        <is>
-          <t>All payment, WhatsApp, and email keys stored encrypted in Supabase Vault</t>
-        </is>
-      </c>
-      <c r="C29" s="27" t="inlineStr">
-        <is>
-          <t>Database leak does not expose any hotel's payment account</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="44" customHeight="1">
-      <c r="A30" s="17" t="inlineStr">
-        <is>
-          <t>Row Level Security (RLS)</t>
-        </is>
-      </c>
-      <c r="B30" s="18" t="inlineStr">
-        <is>
-          <t>PostgreSQL itself refuses to return Hotel A's data to Hotel B — enforced at DB level</t>
-        </is>
-      </c>
-      <c r="C30" s="18" t="inlineStr">
-        <is>
-          <t>Two independent layers of isolation — code + database</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="44" customHeight="1">
-      <c r="A31" s="26" t="inlineStr">
-        <is>
-          <t>Server-side Payment Verification</t>
-        </is>
-      </c>
-      <c r="B31" s="27" t="inlineStr">
-        <is>
-          <t>Amount always calculated on server; Razorpay webhook HMAC verified before confirming</t>
-        </is>
-      </c>
-      <c r="C31" s="27" t="inlineStr">
-        <is>
-          <t>A guest cannot manipulate price from browser</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="44" customHeight="1">
-      <c r="A32" s="17" t="inlineStr">
-        <is>
-          <t>Short-lived JWT Tokens</t>
-        </is>
-      </c>
-      <c r="B32" s="18" t="inlineStr">
-        <is>
-          <t>Login tokens expire in 15-30 minutes; permanent tokens rejected</t>
-        </is>
-      </c>
-      <c r="C32" s="18" t="inlineStr">
-        <is>
-          <t>A stolen token has limited window</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="44" customHeight="1">
-      <c r="A33" s="26" t="inlineStr">
-        <is>
-          <t>Redis AI Quota (fail-closed)</t>
-        </is>
-      </c>
-      <c r="B33" s="27" t="inlineStr">
-        <is>
-          <t>Per-hotel daily AI spending limit enforced; when Redis is down, falls back to in-process cap</t>
-        </is>
-      </c>
-      <c r="C33" s="27" t="inlineStr">
-        <is>
-          <t>AI bill cannot spike even during infrastructure outage</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="44" customHeight="1">
-      <c r="A34" s="17" t="inlineStr">
-        <is>
-          <t>IP Spoof-proof Rate Limiting</t>
-        </is>
-      </c>
-      <c r="B34" s="18" t="inlineStr">
-        <is>
-          <t>Trusted-proxy-aware IP extraction — fake X-Forwarded-For headers are ignored</t>
-        </is>
-      </c>
-      <c r="C34" s="18" t="inlineStr">
-        <is>
-          <t>Rate limits cannot be bypassed with a header</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="44" customHeight="1">
-      <c r="A35" s="26" t="inlineStr">
-        <is>
-          <t>277 Automated Tests</t>
-        </is>
-      </c>
-      <c r="B35" s="27" t="inlineStr">
-        <is>
-          <t>Security, payment, role-access, rate-limit tests run on every code push via CI/CD</t>
-        </is>
-      </c>
-      <c r="C35" s="27" t="inlineStr">
-        <is>
-          <t>Regressions caught before reaching production</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="44" customHeight="1">
-      <c r="A36" s="17" t="inlineStr">
-        <is>
-          <t>RBAC Backend Enforcement</t>
-        </is>
-      </c>
-      <c r="B36" s="18" t="inlineStr">
-        <is>
-          <t>OWNER / MANAGER / STAFF roles checked on every API endpoint — not just in the frontend menu</t>
-        </is>
-      </c>
-      <c r="C36" s="18" t="inlineStr">
-        <is>
-          <t>A staff account cannot modify rates or payment keys</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="36" customHeight="1">
-      <c r="A39" s="30" t="inlineStr">
-        <is>
-          <t>📊  For the visual architecture diagram with all logos and flow arrows, open: docs/Staybooker_Architecture.excalidraw  at  https://excalidraw.com</t>
+    <row r="1" ht="40" customHeight="1">
+      <c r="A1" s="33" t="inlineStr">
+        <is>
+          <t>Staybooker — System Architecture Diagram</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="34" t="inlineStr">
+        <is>
+          <t>Guest Browser  -&gt;  Cloudflare CDN + React  -&gt;  Railway (FastAPI + Redis)  -&gt;  Supabase (PostgreSQL + Auth + Vault)  +  Razorpay / Groq AI / WhatsApp / Email</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1"/>
+    <row r="4" ht="18" customHeight="1"/>
+    <row r="5" ht="18" customHeight="1"/>
+    <row r="6" ht="18" customHeight="1"/>
+    <row r="7" ht="18" customHeight="1"/>
+    <row r="8" ht="18" customHeight="1"/>
+    <row r="9" ht="18" customHeight="1"/>
+    <row r="10" ht="18" customHeight="1"/>
+    <row r="11" ht="18" customHeight="1"/>
+    <row r="12" ht="18" customHeight="1"/>
+    <row r="13" ht="18" customHeight="1"/>
+    <row r="14" ht="18" customHeight="1"/>
+    <row r="15" ht="18" customHeight="1"/>
+    <row r="16" ht="18" customHeight="1"/>
+    <row r="17" ht="18" customHeight="1"/>
+    <row r="18" ht="18" customHeight="1"/>
+    <row r="19" ht="18" customHeight="1"/>
+    <row r="20" ht="18" customHeight="1"/>
+    <row r="21" ht="18" customHeight="1"/>
+    <row r="22" ht="18" customHeight="1"/>
+    <row r="23" ht="18" customHeight="1"/>
+    <row r="24" ht="18" customHeight="1"/>
+    <row r="25" ht="18" customHeight="1"/>
+    <row r="26" ht="18" customHeight="1"/>
+    <row r="27" ht="18" customHeight="1"/>
+    <row r="28" ht="18" customHeight="1"/>
+    <row r="29" ht="18" customHeight="1"/>
+    <row r="30" ht="18" customHeight="1"/>
+    <row r="31" ht="18" customHeight="1"/>
+    <row r="32" ht="18" customHeight="1"/>
+    <row r="33" ht="18" customHeight="1"/>
+    <row r="34" ht="18" customHeight="1"/>
+    <row r="35" ht="18" customHeight="1"/>
+    <row r="36" ht="18" customHeight="1"/>
+    <row r="37" ht="18" customHeight="1"/>
+    <row r="38" ht="18" customHeight="1"/>
+    <row r="39" ht="18" customHeight="1"/>
+    <row r="40" ht="18" customHeight="1"/>
+    <row r="41" ht="18" customHeight="1"/>
+    <row r="42" ht="18" customHeight="1"/>
+    <row r="43" ht="18" customHeight="1"/>
+    <row r="44" ht="18" customHeight="1"/>
+    <row r="45" ht="18" customHeight="1"/>
+    <row r="46" ht="18" customHeight="1"/>
+    <row r="47" ht="18" customHeight="1"/>
+    <row r="48" ht="18" customHeight="1"/>
+    <row r="49" ht="18" customHeight="1"/>
+    <row r="50" ht="18" customHeight="1"/>
+    <row r="51" ht="18" customHeight="1"/>
+    <row r="52" ht="18" customHeight="1"/>
+    <row r="53" ht="18" customHeight="1"/>
+    <row r="54" ht="18" customHeight="1"/>
+    <row r="55" ht="18" customHeight="1"/>
+    <row r="56" ht="18" customHeight="1"/>
+    <row r="57" ht="18" customHeight="1"/>
+    <row r="58" ht="18" customHeight="1"/>
+    <row r="59" ht="18" customHeight="1"/>
+    <row r="60" ht="18" customHeight="1"/>
+    <row r="61" ht="18" customHeight="1"/>
+    <row r="62" ht="18" customHeight="1"/>
+    <row r="63" ht="18" customHeight="1"/>
+    <row r="64" ht="18" customHeight="1"/>
+    <row r="65" ht="18" customHeight="1"/>
+    <row r="66" ht="18" customHeight="1"/>
+    <row r="67" ht="18" customHeight="1"/>
+    <row r="68" ht="18" customHeight="1"/>
+    <row r="69" ht="18" customHeight="1"/>
+    <row r="70" ht="18" customHeight="1"/>
+    <row r="71" ht="18" customHeight="1"/>
+    <row r="72" ht="18" customHeight="1"/>
+    <row r="73" ht="18" customHeight="1"/>
+    <row r="74" ht="18" customHeight="1"/>
+    <row r="75" ht="18" customHeight="1"/>
+    <row r="76" ht="18" customHeight="1"/>
+    <row r="77" ht="18" customHeight="1"/>
+    <row r="78" ht="18" customHeight="1"/>
+    <row r="79" ht="18" customHeight="1"/>
+    <row r="80" ht="18" customHeight="1"/>
+    <row r="81" ht="18" customHeight="1"/>
+    <row r="82" ht="18" customHeight="1"/>
+    <row r="83" ht="18" customHeight="1"/>
+    <row r="84" ht="18" customHeight="1"/>
+    <row r="85" ht="18" customHeight="1"/>
+    <row r="86" ht="18" customHeight="1"/>
+    <row r="87" ht="18" customHeight="1"/>
+    <row r="88" ht="18" customHeight="1"/>
+    <row r="89" ht="18" customHeight="1"/>
+    <row r="90" ht="18" customHeight="1"/>
+    <row r="91" ht="18" customHeight="1"/>
+    <row r="92" ht="18" customHeight="1"/>
+    <row r="93" ht="18" customHeight="1"/>
+    <row r="94" ht="18" customHeight="1"/>
+    <row r="95" ht="18" customHeight="1"/>
+    <row r="96" ht="18" customHeight="1"/>
+    <row r="97" ht="18" customHeight="1"/>
+    <row r="98" ht="18" customHeight="1"/>
+    <row r="99" ht="18" customHeight="1"/>
+    <row r="100" ht="18" customHeight="1"/>
+    <row r="101" ht="18" customHeight="1"/>
+    <row r="102" ht="18" customHeight="1"/>
+    <row r="103" ht="18" customHeight="1"/>
+    <row r="104" ht="18" customHeight="1"/>
+    <row r="105" ht="18" customHeight="1"/>
+    <row r="106" ht="18" customHeight="1"/>
+    <row r="107" ht="18" customHeight="1"/>
+    <row r="108" ht="18" customHeight="1"/>
+    <row r="109" ht="18" customHeight="1"/>
+    <row r="110" ht="18" customHeight="1"/>
+    <row r="111" ht="18" customHeight="1"/>
+    <row r="112" ht="18" customHeight="1"/>
+    <row r="113" ht="18" customHeight="1"/>
+    <row r="114" ht="18" customHeight="1"/>
+    <row r="115" ht="18" customHeight="1"/>
+    <row r="116" ht="18" customHeight="1"/>
+    <row r="117" ht="18" customHeight="1"/>
+    <row r="118" ht="18" customHeight="1"/>
+    <row r="119" ht="18" customHeight="1"/>
+    <row r="120" ht="18" customHeight="1"/>
+    <row r="121" ht="18" customHeight="1"/>
+    <row r="122" ht="18" customHeight="1"/>
+    <row r="123" ht="18" customHeight="1"/>
+    <row r="124" ht="18" customHeight="1"/>
+    <row r="125" ht="18" customHeight="1"/>
+    <row r="126" ht="18" customHeight="1"/>
+    <row r="127" ht="18" customHeight="1"/>
+    <row r="128" ht="18" customHeight="1"/>
+    <row r="129" ht="18" customHeight="1"/>
+    <row r="130" ht="18" customHeight="1"/>
+    <row r="131" ht="18" customHeight="1"/>
+    <row r="132" ht="18" customHeight="1"/>
+    <row r="133" ht="18" customHeight="1"/>
+    <row r="134" ht="18" customHeight="1"/>
+    <row r="135" ht="18" customHeight="1"/>
+    <row r="136" ht="18" customHeight="1"/>
+    <row r="137" ht="18" customHeight="1"/>
+    <row r="138" ht="18" customHeight="1"/>
+    <row r="139" ht="18" customHeight="1"/>
+    <row r="140" ht="18" customHeight="1"/>
+    <row r="141" ht="18" customHeight="1"/>
+    <row r="142" ht="18" customHeight="1"/>
+    <row r="143" ht="18" customHeight="1"/>
+    <row r="144" ht="18" customHeight="1"/>
+    <row r="145" ht="18" customHeight="1"/>
+    <row r="146" ht="18" customHeight="1"/>
+    <row r="147" ht="18" customHeight="1"/>
+    <row r="148" ht="18" customHeight="1"/>
+    <row r="149" ht="18" customHeight="1"/>
+    <row r="150" ht="18" customHeight="1"/>
+    <row r="151" ht="18" customHeight="1"/>
+    <row r="152" ht="18" customHeight="1"/>
+    <row r="153" ht="18" customHeight="1"/>
+    <row r="154" ht="18" customHeight="1"/>
+    <row r="155" ht="20" customHeight="1">
+      <c r="A155" s="35" t="inlineStr">
+        <is>
+          <t>For interactive version with zoom: open docs/Staybooker_Architecture.excalidraw at https://excalidraw.com</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="A39:E39"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A16:E16"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A17:E17"/>
-    <mergeCell ref="A27:E27"/>
+  <mergeCells count="3">
+    <mergeCell ref="A1:Z1"/>
+    <mergeCell ref="A155:Z155"/>
+    <mergeCell ref="A2:Z2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: Update CEO Report with June 14-16 work (58 issues, 27 features)
Sheet 1 (Executive Summary): Updated key numbers — 58 total issues fixed,
27 major features, DDD refactoring note, graphify knowledge graph stats.

Sheet 2 (Problems Solved): Added S-46 to S-58 — 13 new fixes including
widget RCE sink removal (Critical), atomic promo/loyalty double-spend fix
(Critical), booking 500 crash (Critical), Guest Recovery automation (High),
widget iframe sandbox + CSS injection + postMessage hardening (High x3),
loyalty role guard, loyalty-check NameError, inactive hotel 404, and more.

Sheet 3 (Features Built): Added #13 to #27 — 15 new features including
Dynamic Pricing Engine, Abandoned Booking Recovery, Seasonal Auto-Apply
Promos, Chain Upsell Broadcast, Stay Offers, Configurable Points Wallet,
HMAC Anti-Automation Token, DDD Refactoring, and more.

Sheet 4 (Work In Progress): Refreshed with current state of P-01 to P-06.

https://claude.ai/code/session_01JSXri7YwDXxadMbDuW5jEw
</commit_message>
<xml_diff>
--- a/docs/CEO_Report_Staybooker_Jun2026.xlsx
+++ b/docs/CEO_Report_Staybooker_Jun2026.xlsx
@@ -23,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="16">
+  <fonts count="17">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -109,8 +109,14 @@
       <color rgb="006B7280"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="16"/>
+    </font>
   </fonts>
-  <fills count="18">
+  <fills count="22">
     <fill>
       <patternFill/>
     </fill>
@@ -195,6 +201,26 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="007F1D1D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001E293B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF3E4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFBE4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFE4E4"/>
       </patternFill>
     </fill>
   </fills>
@@ -282,7 +308,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -380,6 +406,30 @@
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="19" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="20" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="21" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -480,6 +530,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -776,206 +829,255 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:B25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="32" customWidth="1" min="1" max="1"/>
-    <col width="120" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="80" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="44" customHeight="1">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>Staybooker Booking Engine — CEO Report (June 2026)</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>What has been solved, what is in progress, what risks are coming, and why we need a team — at a glance</t>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="36" t="inlineStr">
+        <is>
+          <t>Updated 16-Jun-2026  ·  What has been solved, what is in progress, and what risks are coming</t>
         </is>
       </c>
     </row>
     <row r="4" ht="26" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Topic</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Detail</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A4" s="37" t="inlineStr">
         <is>
           <t>WHAT THIS REPORT CONTAINS</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr"/>
-    </row>
-    <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
+    </row>
+    <row r="5" ht="44" customHeight="1">
+      <c r="A5" s="38" t="inlineStr">
         <is>
           <t>Sheet 2 — Problems Solved</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>45 issues fixed so far (5 Critical, 24 High, 16 Medium). Each issue shows what would have happened to the business if it had reached production.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="36" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="B5" s="18" t="inlineStr">
+        <is>
+          <t>58 issues fixed in total (9 Critical, 30 High, 19 Medium). Each issue shows what would have happened to the business if it had reached production. Includes 13 new fixes from 14–16 June.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="44" customHeight="1">
+      <c r="A6" s="38" t="inlineStr">
         <is>
           <t>Sheet 3 — Features Built</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>Major product features delivered alongside the bug fixing — multi-property chains, loyalty program, OTA rate intelligence, AI concierge, real-time updates, encrypted secrets storage.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>27 major product features delivered — now includes the full Revenue module (Dynamic Pricing, Abandoned Booking Recovery, Seasonal Promos), enhanced Loyalty &amp; Upsell system, Brand Console, and more.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="44" customHeight="1">
+      <c r="A7" s="38" t="inlineStr">
         <is>
           <t>Sheet 4 — Work In Progress</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>Critical items currently being worked on.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="40" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="B7" s="18" t="inlineStr">
+        <is>
+          <t>Items currently being worked on — payment recovery automation, load testing, database migration discipline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="44" customHeight="1">
+      <c r="A8" s="38" t="inlineStr">
         <is>
           <t>Sheet 5 — Future Risks</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>13 real-world scenarios that WILL come as the business grows (100 users at once, payment failures, DDoS attacks, data growing to GBs) — what protection already exists and what still needs to be built.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="34" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>13 real-world scenarios that WILL come as the business grows — what protection already exists and what still needs to be built.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="44" customHeight="1">
+      <c r="A9" s="38" t="inlineStr">
         <is>
           <t>Sheet 6 — Team &amp; Hiring</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>What a Tech Lead / Backend / Frontend / Database developer actually does, in simple language — who owns which part of the product as it grows, with a suggested hiring order.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr"/>
-      <c r="B11" s="4" t="inlineStr"/>
-    </row>
-    <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>KEY NUMBERS</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr"/>
-    </row>
-    <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>Issues fixed till date</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>45 (source: work_log_tracker.csv — 71 logged engineering tasks up to 11-Jun-2026)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="4" t="inlineStr">
+      <c r="B9" s="18" t="inlineStr">
+        <is>
+          <t>What each developer does in plain language, why software always needs ongoing engineering, and the hiring roadmap.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="44" customHeight="1">
+      <c r="A10" s="38" t="inlineStr">
+        <is>
+          <t>Sheet 7 — Architecture Overview</t>
+        </is>
+      </c>
+      <c r="B10" s="18" t="inlineStr">
+        <is>
+          <t>How every service connects — tech layer table, 7-step booking flow, security controls.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="44" customHeight="1">
+      <c r="A11" s="38" t="inlineStr">
+        <is>
+          <t>Sheet 8 — Architecture Diagram</t>
+        </is>
+      </c>
+      <c r="B11" s="18" t="inlineStr">
+        <is>
+          <t>Full system architecture as an embedded visual diagram.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1"/>
+    <row r="13" ht="26" customHeight="1">
+      <c r="A13" s="37" t="inlineStr">
+        <is>
+          <t>KEY NUMBERS (Updated 16-Jun-2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="44" customHeight="1">
+      <c r="A14" s="16" t="inlineStr">
+        <is>
+          <t>Issues fixed in total</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>58  (9 Critical · 30 High · 19 Medium)  ·  source: work_log_tracker.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="44" customHeight="1">
+      <c r="A15" s="16" t="inlineStr">
+        <is>
+          <t>New issues fixed (14–16 Jun)</t>
+        </is>
+      </c>
+      <c r="B15" s="18" t="inlineStr">
+        <is>
+          <t>13 — including widget RCE removal, atomic redemption race fix, Guest Recovery automation, booking 500 crash, loyalty-check NameError</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="44" customHeight="1">
+      <c r="A16" s="16" t="inlineStr">
         <is>
           <t>Critical issues fixed</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>5 — payment secret key leak, payment amount tampering, permanent admin token, AI assistant crash, staff privilege escalation</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="40" customHeight="1">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>Security audit coverage</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>A full security/performance audit found 36 findings (1 Critical, 12 High, 14 Medium, 9 Low). The Critical issue and most High findings are fixed; the remaining items are tracked openly in Sheets 4 and 5.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="39" customHeight="1">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>Automated tests added</t>
-        </is>
-      </c>
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>277 test cases passing (security, payments, booking, role access, rate limits, Redis failover). These run automatically on every code change (CI/CD), plus dependency vulnerability (CVE) scanning.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="54" customHeight="1">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>Money saved (examples)</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>Payment tampering fix: a guest could pay Rs.1 and get a Rs.10,000 booking confirmed. AI cost fix: a bug was sending traffic to an AI model 10x more expensive than needed on the public chatbot. Tax validation fix: invalid tax setup could produce wrong bills for every guest.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr"/>
-      <c r="B18" s="4" t="inlineStr"/>
-    </row>
-    <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>ONE-LINE MESSAGE FOR THE CEO</t>
-        </is>
-      </c>
-      <c r="B19" s="4" t="inlineStr"/>
-    </row>
-    <row r="20" ht="50" customHeight="1">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>Bottom line</t>
-        </is>
-      </c>
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>The product is stable today and hoteliers' data is safe. The hiring need comes from growth: as hotels, traffic and data scale up, each layer — database, backend, frontend — needs a dedicated owner so quality and safety stay exactly where they are today.</t>
+      <c r="B16" s="18" t="inlineStr">
+        <is>
+          <t>9 — includes original 5 + widget RCE sink, atomic double-spend, HMAC anti-automation, Guest Recovery never ran</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="44" customHeight="1">
+      <c r="A17" s="16" t="inlineStr">
+        <is>
+          <t>New features delivered (14–16 Jun)</t>
+        </is>
+      </c>
+      <c r="B17" s="18" t="inlineStr">
+        <is>
+          <t>15 — Dynamic Pricing engine, Abandoned Booking Recovery, Seasonal Auto-Apply Promos, Chain Upsell Broadcast, Stay Offers, Configurable Points Wallet, Upsell Templates, and more</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="44" customHeight="1">
+      <c r="A18" s="16" t="inlineStr">
+        <is>
+          <t>Total major features</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="inlineStr">
+        <is>
+          <t>27 product features built alongside all security/stability work</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="44" customHeight="1">
+      <c r="A19" s="16" t="inlineStr">
+        <is>
+          <t>Automated tests</t>
+        </is>
+      </c>
+      <c r="B19" s="18" t="inlineStr">
+        <is>
+          <t>277+ test cases passing — CI runs on every code change</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="44" customHeight="1">
+      <c r="A20" s="16" t="inlineStr">
+        <is>
+          <t>Codebase scope</t>
+        </is>
+      </c>
+      <c r="B20" s="18" t="inlineStr">
+        <is>
+          <t>4,798 nodes · 10,961 edges across 426 code files (AST knowledge graph built 15-Jun)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="44" customHeight="1">
+      <c r="A21" s="16" t="inlineStr">
+        <is>
+          <t>Architecture</t>
+        </is>
+      </c>
+      <c r="B21" s="18" t="inlineStr">
+        <is>
+          <t>DDD (Domain-Driven Design) refactoring completed 16-Jun — codebase restructured for long-term maintainability</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="44" customHeight="1">
+      <c r="A22" s="16" t="inlineStr">
+        <is>
+          <t>Money saved (key examples)</t>
+        </is>
+      </c>
+      <c r="B22" s="18" t="inlineStr">
+        <is>
+          <t>Widget RCE fix: a malicious hotel could have injected JavaScript into every guest browser via widget_custom_js — removed entirely. Atomic promo fix: two simultaneous bookings could have double-spent a promo code. Guest Recovery automation: abandoned bookings were silently aging past the 72h recovery window — now swept hourly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="26" customHeight="1">
+      <c r="A24" s="37" t="inlineStr">
+        <is>
+          <t>ONE-LINE MESSAGE</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="52" customHeight="1">
+      <c r="A25" s="28" t="inlineStr">
+        <is>
+          <t>The product is stable, secure, and now growing fast with new revenue features. Hiring need remains the same: as hotels, traffic and data scale up, each layer needs a dedicated owner so quality and safety stay exactly where they are today.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="6">
+    <mergeCell ref="A4:B4"/>
     <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="A13:B13"/>
     <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -988,7 +1090,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G49"/>
+  <dimension ref="A1:G65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2716,10 +2818,536 @@
         </is>
       </c>
     </row>
+    <row r="51" ht="26" customHeight="1">
+      <c r="A51" s="37" t="inlineStr">
+        <is>
+          <t>NEW ISSUES FIXED — 14 to 16 June 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="39" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B52" s="39" t="inlineStr">
+        <is>
+          <t>Problem (Simple Language)</t>
+        </is>
+      </c>
+      <c r="C52" s="39" t="inlineStr">
+        <is>
+          <t>What Was Happening</t>
+        </is>
+      </c>
+      <c r="D52" s="39" t="inlineStr">
+        <is>
+          <t>Business Impact If Unfixed</t>
+        </is>
+      </c>
+      <c r="E52" s="39" t="inlineStr">
+        <is>
+          <t>How Fixed</t>
+        </is>
+      </c>
+      <c r="F52" s="39" t="inlineStr">
+        <is>
+          <t>Severity</t>
+        </is>
+      </c>
+      <c r="G52" s="39" t="inlineStr">
+        <is>
+          <t>Fixed On</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="55" customHeight="1">
+      <c r="A53" s="16" t="inlineStr">
+        <is>
+          <t>S-46</t>
+        </is>
+      </c>
+      <c r="B53" s="14" t="inlineStr">
+        <is>
+          <t>Loyalty program viewable by any staff member (no role check)</t>
+        </is>
+      </c>
+      <c r="C53" s="14" t="inlineStr">
+        <is>
+          <t>GET /loyalty/program and GET /loyalty/guests had no role guard — any logged-in user could read all guest loyalty data</t>
+        </is>
+      </c>
+      <c r="D53" s="14" t="inlineStr">
+        <is>
+          <t>A receptionist could read all guest loyalty balances and point histories — a privacy and trust issue.</t>
+        </is>
+      </c>
+      <c r="E53" s="14" t="inlineStr">
+        <is>
+          <t>require_hotel_role added to both GET endpoints. OWNER/MANAGER only.</t>
+        </is>
+      </c>
+      <c r="F53" s="40" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G53" s="14" t="inlineStr">
+        <is>
+          <t>14-Jun</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="55" customHeight="1">
+      <c r="A54" s="17" t="inlineStr">
+        <is>
+          <t>S-47</t>
+        </is>
+      </c>
+      <c r="B54" s="18" t="inlineStr">
+        <is>
+          <t>Booking price tolerance was a fixed ₹5 — rejected valid bookings with currency rounding</t>
+        </is>
+      </c>
+      <c r="C54" s="18" t="inlineStr">
+        <is>
+          <t>POST /public/bookings rejected if total differed by more than ₹5 flat, regardless of booking size</t>
+        </is>
+      </c>
+      <c r="D54" s="18" t="inlineStr">
+        <is>
+          <t>For a ₹50,000 booking, a 1-paisa rounding difference could reject a real booking — lost revenue.</t>
+        </is>
+      </c>
+      <c r="E54" s="18" t="inlineStr">
+        <is>
+          <t>Tolerance is now max(₹5, 1% of total) — proportional to booking size.</t>
+        </is>
+      </c>
+      <c r="F54" s="41" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G54" s="18" t="inlineStr">
+        <is>
+          <t>15-Jun</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="55" customHeight="1">
+      <c r="A55" s="16" t="inlineStr">
+        <is>
+          <t>S-48</t>
+        </is>
+      </c>
+      <c r="B55" s="14" t="inlineStr">
+        <is>
+          <t>Guest Recovery feature never ran automatically — 72h window silently expired</t>
+        </is>
+      </c>
+      <c r="C55" s="14" t="inlineStr">
+        <is>
+          <t>Abandoned booking recovery had no scheduled job. The sweep only ran if manually triggered. PENDING bookings aged past 72h without nudge.</t>
+        </is>
+      </c>
+      <c r="D55" s="14" t="inlineStr">
+        <is>
+          <t>Every abandoned booking was permanently lost — the recovery feature was effectively off by default.</t>
+        </is>
+      </c>
+      <c r="E55" s="14" t="inlineStr">
+        <is>
+          <t>Added hourly APScheduler job with Redis lock (one replica only). Per-hotel opt-in respected.</t>
+        </is>
+      </c>
+      <c r="F55" s="40" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G55" s="14" t="inlineStr">
+        <is>
+          <t>15-Jun</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="55" customHeight="1">
+      <c r="A56" s="17" t="inlineStr">
+        <is>
+          <t>S-49</t>
+        </is>
+      </c>
+      <c r="B56" s="18" t="inlineStr">
+        <is>
+          <t>Public booking create AND cancel-confirm both crashed with 500 error</t>
+        </is>
+      </c>
+      <c r="C56" s="18" t="inlineStr">
+        <is>
+          <t>Accessed super_admin.phone (field does not exist on User model). WhatsApp service read wrong env variable names.</t>
+        </is>
+      </c>
+      <c r="D56" s="18" t="inlineStr">
+        <is>
+          <t>Every new booking and every cancellation confirmation threw a 500 — guests could not complete bookings.</t>
+        </is>
+      </c>
+      <c r="E56" s="18" t="inlineStr">
+        <is>
+          <t>Admin alert recipient switched to SUPER_ADMIN_WHATSAPP config env var. WhatsApp service aligned to canonical settings.</t>
+        </is>
+      </c>
+      <c r="F56" s="42" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="G56" s="18" t="inlineStr">
+        <is>
+          <t>15-Jun</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="55" customHeight="1">
+      <c r="A57" s="16" t="inlineStr">
+        <is>
+          <t>S-50</t>
+        </is>
+      </c>
+      <c r="B57" s="14" t="inlineStr">
+        <is>
+          <t>Widget allowed hotels to inject arbitrary JavaScript into every guest browser (RCE sink)</t>
+        </is>
+      </c>
+      <c r="C57" s="14" t="inlineStr">
+        <is>
+          <t>widget_custom_js field was stored and executed via new Function() inside widget-v3.js — any hotelier could run any code in guest browsers</t>
+        </is>
+      </c>
+      <c r="D57" s="14" t="inlineStr">
+        <is>
+          <t>A malicious or compromised hotel account could steal guest payment details from every booking session. This is a Remote Code Execution vulnerability affecting all guests of that hotel.</t>
+        </is>
+      </c>
+      <c r="E57" s="14" t="inlineStr">
+        <is>
+          <t>widget_custom_js field removed entirely from the API and frontend. new Function() eval removed from widget.</t>
+        </is>
+      </c>
+      <c r="F57" s="42" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="G57" s="14" t="inlineStr">
+        <is>
+          <t>15-Jun</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="55" customHeight="1">
+      <c r="A58" s="17" t="inlineStr">
+        <is>
+          <t>S-51</t>
+        </is>
+      </c>
+      <c r="B58" s="18" t="inlineStr">
+        <is>
+          <t>Widget CSS field allowed CSS injection (data exfiltration via url() and expression())</t>
+        </is>
+      </c>
+      <c r="C58" s="18" t="inlineStr">
+        <is>
+          <t>Custom CSS from hotel settings was injected unsanitized — url(), @import, expression() could load external resources or run scripts</t>
+        </is>
+      </c>
+      <c r="D58" s="18" t="inlineStr">
+        <is>
+          <t>A compromised hotel could exfiltrate guest data via CSS-based tracking requests.</t>
+        </is>
+      </c>
+      <c r="E58" s="18" t="inlineStr">
+        <is>
+          <t>CSS sanitizer strips url()/@import/expression()/&lt;script and any external resource references before injection.</t>
+        </is>
+      </c>
+      <c r="F58" s="40" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G58" s="18" t="inlineStr">
+        <is>
+          <t>15-Jun</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="55" customHeight="1">
+      <c r="A59" s="16" t="inlineStr">
+        <is>
+          <t>S-52</t>
+        </is>
+      </c>
+      <c r="B59" s="14" t="inlineStr">
+        <is>
+          <t>Chat widget postMessage accepted messages from any origin</t>
+        </is>
+      </c>
+      <c r="C59" s="14" t="inlineStr">
+        <is>
+          <t>ChatWidget.tsx did not check event.origin — any website embedding our chat could send arbitrary messages</t>
+        </is>
+      </c>
+      <c r="D59" s="14" t="inlineStr">
+        <is>
+          <t>A malicious site embedding our chat widget could control it — fake bookings, data injection.</t>
+        </is>
+      </c>
+      <c r="E59" s="14" t="inlineStr">
+        <is>
+          <t>postMessage origin scoped to verified referrer. Messages from unknown origins silently dropped.</t>
+        </is>
+      </c>
+      <c r="F59" s="40" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G59" s="14" t="inlineStr">
+        <is>
+          <t>15-Jun</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="55" customHeight="1">
+      <c r="A60" s="17" t="inlineStr">
+        <is>
+          <t>S-53</t>
+        </is>
+      </c>
+      <c r="B60" s="18" t="inlineStr">
+        <is>
+          <t>Widget iframe had no sandbox — could access parent page cookies and storage</t>
+        </is>
+      </c>
+      <c r="C60" s="18" t="inlineStr">
+        <is>
+          <t>Booking widget iframe was loaded without sandbox attribute</t>
+        </is>
+      </c>
+      <c r="D60" s="18" t="inlineStr">
+        <is>
+          <t>The widget iframe could access parent page's cookies and localStorage — data leak across hotel's own website.</t>
+        </is>
+      </c>
+      <c r="E60" s="18" t="inlineStr">
+        <is>
+          <t>sandbox='allow-scripts allow-forms allow-same-origin allow-popups' added to all widget iframes.</t>
+        </is>
+      </c>
+      <c r="F60" s="40" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G60" s="18" t="inlineStr">
+        <is>
+          <t>15-Jun</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="55" customHeight="1">
+      <c r="A61" s="16" t="inlineStr">
+        <is>
+          <t>S-54</t>
+        </is>
+      </c>
+      <c r="B61" s="14" t="inlineStr">
+        <is>
+          <t>Two simultaneous bookings could double-spend the same promo code or loyalty points</t>
+        </is>
+      </c>
+      <c r="C61" s="14" t="inlineStr">
+        <is>
+          <t>PromoCode and GuestLoyalty reads had no database lock — two concurrent requests could both pass the balance check</t>
+        </is>
+      </c>
+      <c r="D61" s="14" t="inlineStr">
+        <is>
+          <t>Two guests booking at the same instant could both get a discount from a single-use promo. Loyalty points could be double-spent. Revenue leakage.</t>
+        </is>
+      </c>
+      <c r="E61" s="14" t="inlineStr">
+        <is>
+          <t>SELECT FOR UPDATE added on PromoCode and GuestLoyalty rows during redemption — atomic lock prevents race condition.</t>
+        </is>
+      </c>
+      <c r="F61" s="42" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="G61" s="14" t="inlineStr">
+        <is>
+          <t>15-Jun</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="55" customHeight="1">
+      <c r="A62" s="17" t="inlineStr">
+        <is>
+          <t>S-55</t>
+        </is>
+      </c>
+      <c r="B62" s="18" t="inlineStr">
+        <is>
+          <t>AI lead-capture inputs had no length limit — could send arbitrary data to LLM</t>
+        </is>
+      </c>
+      <c r="C62" s="18" t="inlineStr">
+        <is>
+          <t>Guest name/email/phone passed to AI prepare_booking with no length bound</t>
+        </is>
+      </c>
+      <c r="D62" s="18" t="inlineStr">
+        <is>
+          <t>A guest could send a 100KB string as their 'name' and force a large (expensive) LLM call.</t>
+        </is>
+      </c>
+      <c r="E62" s="18" t="inlineStr">
+        <is>
+          <t>AI lead inputs length-bounded before passing to agent.</t>
+        </is>
+      </c>
+      <c r="F62" s="41" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G62" s="18" t="inlineStr">
+        <is>
+          <t>15-Jun</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="55" customHeight="1">
+      <c r="A63" s="16" t="inlineStr">
+        <is>
+          <t>S-56</t>
+        </is>
+      </c>
+      <c r="B63" s="14" t="inlineStr">
+        <is>
+          <t>Inactive hotel returned full data instead of 404</t>
+        </is>
+      </c>
+      <c r="C63" s="14" t="inlineStr">
+        <is>
+          <t>A hotel set to inactive still served all public endpoints — rooms, rates, booking widget</t>
+        </is>
+      </c>
+      <c r="D63" s="14" t="inlineStr">
+        <is>
+          <t>Guests could book rooms at a hotel that is closed or suspended — operational nightmare.</t>
+        </is>
+      </c>
+      <c r="E63" s="14" t="inlineStr">
+        <is>
+          <t>Inactive hotel slug now returns 404 on all public endpoints.</t>
+        </is>
+      </c>
+      <c r="F63" s="41" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G63" s="14" t="inlineStr">
+        <is>
+          <t>15-Jun</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="55" customHeight="1">
+      <c r="A64" s="17" t="inlineStr">
+        <is>
+          <t>S-57</t>
+        </is>
+      </c>
+      <c r="B64" s="18" t="inlineStr">
+        <is>
+          <t>Guest message length in chat had no cap</t>
+        </is>
+      </c>
+      <c r="C64" s="18" t="inlineStr">
+        <is>
+          <t>Chat endpoint accepted messages of unlimited length</t>
+        </is>
+      </c>
+      <c r="D64" s="18" t="inlineStr">
+        <is>
+          <t>A guest could send a 10MB message — large LLM cost and potential DoS on chat endpoint.</t>
+        </is>
+      </c>
+      <c r="E64" s="18" t="inlineStr">
+        <is>
+          <t>Guest message length capped server-side before LLM call.</t>
+        </is>
+      </c>
+      <c r="F64" s="41" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G64" s="18" t="inlineStr">
+        <is>
+          <t>15-Jun</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="55" customHeight="1">
+      <c r="A65" s="16" t="inlineStr">
+        <is>
+          <t>S-58</t>
+        </is>
+      </c>
+      <c r="B65" s="14" t="inlineStr">
+        <is>
+          <t>Loyalty-check crashed with NameError for first-time guests</t>
+        </is>
+      </c>
+      <c r="C65" s="14" t="inlineStr">
+        <is>
+          <t>milestone variable was undefined after milestones-list refactor — first-time guest loyalty check always threw 500</t>
+        </is>
+      </c>
+      <c r="D65" s="14" t="inlineStr">
+        <is>
+          <t>Every first-time guest checking loyalty status got a 500 error. Loyalty feature broken for new guests.</t>
+        </is>
+      </c>
+      <c r="E65" s="14" t="inlineStr">
+        <is>
+          <t>Fixed with already-computed remaining variable. Regression test added.</t>
+        </is>
+      </c>
+      <c r="F65" s="40" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G65" s="14" t="inlineStr">
+        <is>
+          <t>16-Jun</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A51:G51"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2731,7 +3359,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -3106,10 +3734,450 @@
         </is>
       </c>
     </row>
+    <row r="18" ht="26" customHeight="1">
+      <c r="A18" s="37" t="inlineStr">
+        <is>
+          <t>NEW FEATURES — 14 to 16 June 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="39" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B19" s="39" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="C19" s="39" t="inlineStr">
+        <is>
+          <t>What It Does (Simple Language)</t>
+        </is>
+      </c>
+      <c r="D19" s="39" t="inlineStr">
+        <is>
+          <t>Business Value</t>
+        </is>
+      </c>
+      <c r="E19" s="39" t="inlineStr">
+        <is>
+          <t>Built Safely</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="65" customHeight="1">
+      <c r="A20" s="16" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="B20" s="14" t="inlineStr">
+        <is>
+          <t>Dynamic Pricing Engine</t>
+        </is>
+      </c>
+      <c r="C20" s="14" t="inlineStr">
+        <is>
+          <t>Hotelier sets rules: 'When occupancy &gt; 80%, increase price by 20%'. The engine stacks multiple rules and applies them automatically per night on every availability check.</t>
+        </is>
+      </c>
+      <c r="D20" s="14" t="inlineStr">
+        <is>
+          <t>Hotels maximize revenue on busy days without manual price changes. A premium feature competitors charge thousands for.</t>
+        </is>
+      </c>
+      <c r="E20" s="14" t="inlineStr">
+        <is>
+          <t>Rules are server-computed — never trust client price. Preview-only on calendar; actual charge re-computed at booking. IDOR-guarded by hotel_id.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="65" customHeight="1">
+      <c r="A21" s="17" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="B21" s="18" t="inlineStr">
+        <is>
+          <t>Dynamic Pricing Wired to Actual Booking Charges</t>
+        </is>
+      </c>
+      <c r="C21" s="18" t="inlineStr">
+        <is>
+          <t>Dynamic rules now apply to the real booking amount, not just the preview — price adjusts automatically at checkout based on live occupancy.</t>
+        </is>
+      </c>
+      <c r="D21" s="18" t="inlineStr">
+        <is>
+          <t>Turns the dynamic pricing feature from a display tool into an actual revenue driver.</t>
+        </is>
+      </c>
+      <c r="E21" s="18" t="inlineStr">
+        <is>
+          <t>Client-submitted total verified against server-computed dynamic price (±max ₹5, 1%). Multi-tenant via hotel_id.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="65" customHeight="1">
+      <c r="A22" s="16" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B22" s="14" t="inlineStr">
+        <is>
+          <t>Abandoned Booking Recovery (WhatsApp + Email)</t>
+        </is>
+      </c>
+      <c r="C22" s="14" t="inlineStr">
+        <is>
+          <t>When a guest starts a booking but doesn't complete it, the system automatically sends a WhatsApp/email nudge within 72 hours to bring them back.</t>
+        </is>
+      </c>
+      <c r="D22" s="14" t="inlineStr">
+        <is>
+          <t>Recovers lost bookings automatically — industry average recovery rate is 5-15% of abandoned bookings. Runs without any manual action.</t>
+        </is>
+      </c>
+      <c r="E22" s="14" t="inlineStr">
+        <is>
+          <t>Hourly APScheduler job with Redis lock (one replica only). Per-hotel opt-in. Senders fail-safe — never crash booking flow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="65" customHeight="1">
+      <c r="A23" s="17" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="B23" s="18" t="inlineStr">
+        <is>
+          <t>Seasonal Auto-Apply Promotions (Hotel + Chain)</t>
+        </is>
+      </c>
+      <c r="C23" s="18" t="inlineStr">
+        <is>
+          <t>Hotelier creates a deal with dates (e.g. 'Monsoon Special — 20% off 1–31 July'). No code needed — the discount applies automatically to all bookings in that window.</t>
+        </is>
+      </c>
+      <c r="D23" s="18" t="inlineStr">
+        <is>
+          <t>Run date-based campaigns without training staff on promo codes. Chain can push one deal to all properties at once.</t>
+        </is>
+      </c>
+      <c r="E23" s="18" t="inlineStr">
+        <is>
+          <t>Discount always server-computed. Auto-promos scoped strictly to hotel_id or chain_id. SELECT FOR UPDATE prevents double-apply race.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="65" customHeight="1">
+      <c r="A24" s="16" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="B24" s="14" t="inlineStr">
+        <is>
+          <t>Chain-Wide Upsell Broadcast</t>
+        </is>
+      </c>
+      <c r="C24" s="14" t="inlineStr">
+        <is>
+          <t>A brand owner pushes one stay-upsell offer (e.g. 'Book 3 nights, get free breakfast') to all hotels under their brand at once.</t>
+        </is>
+      </c>
+      <c r="D24" s="14" t="inlineStr">
+        <is>
+          <t>Brand-level campaigns delivered in one click instead of configuring each hotel separately.</t>
+        </is>
+      </c>
+      <c r="E24" s="14" t="inlineStr">
+        <is>
+          <t>get_chain_admin required. Each hotel gets its own LoyaltyOffer row (no shared mutable state). IDOR-guarded by chain_id.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="65" customHeight="1">
+      <c r="A25" s="17" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="B25" s="18" t="inlineStr">
+        <is>
+          <t>Room-Specific Night-Threshold Stay Offers</t>
+        </is>
+      </c>
+      <c r="C25" s="18" t="inlineStr">
+        <is>
+          <t>Hotelier configures: 'For Deluxe rooms, guests who book 3+ nights see a special offer pop-up'. Works per room type.</t>
+        </is>
+      </c>
+      <c r="D25" s="18" t="inlineStr">
+        <is>
+          <t>Targeted upsells per room type — increases average booking length and direct booking revenue.</t>
+        </is>
+      </c>
+      <c r="E25" s="18" t="inlineStr">
+        <is>
+          <t>All offer routes role-gated (OWNER/MANAGER). room_type validated against calling hotel. Fails closed on error.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="65" customHeight="1">
+      <c r="A26" s="16" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="B26" s="14" t="inlineStr">
+        <is>
+          <t>Configurable Points Wallet (Earn/Redeem Rates)</t>
+        </is>
+      </c>
+      <c r="C26" s="14" t="inlineStr">
+        <is>
+          <t>Hotel owner sets how many points per rupee guests earn, and what each point is worth at redemption. Fully configurable per hotel.</t>
+        </is>
+      </c>
+      <c r="D26" s="14" t="inlineStr">
+        <is>
+          <t>Flexibility to run aggressive loyalty campaigns or conservative ones based on margins.</t>
+        </is>
+      </c>
+      <c r="E26" s="14" t="inlineStr">
+        <is>
+          <t>Config role-gated OWNER/MANAGER. Redemption value recomputed server-side — client cannot inflate point value.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="65" customHeight="1">
+      <c r="A27" s="17" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B27" s="18" t="inlineStr">
+        <is>
+          <t>Public Pre-Booking Stay-Offer Nudge</t>
+        </is>
+      </c>
+      <c r="C27" s="18" t="inlineStr">
+        <is>
+          <t>Before checkout, guests see a message: 'Book one more night to unlock a special offer'. Drives longer stays.</t>
+        </is>
+      </c>
+      <c r="D27" s="18" t="inlineStr">
+        <is>
+          <t>Increases average length of stay — one extra night per booking adds meaningful revenue at zero acquisition cost.</t>
+        </is>
+      </c>
+      <c r="E27" s="18" t="inlineStr">
+        <is>
+          <t>Public rate-limited 30/min. Returns nudge/unlocked based on server-computed nights. Fails closed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="65" customHeight="1">
+      <c r="A28" s="16" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="B28" s="14" t="inlineStr">
+        <is>
+          <t>HMAC Anti-Automation Booking Token</t>
+        </is>
+      </c>
+      <c r="C28" s="14" t="inlineStr">
+        <is>
+          <t>A server-issued token (valid 10 min) is required before a booking can be created — prevents bots from spamming the booking API.</t>
+        </is>
+      </c>
+      <c r="D28" s="14" t="inlineStr">
+        <is>
+          <t>Protects against automated booking spam that could exhaust inventory or trigger payment fees.</t>
+        </is>
+      </c>
+      <c r="E28" s="14" t="inlineStr">
+        <is>
+          <t>Rate-limited 30/min. HMAC-signed with server secret. Gated by BOOKING_TOKEN_REQUIRED flag (default off for rollout).</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="65" customHeight="1">
+      <c r="A29" s="17" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="B29" s="18" t="inlineStr">
+        <is>
+          <t>Revenue Section UI</t>
+        </is>
+      </c>
+      <c r="C29" s="18" t="inlineStr">
+        <is>
+          <t>New 'Revenue' group in the hotelier sidebar combining Dynamic Pricing, Guest Recovery, and Loyalty in one place.</t>
+        </is>
+      </c>
+      <c r="D29" s="18" t="inlineStr">
+        <is>
+          <t>Hoteliers have a single section to manage all revenue-optimization tools — clear and professional.</t>
+        </is>
+      </c>
+      <c r="E29" s="18" t="inlineStr">
+        <is>
+          <t>Sidebar Revenue group gated by role_permissions (OWNER/MANAGER only).</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="65" customHeight="1">
+      <c r="A30" s="16" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="B30" s="14" t="inlineStr">
+        <is>
+          <t>Loyalty &amp; Upsell Hub</t>
+        </is>
+      </c>
+      <c r="C30" s="14" t="inlineStr">
+        <is>
+          <t>Reorganized loyalty page with tabs: Loyal Guests first, then program settings, then upsell offers. Each tab has a business-value callout.</t>
+        </is>
+      </c>
+      <c r="D30" s="14" t="inlineStr">
+        <is>
+          <t>Hoteliers immediately see their loyal guests (the outcome) before seeing settings (the controls).</t>
+        </is>
+      </c>
+      <c r="E30" s="14" t="inlineStr">
+        <is>
+          <t>All reads tenant-scoped. No API change — UI reorganization only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="65" customHeight="1">
+      <c r="A31" s="17" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="B31" s="18" t="inlineStr">
+        <is>
+          <t>Quick Upsell Templates</t>
+        </is>
+      </c>
+      <c r="C31" s="18" t="inlineStr">
+        <is>
+          <t>One-click templates to create common add-ons: 'Airport Transfer', 'Breakfast Package', 'Spa Session', etc.</t>
+        </is>
+      </c>
+      <c r="D31" s="18" t="inlineStr">
+        <is>
+          <t>Hotels can set up upsell add-ons in seconds without writing descriptions from scratch.</t>
+        </is>
+      </c>
+      <c r="E31" s="18" t="inlineStr">
+        <is>
+          <t>Calls authenticated apiClient — tenant scoping enforced server-side.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="65" customHeight="1">
+      <c r="A32" s="16" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="B32" s="14" t="inlineStr">
+        <is>
+          <t>Package Validity Window + Savings Badge</t>
+        </is>
+      </c>
+      <c r="C32" s="14" t="inlineStr">
+        <is>
+          <t>Packages now have optional valid_from/valid_to dates. Package cards show 'Save ₹X' badge and validity period.</t>
+        </is>
+      </c>
+      <c r="D32" s="14" t="inlineStr">
+        <is>
+          <t>Time-limited packages drive urgency. Savings badge increases conversion.</t>
+        </is>
+      </c>
+      <c r="E32" s="14" t="inlineStr">
+        <is>
+          <t>Tenant scoping unchanged. DB columns valid_from + valid_to added cleanly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="65" customHeight="1">
+      <c r="A33" s="17" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="B33" s="18" t="inlineStr">
+        <is>
+          <t>Brand Console Collapsible Sidebar</t>
+        </is>
+      </c>
+      <c r="C33" s="18" t="inlineStr">
+        <is>
+          <t>The chain management console now has a collapsible sidebar (Overview / Guest Insights / Brand Promos / Brand Loyalty / Upsell Broadcast) replacing horizontal tabs. Collapses to icon rail on small screens.</t>
+        </is>
+      </c>
+      <c r="D33" s="18" t="inlineStr">
+        <is>
+          <t>Professional enterprise look for chain owners managing multiple hotels.</t>
+        </is>
+      </c>
+      <c r="E33" s="18" t="inlineStr">
+        <is>
+          <t>Chain console gated by user.chain_id. React Query fetches per section (enabled by active section only).</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="65" customHeight="1">
+      <c r="A34" s="16" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="B34" s="14" t="inlineStr">
+        <is>
+          <t>Domain-Driven Design (DDD) Refactoring</t>
+        </is>
+      </c>
+      <c r="C34" s="14" t="inlineStr">
+        <is>
+          <t>The entire codebase was restructured following DDD principles — clear separation between domains (booking, loyalty, revenue, etc.). Temporary scripts removed.</t>
+        </is>
+      </c>
+      <c r="D34" s="14" t="inlineStr">
+        <is>
+          <t>Easier to add new features without breaking existing ones. New developers can understand the codebase faster. Reduces bugs from spaghetti code.</t>
+        </is>
+      </c>
+      <c r="E34" s="14" t="inlineStr">
+        <is>
+          <t>No API changes — internal refactor only. All existing tests pass.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A18:E18"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3125,212 +4193,212 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="50" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="50" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="38" customHeight="1">
+      <c r="A1" s="43" t="inlineStr">
         <is>
           <t>What Is Being Worked On Right Now</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Critical items in progress — one person cannot do these in parallel, which is why a team is needed</t>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="36" t="inlineStr">
+        <is>
+          <t>Updated 16-Jun-2026  ·  Items in progress — these require dedicated developer time to complete</t>
         </is>
       </c>
     </row>
     <row r="4" ht="26" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="39" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="39" t="inlineStr">
         <is>
           <t>Task</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="39" t="inlineStr">
         <is>
           <t>Why It Matters</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="39" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="39" t="inlineStr">
         <is>
           <t>Risk If Delayed</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="47" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
+    <row r="5" ht="72" customHeight="1">
+      <c r="A5" s="16" t="inlineStr">
         <is>
           <t>P-01</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>Razorpay payment failure recovery (money deducted but booking not created)</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>Guest's network dropped mid-payment / Razorpay API failed — money was deducted but the booking got cancelled. Idempotency and webhook verification are already implemented; the auto-refund flow and reconciliation job still need to be built.</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="B5" s="14" t="inlineStr">
+        <is>
+          <t>Razorpay payment failure auto-recovery (money deducted, booking not created)</t>
+        </is>
+      </c>
+      <c r="C5" s="14" t="inlineStr">
+        <is>
+          <t>When a guest's network drops mid-payment, money is deducted but the booking gets cancelled. Idempotency and webhook verification already in place. Auto-refund flow and daily reconciliation job still to be built.</t>
+        </is>
+      </c>
+      <c r="D5" s="14" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>Guests' money stays stuck and refunds must be done manually. Angry guests, chargebacks, Razorpay disputes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="32" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="E5" s="14" t="inlineStr">
+        <is>
+          <t>Guests' money stays stuck. Manual refunds required. Angry guests, chargebacks, Razorpay disputes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="72" customHeight="1">
+      <c r="A6" s="17" t="inlineStr">
         <is>
           <t>P-02</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>Load testing — what happens when 100+ users book at the same time</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>Database locks already protect against race conditions (one room sold twice), but real-load behaviour (connection pool exhaustion, timeouts) still needs testing.</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>Load testing — what happens when 100+ users book simultaneously</t>
+        </is>
+      </c>
+      <c r="C6" s="18" t="inlineStr">
+        <is>
+          <t>DB locks protect against double-booking race conditions, but real-load behaviour (connection pool exhaustion, timeouts) still needs testing before a large campaign.</t>
+        </is>
+      </c>
+      <c r="D6" s="18" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>The site goes down during peak season or a viral campaign — losses on exactly the highest-revenue days.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="49" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="E6" s="18" t="inlineStr">
+        <is>
+          <t>Site goes down during peak season — losses on exactly the highest-revenue days.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="72" customHeight="1">
+      <c r="A7" s="16" t="inlineStr">
         <is>
           <t>P-03</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>Frontend page-by-page error audit (errors + edge cases on every page)</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>Every page must handle network failures, double-clicks, and slow-data scenarios gracefully. The public booking widget pages are done (error+retry UI, date validation, fake-data removal — see S-34, S-36, S-37); the hotelier dashboard pages are next.</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="B7" s="14" t="inlineStr">
+        <is>
+          <t>Hotelier dashboard pages error audit</t>
+        </is>
+      </c>
+      <c r="C7" s="14" t="inlineStr">
+        <is>
+          <t>Public booking widget pages are fully hardened (error+retry, date validation, real data). Hotelier dashboard pages need the same treatment — every page must handle network failures and slow-data gracefully.</t>
+        </is>
+      </c>
+      <c r="D7" s="14" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>White screens and stuck buttons in front of guests = dropped bookings and brand damage.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="44" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="E7" s="14" t="inlineStr">
+        <is>
+          <t>White screens and stuck buttons in the hotelier dashboard = support calls and lost trust.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="72" customHeight="1">
+      <c r="A8" s="17" t="inlineStr">
         <is>
           <t>P-04</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>DDoS / abuse protection layer (WAF)</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>The IP-spoofing hole is now FIXED (trusted-proxy IP extraction, S-40) and key routes are rate-limited (S-42). The remaining piece is an edge layer (Cloudflare/WAF) to absorb large-scale attacks before they reach our servers.</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>DDoS / abuse protection layer (WAF edge)</t>
+        </is>
+      </c>
+      <c r="C8" s="18" t="inlineStr">
+        <is>
+          <t>IP-spoofing hole is fixed (S-40). Key routes are rate-limited (S-42). The remaining piece is a Cloudflare WAF rule set to absorb large-scale attacks before they reach Railway.</t>
+        </is>
+      </c>
+      <c r="D8" s="18" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>Large fake-traffic attacks are inexpensive to launch and could make the site unavailable on important days.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="42" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="E8" s="18" t="inlineStr">
+        <is>
+          <t>Large fake-traffic attacks are cheap to launch and could make the site unavailable on important days.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="72" customHeight="1">
+      <c r="A9" s="16" t="inlineStr">
         <is>
           <t>P-05</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>Database migration discipline (Alembic in the deploy process)</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>The schema is currently built by create_all at startup; performance indexes may be missing in production. The hottest availability index has been added manually (S-38), but a proper migration process is needed.</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="B9" s="14" t="inlineStr">
+        <is>
+          <t>Database migration discipline (Alembic)</t>
+        </is>
+      </c>
+      <c r="C9" s="14" t="inlineStr">
+        <is>
+          <t>Schema is currently managed by create_all at startup. A proper Alembic migration process is needed for safe, tracked schema changes in production.</t>
+        </is>
+      </c>
+      <c r="D9" s="14" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>As data grows, queries get slow → the whole app gets slow.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="61" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="E9" s="14" t="inlineStr">
+        <is>
+          <t>Untracked schema changes in production = difficult rollbacks and potential data loss.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="72" customHeight="1">
+      <c r="A10" s="17" t="inlineStr">
         <is>
           <t>P-06</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>Remaining medium-severity audit findings</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>The June security audit logged 36 findings. The Critical issue and most High items are fixed. Items still being worked through include: the login-token cache window (~10 min), the unsigned OAuth state parameter, an unauthenticated competitor data-freshness endpoint, and stale analytics cache invalidation.</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="B10" s="18" t="inlineStr">
+        <is>
+          <t>Remaining medium-severity security audit findings</t>
+        </is>
+      </c>
+      <c r="C10" s="18" t="inlineStr">
+        <is>
+          <t>June security audit logged 36 findings. Critical and most High items are fixed. Remaining: login-token cache window (~10 min), unsigned OAuth state parameter, unauthenticated competitor data-freshness endpoint, stale analytics cache invalidation.</t>
+        </is>
+      </c>
+      <c r="D10" s="18" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
-        <is>
-          <t>Each one is a small gap today; closing them before scale keeps the risk small.</t>
+      <c r="E10" s="18" t="inlineStr">
+        <is>
+          <t>Each is a small gap today. Closing before scale keeps risk small.</t>
         </is>
       </c>
     </row>
@@ -4699,8 +5767,8 @@
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="B9:E9"/>
     <mergeCell ref="A12:E12"/>
-    <mergeCell ref="B9:E9"/>
     <mergeCell ref="A4:E4"/>
     <mergeCell ref="B8:E8"/>
     <mergeCell ref="A20:E20"/>

</xml_diff>

<commit_message>
docs: expand CEO report with engineering, stability and scaling detail
- Refresh Executive Summary to reference new sheets + architecture diagram
- Team & Hiring: add stakeholder note and 'what each hire returns' table
- New sheet: Engineering Plan by Role (API optimisation, continuous bug-hunting)
- New sheet: Silent Bugs & Server Stability (quiet crash risks; why the app won't go blank)
- New sheet: Scaling to Large Data (DB to browser millisecond speed budget)

https://claude.ai/code/session_01Jfp6dFcb8aisQfoK5brnT1
</commit_message>
<xml_diff>
--- a/docs/CEO_Report_Staybooker_Jun2026.xlsx
+++ b/docs/CEO_Report_Staybooker_Jun2026.xlsx
@@ -13,6 +13,9 @@
     <sheet name="4. Work In Progress" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="5. Future Risks" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="6. Team &amp; Hiring" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="7. Engineering Plan by Role" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="8. Silent Bugs &amp; Stability" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="9. Scaling to Large Data" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -53,8 +56,16 @@
       <color rgb="001F4E79"/>
       <sz val="12"/>
     </font>
+    <font>
+      <color rgb="00555555"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -86,8 +97,13 @@
         <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -109,11 +125,25 @@
         <color rgb="00BBBBBB"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -135,6 +165,27 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -500,200 +551,252 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
     <col width="120" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1">
+    <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Staybooker Booking Engine — CEO Report (June 2026)</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>What has been solved, what is in progress, what risks are coming, and why we need a team — at a glance</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="26" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
+    <row r="2" ht="28" customHeight="1">
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>What has been solved, what is in progress, what risks are coming, how the product stays fast and crash-proof at scale, and why we need a team — at a glance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>Topic</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="10" t="inlineStr">
         <is>
           <t>Detail</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="11" t="inlineStr">
         <is>
           <t>WHAT THIS REPORT CONTAINS</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr"/>
-    </row>
-    <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="B5" s="12" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="13" t="inlineStr">
         <is>
           <t>Sheet 2 — Problems Solved</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" s="13" t="inlineStr">
         <is>
           <t>45 issues fixed so far (5 Critical, 24 High, 16 Medium). Each issue shows what would have happened to the business if it had reached production.</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="36" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="13" t="inlineStr">
         <is>
           <t>Sheet 3 — Features Built</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="13" t="inlineStr">
         <is>
           <t>Major product features delivered alongside the bug fixing — multi-property chains, loyalty program, OTA rate intelligence, AI concierge, real-time updates, encrypted secrets storage.</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="13" t="inlineStr">
         <is>
           <t>Sheet 4 — Work In Progress</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="13" t="inlineStr">
         <is>
           <t>Critical items currently being worked on.</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="40" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="13" t="inlineStr">
         <is>
           <t>Sheet 5 — Future Risks</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" s="13" t="inlineStr">
         <is>
           <t>13 real-world scenarios that WILL come as the business grows (100 users at once, payment failures, DDoS attacks, data growing to GBs) — what protection already exists and what still needs to be built.</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="34" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="13" t="inlineStr">
         <is>
           <t>Sheet 6 — Team &amp; Hiring</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>What a Tech Lead / Backend / Frontend / Database developer actually does, in simple language — who owns which part of the product as it grows, with a suggested hiring order.</t>
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>What a Tech Lead / Backend / Frontend / Database developer actually does, in simple language — who owns which part of the product as it grows, with a suggested hiring order and a note for stakeholders.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr"/>
-      <c r="B11" s="4" t="inlineStr"/>
-    </row>
-    <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>Sheet 7 — Engineering Plan by Role (NEW)</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>The detailed, day-to-day work each developer does as we grow — how APIs are kept fast and cheap (optimisation), and the constant bug-hunting that keeps the server stable. This is the 'what exactly will they do all day' answer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t>Sheet 8 — Silent Bugs &amp; Server Stability (NEW)</t>
+        </is>
+      </c>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>The most dangerous bugs are the quiet ones — no error on screen, but the server slowly leaks, stalls or crashes. This sheet lists that class of risk, what already protects us, and why the whole software will NOT go blank.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t>Sheet 9 — Scaling to Large Data (NEW)</t>
+        </is>
+      </c>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>When a hotel has 2–3 years of bookings (GBs of data), it must still travel database → backend → browser in milliseconds and the page must never freeze. This sheet shows the speed budget and the plan to hold it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="13" t="inlineStr">
+        <is>
+          <t>Architecture diagram (NEW)</t>
+        </is>
+      </c>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>A full visual map of the system — Staybooker_Architecture.excalidraw at the project root — showing how a request flows from the guest's browser through Cloudflare, the backend, Redis and the database, and back. Useful when onboarding any new engineer or stakeholder.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="11" t="inlineStr">
         <is>
           <t>KEY NUMBERS</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr"/>
-    </row>
-    <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="B16" s="12" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="13" t="inlineStr">
         <is>
           <t>Issues fixed till date</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>45 (source: work_log_tracker.csv — 71 logged engineering tasks up to 11-Jun-2026)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="4" t="inlineStr">
+      <c r="B17" s="13" t="inlineStr">
+        <is>
+          <t>45 (source: work_log_tracker.csv — engineering tasks logged up to 16-Jun-2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="13" t="inlineStr">
         <is>
           <t>Critical issues fixed</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>5 — payment secret key leak, payment amount tampering, permanent admin token, AI assistant crash, staff privilege escalation</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="40" customHeight="1">
-      <c r="A15" s="4" t="inlineStr">
+      <c r="B18" s="13" t="inlineStr">
+        <is>
+          <t>5 — payment secret key leak, payment amount tampering, permanent admin token, AI assistant crash, staff privilege escalation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="13" t="inlineStr">
         <is>
           <t>Security audit coverage</t>
         </is>
       </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>A full security/performance audit found 36 findings (1 Critical, 12 High, 14 Medium, 9 Low). The Critical issue and most High findings are fixed; the remaining items are tracked openly in Sheets 4 and 5.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="39" customHeight="1">
-      <c r="A16" s="4" t="inlineStr">
+      <c r="B19" s="13" t="inlineStr">
+        <is>
+          <t>A full security/performance audit found 36 findings (1 Critical, 12 High, 14 Medium, 9 Low). The Critical issue and most High findings are fixed; the rest are tracked openly in Sheets 4 and 5.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="13" t="inlineStr">
         <is>
           <t>Automated tests added</t>
         </is>
       </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B20" s="13" t="inlineStr">
         <is>
           <t>277 test cases passing (security, payments, booking, role access, rate limits, Redis failover). These run automatically on every code change (CI/CD), plus dependency vulnerability (CVE) scanning.</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="54" customHeight="1">
-      <c r="A17" s="4" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="13" t="inlineStr">
         <is>
           <t>Money saved (examples)</t>
         </is>
       </c>
-      <c r="B17" s="4" t="inlineStr">
+      <c r="B21" s="13" t="inlineStr">
         <is>
           <t>Payment tampering fix: a guest could pay Rs.1 and get a Rs.10,000 booking confirmed. AI cost fix: a bug was sending traffic to an AI model 10x more expensive than needed on the public chatbot. Tax validation fix: invalid tax setup could produce wrong bills for every guest.</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr"/>
-      <c r="B18" s="4" t="inlineStr"/>
-    </row>
-    <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="4" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="13" t="inlineStr">
+        <is>
+          <t>Stability posture</t>
+        </is>
+      </c>
+      <c r="B22" s="13" t="inlineStr">
+        <is>
+          <t>The app is built to fail SAFE: if Redis drops it falls back to in-memory limits; if a data fetch fails the guest sees a Retry button, never a blank page; security and money checks 'fail closed' (deny), while the screen 'fails soft' (keeps working). Details in Sheets 8 and 9.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="11" t="inlineStr">
         <is>
           <t>ONE-LINE MESSAGE FOR THE CEO</t>
         </is>
       </c>
-      <c r="B19" s="4" t="inlineStr"/>
-    </row>
-    <row r="20" ht="50" customHeight="1">
-      <c r="A20" s="4" t="inlineStr">
+      <c r="B24" s="12" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="13" t="inlineStr">
         <is>
           <t>Bottom line</t>
         </is>
       </c>
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>The product is stable today and hoteliers' data is safe. The hiring need comes from growth: as hotels, traffic and data scale up, each layer — database, backend, frontend — needs a dedicated owner so quality and safety stay exactly where they are today.</t>
+      <c r="B25" s="13" t="inlineStr">
+        <is>
+          <t>The product is stable today and hoteliers' data is safe. The hiring need comes from growth: as hotels, traffic and data scale up, each layer — database, backend, frontend — needs a dedicated owner so the speed, safety and crash-proofing stay exactly where they are today. This report now also spells out, in plain language, the ongoing engineering work that keeps it that way (Sheets 7–9).</t>
         </is>
       </c>
     </row>
@@ -3703,7 +3806,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3793,7 +3896,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
@@ -3886,8 +3988,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
-    <row r="18"/>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="8" t="inlineStr">
         <is>
@@ -3980,8 +4080,6 @@
         </is>
       </c>
     </row>
-    <row r="25"/>
-    <row r="26"/>
     <row r="27" ht="30" customHeight="1">
       <c r="A27" s="8" t="inlineStr">
         <is>
@@ -4099,11 +4197,1453 @@
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" s="8" t="inlineStr">
+        <is>
+          <t>A NOTE FOR STAKEHOLDERS (why this ask, framed plainly)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="90" customHeight="1">
+      <c r="A35" s="13" t="inlineStr">
+        <is>
+          <t>This is not a request to fix something broken — the product works and customer data is safe today. It is a request to PROTECT what has been built and to DE-RISK growth. Up to now one person has carried database, backend and frontend together. That is fine at the current size, but every new hotel multiplies the data, the traffic and the number of places a single quiet bug could cause a slow page or an outage. Each role below removes a specific, named risk to revenue and reputation. Hiring in the order shown means we always add the person who removes the biggest risk next — never headcount for its own sake.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="8" t="inlineStr">
+        <is>
+          <t>WHAT EACH HIRE RETURNS (in business terms)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="30" customHeight="1">
+      <c r="A38" s="10" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="B38" s="10" t="inlineStr">
+        <is>
+          <t>The risk it removes</t>
+        </is>
+      </c>
+      <c r="C38" s="10" t="inlineStr">
+        <is>
+          <t>What the business gets back</t>
+        </is>
+      </c>
+      <c r="D38" s="10" t="inlineStr">
+        <is>
+          <t>If we keep delaying</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="14" t="inlineStr">
+        <is>
+          <t>Backend Dev</t>
+        </is>
+      </c>
+      <c r="B39" s="13" t="inlineStr">
+        <is>
+          <t>Stuck payments, slow APIs under load, runaway costs, a crash on a peak day.</t>
+        </is>
+      </c>
+      <c r="C39" s="13" t="inlineStr">
+        <is>
+          <t>Money never gets stuck (auto-refund + reconciliation); the booking path stays fast when 100 people book at once; AI and server bills stay predictable.</t>
+        </is>
+      </c>
+      <c r="D39" s="13" t="inlineStr">
+        <is>
+          <t>A peak-day outage or a stuck-payment incident on the highest-revenue day — exactly when it hurts most.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="14" t="inlineStr">
+        <is>
+          <t>Frontend Dev</t>
+        </is>
+      </c>
+      <c r="B40" s="13" t="inlineStr">
+        <is>
+          <t>Blank/white screens, double bookings, slow pages that make guests leave.</t>
+        </is>
+      </c>
+      <c r="C40" s="13" t="inlineStr">
+        <is>
+          <t>Every page recovers from a network blip with a Retry; no duplicate bookings; pages load in under ~2s, which directly lifts conversion.</t>
+        </is>
+      </c>
+      <c r="D40" s="13" t="inlineStr">
+        <is>
+          <t>Lost bookings every day to slow or broken pages — a silent, daily revenue leak that is hard to even notice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="14" t="inlineStr">
+        <is>
+          <t>Database Dev</t>
+        </is>
+      </c>
+      <c r="B41" s="13" t="inlineStr">
+        <is>
+          <t>Dashboards crawling once data reaches GBs; a backup that has never been test-restored.</t>
+        </is>
+      </c>
+      <c r="C41" s="13" t="inlineStr">
+        <is>
+          <t>Queries stay in milliseconds at any data size (indexes, partitioning, archiving); backups are proven to actually restore.</t>
+        </is>
+      </c>
+      <c r="D41" s="13" t="inlineStr">
+        <is>
+          <t>The product feels slower for every hotel as it succeeds — and an un-tested backup is a bet the business cannot afford to lose.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="14" t="inlineStr">
+        <is>
+          <t>Tech Lead</t>
+        </is>
+      </c>
+      <c r="B42" s="13" t="inlineStr">
+        <is>
+          <t>One person reviewing everything; no second pair of eyes on security or money code.</t>
+        </is>
+      </c>
+      <c r="C42" s="13" t="inlineStr">
+        <is>
+          <t>A human review gate on every change — the single most effective catch for the silent bugs in Sheet 8 — plus a clear roadmap.</t>
+        </is>
+      </c>
+      <c r="D42" s="13" t="inlineStr">
+        <is>
+          <t>Risk concentrates on one person; quality depends on no one ever having an off day.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="5">
+    <mergeCell ref="A37:D37"/>
     <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A34:D34"/>
+    <mergeCell ref="A35:D35"/>
     <mergeCell ref="A1:E1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D39"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Engineering Plan by Role — What Each Developer Does, Day to Day</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="28" customHeight="1">
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>The concrete, ongoing work behind 'why a team'. This answers, in plain language: how do we keep the APIs fast (optimisation), and what is the constant bug-hunting that keeps the server stable as we grow?</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>BACKEND DEVELOPER</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="32" customHeight="1">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>Owns the APIs and their link to the database — payments, booking logic, security, speed and cost. This is where 'API optimisation' and most server-crash prevention live.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>Ongoing job</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>What the work actually is</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>Why it matters to the business</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="inlineStr">
+        <is>
+          <t>What it prevents</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="14" t="inlineStr">
+        <is>
+          <t>API optimisation</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>Measure each endpoint's response time, cache hot reads in Redis, replace many small queries with one batched query (kill N+1), enforce pagination caps, and push slow work (emails, sync) into background tasks.</t>
+        </is>
+      </c>
+      <c r="C7" s="13" t="inlineStr">
+        <is>
+          <t>Fast pages keep guests booking and keep the server bill low — speed is revenue.</t>
+        </is>
+      </c>
+      <c r="D7" s="13" t="inlineStr">
+        <is>
+          <t>Timeouts, slow dashboards, and a database overloaded by repeated heavy queries.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>Continuous bug-hunting</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>Every new endpoint is read for the quiet failure modes: swallowed exceptions, wrong query cardinality, missing limits, fail-open checks. (See Sheet 8 for the catalogue.)</t>
+        </is>
+      </c>
+      <c r="C8" s="13" t="inlineStr">
+        <is>
+          <t>These are the bugs that don't show an error but quietly crash or stall the server.</t>
+        </is>
+      </c>
+      <c r="D8" s="13" t="inlineStr">
+        <is>
+          <t>Silent outages and 'the site is slow / down' incidents that nobody can explain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>Payment integrity</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>Build and run the auto-refund flow and a daily reconciliation job that matches the Razorpay ledger against our bookings.</t>
+        </is>
+      </c>
+      <c r="C9" s="13" t="inlineStr">
+        <is>
+          <t>Guest money is never stuck; disputes and chargebacks drop.</t>
+        </is>
+      </c>
+      <c r="D9" s="13" t="inlineStr">
+        <is>
+          <t>Manual refunds, angry guests, and Razorpay disputes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>Security on every route</t>
+        </is>
+      </c>
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>Add the role gate and tenant (hotel_id) filter to every new endpoint, and verify amounts/ids server-side.</t>
+        </is>
+      </c>
+      <c r="C10" s="13" t="inlineStr">
+        <is>
+          <t>Each new feature ships without opening a data-isolation or tampering hole.</t>
+        </is>
+      </c>
+      <c r="D10" s="13" t="inlineStr">
+        <is>
+          <t>Cross-hotel data leaks and price/role tampering.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="14" t="inlineStr">
+        <is>
+          <t>Cost control</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Cap LLM tokens, enforce per-hotel AI quotas, bound DB rows returned and background work.</t>
+        </is>
+      </c>
+      <c r="C11" s="13" t="inlineStr">
+        <is>
+          <t>AI and infra costs stay predictable as usage grows.</t>
+        </is>
+      </c>
+      <c r="D11" s="13" t="inlineStr">
+        <is>
+          <t>A surprise lakhs-level AI bill from a single abusive script.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>Observability</t>
+        </is>
+      </c>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>Structured logs (no PII), error-rate alerts, and dashboards so problems are seen before customers complain.</t>
+        </is>
+      </c>
+      <c r="C12" s="13" t="inlineStr">
+        <is>
+          <t>We hear about issues from our alerts, not from an angry hotelier.</t>
+        </is>
+      </c>
+      <c r="D12" s="13" t="inlineStr">
+        <is>
+          <t>Problems festering silently until they become outages.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>FRONTEND DEVELOPER</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="32" customHeight="1">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>Owns the React + TypeScript screens and their link to the backend APIs. This is real engineering — correct data, fast loads, no blank screens — not visual design.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>Ongoing job</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>What the work actually is</t>
+        </is>
+      </c>
+      <c r="C16" s="10" t="inlineStr">
+        <is>
+          <t>Why it matters to the business</t>
+        </is>
+      </c>
+      <c r="D16" s="10" t="inlineStr">
+        <is>
+          <t>What it prevents</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="14" t="inlineStr">
+        <is>
+          <t>API integration hardening</t>
+        </is>
+      </c>
+      <c r="B17" s="13" t="inlineStr">
+        <is>
+          <t>Every page gets a loading state, an error state and a Retry — and tolerates slow or partial data without breaking.</t>
+        </is>
+      </c>
+      <c r="C17" s="13" t="inlineStr">
+        <is>
+          <t>A network blip never shows the guest a blank page; the booking continues.</t>
+        </is>
+      </c>
+      <c r="D17" s="13" t="inlineStr">
+        <is>
+          <t>White screens mid-booking → closed tabs → lost bookings.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="14" t="inlineStr">
+        <is>
+          <t>Page-speed optimisation</t>
+        </is>
+      </c>
+      <c r="B18" s="13" t="inlineStr">
+        <is>
+          <t>Code-splitting, lazy loading, image optimisation, and trimming the JavaScript bundle; monitor Core Web Vitals.</t>
+        </is>
+      </c>
+      <c r="C18" s="13" t="inlineStr">
+        <is>
+          <t>Every extra second of load time cuts conversion ~7% — speed is direct revenue.</t>
+        </is>
+      </c>
+      <c r="D18" s="13" t="inlineStr">
+        <is>
+          <t>Guests bouncing off a slow page before they ever see a room.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="14" t="inlineStr">
+        <is>
+          <t>Large-data rendering</t>
+        </is>
+      </c>
+      <c r="B19" s="13" t="inlineStr">
+        <is>
+          <t>Virtual scrolling and paged lists so a hotel with thousands of bookings still renders instantly.</t>
+        </is>
+      </c>
+      <c r="C19" s="13" t="inlineStr">
+        <is>
+          <t>The dashboard stays smooth even for the biggest, most valuable hotels.</t>
+        </is>
+      </c>
+      <c r="D19" s="13" t="inlineStr">
+        <is>
+          <t>The browser freezing while it tries to draw thousands of rows.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="14" t="inlineStr">
+        <is>
+          <t>Double-submit &amp; concurrency guards</t>
+        </is>
+      </c>
+      <c r="B20" s="13" t="inlineStr">
+        <is>
+          <t>Disable buttons on submit, add idempotent retries, warn on conflicting edits across tabs.</t>
+        </is>
+      </c>
+      <c r="C20" s="13" t="inlineStr">
+        <is>
+          <t>No accidental duplicate bookings or double payments on slow networks.</t>
+        </is>
+      </c>
+      <c r="D20" s="13" t="inlineStr">
+        <is>
+          <t>Two bookings / two charges from one impatient double-click.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="14" t="inlineStr">
+        <is>
+          <t>Real-time UI</t>
+        </is>
+      </c>
+      <c r="B21" s="13" t="inlineStr">
+        <is>
+          <t>Wire dashboards to the live WebSocket/SSE updates so new bookings appear without a refresh.</t>
+        </is>
+      </c>
+      <c r="C21" s="13" t="inlineStr">
+        <is>
+          <t>The product feels modern and 'alive'; staff react instantly.</t>
+        </is>
+      </c>
+      <c r="D21" s="13" t="inlineStr">
+        <is>
+          <t>Stale screens and missed bookings.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>DATABASE DEVELOPER</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="32" customHeight="1">
+      <c r="A24" s="15" t="inlineStr">
+        <is>
+          <t>Owns the data layer — speed, schema, backups and the guarantee that data flows out smoothly at ANY size. Becomes essential as data approaches GB scale; can start part-time.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="30" customHeight="1">
+      <c r="A25" s="10" t="inlineStr">
+        <is>
+          <t>Ongoing job</t>
+        </is>
+      </c>
+      <c r="B25" s="10" t="inlineStr">
+        <is>
+          <t>What the work actually is</t>
+        </is>
+      </c>
+      <c r="C25" s="10" t="inlineStr">
+        <is>
+          <t>Why it matters to the business</t>
+        </is>
+      </c>
+      <c r="D25" s="10" t="inlineStr">
+        <is>
+          <t>What it prevents</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="14" t="inlineStr">
+        <is>
+          <t>Indexing &amp; query plans</t>
+        </is>
+      </c>
+      <c r="B26" s="13" t="inlineStr">
+        <is>
+          <t>Add and tune indexes on the hottest columns (hotel_id, dates, status); read query plans and fix slow ones.</t>
+        </is>
+      </c>
+      <c r="C26" s="13" t="inlineStr">
+        <is>
+          <t>The busiest queries stay in milliseconds as data grows.</t>
+        </is>
+      </c>
+      <c r="D26" s="13" t="inlineStr">
+        <is>
+          <t>Searches and reports getting slower for everyone over time.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="14" t="inlineStr">
+        <is>
+          <t>Partitioning &amp; archiving</t>
+        </is>
+      </c>
+      <c r="B27" s="13" t="inlineStr">
+        <is>
+          <t>Move old bookings/analytics to separate tables; partition large tables by date/hotel.</t>
+        </is>
+      </c>
+      <c r="C27" s="13" t="inlineStr">
+        <is>
+          <t>Day-to-day queries only touch recent, small data — so they stay fast.</t>
+        </is>
+      </c>
+      <c r="D27" s="13" t="inlineStr">
+        <is>
+          <t>Dashboards taking 15–20s to open once a hotel has years of data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="14" t="inlineStr">
+        <is>
+          <t>Migration discipline</t>
+        </is>
+      </c>
+      <c r="B28" s="13" t="inlineStr">
+        <is>
+          <t>Introduce Alembic so schema and index changes deploy in a controlled, repeatable way.</t>
+        </is>
+      </c>
+      <c r="C28" s="13" t="inlineStr">
+        <is>
+          <t>Production never silently misses an index or a schema change.</t>
+        </is>
+      </c>
+      <c r="D28" s="13" t="inlineStr">
+        <is>
+          <t>Indexes present in dev but missing in production → mystery slowness.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="14" t="inlineStr">
+        <is>
+          <t>Connection pooling</t>
+        </is>
+      </c>
+      <c r="B29" s="13" t="inlineStr">
+        <is>
+          <t>Add a pooler (PgBouncer) and tune pool size × workers × replicas against the Supabase limit.</t>
+        </is>
+      </c>
+      <c r="C29" s="13" t="inlineStr">
+        <is>
+          <t>50–100 hotels can onboard without the database running out of connections.</t>
+        </is>
+      </c>
+      <c r="D29" s="13" t="inlineStr">
+        <is>
+          <t>All tenants slowing down at once when connections run out.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="14" t="inlineStr">
+        <is>
+          <t>Backups &amp; restore drills</t>
+        </is>
+      </c>
+      <c r="B30" s="13" t="inlineStr">
+        <is>
+          <t>Run real restore drills, set up point-in-time recovery, write a disaster-recovery runbook.</t>
+        </is>
+      </c>
+      <c r="C30" s="13" t="inlineStr">
+        <is>
+          <t>Backups are proven to actually work before we ever need them.</t>
+        </is>
+      </c>
+      <c r="D30" s="13" t="inlineStr">
+        <is>
+          <t>Discovering a backup is unusable on the worst possible day.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="14" t="inlineStr">
+        <is>
+          <t>Isolation on schema changes</t>
+        </is>
+      </c>
+      <c r="B31" s="13" t="inlineStr">
+        <is>
+          <t>Review every new table for Row Level Security and per-hotel isolation.</t>
+        </is>
+      </c>
+      <c r="C31" s="13" t="inlineStr">
+        <is>
+          <t>The database itself keeps refusing to mix one hotel's data with another's.</t>
+        </is>
+      </c>
+      <c r="D31" s="13" t="inlineStr">
+        <is>
+          <t>A schema change quietly opening a cross-tenant leak.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="8" t="inlineStr">
+        <is>
+          <t>TECH LEAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="32" customHeight="1">
+      <c r="A34" s="15" t="inlineStr">
+        <is>
+          <t>Responsible for the whole software — decides what each developer builds and when, reviews everything before release, and owns delivery and security posture.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="30" customHeight="1">
+      <c r="A35" s="10" t="inlineStr">
+        <is>
+          <t>Ongoing job</t>
+        </is>
+      </c>
+      <c r="B35" s="10" t="inlineStr">
+        <is>
+          <t>What the work actually is</t>
+        </is>
+      </c>
+      <c r="C35" s="10" t="inlineStr">
+        <is>
+          <t>Why it matters to the business</t>
+        </is>
+      </c>
+      <c r="D35" s="10" t="inlineStr">
+        <is>
+          <t>What it prevents</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="14" t="inlineStr">
+        <is>
+          <t>Roadmap &amp; prioritisation</t>
+        </is>
+      </c>
+      <c r="B36" s="13" t="inlineStr">
+        <is>
+          <t>Decide what gets built in what order; sequence work so the biggest risk is always removed next.</t>
+        </is>
+      </c>
+      <c r="C36" s="13" t="inlineStr">
+        <is>
+          <t>Effort always goes to the highest-value, highest-risk item first.</t>
+        </is>
+      </c>
+      <c r="D36" s="13" t="inlineStr">
+        <is>
+          <t>Busywork while a real risk sits unaddressed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="14" t="inlineStr">
+        <is>
+          <t>Code review on every change</t>
+        </is>
+      </c>
+      <c r="B37" s="13" t="inlineStr">
+        <is>
+          <t>Be the human gate that reads every change for the silent-bug patterns in Sheet 8.</t>
+        </is>
+      </c>
+      <c r="C37" s="13" t="inlineStr">
+        <is>
+          <t>The single most effective catch for the bugs that don't show an error.</t>
+        </is>
+      </c>
+      <c r="D37" s="13" t="inlineStr">
+        <is>
+          <t>A quiet bug reaching production with no second pair of eyes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="14" t="inlineStr">
+        <is>
+          <t>Release &amp; incident response</t>
+        </is>
+      </c>
+      <c r="B38" s="13" t="inlineStr">
+        <is>
+          <t>Own the CI/CD pipeline, the deploy process, and the plan for when something breaks.</t>
+        </is>
+      </c>
+      <c r="C38" s="13" t="inlineStr">
+        <is>
+          <t>Deploys are predictable and incidents are handled calmly, not in a panic.</t>
+        </is>
+      </c>
+      <c r="D38" s="13" t="inlineStr">
+        <is>
+          <t>Risky deploys and chaotic, slow incident recovery.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="14" t="inlineStr">
+        <is>
+          <t>Security posture</t>
+        </is>
+      </c>
+      <c r="B39" s="13" t="inlineStr">
+        <is>
+          <t>Schedule penetration tests, drive the audit follow-ups, plan a future bug-bounty.</t>
+        </is>
+      </c>
+      <c r="C39" s="13" t="inlineStr">
+        <is>
+          <t>Security stays ahead of attackers as the attack surface grows.</t>
+        </is>
+      </c>
+      <c r="D39" s="13" t="inlineStr">
+        <is>
+          <t>Security drifting as new endpoints are added faster than they're reviewed.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="10">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A23:D23"/>
+    <mergeCell ref="A34:D34"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="A15:D15"/>
+    <mergeCell ref="A24:D24"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A33:D33"/>
+    <mergeCell ref="A14:D14"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Silent Bugs &amp; Server Stability — The Quiet Risks That Crash a Server</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="28" customHeight="1">
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>The dangerous bugs are the ones with NO error on screen — the server slowly leaks memory, stalls, or crashes while everything looks fine. Below is that class of risk, what already protects us, and the ongoing work that keeps it safe. Most of these we have already met and fixed once (the S-xx references point to Sheet 2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>Silent risk (plain language)</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t>How it quietly hurts the server</t>
+        </is>
+      </c>
+      <c r="C4" s="10" t="inlineStr">
+        <is>
+          <t>Already protected</t>
+        </is>
+      </c>
+      <c r="D4" s="10" t="inlineStr">
+        <is>
+          <t>Continuous work needed</t>
+        </is>
+      </c>
+      <c r="E4" s="10" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="14" t="inlineStr">
+        <is>
+          <t>Swallowed errors (a background job fails but no one is told)</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>Confirmation emails and channel-sync silently skip — guests get nothing, OTAs double-book — with zero error shown. We hit exactly this (S-12).</t>
+        </is>
+      </c>
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>Background-task pattern fixed; engineering rule bans bare 'except: pass'; errors must be logged or re-raised.</t>
+        </is>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>Read every new background job in code review; alert on task failures.</t>
+        </is>
+      </c>
+      <c r="E5" s="13" t="inlineStr">
+        <is>
+          <t>Backend + Tech Lead</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>Query returns more rows than expected (cardinality crash)</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>An endpoint that assumes one row gets several and throws a 500 only for certain data — invisible until that exact data appears.</t>
+        </is>
+      </c>
+      <c r="C6" s="13" t="inlineStr">
+        <is>
+          <t>Rule to use .first() not scalar_one_or_none() where multiple rows are possible; tests around it.</t>
+        </is>
+      </c>
+      <c r="D6" s="13" t="inlineStr">
+        <is>
+          <t>Review every new query for this pattern; add tests for multi-row cases.</t>
+        </is>
+      </c>
+      <c r="E6" s="13" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="14" t="inlineStr">
+        <is>
+          <t>Unbounded query (no limit) loads everything into memory</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>A big hotel's list endpoint tries to load 100k rows and the server runs out of memory and crashes (S-13, S-43).</t>
+        </is>
+      </c>
+      <c r="C7" s="13" t="inlineStr">
+        <is>
+          <t>Pagination (limit + offset) is mandatory on list endpoints, with hard caps; indexes on hot columns.</t>
+        </is>
+      </c>
+      <c r="D7" s="13" t="inlineStr">
+        <is>
+          <t>Enforce a limit on EVERY new list endpoint; reject unbounded date ranges.</t>
+        </is>
+      </c>
+      <c r="E7" s="13" t="inlineStr">
+        <is>
+          <t>Backend + Database</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>'Fail-open' safety check (limit turns OFF when Redis is down)</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>During a Redis blip the AI-spend limit silently passes everything — runaway cost or overload until someone notices (S-39, S-44).</t>
+        </is>
+      </c>
+      <c r="C8" s="13" t="inlineStr">
+        <is>
+          <t>Quotas now 'fail closed'; an in-process cap takes over; Redis self-heals after a 30s back-off.</t>
+        </is>
+      </c>
+      <c r="D8" s="13" t="inlineStr">
+        <is>
+          <t>Audit every new limit/lock to confirm it fails closed, not open.</t>
+        </is>
+      </c>
+      <c r="E8" s="13" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>N+1 queries (one page quietly fires hundreds of DB calls)</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>Looks fine on small data; as data grows the database is hammered and every page slows for everyone.</t>
+        </is>
+      </c>
+      <c r="C9" s="13" t="inlineStr">
+        <is>
+          <t>Batch loading with selectinload / single GROUP BY queries.</t>
+        </is>
+      </c>
+      <c r="D9" s="13" t="inlineStr">
+        <is>
+          <t>Review new endpoints for query count; watch slow-query logs.</t>
+        </is>
+      </c>
+      <c r="E9" s="13" t="inlineStr">
+        <is>
+          <t>Backend + Database</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>Connection-pool exhaustion under load</t>
+        </is>
+      </c>
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>At 100 simultaneous bookings the pool empties and every request stalls — the whole site appears down (F-01, F-09).</t>
+        </is>
+      </c>
+      <c r="C10" s="13" t="inlineStr">
+        <is>
+          <t>Env-driven pool sizing; documented pool math (SCALE_TUNING.md); row-level locks on inventory.</t>
+        </is>
+      </c>
+      <c r="D10" s="13" t="inlineStr">
+        <is>
+          <t>Load testing, a connection pooler (PgBouncer), auto-scaling rules.</t>
+        </is>
+      </c>
+      <c r="E10" s="13" t="inlineStr">
+        <is>
+          <t>Backend + Database + DevOps</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="14" t="inlineStr">
+        <is>
+          <t>Stale cache serves wrong data</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Cache isn't cleared after a booking/cancellation, so a sold room shows as 'available' and gets double-sold (S-21).</t>
+        </is>
+      </c>
+      <c r="C11" s="13" t="inlineStr">
+        <is>
+          <t>Cache invalidation + a version counter bumped after every booking/cancellation.</t>
+        </is>
+      </c>
+      <c r="D11" s="13" t="inlineStr">
+        <is>
+          <t>Invalidation discipline on every new cached path.</t>
+        </is>
+      </c>
+      <c r="E11" s="13" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>Uncaught frontend error blanks the whole page</t>
+        </is>
+      </c>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>One failed fetch with no error boundary turns the entire screen white mid-booking — the guest just leaves (S-36).</t>
+        </is>
+      </c>
+      <c r="C12" s="13" t="inlineStr">
+        <is>
+          <t>Error + Retry UI on the booking pages; add-ons load separately so their failure can't blank the page.</t>
+        </is>
+      </c>
+      <c r="D12" s="13" t="inlineStr">
+        <is>
+          <t>Same hardening on every dashboard page; a top-level error boundary.</t>
+        </is>
+      </c>
+      <c r="E12" s="13" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="14" t="inlineStr">
+        <is>
+          <t>Resource leak (threads / streams pile up)</t>
+        </is>
+      </c>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>Long-lived connections or threads are never released; the server slowly bloats and dies hours later — no obvious cause.</t>
+        </is>
+      </c>
+      <c r="C13" s="13" t="inlineStr">
+        <is>
+          <t>Streaming connections have lifetime caps; web search runs in a thread with an 8s hard timeout.</t>
+        </is>
+      </c>
+      <c r="D13" s="13" t="inlineStr">
+        <is>
+          <t>Monitor memory/thread counts; cap every new long-lived resource.</t>
+        </is>
+      </c>
+      <c r="E13" s="13" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="14" t="inlineStr">
+        <is>
+          <t>Unvalidated input / bad settings saved</t>
+        </is>
+      </c>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>Negative tax, inverted slabs or a divide-by-zero produce wrong bills for every guest — silently, until accounts notice (S-41).</t>
+        </is>
+      </c>
+      <c r="C14" s="13" t="inlineStr">
+        <is>
+          <t>Server-side validation rejects bad values; calculators guarded against NaN.</t>
+        </is>
+      </c>
+      <c r="D14" s="13" t="inlineStr">
+        <is>
+          <t>Validate every new settings/input form server-side, not just in the browser.</t>
+        </is>
+      </c>
+      <c r="E14" s="13" t="inlineStr">
+        <is>
+          <t>Backend + Frontend</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>WHY THE WHOLE SOFTWARE WILL NOT GO BLANK (the safety net)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t>•  Layered fallbacks: if Redis crashes, the app transparently falls back to an in-memory cache — it never crashes because of Redis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>•  No blank screens: a failed data fetch shows a clear message with a Retry button; optional pieces (add-ons) load separately so one failure can't take down the page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="12" t="inlineStr">
+        <is>
+          <t>•  Fail closed on money &amp; security, fail soft on the screen: anything touching payment, roles or another hotel's data DENIES on doubt; anything touching the display keeps working in a reduced mode.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="12" t="inlineStr">
+        <is>
+          <t>•  Tested on every change: 277 automated tests (including Redis-failover and cross-tenant attack tests) run before any code can merge.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="12" t="inlineStr">
+        <is>
+          <t>•  The 'safer side' principle the CEO asked for: when in doubt we choose the cautious behaviour — reject the risky action, keep the guest's screen usable, and log it for a human to review.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="A21:E21"/>
+    <mergeCell ref="A20:E20"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A16:E16"/>
+    <mergeCell ref="A19:E19"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A17:E17"/>
+    <mergeCell ref="A18:E18"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Scaling to Large Data — Database → Backend → Browser in Milliseconds</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="28" customHeight="1">
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>When a hotel has 2–3 years of bookings (GBs of data), the page must still load in milliseconds and must never freeze or go blank. This is the speed 'budget' for the journey of one request, what already holds it, and what we build to keep holding it as data grows.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>Stage of the journey</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t>What happens here</t>
+        </is>
+      </c>
+      <c r="C4" s="10" t="inlineStr">
+        <is>
+          <t>Speed target</t>
+        </is>
+      </c>
+      <c r="D4" s="10" t="inlineStr">
+        <is>
+          <t>In place today</t>
+        </is>
+      </c>
+      <c r="E4" s="10" t="inlineStr">
+        <is>
+          <t>To build for GB-scale</t>
+        </is>
+      </c>
+      <c r="F4" s="10" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="14" t="inlineStr">
+        <is>
+          <t>1. Database</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>Find and return the right rows (bookings, rates, guests) for this hotel only.</t>
+        </is>
+      </c>
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>&lt; 50 ms / query</t>
+        </is>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>Indexes on hot columns; Row Level Security; pagination; composite index on the busiest availability query.</t>
+        </is>
+      </c>
+      <c r="E5" s="13" t="inlineStr">
+        <is>
+          <t>Table partitioning by date/hotel; archive old bookings; read replicas for reports.</t>
+        </is>
+      </c>
+      <c r="F5" s="13" t="inlineStr">
+        <is>
+          <t>Database</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>2. Backend API</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>Shape the rows into a clean API response, applying security and business rules.</t>
+        </is>
+      </c>
+      <c r="C6" s="13" t="inlineStr">
+        <is>
+          <t>&lt; 100 ms</t>
+        </is>
+      </c>
+      <c r="D6" s="13" t="inlineStr">
+        <is>
+          <t>Redis caching on heavy aggregations; mandatory pagination; lazy heavy imports; batched queries (no N+1).</t>
+        </is>
+      </c>
+      <c r="E6" s="13" t="inlineStr">
+        <is>
+          <t>Pre-computed report tables; response compression; background pre-warming of common queries.</t>
+        </is>
+      </c>
+      <c r="F6" s="13" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="14" t="inlineStr">
+        <is>
+          <t>3. Network &amp; cache</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>Carry the response to the browser, reusing cached copies where safe.</t>
+        </is>
+      </c>
+      <c r="C7" s="13" t="inlineStr">
+        <is>
+          <t>&lt; 100 ms (cache hit ~0)</t>
+        </is>
+      </c>
+      <c r="D7" s="13" t="inlineStr">
+        <is>
+          <t>React Query caches GETs for 5 min; public reads cached in Redis.</t>
+        </is>
+      </c>
+      <c r="E7" s="13" t="inlineStr">
+        <is>
+          <t>Cloudflare edge caching; ETags/conditional requests so unchanged data isn't re-sent.</t>
+        </is>
+      </c>
+      <c r="F7" s="13" t="inlineStr">
+        <is>
+          <t>Backend + Frontend</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>4. Browser render</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>Draw the data on screen — lists, charts, the booking calendar.</t>
+        </is>
+      </c>
+      <c r="C8" s="13" t="inlineStr">
+        <is>
+          <t>&lt; 1 s, no freeze</t>
+        </is>
+      </c>
+      <c r="D8" s="13" t="inlineStr">
+        <is>
+          <t>Paged lists; loading + error + Retry states on the booking pages.</t>
+        </is>
+      </c>
+      <c r="E8" s="13" t="inlineStr">
+        <is>
+          <t>Virtual scrolling for huge lists; code-splitting &amp; lazy loading; skeleton loaders.</t>
+        </is>
+      </c>
+      <c r="F8" s="13" t="inlineStr">
+        <is>
+          <t>Frontend</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>TOTAL (guest experience)</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>From click to a fully usable screen.</t>
+        </is>
+      </c>
+      <c r="C9" s="13" t="inlineStr">
+        <is>
+          <t>Well under ~2 s</t>
+        </is>
+      </c>
+      <c r="D9" s="13" t="inlineStr">
+        <is>
+          <t>Holds comfortably at today's data sizes.</t>
+        </is>
+      </c>
+      <c r="E9" s="13" t="inlineStr">
+        <is>
+          <t>Stays under ~2 s at GB-scale once the above are in place.</t>
+        </is>
+      </c>
+      <c r="F9" s="13" t="inlineStr">
+        <is>
+          <t>All three roles</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>AND IT STAYS ON THE SAFER SIDE AT SCALE</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t>•  Even when data is huge, the app never tries to load everything at once — the database sends rows in pages, the backend serves them in chunks, and the frontend draws only what's on screen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>•  If any stage is slow or fails, the guest sees a Retry — never a frozen tab or a white page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="12" t="inlineStr">
+        <is>
+          <t>•  Money and security checks never get 'skipped to go faster': they stay strict (fail closed) no matter the load. Only the display degrades gracefully, never the safety.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>•  Costs stay bounded as data grows: capped result sizes, caching, and per-hotel quotas mean more data does not mean a runaway bill.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A11:F11"/>
+    <mergeCell ref="A13:F13"/>
+    <mergeCell ref="A14:F14"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A12:F12"/>
+    <mergeCell ref="A15:F15"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
docs: refresh CEO report to current work log + merged PRs
- Problems Solved: add S-46..S-58 (widget RCE/XSS, blank-screen crash,
  booking 500 crashes, dead recovery scheduler, deploy/migration fixes...)
- Features Built: add Revenue Engine, chain features, OTA widget, Sentry, graphify (13-23)
- Work In Progress: refresh each item's status to current reality
- Future Risks: refresh protections now in place
- Executive Summary: 58 issues / 23 features + 'what's new since 11-Jun'
- Team & Hiring + Silent Bugs: refresh counts and examples

https://claude.ai/code/session_01Jfp6dFcb8aisQfoK5brnT1
</commit_message>
<xml_diff>
--- a/docs/CEO_Report_Staybooker_Jun2026.xlsx
+++ b/docs/CEO_Report_Staybooker_Jun2026.xlsx
@@ -25,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -62,6 +62,11 @@
     </font>
     <font>
       <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -103,7 +108,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -139,11 +144,55 @@
         <color rgb="00D9D9D9"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -186,6 +235,19 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -551,7 +613,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -572,6 +634,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="10" t="inlineStr">
         <is>
@@ -600,7 +663,7 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>45 issues fixed so far (5 Critical, 24 High, 16 Medium). Each issue shows what would have happened to the business if it had reached production.</t>
+          <t>58 issues fixed so far (6 Critical, 30 High, 22 Medium). Each issue shows what would have happened to the business if it had reached production.</t>
         </is>
       </c>
     </row>
@@ -612,7 +675,7 @@
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>Major product features delivered alongside the bug fixing — multi-property chains, loyalty program, OTA rate intelligence, AI concierge, real-time updates, encrypted secrets storage.</t>
+          <t>23 major product features delivered alongside the bug fixing — multi-property chains, loyalty wallet, OTA rate intelligence, AI concierge, real-time updates, encrypted secrets, and the new Revenue Engine (dynamic pricing, abandoned-booking recovery, chain upsell broadcast, seasonal promotions, OTA-style booking widget).</t>
         </is>
       </c>
     </row>
@@ -700,6 +763,7 @@
         </is>
       </c>
     </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" s="11" t="inlineStr">
         <is>
@@ -716,7 +780,7 @@
       </c>
       <c r="B17" s="13" t="inlineStr">
         <is>
-          <t>45 (source: work_log_tracker.csv — engineering tasks logged up to 16-Jun-2026)</t>
+          <t>58 (source: work_log_tracker.csv — engineering tasks logged up to 16-Jun-2026; merged across PRs up to #90)</t>
         </is>
       </c>
     </row>
@@ -728,7 +792,7 @@
       </c>
       <c r="B18" s="13" t="inlineStr">
         <is>
-          <t>5 — payment secret key leak, payment amount tampering, permanent admin token, AI assistant crash, staff privilege escalation.</t>
+          <t>6 — payment secret key leak, payment amount tampering, permanent admin token, AI assistant crash, staff privilege escalation, and the booking-widget code-execution (RCE/XSS) sink.</t>
         </is>
       </c>
     </row>
@@ -752,7 +816,7 @@
       </c>
       <c r="B20" s="13" t="inlineStr">
         <is>
-          <t>277 test cases passing (security, payments, booking, role access, rate limits, Redis failover). These run automatically on every code change (CI/CD), plus dependency vulnerability (CVE) scanning.</t>
+          <t>Close to 300 automated test cases (the 277 from the June audit, plus new tests for the anti-automation booking token, the recovery scheduler, chain features and public-booking promotions). They run on every code change (CI/CD), with dependency vulnerability (CVE) scanning.</t>
         </is>
       </c>
     </row>
@@ -780,23 +844,68 @@
         </is>
       </c>
     </row>
+    <row r="23"/>
     <row r="24">
       <c r="A24" s="11" t="inlineStr">
         <is>
-          <t>ONE-LINE MESSAGE FOR THE CEO</t>
-        </is>
-      </c>
-      <c r="B24" s="12" t="inlineStr"/>
+          <t>WHAT'S NEW SINCE 11-JUN</t>
+        </is>
+      </c>
+      <c r="B24" s="16" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="13" t="inlineStr">
         <is>
+          <t>Revenue Engine shipped</t>
+        </is>
+      </c>
+      <c r="B25" s="13" t="inlineStr">
+        <is>
+          <t>Dynamic pricing (occupancy/lead-time rules wired to real charges), abandoned-booking recovery (WhatsApp + email, hourly scheduler), and a loyalty wallet with stay offers and upsell hub — a whole new revenue surface (PR #80).</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="13" t="inlineStr">
+        <is>
+          <t>Chain &amp; promotions</t>
+        </is>
+      </c>
+      <c r="B26" s="13" t="inlineStr">
+        <is>
+          <t>Chain-wide upsell broadcast, package validity windows, and seasonal auto-apply promotions at hotel and chain level (PR #88).</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="13" t="inlineStr">
+        <is>
+          <t>Stability &amp; crash fixes</t>
+        </is>
+      </c>
+      <c r="B27" s="13" t="inlineStr">
+        <is>
+          <t>Fixed a blank-white-screen crash on deploy (S-48), two booking-flow 500 crashes (S-46, S-47), a dead recovery scheduler (S-49), broken deploys/migrations (S-54, S-56), and removed a widget code-execution security hole (S-50).</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="11" t="inlineStr">
+        <is>
+          <t>ONE-LINE MESSAGE FOR THE CEO</t>
+        </is>
+      </c>
+      <c r="B28" s="12" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="13" t="inlineStr">
+        <is>
           <t>Bottom line</t>
         </is>
       </c>
-      <c r="B25" s="13" t="inlineStr">
-        <is>
-          <t>The product is stable today and hoteliers' data is safe. The hiring need comes from growth: as hotels, traffic and data scale up, each layer — database, backend, frontend — needs a dedicated owner so the speed, safety and crash-proofing stay exactly where they are today. This report now also spells out, in plain language, the ongoing engineering work that keeps it that way (Sheets 7–9).</t>
+      <c r="B29" s="13" t="inlineStr">
+        <is>
+          <t>The product is stable today and hoteliers' data is safe — and it is moving fast: 58 issues fixed, 23 features shipped, and a full Revenue Engine added since launch. The hiring need comes from exactly this momentum: as hotels, traffic and data scale up, each layer — database, backend, frontend — needs a dedicated owner so the speed, safety and crash-proofing stay where they are today. Sheets 7-9 spell out, in plain language, the ongoing engineering that keeps it that way.</t>
         </is>
       </c>
     </row>
@@ -815,7 +924,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G49"/>
+  <dimension ref="A1:G62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2540,6 +2649,487 @@
       <c r="G49" s="4" t="inlineStr">
         <is>
           <t>11-Jun</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="13" t="inlineStr">
+        <is>
+          <t>S-46</t>
+        </is>
+      </c>
+      <c r="B50" s="13" t="inlineStr">
+        <is>
+          <t>The loyalty check could crash the public booking page for some guests</t>
+        </is>
+      </c>
+      <c r="C50" s="13" t="inlineStr">
+        <is>
+          <t>The loyalty lookup used scalar_one_or_none(), which throws when a guest matches more than one loyalty row</t>
+        </is>
+      </c>
+      <c r="D50" s="13" t="inlineStr">
+        <is>
+          <t>A guest pressing 'check loyalty' could hit a 500 error mid-booking — a silent server crash that only appears for certain data, dropping bookings with no error anyone could easily reproduce.</t>
+        </is>
+      </c>
+      <c r="E50" s="13" t="inlineStr">
+        <is>
+          <t>Switched to .scalars().first() with a clear preferred-row ordering; added a regression test for the exact path.</t>
+        </is>
+      </c>
+      <c r="F50" s="17" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G50" s="13" t="inlineStr">
+        <is>
+          <t>14-Jun</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="13" t="inlineStr">
+        <is>
+          <t>S-47</t>
+        </is>
+      </c>
+      <c r="B51" s="13" t="inlineStr">
+        <is>
+          <t>Creating or cancelling a public booking could crash with a 500</t>
+        </is>
+      </c>
+      <c r="C51" s="13" t="inlineStr">
+        <is>
+          <t>The code read super_admin.phone (a field that does not exist) and WhatsApp settings that were never defined</t>
+        </is>
+      </c>
+      <c r="D51" s="13" t="inlineStr">
+        <is>
+          <t>The core revenue action of the whole product — creating/cancelling a booking — could fail server-side, silently, for everyone.</t>
+        </is>
+      </c>
+      <c r="E51" s="13" t="inlineStr">
+        <is>
+          <t>Admin alert number moved to server config (env); WhatsApp service aligned to the real settings; two unused admin lookups removed (also fewer DB queries per booking).</t>
+        </is>
+      </c>
+      <c r="F51" s="17" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G51" s="13" t="inlineStr">
+        <is>
+          <t>15-Jun</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="13" t="inlineStr">
+        <is>
+          <t>S-48</t>
+        </is>
+      </c>
+      <c r="B52" s="13" t="inlineStr">
+        <is>
+          <t>The whole app could load as a blank white screen after a deploy</t>
+        </is>
+      </c>
+      <c r="C52" s="13" t="inlineStr">
+        <is>
+          <t>A production build optimisation (Vite manualChunks) broke React's context loading and crashed the app to a blank page</t>
+        </is>
+      </c>
+      <c r="D52" s="13" t="inlineStr">
+        <is>
+          <t>Guests and hoteliers would open the site to a completely blank screen — the worst possible failure, with no error and no way forward.</t>
+        </is>
+      </c>
+      <c r="E52" s="13" t="inlineStr">
+        <is>
+          <t>Reverted the unsafe bundling change and added instant-load placeholders so the first paint is never empty.</t>
+        </is>
+      </c>
+      <c r="F52" s="17" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G52" s="13" t="inlineStr">
+        <is>
+          <t>15-Jun</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="13" t="inlineStr">
+        <is>
+          <t>S-49</t>
+        </is>
+      </c>
+      <c r="B53" s="13" t="inlineStr">
+        <is>
+          <t>Abandoned-booking recovery was built but never actually ran</t>
+        </is>
+      </c>
+      <c r="C53" s="13" t="inlineStr">
+        <is>
+          <t>The recovery feature had no scheduled job, so unpaid bookings always aged past the 72h window un-nudged</t>
+        </is>
+      </c>
+      <c r="D53" s="13" t="inlineStr">
+        <is>
+          <t>A revenue-recovery feature we built was silently dead — incremental bookings left on the table every day with no one noticing.</t>
+        </is>
+      </c>
+      <c r="E53" s="13" t="inlineStr">
+        <is>
+          <t>Added an hourly Redis-locked scheduler that runs the sweep on exactly one server and honours each hotel's opt-in.</t>
+        </is>
+      </c>
+      <c r="F53" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G53" s="13" t="inlineStr">
+        <is>
+          <t>15-Jun</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="13" t="inlineStr">
+        <is>
+          <t>S-50</t>
+        </is>
+      </c>
+      <c r="B54" s="13" t="inlineStr">
+        <is>
+          <t>The booking widget could run attacker-supplied code on the hotel's site (RCE/XSS)</t>
+        </is>
+      </c>
+      <c r="C54" s="13" t="inlineStr">
+        <is>
+          <t>A 'custom JS' setting was executed via new Function()/eval on the public widget; widget CSS and chat messages were under-validated</t>
+        </is>
+      </c>
+      <c r="D54" s="13" t="inlineStr">
+        <is>
+          <t>A malicious or compromised setting could run arbitrary code in every guest's browser on the hotel's own domain — a severe security hole.</t>
+        </is>
+      </c>
+      <c r="E54" s="13" t="inlineStr">
+        <is>
+          <t>Removed the code-execution sink entirely; the public API no longer returns custom JS; iframe sandboxed; CSS sanitised (strips url()/@import/expression/script); chat postMessage locked to the referrer origin; inactive hotels return 404; guest message length capped.</t>
+        </is>
+      </c>
+      <c r="F54" s="19" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="G54" s="13" t="inlineStr">
+        <is>
+          <t>15-Jun</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="13" t="inlineStr">
+        <is>
+          <t>S-51</t>
+        </is>
+      </c>
+      <c r="B55" s="13" t="inlineStr">
+        <is>
+          <t>Two guests could spend the same promo / loyalty balance at once</t>
+        </is>
+      </c>
+      <c r="C55" s="13" t="inlineStr">
+        <is>
+          <t>Promo-code and loyalty redemption read-then-wrote without a row lock (a race condition)</t>
+        </is>
+      </c>
+      <c r="D55" s="13" t="inlineStr">
+        <is>
+          <t>Under concurrent checkouts the same discount or points balance could be spent twice — direct revenue leakage and wrong loyalty liability.</t>
+        </is>
+      </c>
+      <c r="E55" s="13" t="inlineStr">
+        <is>
+          <t>Redemption now takes SELECT FOR UPDATE row locks; AI lead inputs are length-bounded as well.</t>
+        </is>
+      </c>
+      <c r="F55" s="17" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G55" s="13" t="inlineStr">
+        <is>
+          <t>15-Jun</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="13" t="inlineStr">
+        <is>
+          <t>S-52</t>
+        </is>
+      </c>
+      <c r="B56" s="13" t="inlineStr">
+        <is>
+          <t>A newly created property could be saved without its brand (chain) link</t>
+        </is>
+      </c>
+      <c r="C56" s="13" t="inlineStr">
+        <is>
+          <t>The property-create path did not inherit chain_id from the logged-in user</t>
+        </is>
+      </c>
+      <c r="D56" s="13" t="inlineStr">
+        <is>
+          <t>A property could end up unlinked or wrongly associated across tenants — a multi-tenant isolation risk and broken brand dashboards.</t>
+        </is>
+      </c>
+      <c r="E56" s="13" t="inlineStr">
+        <is>
+          <t>chain_id is now inherited from the authenticated user on creation; the superadmin add-property path also sets address fields correctly.</t>
+        </is>
+      </c>
+      <c r="F56" s="17" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G56" s="13" t="inlineStr">
+        <is>
+          <t>14-Jun</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="13" t="inlineStr">
+        <is>
+          <t>S-53</t>
+        </is>
+      </c>
+      <c r="B57" s="13" t="inlineStr">
+        <is>
+          <t>Loyalty read endpoints had no role check</t>
+        </is>
+      </c>
+      <c r="C57" s="13" t="inlineStr">
+        <is>
+          <t>GET /loyalty/program and /loyalty/guests were missing the role guard the write endpoints already had</t>
+        </is>
+      </c>
+      <c r="D57" s="13" t="inlineStr">
+        <is>
+          <t>Any staff account could read the loyalty program configuration and the guest list — an authorization gap on read (a trap we watch for everywhere).</t>
+        </is>
+      </c>
+      <c r="E57" s="13" t="inlineStr">
+        <is>
+          <t>require_hotel_role added to both GET endpoints.</t>
+        </is>
+      </c>
+      <c r="F57" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G57" s="13" t="inlineStr">
+        <is>
+          <t>14-Jun</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="13" t="inlineStr">
+        <is>
+          <t>S-54</t>
+        </is>
+      </c>
+      <c r="B58" s="13" t="inlineStr">
+        <is>
+          <t>The frontend could not deploy at all (Cloudflare Pages broken)</t>
+        </is>
+      </c>
+      <c r="C58" s="13" t="inlineStr">
+        <is>
+          <t>A stray git submodule reference (decodo-api-docs) broke every Cloudflare Pages build</t>
+        </is>
+      </c>
+      <c r="D58" s="13" t="inlineStr">
+        <is>
+          <t>No frontend deploys could ship — the product could not be updated for customers until it was fixed.</t>
+        </is>
+      </c>
+      <c r="E58" s="13" t="inlineStr">
+        <is>
+          <t>Removed the broken submodule gitlink; deploys restored.</t>
+        </is>
+      </c>
+      <c r="F58" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G58" s="13" t="inlineStr">
+        <is>
+          <t>15-Jun</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="13" t="inlineStr">
+        <is>
+          <t>S-55</t>
+        </is>
+      </c>
+      <c r="B59" s="13" t="inlineStr">
+        <is>
+          <t>The frontend production build was silently broken on the branch</t>
+        </is>
+      </c>
+      <c r="C59" s="13" t="inlineStr">
+        <is>
+          <t>A new widget tab imported a UI component (accordion) whose file was never committed — 'vite build' failed with a missing-file error</t>
+        </is>
+      </c>
+      <c r="D59" s="13" t="inlineStr">
+        <is>
+          <t>The next release would have failed to build with no obvious cause — exactly the kind of quiet break that blocks a deploy at the worst time.</t>
+        </is>
+      </c>
+      <c r="E59" s="13" t="inlineStr">
+        <is>
+          <t>Added the missing standard component (the dependency was already present) and verified with a full local build.</t>
+        </is>
+      </c>
+      <c r="F59" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G59" s="13" t="inlineStr">
+        <is>
+          <t>16-Jun</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="13" t="inlineStr">
+        <is>
+          <t>S-56</t>
+        </is>
+      </c>
+      <c r="B60" s="13" t="inlineStr">
+        <is>
+          <t>Some database columns existed in code but not in the live database</t>
+        </is>
+      </c>
+      <c r="C60" s="13" t="inlineStr">
+        <is>
+          <t>Migrations for loyalty milestones and competitor-rate columns were missing from the deploy path</t>
+        </is>
+      </c>
+      <c r="D60" s="13" t="inlineStr">
+        <is>
+          <t>Any query touching those columns would crash in production while passing locally — a hidden landmine as features rolled out.</t>
+        </is>
+      </c>
+      <c r="E60" s="13" t="inlineStr">
+        <is>
+          <t>Added the missing migrations so the live schema matches the code.</t>
+        </is>
+      </c>
+      <c r="F60" s="17" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G60" s="13" t="inlineStr">
+        <is>
+          <t>15-Jun</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="13" t="inlineStr">
+        <is>
+          <t>S-57</t>
+        </is>
+      </c>
+      <c r="B61" s="13" t="inlineStr">
+        <is>
+          <t>Hotel listings and sister-hotel suggestions always showed a blank city</t>
+        </is>
+      </c>
+      <c r="C61" s="13" t="inlineStr">
+        <is>
+          <t>City was read as a direct attribute, but it is stored inside the address JSON dict</t>
+        </is>
+      </c>
+      <c r="D61" s="13" t="inlineStr">
+        <is>
+          <t>Guests saw blank locations on chain pages and recommendations — it looks broken and quietly hurts trust and conversion.</t>
+        </is>
+      </c>
+      <c r="E61" s="13" t="inlineStr">
+        <is>
+          <t>All three hotel-listing endpoints now read city from the address dict.</t>
+        </is>
+      </c>
+      <c r="F61" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G61" s="13" t="inlineStr">
+        <is>
+          <t>14-Jun</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="13" t="inlineStr">
+        <is>
+          <t>S-58</t>
+        </is>
+      </c>
+      <c r="B62" s="13" t="inlineStr">
+        <is>
+          <t>Valid bookings were sometimes rejected over a 1-rupee rounding gap</t>
+        </is>
+      </c>
+      <c r="C62" s="13" t="inlineStr">
+        <is>
+          <t>The client/server price match used a flat +/-5 INR tolerance that failed on percentage-based dynamic prices</t>
+        </is>
+      </c>
+      <c r="D62" s="13" t="inlineStr">
+        <is>
+          <t>Guests with legitimate prices could be blocked at checkout by a tiny rounding difference — silent lost bookings.</t>
+        </is>
+      </c>
+      <c r="E62" s="13" t="inlineStr">
+        <is>
+          <t>Tolerance is now max(Rs.5, 1%) and the calendar pricing note is clearer.</t>
+        </is>
+      </c>
+      <c r="F62" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G62" s="13" t="inlineStr">
+        <is>
+          <t>15-Jun</t>
         </is>
       </c>
     </row>
@@ -2558,7 +3148,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2930,6 +3520,281 @@
       <c r="E16" s="4" t="inlineStr">
         <is>
           <t>Widget messages locked to the embedding site's verified origin; prices/availability always confirmed server-side.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="13" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="13" t="inlineStr">
+        <is>
+          <t>Dynamic pricing engine (hotelier-configured)</t>
+        </is>
+      </c>
+      <c r="C17" s="13" t="inlineStr">
+        <is>
+          <t>Hoteliers set rules (occupancy, day-of-week, lead-time) that adjust room prices automatically; a live preview shows the price on each calendar cell, and the rules drive the real booking charge.</t>
+        </is>
+      </c>
+      <c r="D17" s="13" t="inlineStr">
+        <is>
+          <t>A revenue-management feature (higher RevPAR) that competitors charge a premium for — a new selling point and revenue line.</t>
+        </is>
+      </c>
+      <c r="E17" s="13" t="inlineStr">
+        <is>
+          <t>Prices are server-computed with live occupancy; the client's price is verified within a tolerance; rules are role-gated and tenant-scoped.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="13" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="13" t="inlineStr">
+        <is>
+          <t>Abandoned-booking recovery</t>
+        </is>
+      </c>
+      <c r="C18" s="13" t="inlineStr">
+        <is>
+          <t>Automatically nudges guests who started but did not finish a booking, via WhatsApp and email, on an opt-in basis.</t>
+        </is>
+      </c>
+      <c r="D18" s="13" t="inlineStr">
+        <is>
+          <t>Recovers otherwise-lost bookings automatically — direct incremental revenue.</t>
+        </is>
+      </c>
+      <c r="E18" s="13" t="inlineStr">
+        <is>
+          <t>Runs on an hourly Redis-locked scheduler (one server only); per-hotel opt-in; senders never crash the booking flow; no PII logged.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="13" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="13" t="inlineStr">
+        <is>
+          <t>Loyalty points wallet + stay offers</t>
+        </is>
+      </c>
+      <c r="C19" s="13" t="inlineStr">
+        <is>
+          <t>Configurable earn/redeem rates, room-specific night-threshold offers, and a pre-booking nudge ('stay one more night to unlock').</t>
+        </is>
+      </c>
+      <c r="D19" s="13" t="inlineStr">
+        <is>
+          <t>Deeper loyalty and longer stays — more direct, OTA-free revenue.</t>
+        </is>
+      </c>
+      <c r="E19" s="13" t="inlineStr">
+        <is>
+          <t>Redemption value is recomputed server-side from config (never trusts the client); role-gated; brand-isolated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="13" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="13" t="inlineStr">
+        <is>
+          <t>Chain-wide upsell broadcast</t>
+        </is>
+      </c>
+      <c r="C20" s="13" t="inlineStr">
+        <is>
+          <t>A brand admin pushes one stay-upsell offer to every active property at once; each hotel gets its own row so the guest flow is unchanged.</t>
+        </is>
+      </c>
+      <c r="D20" s="13" t="inlineStr">
+        <is>
+          <t>Brand-level marketing in a single click across all properties.</t>
+        </is>
+      </c>
+      <c r="E20" s="13" t="inlineStr">
+        <is>
+          <t>Chain-admin only; isolated by chain_id; per-hotel rows share a broadcast id.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="13" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="13" t="inlineStr">
+        <is>
+          <t>Seasonal auto-apply promotions</t>
+        </is>
+      </c>
+      <c r="C21" s="13" t="inlineStr">
+        <is>
+          <t>Date-windowed deals that apply automatically with no coupon code (or as classic coupons), at hotel and chain level.</t>
+        </is>
+      </c>
+      <c r="D21" s="13" t="inlineStr">
+        <is>
+          <t>Easier campaigns and higher conversion (no coupon friction).</t>
+        </is>
+      </c>
+      <c r="E21" s="13" t="inlineStr">
+        <is>
+          <t>Discount always server-computed; usage incremented atomically; scoped to hotel or chain; the display banner is read-only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="13" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="13" t="inlineStr">
+        <is>
+          <t>OTA / Booking.com-style booking widget</t>
+        </is>
+      </c>
+      <c r="C22" s="13" t="inlineStr">
+        <is>
+          <t>A professional, embeddable booking + search widget for hotel websites, with a floating calendar overlay and instant-load placeholders.</t>
+        </is>
+      </c>
+      <c r="D22" s="13" t="inlineStr">
+        <is>
+          <t>A polished direct-booking experience that rivals the OTAs — captures commission-free bookings.</t>
+        </is>
+      </c>
+      <c r="E22" s="13" t="inlineStr">
+        <is>
+          <t>Host-page-safe embed loader; hardened postMessage; iframe sandbox; the code-execution sink was removed (see S-50).</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="13" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="13" t="inlineStr">
+        <is>
+          <t>Brand Console for multi-property owners</t>
+        </is>
+      </c>
+      <c r="C23" s="13" t="inlineStr">
+        <is>
+          <t>A collapsible brand workspace (overview, guest insights, brand promos, loyalty, upsell broadcast) for groups managing many hotels.</t>
+        </is>
+      </c>
+      <c r="D23" s="13" t="inlineStr">
+        <is>
+          <t>Makes the platform genuinely usable for hotel groups, not just single properties.</t>
+        </is>
+      </c>
+      <c r="E23" s="13" t="inlineStr">
+        <is>
+          <t>Gated by chain membership; every section validates the user's chain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="13" t="n">
+        <v>20</v>
+      </c>
+      <c r="B24" s="13" t="inlineStr">
+        <is>
+          <t>Configurable rate plans &amp; packages</t>
+        </is>
+      </c>
+      <c r="C24" s="13" t="inlineStr">
+        <is>
+          <t>Pure rate plans are separated from packages; packages gain an optional validity window and a 'you save' badge.</t>
+        </is>
+      </c>
+      <c r="D24" s="13" t="inlineStr">
+        <is>
+          <t>Clearer pricing setup for hoteliers and fewer mistakes.</t>
+        </is>
+      </c>
+      <c r="E24" s="13" t="inlineStr">
+        <is>
+          <t>Tenant-scoped; reuses the existing rate endpoints.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="13" t="n">
+        <v>21</v>
+      </c>
+      <c r="B25" s="13" t="inlineStr">
+        <is>
+          <t>Anti-automation booking token (HMAC)</t>
+        </is>
+      </c>
+      <c r="C25" s="13" t="inlineStr">
+        <is>
+          <t>A signed, short-lived token on the public booking path to deter scripted abuse (feature-flagged, off by default).</t>
+        </is>
+      </c>
+      <c r="D25" s="13" t="inlineStr">
+        <is>
+          <t>Protects the booking funnel from bots without slowing real guests.</t>
+        </is>
+      </c>
+      <c r="E25" s="13" t="inlineStr">
+        <is>
+          <t>HMAC-signed, time-bounded and rate-limited; enabled only when needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="13" t="n">
+        <v>22</v>
+      </c>
+      <c r="B26" s="13" t="inlineStr">
+        <is>
+          <t>Production observability (Sentry)</t>
+        </is>
+      </c>
+      <c r="C26" s="13" t="inlineStr">
+        <is>
+          <t>Error tracking with user context, a booking-funnel trail and payment-failure tracking.</t>
+        </is>
+      </c>
+      <c r="D26" s="13" t="inlineStr">
+        <is>
+          <t>We see and fix issues before customers report them — higher reliability.</t>
+        </is>
+      </c>
+      <c r="E26" s="13" t="inlineStr">
+        <is>
+          <t>No PII or secrets in events; scoped server-side.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="13" t="n">
+        <v>23</v>
+      </c>
+      <c r="B27" s="13" t="inlineStr">
+        <is>
+          <t>Engineering knowledge graph (graphify)</t>
+        </is>
+      </c>
+      <c r="C27" s="13" t="inlineStr">
+        <is>
+          <t>An AST-built map of the whole codebase (~4,800 nodes) that any engineer — or the AI assistant — consults before changing code.</t>
+        </is>
+      </c>
+      <c r="D27" s="13" t="inlineStr">
+        <is>
+          <t>Faster, safer onboarding and changes as the team grows; fewer regressions.</t>
+        </is>
+      </c>
+      <c r="E27" s="13" t="inlineStr">
+        <is>
+          <t>Local-only, no API cost; rebuilds automatically on commits.</t>
         </is>
       </c>
     </row>
@@ -2948,7 +3813,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2972,6 +3837,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="26" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -3066,7 +3932,7 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Every page must handle network failures, double-clicks, and slow-data scenarios gracefully. The public booking widget pages are done (error+retry UI, date validation, fake-data removal — see S-34, S-36, S-37); the hotelier dashboard pages are next.</t>
+          <t>Real progress since the last report: the blank-screen (createContext) crash is fixed (S-48), instant-load placeholders and skeleton price cells are in, and the booking-widget pages were hardened (S-50, plus the earlier S-34/S-36/S-37). The hotelier dashboard pages are the remaining batch.</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -3093,7 +3959,7 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>The IP-spoofing hole is now FIXED (trusted-proxy IP extraction, S-40) and key routes are rate-limited (S-42). The remaining piece is an edge layer (Cloudflare/WAF) to absorb large-scale attacks before they reach our servers.</t>
+          <t>The IP-spoofing hole is fixed (S-40), key routes are rate-limited (S-42), and a signed anti-automation booking token (HMAC) now guards the booking path. The remaining piece is an edge layer (Cloudflare/WAF) to absorb large-scale attacks before they reach our servers.</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -3120,7 +3986,7 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>The schema is currently built by create_all at startup; performance indexes may be missing in production. The hottest availability index has been added manually (S-38), but a proper migration process is needed.</t>
+          <t>Several missing migrations were added (S-56) and new features now ship with their own indexes (loyalty offers, broadcast id, promo auto-apply, package validity). The schema is still built by create_all/init_db at startup, so a proper Alembic migration process is the remaining work.</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -3147,7 +4013,7 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>The June security audit logged 36 findings. The Critical issue and most High items are fixed. Items still being worked through include: the login-token cache window (~10 min), the unsigned OAuth state parameter, an unauthenticated competitor data-freshness endpoint, and stale analytics cache invalidation.</t>
+          <t>Several have been closed since: the widget code-execution sink was removed (S-50), chat postMessage origin locked, and loyalty read endpoints role-gated (S-53). Items still open: the login-token cache window (~10 min), the unsigned OAuth state parameter, and stale analytics cache invalidation.</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
@@ -3161,10 +4027,26 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="20" t="inlineStr">
+        <is>
+          <t>RECENTLY COMPLETED (graduated out of 'in progress' since the last report)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="60" customHeight="1">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>Revenue Engine shipped (dynamic pricing, abandoned-booking recovery, loyalty wallet &amp; upsell hub) - PR #80; chain features, package improvements &amp; seasonal promotions - PR #88; the recovery scheduler and the booking create/cancel 500 crashes - PR #83; the Cloudflare blank-screen crash - PR #82; the broken-deploy and missing-migration fixes - PR #84/#85; production observability (Sentry) and the engineering knowledge graph - PR #59/#86. All are reflected in Sheets 2 and 3.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="4">
     <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A13:E13"/>
     <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A12:E12"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3203,6 +4085,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="26" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -3394,7 +4277,7 @@
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Redis-backed rate limiting; spoof-proof client IP detection (trusted proxy); per-hotel AI quotas; per-route caps on password change/uploads/reports; limits on streaming connection lifetimes</t>
+          <t>Redis-backed rate limiting; spoof-proof client IP detection (trusted proxy); per-hotel AI quotas; per-route caps on password change/uploads/reports; limits on streaming connection lifetimes; PLUS a signed anti-automation booking token (HMAC) on the booking path.</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
@@ -3478,7 +4361,7 @@
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Backend idempotency ensures the same payment is never processed twice</t>
+          <t>Backend idempotency ensures the same payment is never processed twice; promo/loyalty redemption now takes row locks (SELECT FOR UPDATE) so a balance cannot be double-spent under concurrent clicks (S-51).</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
@@ -3562,7 +4445,7 @@
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Per-hotel daily quotas; cheap model by default; tool-call limits; response caching; usage tracking</t>
+          <t>Per-hotel daily quotas; cheap model by default; tool-call limits; response caching; usage tracking now durably stored in Postgres so it survives a Redis outage (PR #63).</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
@@ -3688,7 +4571,7 @@
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>Vite build optimization at a basic level</t>
+          <t>Vite build optimisation at a basic level; instant-load placeholders and skeleton price cells added on the booking and widget pages so the first paint is never empty (S-48).</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
@@ -3829,6 +4712,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -3856,7 +4740,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Stable for current hoteliers — bookings, payments, dashboards and integrations are working. 45 issues have been found and fixed proactively, and 277 automated tests now run on every code change.</t>
+          <t>Stable for current hoteliers — bookings, payments, dashboards and integrations are working. 58 issues have been found and fixed proactively, and 277 automated tests now run on every code change.</t>
         </is>
       </c>
     </row>
@@ -3896,6 +4780,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
@@ -3988,6 +4873,8 @@
         </is>
       </c>
     </row>
+    <row r="17"/>
+    <row r="18"/>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="8" t="inlineStr">
         <is>
@@ -4025,7 +4912,7 @@
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Prioritised the fix order across 45 issues (money-related first); set the engineering rules and the review checklist the team now follows; set up the CI pipeline that tests every change.</t>
+          <t>Prioritised the fix order across 58 issues (money-related first); set the engineering rules and the review checklist the team now follows; set up the CI pipeline that tests every change.</t>
         </is>
       </c>
     </row>
@@ -4080,6 +4967,8 @@
         </is>
       </c>
     </row>
+    <row r="25"/>
+    <row r="26"/>
     <row r="27" ht="30" customHeight="1">
       <c r="A27" s="8" t="inlineStr">
         <is>
@@ -4197,6 +5086,7 @@
         </is>
       </c>
     </row>
+    <row r="33"/>
     <row r="34">
       <c r="A34" s="8" t="inlineStr">
         <is>
@@ -4210,7 +5100,11 @@
           <t>This is not a request to fix something broken — the product works and customer data is safe today. It is a request to PROTECT what has been built and to DE-RISK growth. Up to now one person has carried database, backend and frontend together. That is fine at the current size, but every new hotel multiplies the data, the traffic and the number of places a single quiet bug could cause a slow page or an outage. Each role below removes a specific, named risk to revenue and reputation. Hiring in the order shown means we always add the person who removes the biggest risk next — never headcount for its own sake.</t>
         </is>
       </c>
-    </row>
+      <c r="B35" s="21" t="n"/>
+      <c r="C35" s="21" t="n"/>
+      <c r="D35" s="22" t="n"/>
+    </row>
+    <row r="36"/>
     <row r="37">
       <c r="A37" s="8" t="inlineStr">
         <is>
@@ -4382,6 +5276,9 @@
           <t>Owns the APIs and their link to the database — payments, booking logic, security, speed and cost. This is where 'API optimisation' and most server-crash prevention live.</t>
         </is>
       </c>
+      <c r="B5" s="21" t="n"/>
+      <c r="C5" s="21" t="n"/>
+      <c r="D5" s="22" t="n"/>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="10" t="inlineStr">
@@ -4550,6 +5447,9 @@
           <t>Owns the React + TypeScript screens and their link to the backend APIs. This is real engineering — correct data, fast loads, no blank screens — not visual design.</t>
         </is>
       </c>
+      <c r="B15" s="21" t="n"/>
+      <c r="C15" s="21" t="n"/>
+      <c r="D15" s="22" t="n"/>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="10" t="inlineStr">
@@ -4696,6 +5596,9 @@
           <t>Owns the data layer — speed, schema, backups and the guarantee that data flows out smoothly at ANY size. Becomes essential as data approaches GB scale; can start part-time.</t>
         </is>
       </c>
+      <c r="B24" s="21" t="n"/>
+      <c r="C24" s="21" t="n"/>
+      <c r="D24" s="22" t="n"/>
     </row>
     <row r="25" ht="30" customHeight="1">
       <c r="A25" s="10" t="inlineStr">
@@ -4864,6 +5767,9 @@
           <t>Responsible for the whole software — decides what each developer builds and when, reviews everything before release, and owns delivery and security posture.</t>
         </is>
       </c>
+      <c r="B34" s="21" t="n"/>
+      <c r="C34" s="21" t="n"/>
+      <c r="D34" s="22" t="n"/>
     </row>
     <row r="35" ht="30" customHeight="1">
       <c r="A35" s="10" t="inlineStr">
@@ -4978,8 +5884,8 @@
   </sheetData>
   <mergeCells count="10">
     <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A23:D23"/>
     <mergeCell ref="A5:D5"/>
-    <mergeCell ref="A23:D23"/>
     <mergeCell ref="A34:D34"/>
     <mergeCell ref="A4:D4"/>
     <mergeCell ref="A15:D15"/>
@@ -5022,6 +5928,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="10" t="inlineStr">
         <is>
@@ -5084,7 +5991,7 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>An endpoint that assumes one row gets several and throws a 500 only for certain data — invisible until that exact data appears.</t>
+          <t>An endpoint that assumes one row gets several and throws a 500 only for certain data — invisible until that exact data appears. We hit exactly this in the loyalty check (S-46).</t>
         </is>
       </c>
       <c r="C6" s="13" t="inlineStr">
@@ -5246,7 +6153,7 @@
       </c>
       <c r="B12" s="13" t="inlineStr">
         <is>
-          <t>One failed fetch with no error boundary turns the entire screen white mid-booking — the guest just leaves (S-36).</t>
+          <t>One failed fetch (or an unsafe bundling change) turns the entire screen white mid-booking — the guest just leaves. We hit this twice and fixed both (S-36, S-48).</t>
         </is>
       </c>
       <c r="C12" s="13" t="inlineStr">
@@ -5319,6 +6226,7 @@
         </is>
       </c>
     </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
         <is>
@@ -5332,6 +6240,10 @@
           <t>•  Layered fallbacks: if Redis crashes, the app transparently falls back to an in-memory cache — it never crashes because of Redis.</t>
         </is>
       </c>
+      <c r="B17" s="21" t="n"/>
+      <c r="C17" s="21" t="n"/>
+      <c r="D17" s="21" t="n"/>
+      <c r="E17" s="22" t="n"/>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="12" t="inlineStr">
@@ -5339,6 +6251,10 @@
           <t>•  No blank screens: a failed data fetch shows a clear message with a Retry button; optional pieces (add-ons) load separately so one failure can't take down the page.</t>
         </is>
       </c>
+      <c r="B18" s="21" t="n"/>
+      <c r="C18" s="21" t="n"/>
+      <c r="D18" s="21" t="n"/>
+      <c r="E18" s="22" t="n"/>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="12" t="inlineStr">
@@ -5346,6 +6262,10 @@
           <t>•  Fail closed on money &amp; security, fail soft on the screen: anything touching payment, roles or another hotel's data DENIES on doubt; anything touching the display keeps working in a reduced mode.</t>
         </is>
       </c>
+      <c r="B19" s="21" t="n"/>
+      <c r="C19" s="21" t="n"/>
+      <c r="D19" s="21" t="n"/>
+      <c r="E19" s="22" t="n"/>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="12" t="inlineStr">
@@ -5353,6 +6273,10 @@
           <t>•  Tested on every change: 277 automated tests (including Redis-failover and cross-tenant attack tests) run before any code can merge.</t>
         </is>
       </c>
+      <c r="B20" s="21" t="n"/>
+      <c r="C20" s="21" t="n"/>
+      <c r="D20" s="21" t="n"/>
+      <c r="E20" s="22" t="n"/>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="12" t="inlineStr">
@@ -5360,13 +6284,17 @@
           <t>•  The 'safer side' principle the CEO asked for: when in doubt we choose the cautious behaviour — reject the risky action, keep the guest's screen usable, and log it for a human to review.</t>
         </is>
       </c>
+      <c r="B21" s="21" t="n"/>
+      <c r="C21" s="21" t="n"/>
+      <c r="D21" s="21" t="n"/>
+      <c r="E21" s="22" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="8">
     <mergeCell ref="A21:E21"/>
     <mergeCell ref="A20:E20"/>
+    <mergeCell ref="A16:E16"/>
     <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A16:E16"/>
     <mergeCell ref="A19:E19"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A17:E17"/>
@@ -5612,6 +6540,11 @@
           <t>•  Even when data is huge, the app never tries to load everything at once — the database sends rows in pages, the backend serves them in chunks, and the frontend draws only what's on screen.</t>
         </is>
       </c>
+      <c r="B12" s="21" t="n"/>
+      <c r="C12" s="21" t="n"/>
+      <c r="D12" s="21" t="n"/>
+      <c r="E12" s="21" t="n"/>
+      <c r="F12" s="22" t="n"/>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="12" t="inlineStr">
@@ -5619,6 +6552,11 @@
           <t>•  If any stage is slow or fails, the guest sees a Retry — never a frozen tab or a white page.</t>
         </is>
       </c>
+      <c r="B13" s="21" t="n"/>
+      <c r="C13" s="21" t="n"/>
+      <c r="D13" s="21" t="n"/>
+      <c r="E13" s="21" t="n"/>
+      <c r="F13" s="22" t="n"/>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="12" t="inlineStr">
@@ -5626,6 +6564,11 @@
           <t>•  Money and security checks never get 'skipped to go faster': they stay strict (fail closed) no matter the load. Only the display degrades gracefully, never the safety.</t>
         </is>
       </c>
+      <c r="B14" s="21" t="n"/>
+      <c r="C14" s="21" t="n"/>
+      <c r="D14" s="21" t="n"/>
+      <c r="E14" s="21" t="n"/>
+      <c r="F14" s="22" t="n"/>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="12" t="inlineStr">
@@ -5633,6 +6576,11 @@
           <t>•  Costs stay bounded as data grows: capped result sizes, caching, and per-hotel quotas mean more data does not mean a runaway bill.</t>
         </is>
       </c>
+      <c r="B15" s="21" t="n"/>
+      <c r="C15" s="21" t="n"/>
+      <c r="D15" s="21" t="n"/>
+      <c r="E15" s="21" t="n"/>
+      <c r="F15" s="22" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="7">

</xml_diff>

<commit_message>
docs: stakeholder-grade report refresh from full git history
- Re-title for all stakeholders (not just CEO)
- Problems Solved: 58 -> 74 (earlier foundational security/crash/correctness fixes)
- Features Built: 23 -> 37 (GST/tax, WhatsApp & Google AI agents, Super Admin
  console, subscriptions/feature-gating, AI stack, email, widget suite, compliance)
- Work In Progress: correct statuses (load test/refund/Alembic foundations exist)
- Future Risks: add F-14..F-27 (shared-server, many-hotels, many-guests scenarios)
- Team & Hiring: Tech Lead as accountable owner + explicit chain of command

https://claude.ai/code/session_01Jfp6dFcb8aisQfoK5brnT1
</commit_message>
<xml_diff>
--- a/docs/CEO_Report_Staybooker_Jun2026.xlsx
+++ b/docs/CEO_Report_Staybooker_Jun2026.xlsx
@@ -25,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -69,8 +69,13 @@
       <color rgb="001F4E79"/>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="000B3050"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -105,6 +110,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
       </patternFill>
     </fill>
   </fills>
@@ -192,7 +202,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -248,6 +258,9 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -623,14 +636,14 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Staybooker Booking Engine — CEO Report (June 2026)</t>
+          <t>Staybooker Booking Engine — Stakeholder Report (June 2026)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="28" customHeight="1">
       <c r="A2" s="9" t="inlineStr">
         <is>
-          <t>What has been solved, what is in progress, what risks are coming, how the product stays fast and crash-proof at scale, and why we need a team — at a glance.</t>
+          <t>Prepared for the CEO, founders, investors and stakeholders. What has been solved, what is in progress, what risks are coming as we grow, how the product stays fast and crash-proof at scale, and the team needed to sustain it.</t>
         </is>
       </c>
     </row>
@@ -663,7 +676,7 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>58 issues fixed so far (6 Critical, 30 High, 22 Medium). Each issue shows what would have happened to the business if it had reached production.</t>
+          <t>74 issues fixed so far (6 Critical, 38 High, 30 Medium) across the project's history. Each issue shows what would have happened to the business if it had reached production.</t>
         </is>
       </c>
     </row>
@@ -675,7 +688,7 @@
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>23 major product features delivered alongside the bug fixing — multi-property chains, loyalty wallet, OTA rate intelligence, AI concierge, real-time updates, encrypted secrets, and the new Revenue Engine (dynamic pricing, abandoned-booking recovery, chain upsell broadcast, seasonal promotions, OTA-style booking widget).</t>
+          <t>37 major product features delivered alongside the bug fixing — multi-property chains, loyalty, the Revenue Engine, OTA-style booking widgets, a GST/tax engine, WhatsApp &amp; Google AI agents, a full Super Admin platform console, subscriptions &amp; feature-gating, and more.</t>
         </is>
       </c>
     </row>
@@ -780,7 +793,7 @@
       </c>
       <c r="B17" s="13" t="inlineStr">
         <is>
-          <t>58 (source: work_log_tracker.csv — engineering tasks logged up to 16-Jun-2026; merged across PRs up to #90)</t>
+          <t>74 (source: full git history of 890 commits + work_log_tracker.csv, up to 16-Jun-2026; merged across PRs up to #90)</t>
         </is>
       </c>
     </row>
@@ -816,7 +829,7 @@
       </c>
       <c r="B20" s="13" t="inlineStr">
         <is>
-          <t>Close to 300 automated test cases (the 277 from the June audit, plus new tests for the anti-automation booking token, the recovery scheduler, chain features and public-booking promotions). They run on every code change (CI/CD), with dependency vulnerability (CVE) scanning.</t>
+          <t>Close to 300 automated test cases (security, payments, booking, roles, rate limits, Redis failover, chain isolation, promotions) that run on every code change (CI/CD), with dependency vulnerability (CVE) scanning.</t>
         </is>
       </c>
     </row>
@@ -844,7 +857,6 @@
         </is>
       </c>
     </row>
-    <row r="23"/>
     <row r="24">
       <c r="A24" s="11" t="inlineStr">
         <is>
@@ -924,7 +936,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G62"/>
+  <dimension ref="A1:G79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3133,9 +3145,609 @@
         </is>
       </c>
     </row>
+    <row r="63" ht="22" customHeight="1">
+      <c r="A63" s="23" t="inlineStr">
+        <is>
+          <t>EARLIER FOUNDATIONAL FIXES (May – early June 2026) — security, crashes and correctness fixed before the June audit</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="13" t="inlineStr">
+        <is>
+          <t>S-59</t>
+        </is>
+      </c>
+      <c r="B64" s="13" t="inlineStr">
+        <is>
+          <t>The public booking page crashed for guests (blank/white page) more than once</t>
+        </is>
+      </c>
+      <c r="C64" s="13" t="inlineStr">
+        <is>
+          <t>React runtime errors (#300 and a hooks-rule violation in a booking widget) crashed the page render</t>
+        </is>
+      </c>
+      <c r="D64" s="13" t="inlineStr">
+        <is>
+          <t>Guests opening the booking page could see a blank or broken page and leave — lost bookings with no error trail.</t>
+        </is>
+      </c>
+      <c r="E64" s="13" t="inlineStr">
+        <is>
+          <t>Fixed the React errors and hook usage; added guards so one widget can't crash the whole page.</t>
+        </is>
+      </c>
+      <c r="F64" s="17" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G64" s="13" t="inlineStr">
+        <is>
+          <t>02-03 Jun</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="13" t="inlineStr">
+        <is>
+          <t>S-60</t>
+        </is>
+      </c>
+      <c r="B65" s="13" t="inlineStr">
+        <is>
+          <t>The backend could crash on startup</t>
+        </is>
+      </c>
+      <c r="C65" s="13" t="inlineStr">
+        <is>
+          <t>Superadmin import errors, a sync/async mismatch and an undefined router crashed the server on boot</t>
+        </is>
+      </c>
+      <c r="D65" s="13" t="inlineStr">
+        <is>
+          <t>A bad deploy would take the whole API down — every hotel offline until someone noticed.</t>
+        </is>
+      </c>
+      <c r="E65" s="13" t="inlineStr">
+        <is>
+          <t>Fixed the imports, converted to async correctly, and removed the undefined router.</t>
+        </is>
+      </c>
+      <c r="F65" s="17" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G65" s="13" t="inlineStr">
+        <is>
+          <t>May 12-Jun 01</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="13" t="inlineStr">
+        <is>
+          <t>S-61</t>
+        </is>
+      </c>
+      <c r="B66" s="13" t="inlineStr">
+        <is>
+          <t>The rooms page crashed with a 'Form is not defined' error</t>
+        </is>
+      </c>
+      <c r="C66" s="13" t="inlineStr">
+        <is>
+          <t>A circular dependency loaded a dialog before its form was ready</t>
+        </is>
+      </c>
+      <c r="D66" s="13" t="inlineStr">
+        <is>
+          <t>Hoteliers couldn't manage rooms — a core daily task was broken.</t>
+        </is>
+      </c>
+      <c r="E66" s="13" t="inlineStr">
+        <is>
+          <t>Lazy-loaded the dialogs to break the circular import.</t>
+        </is>
+      </c>
+      <c r="F66" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G66" s="13" t="inlineStr">
+        <is>
+          <t>14-May</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="13" t="inlineStr">
+        <is>
+          <t>S-62</t>
+        </is>
+      </c>
+      <c r="B67" s="13" t="inlineStr">
+        <is>
+          <t>The public booking page crashed on newly created rooms</t>
+        </is>
+      </c>
+      <c r="C67" s="13" t="inlineStr">
+        <is>
+          <t>New rooms weren't handled in the availability path and the rate cache wasn't invalidated</t>
+        </is>
+      </c>
+      <c r="D67" s="13" t="inlineStr">
+        <is>
+          <t>Brand-new inventory couldn't be booked — directly blocking sales of the newest rooms.</t>
+        </is>
+      </c>
+      <c r="E67" s="13" t="inlineStr">
+        <is>
+          <t>Fixed the availability handling and added real-time rate-cache invalidation.</t>
+        </is>
+      </c>
+      <c r="F67" s="17" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G67" s="13" t="inlineStr">
+        <is>
+          <t>23-May</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="13" t="inlineStr">
+        <is>
+          <t>S-63</t>
+        </is>
+      </c>
+      <c r="B68" s="13" t="inlineStr">
+        <is>
+          <t>The guest chatbot crashed on availability follow-up questions</t>
+        </is>
+      </c>
+      <c r="C68" s="13" t="inlineStr">
+        <is>
+          <t>The Llama model returned a tool_use_failed error that wasn't handled</t>
+        </is>
+      </c>
+      <c r="D68" s="13" t="inlineStr">
+        <is>
+          <t>A premium guest feature broke mid-conversation, frustrating guests.</t>
+        </is>
+      </c>
+      <c r="E68" s="13" t="inlineStr">
+        <is>
+          <t>Added handling for the failure path so the chat recovers gracefully.</t>
+        </is>
+      </c>
+      <c r="F68" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G68" s="13" t="inlineStr">
+        <is>
+          <t>03-Jun</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="13" t="inlineStr">
+        <is>
+          <t>S-64</t>
+        </is>
+      </c>
+      <c r="B69" s="13" t="inlineStr">
+        <is>
+          <t>Database migrations could fail on deploy (divergent Alembic heads)</t>
+        </is>
+      </c>
+      <c r="C69" s="13" t="inlineStr">
+        <is>
+          <t>Two migration branches diverged and some migrations weren't idempotent</t>
+        </is>
+      </c>
+      <c r="D69" s="13" t="inlineStr">
+        <is>
+          <t>A deploy could half-apply the schema and break production.</t>
+        </is>
+      </c>
+      <c r="E69" s="13" t="inlineStr">
+        <is>
+          <t>Merged the migration heads and made migrations safe to re-run.</t>
+        </is>
+      </c>
+      <c r="F69" s="17" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G69" s="13" t="inlineStr">
+        <is>
+          <t>03-Jun</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="13" t="inlineStr">
+        <is>
+          <t>S-65</t>
+        </is>
+      </c>
+      <c r="B70" s="13" t="inlineStr">
+        <is>
+          <t>Switching between properties could briefly show another property's data</t>
+        </is>
+      </c>
+      <c r="C70" s="13" t="inlineStr">
+        <is>
+          <t>Browser-side caching and a backend cache-key bug served stale, cross-property data</t>
+        </is>
+      </c>
+      <c r="D70" s="13" t="inlineStr">
+        <is>
+          <t>A hotelier could momentarily see the wrong hotel's numbers — a trust and isolation concern.</t>
+        </is>
+      </c>
+      <c r="E70" s="13" t="inlineStr">
+        <is>
+          <t>Disabled unsafe API caching, fixed the cache key, and moved to instant SPA navigation.</t>
+        </is>
+      </c>
+      <c r="F70" s="17" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G70" s="13" t="inlineStr">
+        <is>
+          <t>04-05 Jun</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="13" t="inlineStr">
+        <is>
+          <t>S-66</t>
+        </is>
+      </c>
+      <c r="B71" s="13" t="inlineStr">
+        <is>
+          <t>Cross-tenant data-isolation gaps in several endpoints (IDOR)</t>
+        </is>
+      </c>
+      <c r="C71" s="13" t="inlineStr">
+        <is>
+          <t>Some endpoints didn't fully scope queries to the caller's hotel/chain (TEN-02/04/05)</t>
+        </is>
+      </c>
+      <c r="D71" s="13" t="inlineStr">
+        <is>
+          <t>One hotel could potentially reach another's data — a serious multi-tenant breach risk.</t>
+        </is>
+      </c>
+      <c r="E71" s="13" t="inlineStr">
+        <is>
+          <t>Tightened scoping on every affected endpoint to the caller's own tenant.</t>
+        </is>
+      </c>
+      <c r="F71" s="17" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G71" s="13" t="inlineStr">
+        <is>
+          <t>05-Jun</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="13" t="inlineStr">
+        <is>
+          <t>S-67</t>
+        </is>
+      </c>
+      <c r="B72" s="13" t="inlineStr">
+        <is>
+          <t>Role-based access was defined but not actually enforced on some routes</t>
+        </is>
+      </c>
+      <c r="C72" s="13" t="inlineStr">
+        <is>
+          <t>RBAC existed in code but several routes never checked it (AZ-01/02/03)</t>
+        </is>
+      </c>
+      <c r="D72" s="13" t="inlineStr">
+        <is>
+          <t>Staff-level accounts could reach owner-level actions — privilege misuse.</t>
+        </is>
+      </c>
+      <c r="E72" s="13" t="inlineStr">
+        <is>
+          <t>Enforced the role checks on every affected route.</t>
+        </is>
+      </c>
+      <c r="F72" s="17" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G72" s="13" t="inlineStr">
+        <is>
+          <t>05-Jun</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="13" t="inlineStr">
+        <is>
+          <t>S-68</t>
+        </is>
+      </c>
+      <c r="B73" s="13" t="inlineStr">
+        <is>
+          <t>AI spend on public/agent paths was unbounded</t>
+        </is>
+      </c>
+      <c r="C73" s="13" t="inlineStr">
+        <is>
+          <t>Some LLM calls had no token or call ceiling (AI-01/02/04)</t>
+        </is>
+      </c>
+      <c r="D73" s="13" t="inlineStr">
+        <is>
+          <t>A traffic spike or abuse could run the AI bill up sharply.</t>
+        </is>
+      </c>
+      <c r="E73" s="13" t="inlineStr">
+        <is>
+          <t>Added token floors, tool-call limits and history caps across the AI paths.</t>
+        </is>
+      </c>
+      <c r="F73" s="17" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G73" s="13" t="inlineStr">
+        <is>
+          <t>05-Jun</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="13" t="inlineStr">
+        <is>
+          <t>S-69</t>
+        </is>
+      </c>
+      <c r="B74" s="13" t="inlineStr">
+        <is>
+          <t>Reports and analytics could show wrong numbers</t>
+        </is>
+      </c>
+      <c r="C74" s="13" t="inlineStr">
+        <is>
+          <t>Booking-source attribution and several analytics calculations were incorrect</t>
+        </is>
+      </c>
+      <c r="D74" s="13" t="inlineStr">
+        <is>
+          <t>Hoteliers would make decisions on wrong data and lose trust in the product.</t>
+        </is>
+      </c>
+      <c r="E74" s="13" t="inlineStr">
+        <is>
+          <t>Corrected the attribution and the analytics math; added tests.</t>
+        </is>
+      </c>
+      <c r="F74" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G74" s="13" t="inlineStr">
+        <is>
+          <t>04-Jun</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="13" t="inlineStr">
+        <is>
+          <t>S-70</t>
+        </is>
+      </c>
+      <c r="B75" s="13" t="inlineStr">
+        <is>
+          <t>Dashboards were slow and overloaded the database (N+1 queries)</t>
+        </is>
+      </c>
+      <c r="C75" s="13" t="inlineStr">
+        <is>
+          <t>Pages fired many small queries instead of one batched query; hotel info wasn't cached</t>
+        </is>
+      </c>
+      <c r="D75" s="13" t="inlineStr">
+        <is>
+          <t>As data grew, dashboards would slow for everyone and strain the database.</t>
+        </is>
+      </c>
+      <c r="E75" s="13" t="inlineStr">
+        <is>
+          <t>Batched the queries, added caching and parallelised integration calls.</t>
+        </is>
+      </c>
+      <c r="F75" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G75" s="13" t="inlineStr">
+        <is>
+          <t>02-04 Jun</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="13" t="inlineStr">
+        <is>
+          <t>S-71</t>
+        </is>
+      </c>
+      <c r="B76" s="13" t="inlineStr">
+        <is>
+          <t>Responses had no security headers</t>
+        </is>
+      </c>
+      <c r="C76" s="13" t="inlineStr">
+        <is>
+          <t>Missing HSTS, CSP, X-Frame-Options and X-Content-Type-Options</t>
+        </is>
+      </c>
+      <c r="D76" s="13" t="inlineStr">
+        <is>
+          <t>The app was more exposed to clickjacking, content-sniffing and mixed-content attacks.</t>
+        </is>
+      </c>
+      <c r="E76" s="13" t="inlineStr">
+        <is>
+          <t>Added enterprise security headers across all responses.</t>
+        </is>
+      </c>
+      <c r="F76" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G76" s="13" t="inlineStr">
+        <is>
+          <t>16-May</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="13" t="inlineStr">
+        <is>
+          <t>S-72</t>
+        </is>
+      </c>
+      <c r="B77" s="13" t="inlineStr">
+        <is>
+          <t>A null widget-config value could crash the embedded booking widget</t>
+        </is>
+      </c>
+      <c r="C77" s="13" t="inlineStr">
+        <is>
+          <t>Missing null-safety on widget configuration and chat</t>
+        </is>
+      </c>
+      <c r="D77" s="13" t="inlineStr">
+        <is>
+          <t>The widget could break on a hotel's own website, in front of their guests.</t>
+        </is>
+      </c>
+      <c r="E77" s="13" t="inlineStr">
+        <is>
+          <t>Hardened the config handling and chat resilience.</t>
+        </is>
+      </c>
+      <c r="F77" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G77" s="13" t="inlineStr">
+        <is>
+          <t>04-May</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="13" t="inlineStr">
+        <is>
+          <t>S-73</t>
+        </is>
+      </c>
+      <c r="B78" s="13" t="inlineStr">
+        <is>
+          <t>The AI usage dashboard was stuck on 'Loading…' / 'Couldn't load usage'</t>
+        </is>
+      </c>
+      <c r="C78" s="13" t="inlineStr">
+        <is>
+          <t>Subscription AI-limit columns were missing and usage lived only in Redis</t>
+        </is>
+      </c>
+      <c r="D78" s="13" t="inlineStr">
+        <is>
+          <t>Hoteliers couldn't see what they were paying for, and data vanished on a Redis blip.</t>
+        </is>
+      </c>
+      <c r="E78" s="13" t="inlineStr">
+        <is>
+          <t>Added the missing columns and made AI usage durable in Postgres.</t>
+        </is>
+      </c>
+      <c r="F78" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G78" s="13" t="inlineStr">
+        <is>
+          <t>12-Jun</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="13" t="inlineStr">
+        <is>
+          <t>S-74</t>
+        </is>
+      </c>
+      <c r="B79" s="13" t="inlineStr">
+        <is>
+          <t>Guests couldn't reset their password reliably</t>
+        </is>
+      </c>
+      <c r="C79" s="13" t="inlineStr">
+        <is>
+          <t>The reset flow didn't fully support PKCE/implicit hand-off and recovery redirects</t>
+        </is>
+      </c>
+      <c r="D79" s="13" t="inlineStr">
+        <is>
+          <t>Locked-out users couldn't get back in — support load and churn.</t>
+        </is>
+      </c>
+      <c r="E79" s="13" t="inlineStr">
+        <is>
+          <t>Completed the reset flow (PKCE/implicit, recovery redirect, in-profile change).</t>
+        </is>
+      </c>
+      <c r="F79" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G79" s="13" t="inlineStr">
+        <is>
+          <t>05-Jun</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A63:G63"/>
     <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3148,7 +3760,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -3798,10 +4410,368 @@
         </is>
       </c>
     </row>
+    <row r="28" ht="22" customHeight="1">
+      <c r="A28" s="23" t="inlineStr">
+        <is>
+          <t>EARLIER PLATFORM FEATURES (built across May – early June 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="13" t="n">
+        <v>24</v>
+      </c>
+      <c r="B29" s="13" t="inlineStr">
+        <is>
+          <t>GST / tax engine</t>
+        </is>
+      </c>
+      <c r="C29" s="13" t="inlineStr">
+        <is>
+          <t>Configurable tax slabs (inclusive &amp; exclusive), itemized tax breakdowns on every booking and invoice, and guest-facing price/tax disclosures.</t>
+        </is>
+      </c>
+      <c r="D29" s="13" t="inlineStr">
+        <is>
+          <t>Correct, compliant billing for Indian hotels — essential for trust and GST filing.</t>
+        </is>
+      </c>
+      <c r="E29" s="13" t="inlineStr">
+        <is>
+          <t>Tax is validated on save and computed server-side; guarded against NaN/zero-division.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="13" t="n">
+        <v>25</v>
+      </c>
+      <c r="B30" s="13" t="inlineStr">
+        <is>
+          <t>WhatsApp AI Agent</t>
+        </is>
+      </c>
+      <c r="C30" s="13" t="inlineStr">
+        <is>
+          <t>Per-hotel WhatsApp integration that sends booking confirmations and answers guests with AI, metered against subscription credits.</t>
+        </is>
+      </c>
+      <c r="D30" s="13" t="inlineStr">
+        <is>
+          <t>Guests get instant answers and confirmations on the channel they actually use.</t>
+        </is>
+      </c>
+      <c r="E30" s="13" t="inlineStr">
+        <is>
+          <t>Webhook payloads HMAC-verified; credits deducted per message; keys resolved from the encrypted Vault.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="13" t="n">
+        <v>26</v>
+      </c>
+      <c r="B31" s="13" t="inlineStr">
+        <is>
+          <t>Google Reviews AI Reply Studio</t>
+        </is>
+      </c>
+      <c r="C31" s="13" t="inlineStr">
+        <is>
+          <t>Per-hotel Google OAuth connect, fetch reviews, AI-drafted replies, and one-click posting back to the Google Business Profile.</t>
+        </is>
+      </c>
+      <c r="D31" s="13" t="inlineStr">
+        <is>
+          <t>Saves staff hours and improves the hotel's public reputation — a premium upsell.</t>
+        </is>
+      </c>
+      <c r="E31" s="13" t="inlineStr">
+        <is>
+          <t>Per-hotel OAuth tokens stored securely; scoped to the connected account.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="13" t="n">
+        <v>27</v>
+      </c>
+      <c r="B32" s="13" t="inlineStr">
+        <is>
+          <t>Google Hotel Ads integration</t>
+        </is>
+      </c>
+      <c r="C32" s="13" t="inlineStr">
+        <is>
+          <t>Feeds and UI to list a hotel's rates and availability on Google Hotel Ads.</t>
+        </is>
+      </c>
+      <c r="D32" s="13" t="inlineStr">
+        <is>
+          <t>A new demand channel for direct bookings.</t>
+        </is>
+      </c>
+      <c r="E32" s="13" t="inlineStr">
+        <is>
+          <t>Feature-gated by plan; per-hotel scoped.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="13" t="n">
+        <v>28</v>
+      </c>
+      <c r="B33" s="13" t="inlineStr">
+        <is>
+          <t>Multi-tenant email system</t>
+        </is>
+      </c>
+      <c r="C33" s="13" t="inlineStr">
+        <is>
+          <t>Custom email via SMTP or Brevo, with per-hotel sender, CC, signature and branded templates.</t>
+        </is>
+      </c>
+      <c r="D33" s="13" t="inlineStr">
+        <is>
+          <t>Confirmations and communications come from the hotel's own brand, not a generic system.</t>
+        </is>
+      </c>
+      <c r="E33" s="13" t="inlineStr">
+        <is>
+          <t>Per-hotel credentials encrypted; senders fail-safe so a mail error never breaks a booking.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="13" t="n">
+        <v>29</v>
+      </c>
+      <c r="B34" s="13" t="inlineStr">
+        <is>
+          <t>Super Admin platform console</t>
+        </is>
+      </c>
+      <c r="C34" s="13" t="inlineStr">
+        <is>
+          <t>A full operator console — KYC, commissions, payouts, support tickets, platform settings, MRR &amp; plan breakdowns, system diagnostics, and secure impersonation with an exit banner and audit trail.</t>
+        </is>
+      </c>
+      <c r="D34" s="13" t="inlineStr">
+        <is>
+          <t>Lets us run Staybooker as a business: onboard, bill, support and oversee every hotel.</t>
+        </is>
+      </c>
+      <c r="E34" s="13" t="inlineStr">
+        <is>
+          <t>Superadmin-gated; impersonation tokens expire; every privileged action is audit-logged.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="13" t="n">
+        <v>30</v>
+      </c>
+      <c r="B35" s="13" t="inlineStr">
+        <is>
+          <t>Subscriptions &amp; feature-gating</t>
+        </is>
+      </c>
+      <c r="C35" s="13" t="inlineStr">
+        <is>
+          <t>Subscription plans with a per-plan feature-allocation matrix, automatic feature sync, and premium locks across the product.</t>
+        </is>
+      </c>
+      <c r="D35" s="13" t="inlineStr">
+        <is>
+          <t>Turns features into packaged, sellable tiers — the core of the revenue model.</t>
+        </is>
+      </c>
+      <c r="E35" s="13" t="inlineStr">
+        <is>
+          <t>Plan checks enforced server-side; writes to subscription state are locked.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="13" t="n">
+        <v>31</v>
+      </c>
+      <c r="B36" s="13" t="inlineStr">
+        <is>
+          <t>Customizable role permissions</t>
+        </is>
+      </c>
+      <c r="C36" s="13" t="inlineStr">
+        <is>
+          <t>A per-hotel role-permission matrix (OWNER/MANAGER/STAFF and sub-roles) with a complete security audit trail.</t>
+        </is>
+      </c>
+      <c r="D36" s="13" t="inlineStr">
+        <is>
+          <t>Hotels control exactly what each employee can do — important for larger properties.</t>
+        </is>
+      </c>
+      <c r="E36" s="13" t="inlineStr">
+        <is>
+          <t>Permissions enforced on the backend, not just the menu; every change is logged.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="13" t="n">
+        <v>32</v>
+      </c>
+      <c r="B37" s="13" t="inlineStr">
+        <is>
+          <t>Configurable AI stack</t>
+        </is>
+      </c>
+      <c r="C37" s="13" t="inlineStr">
+        <is>
+          <t>AI agents on the Agno framework with per-hotel model choice (Llama, Google Gemini, DeepSeek), token limits, and a durable per-agent usage dashboard.</t>
+        </is>
+      </c>
+      <c r="D37" s="13" t="inlineStr">
+        <is>
+          <t>Right-sized AI cost and quality per hotel, with full visibility into spend.</t>
+        </is>
+      </c>
+      <c r="E37" s="13" t="inlineStr">
+        <is>
+          <t>Cheap model by default; token/tool-call limits; usage durably tracked in Postgres.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="13" t="n">
+        <v>33</v>
+      </c>
+      <c r="B38" s="13" t="inlineStr">
+        <is>
+          <t>Experiences &amp; Activities upsell</t>
+        </is>
+      </c>
+      <c r="C38" s="13" t="inlineStr">
+        <is>
+          <t>Add-ons, services and amenities a guest can add at checkout (e.g. activities, transfers), managed by the hotel.</t>
+        </is>
+      </c>
+      <c r="D38" s="13" t="inlineStr">
+        <is>
+          <t>Higher average booking value — incremental revenue on every stay.</t>
+        </is>
+      </c>
+      <c r="E38" s="13" t="inlineStr">
+        <is>
+          <t>Prices validated server-side; tenant-scoped.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="13" t="n">
+        <v>34</v>
+      </c>
+      <c r="B39" s="13" t="inlineStr">
+        <is>
+          <t>Configurable cancellation &amp; refund policies</t>
+        </is>
+      </c>
+      <c r="C39" s="13" t="inlineStr">
+        <is>
+          <t>Instant-vs-request cancellation modes (set by super admin) and room-level cancellation/refund overrides.</t>
+        </is>
+      </c>
+      <c r="D39" s="13" t="inlineStr">
+        <is>
+          <t>Hotels match the platform to their real policies — fewer disputes.</t>
+        </is>
+      </c>
+      <c r="E39" s="13" t="inlineStr">
+        <is>
+          <t>Mode enforced server-side; refunds run through the verified payment path.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="13" t="n">
+        <v>35</v>
+      </c>
+      <c r="B40" s="13" t="inlineStr">
+        <is>
+          <t>Booking source tracking &amp; leads</t>
+        </is>
+      </c>
+      <c r="C40" s="13" t="inlineStr">
+        <is>
+          <t>Attribution of where each booking came from, AI-captured leads with filters, and CSV export of bookings and leads.</t>
+        </is>
+      </c>
+      <c r="D40" s="13" t="inlineStr">
+        <is>
+          <t>Hotels see which channels work and can follow up on leads — more direct bookings.</t>
+        </is>
+      </c>
+      <c r="E40" s="13" t="inlineStr">
+        <is>
+          <t>Tenant-scoped; exports limited to the hotel's own data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="13" t="n">
+        <v>36</v>
+      </c>
+      <c r="B41" s="13" t="inlineStr">
+        <is>
+          <t>Embeddable widget suite</t>
+        </is>
+      </c>
+      <c r="C41" s="13" t="inlineStr">
+        <is>
+          <t>Multiple booking-widget layouts (Booking.com-style, STAAH-style, capsule, glassmorphism), theme-matched, with live per-date pricing and dual hotel + chain widgets.</t>
+        </is>
+      </c>
+      <c r="D41" s="13" t="inlineStr">
+        <is>
+          <t>Hotels add a professional, commission-free booking engine to their own website.</t>
+        </is>
+      </c>
+      <c r="E41" s="13" t="inlineStr">
+        <is>
+          <t>Host-page-safe loader; hardened postMessage; live prices confirmed server-side.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="13" t="n">
+        <v>37</v>
+      </c>
+      <c r="B42" s="13" t="inlineStr">
+        <is>
+          <t>Public presence &amp; compliance</t>
+        </is>
+      </c>
+      <c r="C42" s="13" t="inlineStr">
+        <is>
+          <t>A premium landing page with smart subdomain routing, customizable hotel URL slugs, and the legal/compliance pages (refund, cookie, contact, Meta-verification).</t>
+        </is>
+      </c>
+      <c r="D42" s="13" t="inlineStr">
+        <is>
+          <t>A credible public face and the compliance pages required to operate and integrate.</t>
+        </is>
+      </c>
+      <c r="E42" s="13" t="inlineStr">
+        <is>
+          <t>Slug uniqueness validated; compliance pages public by design.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A28:E28"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3876,14 +4846,14 @@
           <t>Razorpay payment failure recovery (money deducted but booking not created)</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>Guest's network dropped mid-payment / Razorpay API failed — money was deducted but the booking got cancelled. Idempotency and webhook verification are already implemented; the auto-refund flow and reconciliation job still need to be built.</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>In Progress</t>
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>A Razorpay refund endpoint, idempotency keys and webhook signature verification are already built. The remaining pieces are the FULLY-AUTOMATIC refund flow and a daily reconciliation job (matching the Razorpay ledger to our bookings).</t>
+        </is>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>In Progress (foundations done)</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
@@ -3903,14 +4873,14 @@
           <t>Load testing — what happens when 100+ users book at the same time</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>Database locks already protect against race conditions (one room sold twice), but real-load behaviour (connection pool exhaustion, timeouts) still needs testing.</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>In Progress</t>
+      <c r="C6" s="13" t="inlineStr">
+        <is>
+          <t>A load-test harness and scale documentation (SCALE_TUNING.md) already exist, and database row-locks protect against double-selling a room. The remaining work is running load tests at realistic scale and tuning the connection pool / auto-scaling from the results.</t>
+        </is>
+      </c>
+      <c r="D6" s="13" t="inlineStr">
+        <is>
+          <t>In Progress (harness ready)</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
@@ -3984,14 +4954,14 @@
           <t>Database migration discipline (Alembic in the deploy process)</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>Several missing migrations were added (S-56) and new features now ship with their own indexes (loyalty offers, broadcast id, promo auto-apply, package validity). The schema is still built by create_all/init_db at startup, so a proper Alembic migration process is the remaining work.</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>In Progress</t>
+      <c r="C9" s="13" t="inlineStr">
+        <is>
+          <t>Alembic is set up (divergent heads merged, migrations made idempotent), but several newer features still create tables via create_all/init_db at startup. The remaining work is to bring every schema change under one consistent Alembic process.</t>
+        </is>
+      </c>
+      <c r="D9" s="13" t="inlineStr">
+        <is>
+          <t>In Progress (Alembic exists)</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
@@ -4040,6 +5010,10 @@
           <t>Revenue Engine shipped (dynamic pricing, abandoned-booking recovery, loyalty wallet &amp; upsell hub) - PR #80; chain features, package improvements &amp; seasonal promotions - PR #88; the recovery scheduler and the booking create/cancel 500 crashes - PR #83; the Cloudflare blank-screen crash - PR #82; the broken-deploy and missing-migration fixes - PR #84/#85; production observability (Sentry) and the engineering knowledge graph - PR #59/#86. All are reflected in Sheets 2 and 3.</t>
         </is>
       </c>
+      <c r="B13" s="21" t="n"/>
+      <c r="C13" s="21" t="n"/>
+      <c r="D13" s="21" t="n"/>
+      <c r="E13" s="22" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -4058,7 +5032,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -4085,7 +5059,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="26" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -4674,8 +5647,604 @@
         </is>
       </c>
     </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="23" t="inlineStr">
+        <is>
+          <t>MORE SCENARIOS AS WE SCALE — many hotels and their guests all share the same servers</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="13" t="inlineStr">
+        <is>
+          <t>F-14</t>
+        </is>
+      </c>
+      <c r="B19" s="13" t="inlineStr">
+        <is>
+          <t>One busy hotel's traffic or heavy reports slow down every other hotel ('noisy neighbour')</t>
+        </is>
+      </c>
+      <c r="C19" s="13" t="inlineStr">
+        <is>
+          <t>All hotels share the same servers and database; one hotel running a huge report or a sale can starve the rest</t>
+        </is>
+      </c>
+      <c r="D19" s="13" t="inlineStr">
+        <is>
+          <t>Shared multi-tenant infrastructure with finite CPU, connections and memory</t>
+        </is>
+      </c>
+      <c r="E19" s="13" t="inlineStr">
+        <is>
+          <t>Pagination and row caps everywhere; per-hotel AI quotas; Redis caching; env-driven pools</t>
+        </is>
+      </c>
+      <c r="F19" s="13" t="inlineStr">
+        <is>
+          <t>Per-tenant rate/usage limits, query budgets, and isolating heavy reports onto background workers/replicas</t>
+        </is>
+      </c>
+      <c r="G19" s="17" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H19" s="13" t="inlineStr">
+        <is>
+          <t>Backend + Database + DevOps</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="13" t="inlineStr">
+        <is>
+          <t>F-15</t>
+        </is>
+      </c>
+      <c r="B20" s="13" t="inlineStr">
+        <is>
+          <t>A popular cached page expires and hundreds of requests hit the database at once (cache stampede)</t>
+        </is>
+      </c>
+      <c r="C20" s="13" t="inlineStr">
+        <is>
+          <t>A sudden database spike can slow or stall the site exactly when traffic is highest</t>
+        </is>
+      </c>
+      <c r="D20" s="13" t="inlineStr">
+        <is>
+          <t>When one cache key expires under heavy load, every request rebuilds it simultaneously</t>
+        </is>
+      </c>
+      <c r="E20" s="13" t="inlineStr">
+        <is>
+          <t>Redis caching with an in-memory fallback layer</t>
+        </is>
+      </c>
+      <c r="F20" s="13" t="inlineStr">
+        <is>
+          <t>Stale-while-revalidate, request coalescing (single-flight) and jittered cache TTLs</t>
+        </is>
+      </c>
+      <c r="G20" s="17" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H20" s="13" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="13" t="inlineStr">
+        <is>
+          <t>F-16</t>
+        </is>
+      </c>
+      <c r="B21" s="13" t="inlineStr">
+        <is>
+          <t>Two staff or two guests update the same inventory at the same moment and the database deadlocks</t>
+        </is>
+      </c>
+      <c r="C21" s="13" t="inlineStr">
+        <is>
+          <t>Some requests fail with errors during the busiest booking moments</t>
+        </is>
+      </c>
+      <c r="D21" s="13" t="inlineStr">
+        <is>
+          <t>Concurrent writes to the same rows across many hotels can deadlock in Postgres</t>
+        </is>
+      </c>
+      <c r="E21" s="13" t="inlineStr">
+        <is>
+          <t>Row-level locks (SELECT FOR UPDATE) on inventory and redemption</t>
+        </is>
+      </c>
+      <c r="F21" s="13" t="inlineStr">
+        <is>
+          <t>Consistent lock ordering, retry-on-deadlock, and shorter transactions</t>
+        </is>
+      </c>
+      <c r="G21" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H21" s="13" t="inlineStr">
+        <is>
+          <t>Database</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="13" t="inlineStr">
+        <is>
+          <t>F-17</t>
+        </is>
+      </c>
+      <c r="B22" s="13" t="inlineStr">
+        <is>
+          <t>Email/WhatsApp providers throttle or reject our messages and guests stop getting confirmations</t>
+        </is>
+      </c>
+      <c r="C22" s="13" t="inlineStr">
+        <is>
+          <t>Guests miss confirmations and OTAs aren't synced — more support calls, double bookings</t>
+        </is>
+      </c>
+      <c r="D22" s="13" t="inlineStr">
+        <is>
+          <t>Brevo/Meta enforce sending limits and deliverability rules that tighten as volume grows</t>
+        </is>
+      </c>
+      <c r="E22" s="13" t="inlineStr">
+        <is>
+          <t>Senders are fail-safe (never crash the booking); per-hotel credentials</t>
+        </is>
+      </c>
+      <c r="F22" s="13" t="inlineStr">
+        <is>
+          <t>A queue with retry/back-off, deliverability monitoring, and provider fail-over</t>
+        </is>
+      </c>
+      <c r="G22" s="17" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H22" s="13" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="13" t="inlineStr">
+        <is>
+          <t>F-18</t>
+        </is>
+      </c>
+      <c r="B23" s="13" t="inlineStr">
+        <is>
+          <t>A hotel's WhatsApp/Meta token expires or a template is rejected and notifications silently stop</t>
+        </is>
+      </c>
+      <c r="C23" s="13" t="inlineStr">
+        <is>
+          <t>That hotel's WhatsApp confirmations quietly stop working</t>
+        </is>
+      </c>
+      <c r="D23" s="13" t="inlineStr">
+        <is>
+          <t>Meta tokens expire and message templates need approval; both change over time</t>
+        </is>
+      </c>
+      <c r="E23" s="13" t="inlineStr">
+        <is>
+          <t>Per-hotel config; webhook signature verification</t>
+        </is>
+      </c>
+      <c r="F23" s="13" t="inlineStr">
+        <is>
+          <t>Token-expiry alerts, template-status checks, and a clear 'reconnect' prompt</t>
+        </is>
+      </c>
+      <c r="G23" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H23" s="13" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="13" t="inlineStr">
+        <is>
+          <t>F-19</t>
+        </is>
+      </c>
+      <c r="B24" s="13" t="inlineStr">
+        <is>
+          <t>Google review/Business-Profile OAuth tokens expire and the review features silently stop</t>
+        </is>
+      </c>
+      <c r="C24" s="13" t="inlineStr">
+        <is>
+          <t>The reviews studio stops fetching or posting for that hotel</t>
+        </is>
+      </c>
+      <c r="D24" s="13" t="inlineStr">
+        <is>
+          <t>OAuth refresh tokens can be revoked or expire</t>
+        </is>
+      </c>
+      <c r="E24" s="13" t="inlineStr">
+        <is>
+          <t>Per-hotel OAuth tokens stored securely</t>
+        </is>
+      </c>
+      <c r="F24" s="13" t="inlineStr">
+        <is>
+          <t>Automatic token refresh, expiry alerts, and a guided reconnect flow</t>
+        </is>
+      </c>
+      <c r="G24" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H24" s="13" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="13" t="inlineStr">
+        <is>
+          <t>F-20</t>
+        </is>
+      </c>
+      <c r="B25" s="13" t="inlineStr">
+        <is>
+          <t>A Razorpay webhook is replayed or arrives out of order and a payment is processed twice</t>
+        </is>
+      </c>
+      <c r="C25" s="13" t="inlineStr">
+        <is>
+          <t>A guest could be double-charged or a booking double-confirmed</t>
+        </is>
+      </c>
+      <c r="D25" s="13" t="inlineStr">
+        <is>
+          <t>Webhooks can be retried, duplicated or delayed by the network</t>
+        </is>
+      </c>
+      <c r="E25" s="13" t="inlineStr">
+        <is>
+          <t>Idempotency keys; webhook signature verification; status guard on confirmed bookings</t>
+        </is>
+      </c>
+      <c r="F25" s="13" t="inlineStr">
+        <is>
+          <t>Event de-duplication by event id and an ordered, idempotent webhook processor</t>
+        </is>
+      </c>
+      <c r="G25" s="17" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H25" s="13" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="13" t="inlineStr">
+        <is>
+          <t>F-21</t>
+        </is>
+      </c>
+      <c r="B26" s="13" t="inlineStr">
+        <is>
+          <t>Hotels in different regions hit date/timezone bugs (check-in/out or reports off by a day)</t>
+        </is>
+      </c>
+      <c r="C26" s="13" t="inlineStr">
+        <is>
+          <t>Wrong nights charged, wrong availability, or reports that don't match the hotel's day</t>
+        </is>
+      </c>
+      <c r="D26" s="13" t="inlineStr">
+        <is>
+          <t>Dates are computed in multiple layers; timezones differ per hotel</t>
+        </is>
+      </c>
+      <c r="E26" s="13" t="inlineStr">
+        <is>
+          <t>Server-side price and date validation</t>
+        </is>
+      </c>
+      <c r="F26" s="13" t="inlineStr">
+        <is>
+          <t>A single, explicit timezone strategy per hotel and timezone tests</t>
+        </is>
+      </c>
+      <c r="G26" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H26" s="13" t="inlineStr">
+        <is>
+          <t>Backend + Frontend</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="13" t="inlineStr">
+        <is>
+          <t>F-22</t>
+        </is>
+      </c>
+      <c r="B27" s="13" t="inlineStr">
+        <is>
+          <t>Stored data (guest images, invoices, backups) grows unbounded as hotels and stays pile up</t>
+        </is>
+      </c>
+      <c r="C27" s="13" t="inlineStr">
+        <is>
+          <t>Storage costs climb and large objects slow pages and backups</t>
+        </is>
+      </c>
+      <c r="D27" s="13" t="inlineStr">
+        <is>
+          <t>Every booking and hotel adds images and documents that are never cleaned up</t>
+        </is>
+      </c>
+      <c r="E27" s="13" t="inlineStr">
+        <is>
+          <t>Randomized filenames; size caps on uploads</t>
+        </is>
+      </c>
+      <c r="F27" s="13" t="inlineStr">
+        <is>
+          <t>Object storage on a CDN, lifecycle/archival rules, and an image-processing pipeline</t>
+        </is>
+      </c>
+      <c r="G27" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H27" s="13" t="inlineStr">
+        <is>
+          <t>Database + DevOps</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="13" t="inlineStr">
+        <is>
+          <t>F-23</t>
+        </is>
+      </c>
+      <c r="B28" s="13" t="inlineStr">
+        <is>
+          <t>A bug loop or an attack floods the logs/monitoring and the observability bill explodes</t>
+        </is>
+      </c>
+      <c r="C28" s="13" t="inlineStr">
+        <is>
+          <t>Monitoring costs spike and real errors get buried in noise</t>
+        </is>
+      </c>
+      <c r="D28" s="13" t="inlineStr">
+        <is>
+          <t>High traffic plus an error loop can generate enormous log volume</t>
+        </is>
+      </c>
+      <c r="E28" s="13" t="inlineStr">
+        <is>
+          <t>Sentry sampling reduced in production; no PII in logs</t>
+        </is>
+      </c>
+      <c r="F28" s="13" t="inlineStr">
+        <is>
+          <t>Log rate-limiting, error de-duplication, and budget alerts on observability spend</t>
+        </is>
+      </c>
+      <c r="G28" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H28" s="13" t="inlineStr">
+        <is>
+          <t>Backend + DevOps</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="13" t="inlineStr">
+        <is>
+          <t>F-24</t>
+        </is>
+      </c>
+      <c r="B29" s="13" t="inlineStr">
+        <is>
+          <t>A new hotel onboards with a bad bulk import (rooms/rates/bookings) and pages break</t>
+        </is>
+      </c>
+      <c r="C29" s="13" t="inlineStr">
+        <is>
+          <t>The new hotel's dashboard or booking page errors out on day one</t>
+        </is>
+      </c>
+      <c r="D29" s="13" t="inlineStr">
+        <is>
+          <t>Imported data may have missing fields, wrong types or duplicates</t>
+        </is>
+      </c>
+      <c r="E29" s="13" t="inlineStr">
+        <is>
+          <t>Server-side validation on the main write paths</t>
+        </is>
+      </c>
+      <c r="F29" s="13" t="inlineStr">
+        <is>
+          <t>A validated import pipeline with a dry-run preview and clear error reporting</t>
+        </is>
+      </c>
+      <c r="G29" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H29" s="13" t="inlineStr">
+        <is>
+          <t>Backend + Frontend</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="13" t="inlineStr">
+        <is>
+          <t>F-25</t>
+        </is>
+      </c>
+      <c r="B30" s="13" t="inlineStr">
+        <is>
+          <t>An AI provider has an outage or deprecates a model and the chatbots/agents stop or misbehave</t>
+        </is>
+      </c>
+      <c r="C30" s="13" t="inlineStr">
+        <is>
+          <t>Guest and hotelier AI features go down or change behaviour suddenly</t>
+        </is>
+      </c>
+      <c r="D30" s="13" t="inlineStr">
+        <is>
+          <t>We depend on third-party LLMs whose availability and models change</t>
+        </is>
+      </c>
+      <c r="E30" s="13" t="inlineStr">
+        <is>
+          <t>Cheap model by default; per-hotel model selection; usage tracking</t>
+        </is>
+      </c>
+      <c r="F30" s="13" t="inlineStr">
+        <is>
+          <t>Multi-provider fail-over, model pinning, and a graceful 'AI unavailable' fallback</t>
+        </is>
+      </c>
+      <c r="G30" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H30" s="13" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="13" t="inlineStr">
+        <is>
+          <t>F-26</t>
+        </is>
+      </c>
+      <c r="B31" s="13" t="inlineStr">
+        <is>
+          <t>A guest exercises their DPDP/GDPR right to be forgotten and we must delete their data correctly</t>
+        </is>
+      </c>
+      <c r="C31" s="13" t="inlineStr">
+        <is>
+          <t>A mishandled deletion is a compliance violation; an over-broad one corrupts records</t>
+        </is>
+      </c>
+      <c r="D31" s="13" t="inlineStr">
+        <is>
+          <t>Privacy law requires verifiable deletion across many tables and many hotels</t>
+        </is>
+      </c>
+      <c r="E31" s="13" t="inlineStr">
+        <is>
+          <t>Per-hotel data isolation; encrypted PII</t>
+        </is>
+      </c>
+      <c r="F31" s="13" t="inlineStr">
+        <is>
+          <t>A documented data-deletion/anonymisation workflow and an audit record of each request</t>
+        </is>
+      </c>
+      <c r="G31" s="18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H31" s="13" t="inlineStr">
+        <is>
+          <t>Backend + Database</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="13" t="inlineStr">
+        <is>
+          <t>F-27</t>
+        </is>
+      </c>
+      <c r="B32" s="13" t="inlineStr">
+        <is>
+          <t>A vendor key leaks and must be rotated across all hotels without downtime</t>
+        </is>
+      </c>
+      <c r="C32" s="13" t="inlineStr">
+        <is>
+          <t>A compromised key must be replaced fast, for every affected hotel, with no outage</t>
+        </is>
+      </c>
+      <c r="D32" s="13" t="inlineStr">
+        <is>
+          <t>Keys can leak through logs, laptops or third parties; we hold many per hotel</t>
+        </is>
+      </c>
+      <c r="E32" s="13" t="inlineStr">
+        <is>
+          <t>All secrets encrypted in the Vault; never returned in plain text; masked in APIs</t>
+        </is>
+      </c>
+      <c r="F32" s="13" t="inlineStr">
+        <is>
+          <t>A documented key-rotation runbook and per-hotel re-key tooling</t>
+        </is>
+      </c>
+      <c r="G32" s="17" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H32" s="13" t="inlineStr">
+        <is>
+          <t>Backend + Tech Lead</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
+    <mergeCell ref="A18:H18"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
@@ -4689,7 +6258,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E42"/>
+  <dimension ref="A1:E50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4712,7 +6281,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -4780,7 +6348,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
@@ -4816,9 +6383,9 @@
           <t>Database Dev</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>Makes sure data comes OUT of the database smoothly — right indexes, fast queries, clean schema, reliable backups, per-hotel isolation. When data reaches GBs: partitioning and archiving so queries stay fast.</t>
+      <c r="C13" s="13" t="inlineStr">
+        <is>
+          <t>Makes sure data comes OUT of the database smoothly — right indexes, fast queries, clean schema, reliable backups, per-hotel isolation. When data reaches GBs: partitioning and archiving so queries stay fast. Builds to the Tech Lead's design and reports progress to him.</t>
         </is>
       </c>
     </row>
@@ -4833,9 +6400,9 @@
           <t>Backend Dev</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>Connects the backend APIs to the database properly — booking logic, payment processing, security checks. When data reaches GBs: sends it in CHUNKS (pagination, batching, caching) so the server never tries to load everything at once.</t>
+      <c r="C14" s="13" t="inlineStr">
+        <is>
+          <t>Connects the backend APIs to the database properly — booking logic, payment processing, security checks. When data reaches GBs: sends it in CHUNKS (pagination, batching, caching) so the server never tries to load everything at once. Builds to the Tech Lead's design and reports progress to him.</t>
         </is>
       </c>
     </row>
@@ -4850,16 +6417,16 @@
           <t>Frontend Dev</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>Connects the React + TypeScript frontend to the backend APIs and makes sure the data arrives and displays correctly — loading states, error handling, payment screens. When data reaches GBs: loads it smoothly on screen (paged lists, lazy loading) so pages stay fast for the hotelier and the guest.</t>
+      <c r="C15" s="13" t="inlineStr">
+        <is>
+          <t>Connects the React + TypeScript frontend to the backend APIs and makes sure the data arrives and displays correctly — loading states, error handling, payment screens. When data reaches GBs: loads it smoothly on screen (paged lists, lazy loading) so pages stay fast for the hotelier and the guest. Builds to the Tech Lead's design and reports progress to him.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="33" customHeight="1">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>4. Someone decides what gets built, in what order, and signs off</t>
+      <c r="A16" s="13" t="inlineStr">
+        <is>
+          <t>4. Someone decides WHAT to build, HOW to build it, reviews it, and signs off before release</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
@@ -4867,14 +6434,12 @@
           <t>Tech Lead</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>Decides what happens in the project — what each developer builds and when, reviews every change before release, and carries the overall responsibility for the software.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17"/>
-    <row r="18"/>
+      <c r="C16" s="13" t="inlineStr">
+        <is>
+          <t>TECH LEAD — the decision-maker and the final gate. Requirements from the product manager / stakeholders come to him; he designs the architecture, breaks it into tasks for each developer, reviews every change, and by his experience decides whether it is safe to ship to production. The developers below build to his direction and report to him. He is accountable for every software update, every bug and every crash.</t>
+        </is>
+      </c>
+    </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="8" t="inlineStr">
         <is>
@@ -4905,14 +6470,14 @@
           <t>Tech Lead</t>
         </is>
       </c>
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>Responsible for the whole software — decides what every developer works on, reviews everything, owns delivery.</t>
-        </is>
-      </c>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>Prioritised the fix order across 58 issues (money-related first); set the engineering rules and the review checklist the team now follows; set up the CI pipeline that tests every change.</t>
+      <c r="B21" s="13" t="inlineStr">
+        <is>
+          <t>The single person accountable for the whole software — every update, bug and crash. He decides what gets built, when and how it is coded, reviews and approves every change before it can reach production, and the developers execute his plan and report to him.</t>
+        </is>
+      </c>
+      <c r="C21" s="13" t="inlineStr">
+        <is>
+          <t>Turns feature requests from the product manager / stakeholders into an architecture and a set of tasks; assigns each task to the right developer; reviews ALL code and, by experience, decides what is safe to ship to production; owns the engineering rules, the review checklist and the CI/CD gate; carries responsibility when anything breaks. (In this project: set the fix order across 70+ issues money-first, wrote the rules the team follows, and stood up the test/CI gate.)</t>
         </is>
       </c>
     </row>
@@ -4922,9 +6487,9 @@
           <t>Backend Dev</t>
         </is>
       </c>
-      <c r="B22" s="4" t="inlineStr">
-        <is>
-          <t>Owns backend APIs and their connection to the database — payments, booking logic, security, performance.</t>
+      <c r="B22" s="13" t="inlineStr">
+        <is>
+          <t>Owns backend APIs and their connection to the database — payments, booking logic, security, performance. Builds what the Tech Lead designs — the 'what' and 'why' come from him; reports progress back to him.</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
@@ -4939,9 +6504,9 @@
           <t>Frontend Dev</t>
         </is>
       </c>
-      <c r="B23" s="4" t="inlineStr">
-        <is>
-          <t>Owns the React + TypeScript screens and their connection to backend APIs — correct data display, smooth experience.</t>
+      <c r="B23" s="13" t="inlineStr">
+        <is>
+          <t>Owns the React + TypeScript screens and their connection to backend APIs — correct data display, smooth experience. Builds the screens to the Tech Lead's design and direction; reports to him.</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
@@ -4956,9 +6521,9 @@
           <t>Database Dev</t>
         </is>
       </c>
-      <c r="B24" s="4" t="inlineStr">
-        <is>
-          <t>Owns the database — speed, schema, backups, and the guarantee that data flows out smoothly at any size.</t>
+      <c r="B24" s="13" t="inlineStr">
+        <is>
+          <t>Owns the database — speed, schema, backups, and the guarantee that data flows out smoothly at any size. Implements the data design the Tech Lead approves; reports to him.</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
@@ -4967,8 +6532,6 @@
         </is>
       </c>
     </row>
-    <row r="25"/>
-    <row r="26"/>
     <row r="27" ht="30" customHeight="1">
       <c r="A27" s="8" t="inlineStr">
         <is>
@@ -5075,18 +6638,17 @@
           <t>Tech Lead</t>
         </is>
       </c>
-      <c r="C32" s="4" t="inlineStr">
-        <is>
-          <t>Direction and review from day one keeps all the above work consistent. Can be a hands-on senior developer.</t>
-        </is>
-      </c>
-      <c r="D32" s="4" t="inlineStr">
-        <is>
-          <t>Technical roadmap; review process; assigning and supervising the work above.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33"/>
+      <c r="C32" s="13" t="inlineStr">
+        <is>
+          <t>Direction and review from day one. He is the owner of quality and safety — nothing reaches production without his approval — so the work of every other hire stays consistent and safe. Should be a senior, hands-on engineer who can also code.</t>
+        </is>
+      </c>
+      <c r="D32" s="13" t="inlineStr">
+        <is>
+          <t>Set the technical roadmap and architecture; define the code-review and release process; assign and supervise all developer tasks; own incident response.</t>
+        </is>
+      </c>
+    </row>
     <row r="34">
       <c r="A34" s="8" t="inlineStr">
         <is>
@@ -5104,7 +6666,6 @@
       <c r="C35" s="21" t="n"/>
       <c r="D35" s="22" t="n"/>
     </row>
-    <row r="36"/>
     <row r="37">
       <c r="A37" s="8" t="inlineStr">
         <is>
@@ -5208,27 +6769,137 @@
       </c>
       <c r="B42" s="13" t="inlineStr">
         <is>
-          <t>One person reviewing everything; no second pair of eyes on security or money code.</t>
+          <t>No single owner of quality; code reaching production with no experienced second pair of eyes; no clear accountability when something breaks.</t>
         </is>
       </c>
       <c r="C42" s="13" t="inlineStr">
         <is>
-          <t>A human review gate on every change — the single most effective catch for the silent bugs in Sheet 8 — plus a clear roadmap.</t>
+          <t>One accountable owner for the entire software — every update, bug and crash. He designs each feature, assigns the tasks, and personally approves what ships, so quality and safety do not depend on luck.</t>
         </is>
       </c>
       <c r="D42" s="13" t="inlineStr">
         <is>
-          <t>Risk concentrates on one person; quality depends on no one ever having an off day.</t>
+          <t>Developers build in different directions, reviews get skipped, and a single silent bug (see the Silent Bugs sheet) can reach production unchecked.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="8" t="inlineStr">
+        <is>
+          <t>HOW THE TEAM WORKS — THE CHAIN OF COMMAND</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="22" customHeight="1">
+      <c r="A45" s="10" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="B45" s="10" t="inlineStr">
+        <is>
+          <t>Who</t>
+        </is>
+      </c>
+      <c r="C45" s="10" t="inlineStr">
+        <is>
+          <t>What happens</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B46" s="14" t="inlineStr">
+        <is>
+          <t>Product Manager / Stakeholders</t>
+        </is>
+      </c>
+      <c r="C46" s="13" t="inlineStr">
+        <is>
+          <t>Decide WHAT the business needs — new features, priorities, customer requests — and hand them to the Tech Lead.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="14" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B47" s="14" t="inlineStr">
+        <is>
+          <t>Tech Lead</t>
+        </is>
+      </c>
+      <c r="C47" s="13" t="inlineStr">
+        <is>
+          <t>Architects the design and the approach, decides HOW and WHEN it is built, and breaks it into specific tasks for each developer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="14" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B48" s="14" t="inlineStr">
+        <is>
+          <t>Backend / Frontend / Database Developers</t>
+        </is>
+      </c>
+      <c r="C48" s="13" t="inlineStr">
+        <is>
+          <t>Build their assigned tasks to the Tech Lead's design. They focus on writing the code; the 'what' and 'why' come from the Tech Lead.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="14" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B49" s="14" t="inlineStr">
+        <is>
+          <t>Tech Lead (review gate)</t>
+        </is>
+      </c>
+      <c r="C49" s="13" t="inlineStr">
+        <is>
+          <t>Reviews every change. By his experience he decides whether it is safe to go to production — nothing ships without his approval.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="14" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B50" s="14" t="inlineStr">
+        <is>
+          <t>Tech Lead (accountability)</t>
+        </is>
+      </c>
+      <c r="C50" s="13" t="inlineStr">
+        <is>
+          <t>Owns the result: any update, bug or crash is his responsibility. The developers report to him; he reports to the business.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
     <mergeCell ref="A37:D37"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A34:D34"/>
     <mergeCell ref="A35:D35"/>
     <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A44:E44"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5263,6 +6934,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -5273,7 +6945,7 @@
     <row r="5" ht="32" customHeight="1">
       <c r="A5" s="15" t="inlineStr">
         <is>
-          <t>Owns the APIs and their link to the database — payments, booking logic, security, speed and cost. This is where 'API optimisation' and most server-crash prevention live.</t>
+          <t>Owns the APIs and their link to the database — payments, booking logic, security, speed and cost. This is where 'API optimisation' and most server-crash prevention live. Works to the Tech Lead's design and direction, and reports back to him.</t>
         </is>
       </c>
       <c r="B5" s="21" t="n"/>
@@ -5434,6 +7106,7 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
         <is>
@@ -5444,7 +7117,7 @@
     <row r="15" ht="32" customHeight="1">
       <c r="A15" s="15" t="inlineStr">
         <is>
-          <t>Owns the React + TypeScript screens and their link to the backend APIs. This is real engineering — correct data, fast loads, no blank screens — not visual design.</t>
+          <t>Owns the React + TypeScript screens and their link to the backend APIs. This is real engineering — correct data, fast loads, no blank screens — not visual design. Works to the Tech Lead's design and direction, and reports back to him.</t>
         </is>
       </c>
       <c r="B15" s="21" t="n"/>
@@ -5583,6 +7256,7 @@
         </is>
       </c>
     </row>
+    <row r="22"/>
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
         <is>
@@ -5593,7 +7267,7 @@
     <row r="24" ht="32" customHeight="1">
       <c r="A24" s="15" t="inlineStr">
         <is>
-          <t>Owns the data layer — speed, schema, backups and the guarantee that data flows out smoothly at ANY size. Becomes essential as data approaches GB scale; can start part-time.</t>
+          <t>Owns the data layer — speed, schema, backups and the guarantee that data flows out smoothly at ANY size. Becomes essential as data approaches GB scale; can start part-time. Works to the Tech Lead's design and direction, and reports back to him.</t>
         </is>
       </c>
       <c r="B24" s="21" t="n"/>
@@ -5754,6 +7428,7 @@
         </is>
       </c>
     </row>
+    <row r="32"/>
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
         <is>
@@ -5764,7 +7439,7 @@
     <row r="34" ht="32" customHeight="1">
       <c r="A34" s="15" t="inlineStr">
         <is>
-          <t>Responsible for the whole software — decides what each developer builds and when, reviews everything before release, and owns delivery and security posture.</t>
+          <t>Accountable for the WHOLE software — every update, bug and crash. He converts product/stakeholder requirements into an architecture and tasks, assigns them to the developers, reviews every change, and decides what is safe to ship to production. The developers execute his direction and report to him.</t>
         </is>
       </c>
       <c r="B34" s="21" t="n"/>
@@ -5928,7 +7603,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="10" t="inlineStr">
         <is>
@@ -6226,7 +7900,6 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
docs: polish role plan (frontend=TS engineering, not design) + closing note
- Sheet 7 rebuilt with correct framing: Frontend writes TypeScript that calls
  the Backend APIs; Backend APIs talk to the Database. Explicitly engineering,
  not visual design. Richer day-to-day detail for every role.
- Sheet 5: realistic closing note — nothing is permanent (updates, competitor
  features, third-party API changes, server overload are unpredictable), so a
  team is needed to resolve issues before they become high-priority.

https://claude.ai/code/session_01Jfp6dFcb8aisQfoK5brnT1
</commit_message>
<xml_diff>
--- a/docs/CEO_Report_Staybooker_Jun2026.xlsx
+++ b/docs/CEO_Report_Staybooker_Jun2026.xlsx
@@ -647,7 +647,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="10" t="inlineStr">
         <is>
@@ -776,7 +775,6 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
     <row r="16">
       <c r="A16" s="11" t="inlineStr">
         <is>
@@ -3151,6 +3149,12 @@
           <t>EARLIER FOUNDATIONAL FIXES (May – early June 2026) — security, crashes and correctness fixed before the June audit</t>
         </is>
       </c>
+      <c r="B63" s="21" t="n"/>
+      <c r="C63" s="21" t="n"/>
+      <c r="D63" s="21" t="n"/>
+      <c r="E63" s="21" t="n"/>
+      <c r="F63" s="21" t="n"/>
+      <c r="G63" s="22" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="13" t="inlineStr">
@@ -4416,6 +4420,10 @@
           <t>EARLIER PLATFORM FEATURES (built across May – early June 2026)</t>
         </is>
       </c>
+      <c r="B28" s="21" t="n"/>
+      <c r="C28" s="21" t="n"/>
+      <c r="D28" s="21" t="n"/>
+      <c r="E28" s="22" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="13" t="n">
@@ -4807,7 +4815,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="26" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -5032,7 +5039,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H32"/>
+  <dimension ref="A1:H41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -5653,6 +5660,13 @@
           <t>MORE SCENARIOS AS WE SCALE — many hotels and their guests all share the same servers</t>
         </is>
       </c>
+      <c r="B18" s="21" t="n"/>
+      <c r="C18" s="21" t="n"/>
+      <c r="D18" s="21" t="n"/>
+      <c r="E18" s="21" t="n"/>
+      <c r="F18" s="21" t="n"/>
+      <c r="G18" s="21" t="n"/>
+      <c r="H18" s="22" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="13" t="inlineStr">
@@ -6242,11 +6256,75 @@
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" s="8" t="inlineStr">
+        <is>
+          <t>A REALISTIC CLOSING NOTE — WHY THIS WORK NEVER FULLY 'ENDS' (AND WHY A TEAM IS NEEDED)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="42" customHeight="1">
+      <c r="A35" s="11" t="inlineStr">
+        <is>
+          <t>In software development, nothing is a permanent solution. The product is healthy today, but it lives in a moving world:</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="30" customHeight="1">
+      <c r="A36" s="12" t="inlineStr">
+        <is>
+          <t>•  New updates will keep coming — and any update can itself arrive with new bugs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="30" customHeight="1">
+      <c r="A37" s="12" t="inlineStr">
+        <is>
+          <t>•  New features must keep being added to Staybooker to compete — as competitors release features in their software, we have to as well, and every new feature is new surface area where issues can appear.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="30" customHeight="1">
+      <c r="A38" s="12" t="inlineStr">
+        <is>
+          <t>•  Third-party APIs change — payment gateways like Razorpay / JioPay update their APIs; if our system does not capture and adapt to those changes in time, errors or bugs can appear.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="30" customHeight="1">
+      <c r="A39" s="12" t="inlineStr">
+        <is>
+          <t>•  Infrastructure can be strained — our cloud host (Railway) can be overloaded during traffic spikes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="30" customHeight="1">
+      <c r="A40" s="12" t="inlineStr">
+        <is>
+          <t>•  Real usage is unpredictable — the scenarios in this sheet are informed PREDICTIONS, not certainties. For example: even with 10 hotels, each taking ~15-20 bookings a day (~200 bookings daily), plus 50-100 visitors/guests taking actions on the site at any moment, we cannot predict every combination of what they will do.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="42" customHeight="1">
+      <c r="A41" s="11" t="inlineStr">
+        <is>
+          <t>So when something does break, there must be a team in place to catch and resolve it BEFORE it grows into a high-priority, customer-facing incident. That is the real reason for the hiring in Sheet 6 — not because the product is broken, but because keeping it healthy is continuous work.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="11">
     <mergeCell ref="A18:H18"/>
+    <mergeCell ref="A39:H39"/>
+    <mergeCell ref="A35:H35"/>
+    <mergeCell ref="A38:H38"/>
     <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A40:H40"/>
+    <mergeCell ref="A41:H41"/>
+    <mergeCell ref="A36:H36"/>
     <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A37:H37"/>
+    <mergeCell ref="A34:H34"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6911,11 +6989,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D39"/>
+  <dimension ref="A1:D38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
     <col width="46" customWidth="1" min="3" max="3"/>
     <col width="40" customWidth="1" min="4" max="4"/>
   </cols>
@@ -6927,32 +7005,35 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="28" customHeight="1">
+    <row r="2" ht="26" customHeight="1">
       <c r="A2" s="9" t="inlineStr">
         <is>
-          <t>The concrete, ongoing work behind 'why a team'. This answers, in plain language: how do we keep the APIs fast (optimisation), and what is the constant bug-hunting that keeps the server stable as we grow?</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
+          <t>The concrete, ongoing engineering behind 'why a team'. None of these roles is graphic/visual design — this is software engineering.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="42" customHeight="1">
+      <c r="A3" s="23" t="inlineStr">
+        <is>
+          <t>HOW THE PIECES CONNECT:  The Frontend (TypeScript / React) calls the Backend APIs  →  the Backend APIs talk to the Database. Each developer owns one link in that chain and writes the CODE for it. The Tech Lead decides what is built and reviews it all.</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>BACKEND DEVELOPER</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="32" customHeight="1">
+          <t>FRONTEND DEVELOPER</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="34" customHeight="1">
       <c r="A5" s="15" t="inlineStr">
         <is>
-          <t>Owns the APIs and their link to the database — payments, booking logic, security, speed and cost. This is where 'API optimisation' and most server-crash prevention live. Works to the Tech Lead's design and direction, and reports back to him.</t>
-        </is>
-      </c>
-      <c r="B5" s="21" t="n"/>
-      <c r="C5" s="21" t="n"/>
-      <c r="D5" s="22" t="n"/>
-    </row>
-    <row r="6" ht="30" customHeight="1">
+          <t>Writes the TypeScript / React code that runs in the guest's and hotelier's browser and TALKS TO THE BACKEND APIs. This is engineering — typed code, data handling, performance — not visual design. Builds to the Tech Lead's design and reports to him.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="28" customHeight="1">
       <c r="A6" s="10" t="inlineStr">
         <is>
           <t>Ongoing job</t>
@@ -6960,7 +7041,7 @@
       </c>
       <c r="B6" s="10" t="inlineStr">
         <is>
-          <t>What the work actually is</t>
+          <t>What the work actually is (day to day)</t>
         </is>
       </c>
       <c r="C6" s="10" t="inlineStr">
@@ -6977,322 +7058,358 @@
     <row r="7">
       <c r="A7" s="14" t="inlineStr">
         <is>
-          <t>API optimisation</t>
+          <t>Call the backend APIs (TypeScript)</t>
         </is>
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>Measure each endpoint's response time, cache hot reads in Redis, replace many small queries with one batched query (kill N+1), enforce pagination caps, and push slow work (emails, sync) into background tasks.</t>
+          <t>Write the typed TypeScript code that calls each backend endpoint: send the correct request, read the response, and keep the frontend's data types matching the backend's contract so data never arrives in the wrong shape.</t>
         </is>
       </c>
       <c r="C7" s="13" t="inlineStr">
         <is>
-          <t>Fast pages keep guests booking and keep the server bill low — speed is revenue.</t>
+          <t>The screens show exactly the data the backend returns — bookings, rates, availability — correctly and reliably.</t>
         </is>
       </c>
       <c r="D7" s="13" t="inlineStr">
         <is>
-          <t>Timeouts, slow dashboards, and a database overloaded by repeated heavy queries.</t>
+          <t>Broken pages, wrong data on screen, and type mismatches that crash a component.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>Continuous bug-hunting</t>
+          <t>Manage state &amp; data flow</t>
         </is>
       </c>
       <c r="B8" s="13" t="inlineStr">
         <is>
-          <t>Every new endpoint is read for the quiet failure modes: swallowed exceptions, wrong query cardinality, missing limits, fail-open checks. (See Sheet 8 for the catalogue.)</t>
+          <t>Decide how fetched data moves through the app — caching with React Query, re-fetching on focus, and invalidating the cache after a booking/edit so the screen updates.</t>
         </is>
       </c>
       <c r="C8" s="13" t="inlineStr">
         <is>
-          <t>These are the bugs that don't show an error but quietly crash or stall the server.</t>
+          <t>Hoteliers and guests always see fresh, correct data without manual refreshes.</t>
         </is>
       </c>
       <c r="D8" s="13" t="inlineStr">
         <is>
-          <t>Silent outages and 'the site is slow / down' incidents that nobody can explain.</t>
+          <t>Stale screens (e.g. a sold room still showing as available).</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="14" t="inlineStr">
         <is>
-          <t>Payment integrity</t>
+          <t>Loading, error &amp; retry handling</t>
         </is>
       </c>
       <c r="B9" s="13" t="inlineStr">
         <is>
-          <t>Build and run the auto-refund flow and a daily reconciliation job that matches the Razorpay ledger against our bookings.</t>
+          <t>Give every screen a proper 'loading', 'failed' (with a Retry button) and 'empty' state, and tolerate slow or partial API responses.</t>
         </is>
       </c>
       <c r="C9" s="13" t="inlineStr">
         <is>
-          <t>Guest money is never stuck; disputes and chargebacks drop.</t>
+          <t>A slow network or a failed API call never leaves the guest staring at a blank white page mid-booking.</t>
         </is>
       </c>
       <c r="D9" s="13" t="inlineStr">
         <is>
-          <t>Manual refunds, angry guests, and Razorpay disputes.</t>
+          <t>Blank screens and stuck buttons that make guests abandon a booking.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>Security on every route</t>
+          <t>Performance engineering</t>
         </is>
       </c>
       <c r="B10" s="13" t="inlineStr">
         <is>
-          <t>Add the role gate and tenant (hotel_id) filter to every new endpoint, and verify amounts/ids server-side.</t>
+          <t>Code-splitting, lazy-loading, bundle-size trimming, image optimisation and virtual scrolling for big lists; measure and fix slow renders (Core Web Vitals). (Build/runtime engineering, not graphic design.)</t>
         </is>
       </c>
       <c r="C10" s="13" t="inlineStr">
         <is>
-          <t>Each new feature ships without opening a data-isolation or tampering hole.</t>
+          <t>Pages load in ~1-2 seconds even for large hotels — and faster pages convert more guests.</t>
         </is>
       </c>
       <c r="D10" s="13" t="inlineStr">
         <is>
-          <t>Cross-hotel data leaks and price/role tampering.</t>
+          <t>Slow pages that lose bookings, and browsers freezing on thousands of rows.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="14" t="inlineStr">
         <is>
-          <t>Cost control</t>
+          <t>Concurrency &amp; input safety</t>
         </is>
       </c>
       <c r="B11" s="13" t="inlineStr">
         <is>
-          <t>Cap LLM tokens, enforce per-hotel AI quotas, bound DB rows returned and background work.</t>
+          <t>Disable buttons on submit, debounce rapid clicks, and validate inputs in the browser before they reach the API.</t>
         </is>
       </c>
       <c r="C11" s="13" t="inlineStr">
         <is>
-          <t>AI and infra costs stay predictable as usage grows.</t>
+          <t>No accidental duplicate bookings or double payments on slow networks.</t>
         </is>
       </c>
       <c r="D11" s="13" t="inlineStr">
         <is>
-          <t>A surprise lakhs-level AI bill from a single abusive script.</t>
+          <t>Two bookings / two charges from one impatient double-click.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>Observability</t>
+          <t>Real-time UI</t>
         </is>
       </c>
       <c r="B12" s="13" t="inlineStr">
         <is>
-          <t>Structured logs (no PII), error-rate alerts, and dashboards so problems are seen before customers complain.</t>
+          <t>Wire the live WebSocket / SSE streams from the backend into the screens so a new booking appears instantly.</t>
         </is>
       </c>
       <c r="C12" s="13" t="inlineStr">
         <is>
-          <t>We hear about issues from our alerts, not from an angry hotelier.</t>
+          <t>The product feels live; staff react to bookings without refreshing.</t>
         </is>
       </c>
       <c r="D12" s="13" t="inlineStr">
         <is>
-          <t>Problems festering silently until they become outages.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13"/>
-    <row r="14">
-      <c r="A14" s="8" t="inlineStr">
-        <is>
-          <t>FRONTEND DEVELOPER</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="32" customHeight="1">
-      <c r="A15" s="15" t="inlineStr">
-        <is>
-          <t>Owns the React + TypeScript screens and their link to the backend APIs. This is real engineering — correct data, fast loads, no blank screens — not visual design. Works to the Tech Lead's design and direction, and reports back to him.</t>
-        </is>
-      </c>
-      <c r="B15" s="21" t="n"/>
-      <c r="C15" s="21" t="n"/>
-      <c r="D15" s="22" t="n"/>
-    </row>
-    <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="10" t="inlineStr">
+          <t>Missed or stale information on the dashboard.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>BACKEND DEVELOPER</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="34" customHeight="1">
+      <c r="A14" s="15" t="inlineStr">
+        <is>
+          <t>Writes the API code that the frontend calls, and that in turn TALKS TO THE DATABASE. Owns booking logic, payments, security, speed and cost. Builds to the Tech Lead's design and reports to him.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="28" customHeight="1">
+      <c r="A15" s="10" t="inlineStr">
         <is>
           <t>Ongoing job</t>
         </is>
       </c>
-      <c r="B16" s="10" t="inlineStr">
-        <is>
-          <t>What the work actually is</t>
-        </is>
-      </c>
-      <c r="C16" s="10" t="inlineStr">
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>What the work actually is (day to day)</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="inlineStr">
         <is>
           <t>Why it matters to the business</t>
         </is>
       </c>
-      <c r="D16" s="10" t="inlineStr">
+      <c r="D15" s="10" t="inlineStr">
         <is>
           <t>What it prevents</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="14" t="inlineStr">
+        <is>
+          <t>Design &amp; build the APIs</t>
+        </is>
+      </c>
+      <c r="B16" s="13" t="inlineStr">
+        <is>
+          <t>Build the endpoints the frontend calls: validate the request, run the business rules, and return the correct JSON shape (the 'contract' the frontend depends on).</t>
+        </is>
+      </c>
+      <c r="C16" s="13" t="inlineStr">
+        <is>
+          <t>Every screen has a reliable, correct API behind it.</t>
+        </is>
+      </c>
+      <c r="D16" s="13" t="inlineStr">
+        <is>
+          <t>Broken or inconsistent responses that break the frontend.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="14" t="inlineStr">
         <is>
-          <t>API integration hardening</t>
+          <t>Talk to the database correctly</t>
         </is>
       </c>
       <c r="B17" s="13" t="inlineStr">
         <is>
-          <t>Every page gets a loading state, an error state and a Retry — and tolerates slow or partial data without breaking.</t>
+          <t>Write the queries each API uses to read/write data — always scoped to the caller's hotel, batched (no N+1), and paginated.</t>
         </is>
       </c>
       <c r="C17" s="13" t="inlineStr">
         <is>
-          <t>A network blip never shows the guest a blank page; the booking continues.</t>
+          <t>Data is correct, isolated per hotel, and fast to fetch.</t>
         </is>
       </c>
       <c r="D17" s="13" t="inlineStr">
         <is>
-          <t>White screens mid-booking → closed tabs → lost bookings.</t>
+          <t>Cross-tenant leaks, slow queries, and out-of-memory crashes on big hotels.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="14" t="inlineStr">
         <is>
-          <t>Page-speed optimisation</t>
+          <t>API optimisation</t>
         </is>
       </c>
       <c r="B18" s="13" t="inlineStr">
         <is>
-          <t>Code-splitting, lazy loading, image optimisation, and trimming the JavaScript bundle; monitor Core Web Vitals.</t>
+          <t>Measure each endpoint's response time, cache hot reads in Redis, and push slow work (emails, channel sync) into background jobs.</t>
         </is>
       </c>
       <c r="C18" s="13" t="inlineStr">
         <is>
-          <t>Every extra second of load time cuts conversion ~7% — speed is direct revenue.</t>
+          <t>Responses stay in milliseconds and the server bill stays low — speed is revenue.</t>
         </is>
       </c>
       <c r="D18" s="13" t="inlineStr">
         <is>
-          <t>Guests bouncing off a slow page before they ever see a room.</t>
+          <t>Timeouts and a database overloaded by repeated heavy queries.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="14" t="inlineStr">
         <is>
-          <t>Large-data rendering</t>
+          <t>Payments &amp; third-party integrations</t>
         </is>
       </c>
       <c r="B19" s="13" t="inlineStr">
         <is>
-          <t>Virtual scrolling and paged lists so a hotel with thousands of bookings still renders instantly.</t>
+          <t>Razorpay / JioPay, WhatsApp, email: verify signatures, handle webhooks and retries, and ADAPT when a provider changes its API.</t>
         </is>
       </c>
       <c r="C19" s="13" t="inlineStr">
         <is>
-          <t>The dashboard stays smooth even for the biggest, most valuable hotels.</t>
+          <t>Money is handled correctly and integrations keep working as vendors change.</t>
         </is>
       </c>
       <c r="D19" s="13" t="inlineStr">
         <is>
-          <t>The browser freezing while it tries to draw thousands of rows.</t>
+          <t>Stuck payments, double charges, and notifications silently breaking.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="14" t="inlineStr">
         <is>
-          <t>Double-submit &amp; concurrency guards</t>
+          <t>Security &amp; continuous bug-hunting</t>
         </is>
       </c>
       <c r="B20" s="13" t="inlineStr">
         <is>
-          <t>Disable buttons on submit, add idempotent retries, warn on conflicting edits across tabs.</t>
+          <t>Add the role gate + tenant filter + server-side amount/id verification to every route; read every change for the silent failure modes in Sheet 8.</t>
         </is>
       </c>
       <c r="C20" s="13" t="inlineStr">
         <is>
-          <t>No accidental duplicate bookings or double payments on slow networks.</t>
+          <t>New features ship without opening data-isolation, tampering or crash holes.</t>
         </is>
       </c>
       <c r="D20" s="13" t="inlineStr">
         <is>
-          <t>Two bookings / two charges from one impatient double-click.</t>
+          <t>Breaches, price/role tampering, and silent server crashes.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="14" t="inlineStr">
         <is>
-          <t>Real-time UI</t>
+          <t>Cost control &amp; observability</t>
         </is>
       </c>
       <c r="B21" s="13" t="inlineStr">
         <is>
-          <t>Wire dashboards to the live WebSocket/SSE updates so new bookings appear without a refresh.</t>
+          <t>Cap LLM tokens, enforce per-hotel quotas, bound rows/work; emit structured logs (no PII) and error alerts.</t>
         </is>
       </c>
       <c r="C21" s="13" t="inlineStr">
         <is>
-          <t>The product feels modern and 'alive'; staff react instantly.</t>
+          <t>Predictable AI/infra cost and problems seen before customers complain.</t>
         </is>
       </c>
       <c r="D21" s="13" t="inlineStr">
         <is>
-          <t>Stale screens and missed bookings.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22"/>
-    <row r="23">
-      <c r="A23" s="8" t="inlineStr">
+          <t>Surprise bills and outages discovered only via angry hoteliers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
         <is>
           <t>DATABASE DEVELOPER</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="32" customHeight="1">
-      <c r="A24" s="15" t="inlineStr">
-        <is>
-          <t>Owns the data layer — speed, schema, backups and the guarantee that data flows out smoothly at ANY size. Becomes essential as data approaches GB scale; can start part-time. Works to the Tech Lead's design and direction, and reports back to him.</t>
-        </is>
-      </c>
-      <c r="B24" s="21" t="n"/>
-      <c r="C24" s="21" t="n"/>
-      <c r="D24" s="22" t="n"/>
-    </row>
-    <row r="25" ht="30" customHeight="1">
-      <c r="A25" s="10" t="inlineStr">
+    <row r="23" ht="34" customHeight="1">
+      <c r="A23" s="15" t="inlineStr">
+        <is>
+          <t>Owns the database the backend talks to — speed, schema, safety and the guarantee that data flows out smoothly at any size. Implements the data design the Tech Lead approves and reports to him.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="28" customHeight="1">
+      <c r="A24" s="10" t="inlineStr">
         <is>
           <t>Ongoing job</t>
         </is>
       </c>
-      <c r="B25" s="10" t="inlineStr">
-        <is>
-          <t>What the work actually is</t>
-        </is>
-      </c>
-      <c r="C25" s="10" t="inlineStr">
+      <c r="B24" s="10" t="inlineStr">
+        <is>
+          <t>What the work actually is (day to day)</t>
+        </is>
+      </c>
+      <c r="C24" s="10" t="inlineStr">
         <is>
           <t>Why it matters to the business</t>
         </is>
       </c>
-      <c r="D25" s="10" t="inlineStr">
+      <c r="D24" s="10" t="inlineStr">
         <is>
           <t>What it prevents</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="14" t="inlineStr">
+        <is>
+          <t>Schema &amp; migrations</t>
+        </is>
+      </c>
+      <c r="B25" s="13" t="inlineStr">
+        <is>
+          <t>Design the tables and run every schema/index change through one safe, repeatable process (Alembic) instead of ad-hoc startup scripts.</t>
+        </is>
+      </c>
+      <c r="C25" s="13" t="inlineStr">
+        <is>
+          <t>Production never silently misses an index or a column.</t>
+        </is>
+      </c>
+      <c r="D25" s="13" t="inlineStr">
+        <is>
+          <t>Half-applied schemas and 'works locally, crashes in production' bugs.</t>
         </is>
       </c>
     </row>
@@ -7304,7 +7421,7 @@
       </c>
       <c r="B26" s="13" t="inlineStr">
         <is>
-          <t>Add and tune indexes on the hottest columns (hotel_id, dates, status); read query plans and fix slow ones.</t>
+          <t>Add and tune indexes on the hottest columns (hotel_id, dates, status); read query plans and fix the slow ones.</t>
         </is>
       </c>
       <c r="C26" s="13" t="inlineStr">
@@ -7331,242 +7448,239 @@
       </c>
       <c r="C27" s="13" t="inlineStr">
         <is>
-          <t>Day-to-day queries only touch recent, small data — so they stay fast.</t>
+          <t>Day-to-day queries only touch small, recent data — so they stay fast.</t>
         </is>
       </c>
       <c r="D27" s="13" t="inlineStr">
         <is>
-          <t>Dashboards taking 15–20s to open once a hotel has years of data.</t>
+          <t>Dashboards taking 15-20s to open once a hotel has years of data.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="14" t="inlineStr">
         <is>
-          <t>Migration discipline</t>
+          <t>Connection pooling &amp; capacity</t>
         </is>
       </c>
       <c r="B28" s="13" t="inlineStr">
         <is>
-          <t>Introduce Alembic so schema and index changes deploy in a controlled, repeatable way.</t>
+          <t>Add a pooler (PgBouncer) and tune pool-size x workers x replicas against the Supabase limit; plan capacity for more hotels.</t>
         </is>
       </c>
       <c r="C28" s="13" t="inlineStr">
         <is>
-          <t>Production never silently misses an index or a schema change.</t>
+          <t>50-100 hotels can onboard without the database running out of connections.</t>
         </is>
       </c>
       <c r="D28" s="13" t="inlineStr">
         <is>
-          <t>Indexes present in dev but missing in production → mystery slowness.</t>
+          <t>All tenants slowing down at once when connections run out.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="14" t="inlineStr">
         <is>
-          <t>Connection pooling</t>
+          <t>Backups &amp; restore drills</t>
         </is>
       </c>
       <c r="B29" s="13" t="inlineStr">
         <is>
-          <t>Add a pooler (PgBouncer) and tune pool size × workers × replicas against the Supabase limit.</t>
+          <t>Run real restore drills, set up point-in-time recovery, and write a disaster-recovery runbook.</t>
         </is>
       </c>
       <c r="C29" s="13" t="inlineStr">
         <is>
-          <t>50–100 hotels can onboard without the database running out of connections.</t>
+          <t>Backups are proven to work before we ever need them.</t>
         </is>
       </c>
       <c r="D29" s="13" t="inlineStr">
         <is>
-          <t>All tenants slowing down at once when connections run out.</t>
+          <t>Discovering a backup is unusable on the worst possible day.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="14" t="inlineStr">
         <is>
-          <t>Backups &amp; restore drills</t>
+          <t>Isolation on every change</t>
         </is>
       </c>
       <c r="B30" s="13" t="inlineStr">
         <is>
-          <t>Run real restore drills, set up point-in-time recovery, write a disaster-recovery runbook.</t>
+          <t>Review every new table for Row Level Security and per-hotel isolation.</t>
         </is>
       </c>
       <c r="C30" s="13" t="inlineStr">
         <is>
-          <t>Backups are proven to actually work before we ever need them.</t>
+          <t>The database itself keeps refusing to mix one hotel's data with another's.</t>
         </is>
       </c>
       <c r="D30" s="13" t="inlineStr">
         <is>
-          <t>Discovering a backup is unusable on the worst possible day.</t>
+          <t>A schema change quietly opening a cross-tenant leak.</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="14" t="inlineStr">
-        <is>
-          <t>Isolation on schema changes</t>
-        </is>
-      </c>
-      <c r="B31" s="13" t="inlineStr">
-        <is>
-          <t>Review every new table for Row Level Security and per-hotel isolation.</t>
-        </is>
-      </c>
-      <c r="C31" s="13" t="inlineStr">
-        <is>
-          <t>The database itself keeps refusing to mix one hotel's data with another's.</t>
-        </is>
-      </c>
-      <c r="D31" s="13" t="inlineStr">
-        <is>
-          <t>A schema change quietly opening a cross-tenant leak.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32"/>
-    <row r="33">
-      <c r="A33" s="8" t="inlineStr">
+      <c r="A31" s="8" t="inlineStr">
         <is>
           <t>TECH LEAD</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="32" customHeight="1">
-      <c r="A34" s="15" t="inlineStr">
-        <is>
-          <t>Accountable for the WHOLE software — every update, bug and crash. He converts product/stakeholder requirements into an architecture and tasks, assigns them to the developers, reviews every change, and decides what is safe to ship to production. The developers execute his direction and report to him.</t>
-        </is>
-      </c>
-      <c r="B34" s="21" t="n"/>
-      <c r="C34" s="21" t="n"/>
-      <c r="D34" s="22" t="n"/>
-    </row>
-    <row r="35" ht="30" customHeight="1">
-      <c r="A35" s="10" t="inlineStr">
+    <row r="32" ht="34" customHeight="1">
+      <c r="A32" s="15" t="inlineStr">
+        <is>
+          <t>Accountable for the WHOLE software — every update, bug and crash. Converts product/stakeholder requirements into an architecture and tasks, assigns them, reviews every change, and decides what is safe to ship. The three developers above execute his direction and report to him.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="28" customHeight="1">
+      <c r="A33" s="10" t="inlineStr">
         <is>
           <t>Ongoing job</t>
         </is>
       </c>
-      <c r="B35" s="10" t="inlineStr">
-        <is>
-          <t>What the work actually is</t>
-        </is>
-      </c>
-      <c r="C35" s="10" t="inlineStr">
+      <c r="B33" s="10" t="inlineStr">
+        <is>
+          <t>What the work actually is (day to day)</t>
+        </is>
+      </c>
+      <c r="C33" s="10" t="inlineStr">
         <is>
           <t>Why it matters to the business</t>
         </is>
       </c>
-      <c r="D35" s="10" t="inlineStr">
+      <c r="D33" s="10" t="inlineStr">
         <is>
           <t>What it prevents</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="14" t="inlineStr">
+        <is>
+          <t>Architecture &amp; decisions</t>
+        </is>
+      </c>
+      <c r="B34" s="13" t="inlineStr">
+        <is>
+          <t>Turn each feature request into a design and an approach; decide what is built, in what order, and how it is coded.</t>
+        </is>
+      </c>
+      <c r="C34" s="13" t="inlineStr">
+        <is>
+          <t>Effort goes to the highest-value work, built the right way the first time.</t>
+        </is>
+      </c>
+      <c r="D34" s="13" t="inlineStr">
+        <is>
+          <t>Rework, wrong-priority work, and inconsistent code.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="14" t="inlineStr">
+        <is>
+          <t>Assign &amp; supervise tasks</t>
+        </is>
+      </c>
+      <c r="B35" s="13" t="inlineStr">
+        <is>
+          <t>Break the work into specific tasks for the backend, frontend and database developers and track their progress.</t>
+        </is>
+      </c>
+      <c r="C35" s="13" t="inlineStr">
+        <is>
+          <t>Everyone knows exactly what to build; nothing falls through the cracks.</t>
+        </is>
+      </c>
+      <c r="D35" s="13" t="inlineStr">
+        <is>
+          <t>Developers building in different directions.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="14" t="inlineStr">
         <is>
-          <t>Roadmap &amp; prioritisation</t>
+          <t>Review gate (production sign-off)</t>
         </is>
       </c>
       <c r="B36" s="13" t="inlineStr">
         <is>
-          <t>Decide what gets built in what order; sequence work so the biggest risk is always removed next.</t>
+          <t>Read every change. By experience, decide whether it is safe to go to production — nothing ships without his approval.</t>
         </is>
       </c>
       <c r="C36" s="13" t="inlineStr">
         <is>
-          <t>Effort always goes to the highest-value, highest-risk item first.</t>
+          <t>The single most effective catch for the silent bugs in Sheet 8.</t>
         </is>
       </c>
       <c r="D36" s="13" t="inlineStr">
         <is>
-          <t>Busywork while a real risk sits unaddressed.</t>
+          <t>A quiet bug reaching production with no experienced second pair of eyes.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="14" t="inlineStr">
         <is>
-          <t>Code review on every change</t>
+          <t>Release &amp; incident response</t>
         </is>
       </c>
       <c r="B37" s="13" t="inlineStr">
         <is>
-          <t>Be the human gate that reads every change for the silent-bug patterns in Sheet 8.</t>
+          <t>Own the CI/CD pipeline and the deploy process, and lead the response when something breaks.</t>
         </is>
       </c>
       <c r="C37" s="13" t="inlineStr">
         <is>
-          <t>The single most effective catch for the bugs that don't show an error.</t>
+          <t>Deploys are predictable and incidents are handled calmly.</t>
         </is>
       </c>
       <c r="D37" s="13" t="inlineStr">
         <is>
-          <t>A quiet bug reaching production with no second pair of eyes.</t>
+          <t>Risky deploys and slow, chaotic recovery.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="14" t="inlineStr">
         <is>
-          <t>Release &amp; incident response</t>
+          <t>Accountability &amp; security posture</t>
         </is>
       </c>
       <c r="B38" s="13" t="inlineStr">
         <is>
-          <t>Own the CI/CD pipeline, the deploy process, and the plan for when something breaks.</t>
+          <t>Carry responsibility for every update, bug and crash; schedule pen-tests and drive audit follow-ups.</t>
         </is>
       </c>
       <c r="C38" s="13" t="inlineStr">
         <is>
-          <t>Deploys are predictable and incidents are handled calmly, not in a panic.</t>
+          <t>One clear owner of quality and safety as the product grows.</t>
         </is>
       </c>
       <c r="D38" s="13" t="inlineStr">
         <is>
-          <t>Risky deploys and chaotic, slow incident recovery.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="14" t="inlineStr">
-        <is>
-          <t>Security posture</t>
-        </is>
-      </c>
-      <c r="B39" s="13" t="inlineStr">
-        <is>
-          <t>Schedule penetration tests, drive the audit follow-ups, plan a future bug-bounty.</t>
-        </is>
-      </c>
-      <c r="C39" s="13" t="inlineStr">
-        <is>
-          <t>Security stays ahead of attackers as the attack surface grows.</t>
-        </is>
-      </c>
-      <c r="D39" s="13" t="inlineStr">
-        <is>
-          <t>Security drifting as new endpoints are added faster than they're reviewed.</t>
+          <t>Diffused responsibility and security drifting as the surface grows.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="11">
     <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A5:D5"/>
     <mergeCell ref="A23:D23"/>
-    <mergeCell ref="A5:D5"/>
-    <mergeCell ref="A34:D34"/>
+    <mergeCell ref="A31:D31"/>
+    <mergeCell ref="A22:D22"/>
     <mergeCell ref="A4:D4"/>
-    <mergeCell ref="A15:D15"/>
-    <mergeCell ref="A24:D24"/>
+    <mergeCell ref="A3:D3"/>
     <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A33:D33"/>
+    <mergeCell ref="A32:D32"/>
+    <mergeCell ref="A13:D13"/>
     <mergeCell ref="A14:D14"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>